<commit_message>
Update team snapshot (2026-03-10)
</commit_message>
<xml_diff>
--- a/team_snapshot_2026.xlsx
+++ b/team_snapshot_2026.xlsx
@@ -1226,22 +1226,22 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="F7" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G7" t="b">
         <v>1</v>
       </c>
       <c r="H7" t="n">
-        <v>1291.479</v>
+        <v>1288.672</v>
       </c>
       <c r="I7" t="n">
-        <v>-2.5457</v>
+        <v>-2.4613</v>
       </c>
       <c r="J7" t="n">
-        <v>1386.1</v>
+        <v>1382</v>
       </c>
       <c r="K7" t="n">
         <v>317</v>
@@ -1262,70 +1262,70 @@
         <v>321</v>
       </c>
       <c r="Q7" t="n">
-        <v>100.633</v>
+        <v>100.336</v>
       </c>
       <c r="R7" t="n">
-        <v>109.066</v>
+        <v>109.176</v>
       </c>
       <c r="S7" t="n">
-        <v>-8.433999999999999</v>
+        <v>-8.840999999999999</v>
       </c>
       <c r="T7" t="n">
-        <v>0.3236</v>
+        <v>0.31821</v>
       </c>
       <c r="U7" t="n">
-        <v>0.17943</v>
+        <v>0.17756</v>
       </c>
       <c r="V7" t="n">
-        <v>71.64</v>
+        <v>71.45</v>
       </c>
       <c r="W7" t="n">
-        <v>77.47</v>
+        <v>77.58</v>
       </c>
       <c r="X7" t="n">
-        <v>0.2969</v>
+        <v>0.2875</v>
       </c>
       <c r="Y7" t="n">
-        <v>24.705</v>
+        <v>24.744</v>
       </c>
       <c r="Z7" t="n">
-        <v>60.055</v>
+        <v>59.856</v>
       </c>
       <c r="AA7" t="n">
-        <v>7.385</v>
+        <v>7.258</v>
       </c>
       <c r="AB7" t="n">
-        <v>23.042</v>
+        <v>22.708</v>
       </c>
       <c r="AC7" t="n">
-        <v>14.847</v>
+        <v>15.206</v>
       </c>
       <c r="AD7" t="n">
-        <v>21.022</v>
+        <v>21.407</v>
       </c>
       <c r="AE7" t="n">
-        <v>10.988</v>
+        <v>10.801</v>
       </c>
       <c r="AF7" t="n">
-        <v>22.513</v>
+        <v>22.749</v>
       </c>
       <c r="AG7" t="n">
-        <v>11.649</v>
+        <v>11.806</v>
       </c>
       <c r="AH7" t="n">
-        <v>7.945</v>
+        <v>7.936</v>
       </c>
       <c r="AI7" t="n">
-        <v>3.778</v>
+        <v>3.828</v>
       </c>
       <c r="AJ7" t="n">
-        <v>19.003</v>
+        <v>18.939</v>
       </c>
       <c r="AK7" t="n">
-        <v>-6.4</v>
+        <v>-6.6</v>
       </c>
       <c r="AL7" t="n">
-        <v>2.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -1466,22 +1466,22 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="F9" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G9" t="b">
         <v>1</v>
       </c>
       <c r="H9" t="n">
-        <v>1267.327</v>
+        <v>1270.134</v>
       </c>
       <c r="I9" t="n">
-        <v>-1.4578</v>
+        <v>-1.4276</v>
       </c>
       <c r="J9" t="n">
-        <v>1413.6</v>
+        <v>1410.3</v>
       </c>
       <c r="K9" t="n">
         <v>351</v>
@@ -1502,70 +1502,70 @@
         <v>352</v>
       </c>
       <c r="Q9" t="n">
-        <v>95.94</v>
+        <v>97.167</v>
       </c>
       <c r="R9" t="n">
-        <v>115.854</v>
+        <v>114.964</v>
       </c>
       <c r="S9" t="n">
-        <v>-19.914</v>
+        <v>-17.798</v>
       </c>
       <c r="T9" t="n">
-        <v>0.30273</v>
+        <v>0.30634</v>
       </c>
       <c r="U9" t="n">
-        <v>0.18876</v>
+        <v>0.18556</v>
       </c>
       <c r="V9" t="n">
-        <v>66.65000000000001</v>
+        <v>67.39</v>
       </c>
       <c r="W9" t="n">
-        <v>81.23</v>
+        <v>80.45999999999999</v>
       </c>
       <c r="X9" t="n">
-        <v>0.2627</v>
+        <v>0.3</v>
       </c>
       <c r="Y9" t="n">
-        <v>24.01</v>
+        <v>24.05</v>
       </c>
       <c r="Z9" t="n">
-        <v>57.149</v>
+        <v>57.477</v>
       </c>
       <c r="AA9" t="n">
-        <v>6.466</v>
+        <v>6.509</v>
       </c>
       <c r="AB9" t="n">
-        <v>19.35</v>
+        <v>19.791</v>
       </c>
       <c r="AC9" t="n">
-        <v>12.167</v>
+        <v>12.236</v>
       </c>
       <c r="AD9" t="n">
-        <v>17.263</v>
+        <v>17.391</v>
       </c>
       <c r="AE9" t="n">
-        <v>8.295999999999999</v>
+        <v>8.558999999999999</v>
       </c>
       <c r="AF9" t="n">
-        <v>19.315</v>
+        <v>19.464</v>
       </c>
       <c r="AG9" t="n">
-        <v>11.12</v>
+        <v>11.295</v>
       </c>
       <c r="AH9" t="n">
-        <v>7.755</v>
+        <v>7.686</v>
       </c>
       <c r="AI9" t="n">
-        <v>3.266</v>
+        <v>3.377</v>
       </c>
       <c r="AJ9" t="n">
-        <v>17.553</v>
+        <v>17.773</v>
       </c>
       <c r="AK9" t="n">
-        <v>-8</v>
+        <v>-9.199999999999999</v>
       </c>
       <c r="AL9" t="n">
-        <v>-6.9</v>
+        <v>-3.3</v>
       </c>
     </row>
     <row r="10">
@@ -5186,22 +5186,22 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F40" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G40" t="b">
         <v>1</v>
       </c>
       <c r="H40" t="n">
-        <v>1405.566</v>
+        <v>1402.226</v>
       </c>
       <c r="I40" t="n">
-        <v>0.1743</v>
+        <v>0.2622</v>
       </c>
       <c r="J40" t="n">
-        <v>1523.3</v>
+        <v>1518.8</v>
       </c>
       <c r="K40" t="n">
         <v>177</v>
@@ -5222,70 +5222,70 @@
         <v>192</v>
       </c>
       <c r="Q40" t="n">
-        <v>109.09</v>
+        <v>108.494</v>
       </c>
       <c r="R40" t="n">
-        <v>112.484</v>
+        <v>112.585</v>
       </c>
       <c r="S40" t="n">
-        <v>-3.395</v>
+        <v>-4.091</v>
       </c>
       <c r="T40" t="n">
-        <v>0.34056</v>
+        <v>0.33944</v>
       </c>
       <c r="U40" t="n">
-        <v>0.15989</v>
+        <v>0.16742</v>
       </c>
       <c r="V40" t="n">
-        <v>76.53</v>
+        <v>75.95</v>
       </c>
       <c r="W40" t="n">
-        <v>78.88</v>
+        <v>78.77</v>
       </c>
       <c r="X40" t="n">
-        <v>0.4569</v>
+        <v>0.4335</v>
       </c>
       <c r="Y40" t="n">
-        <v>25.681</v>
+        <v>25.57</v>
       </c>
       <c r="Z40" t="n">
-        <v>59.078</v>
+        <v>58.52</v>
       </c>
       <c r="AA40" t="n">
-        <v>6.919</v>
+        <v>6.809</v>
       </c>
       <c r="AB40" t="n">
-        <v>21.674</v>
+        <v>21.561</v>
       </c>
       <c r="AC40" t="n">
-        <v>17.406</v>
+        <v>17.323</v>
       </c>
       <c r="AD40" t="n">
-        <v>23.917</v>
+        <v>23.738</v>
       </c>
       <c r="AE40" t="n">
-        <v>10.729</v>
+        <v>10.73</v>
       </c>
       <c r="AF40" t="n">
-        <v>20.751</v>
+        <v>20.881</v>
       </c>
       <c r="AG40" t="n">
-        <v>11.288</v>
+        <v>11.199</v>
       </c>
       <c r="AH40" t="n">
-        <v>6.556</v>
+        <v>6.397</v>
       </c>
       <c r="AI40" t="n">
-        <v>1.489</v>
+        <v>1.465</v>
       </c>
       <c r="AJ40" t="n">
-        <v>18.707</v>
+        <v>18.619</v>
       </c>
       <c r="AK40" t="n">
-        <v>6.2</v>
+        <v>5.2</v>
       </c>
       <c r="AL40" t="n">
-        <v>5.1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41">
@@ -9146,22 +9146,22 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="F73" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G73" t="b">
         <v>1</v>
       </c>
       <c r="H73" t="n">
-        <v>1321.596</v>
+        <v>1327.669</v>
       </c>
       <c r="I73" t="n">
-        <v>1.5666</v>
+        <v>1.6095</v>
       </c>
       <c r="J73" t="n">
-        <v>1449.2</v>
+        <v>1453.9</v>
       </c>
       <c r="K73" t="n">
         <v>222</v>
@@ -9182,70 +9182,70 @@
         <v>229</v>
       </c>
       <c r="Q73" t="n">
-        <v>109.832</v>
+        <v>109.628</v>
       </c>
       <c r="R73" t="n">
-        <v>112.816</v>
+        <v>112.459</v>
       </c>
       <c r="S73" t="n">
-        <v>-2.984</v>
+        <v>-2.831</v>
       </c>
       <c r="T73" t="n">
-        <v>0.31172</v>
+        <v>0.31612</v>
       </c>
       <c r="U73" t="n">
-        <v>0.15656</v>
+        <v>0.16036</v>
       </c>
       <c r="V73" t="n">
-        <v>77.05</v>
+        <v>76.65000000000001</v>
       </c>
       <c r="W73" t="n">
-        <v>79.47</v>
+        <v>78.97</v>
       </c>
       <c r="X73" t="n">
-        <v>0.5062</v>
+        <v>0.5227000000000001</v>
       </c>
       <c r="Y73" t="n">
-        <v>27.319</v>
+        <v>27.182</v>
       </c>
       <c r="Z73" t="n">
-        <v>61.291</v>
+        <v>61.023</v>
       </c>
       <c r="AA73" t="n">
-        <v>6.753</v>
+        <v>6.67</v>
       </c>
       <c r="AB73" t="n">
-        <v>19.247</v>
+        <v>19.375</v>
       </c>
       <c r="AC73" t="n">
-        <v>15.66</v>
+        <v>15.341</v>
       </c>
       <c r="AD73" t="n">
-        <v>19.907</v>
+        <v>19.716</v>
       </c>
       <c r="AE73" t="n">
-        <v>10.739</v>
+        <v>10.841</v>
       </c>
       <c r="AF73" t="n">
-        <v>23.698</v>
+        <v>23.443</v>
       </c>
       <c r="AG73" t="n">
-        <v>13.199</v>
+        <v>13.295</v>
       </c>
       <c r="AH73" t="n">
-        <v>5.658</v>
+        <v>5.648</v>
       </c>
       <c r="AI73" t="n">
-        <v>3.353</v>
+        <v>3.295</v>
       </c>
       <c r="AJ73" t="n">
-        <v>19.388</v>
+        <v>19.239</v>
       </c>
       <c r="AK73" t="n">
-        <v>5</v>
+        <v>5.2</v>
       </c>
       <c r="AL73" t="n">
-        <v>4.7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="74">
@@ -10106,22 +10106,22 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="F81" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G81" t="b">
         <v>1</v>
       </c>
       <c r="H81" t="n">
-        <v>1316.019</v>
+        <v>1318.996</v>
       </c>
       <c r="I81" t="n">
-        <v>-1.332</v>
+        <v>-1.1643</v>
       </c>
       <c r="J81" t="n">
-        <v>1454.6</v>
+        <v>1451.5</v>
       </c>
       <c r="K81" t="n">
         <v>166</v>
@@ -10142,70 +10142,70 @@
         <v>201</v>
       </c>
       <c r="Q81" t="n">
-        <v>111.772</v>
+        <v>112.139</v>
       </c>
       <c r="R81" t="n">
-        <v>113.134</v>
+        <v>113.116</v>
       </c>
       <c r="S81" t="n">
-        <v>-1.362</v>
+        <v>-0.976</v>
       </c>
       <c r="T81" t="n">
-        <v>0.29233</v>
+        <v>0.29289</v>
       </c>
       <c r="U81" t="n">
         <v>0.17069</v>
       </c>
       <c r="V81" t="n">
-        <v>77.79000000000001</v>
+        <v>78.02</v>
       </c>
       <c r="W81" t="n">
-        <v>79.15000000000001</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="X81" t="n">
-        <v>0.3966</v>
+        <v>0.424</v>
       </c>
       <c r="Y81" t="n">
-        <v>27.595</v>
+        <v>27.616</v>
       </c>
       <c r="Z81" t="n">
-        <v>57.766</v>
+        <v>57.68</v>
       </c>
       <c r="AA81" t="n">
-        <v>7.289</v>
+        <v>7.368</v>
       </c>
       <c r="AB81" t="n">
-        <v>20.016</v>
+        <v>20.112</v>
       </c>
       <c r="AC81" t="n">
-        <v>15.316</v>
+        <v>15.416</v>
       </c>
       <c r="AD81" t="n">
-        <v>20.474</v>
+        <v>20.704</v>
       </c>
       <c r="AE81" t="n">
-        <v>8.967000000000001</v>
+        <v>9.007999999999999</v>
       </c>
       <c r="AF81" t="n">
-        <v>21.115</v>
+        <v>21.168</v>
       </c>
       <c r="AG81" t="n">
-        <v>13.421</v>
+        <v>13.616</v>
       </c>
       <c r="AH81" t="n">
-        <v>6.165</v>
+        <v>5.96</v>
       </c>
       <c r="AI81" t="n">
-        <v>3.532</v>
+        <v>3.408</v>
       </c>
       <c r="AJ81" t="n">
-        <v>18.108</v>
+        <v>18.216</v>
       </c>
       <c r="AK81" t="n">
-        <v>11.4</v>
+        <v>10.8</v>
       </c>
       <c r="AL81" t="n">
-        <v>9.4</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="82">
@@ -10586,22 +10586,22 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F85" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G85" t="b">
         <v>1</v>
       </c>
       <c r="H85" t="n">
-        <v>1518.466</v>
+        <v>1511.995</v>
       </c>
       <c r="I85" t="n">
-        <v>0.4929</v>
+        <v>0.4694</v>
       </c>
       <c r="J85" t="n">
-        <v>1416.5</v>
+        <v>1421.6</v>
       </c>
       <c r="K85" t="n">
         <v>147</v>
@@ -10622,70 +10622,70 @@
         <v>126</v>
       </c>
       <c r="Q85" t="n">
-        <v>116.449</v>
+        <v>115.903</v>
       </c>
       <c r="R85" t="n">
-        <v>105.528</v>
+        <v>106.335</v>
       </c>
       <c r="S85" t="n">
-        <v>10.921</v>
+        <v>9.568</v>
       </c>
       <c r="T85" t="n">
-        <v>0.26802</v>
+        <v>0.26977</v>
       </c>
       <c r="U85" t="n">
-        <v>0.14557</v>
+        <v>0.14742</v>
       </c>
       <c r="V85" t="n">
-        <v>77.23999999999999</v>
+        <v>76.67</v>
       </c>
       <c r="W85" t="n">
-        <v>69.91</v>
+        <v>70.18000000000001</v>
       </c>
       <c r="X85" t="n">
-        <v>0.6806</v>
+        <v>0.6503</v>
       </c>
       <c r="Y85" t="n">
-        <v>27.45</v>
+        <v>27.465</v>
       </c>
       <c r="Z85" t="n">
-        <v>56.367</v>
+        <v>56.283</v>
       </c>
       <c r="AA85" t="n">
-        <v>7.521</v>
+        <v>7.615</v>
       </c>
       <c r="AB85" t="n">
-        <v>21.435</v>
+        <v>21.603</v>
       </c>
       <c r="AC85" t="n">
-        <v>14.821</v>
+        <v>14.725</v>
       </c>
       <c r="AD85" t="n">
-        <v>19.722</v>
+        <v>19.521</v>
       </c>
       <c r="AE85" t="n">
-        <v>8.31</v>
+        <v>8.43</v>
       </c>
       <c r="AF85" t="n">
-        <v>22.735</v>
+        <v>22.832</v>
       </c>
       <c r="AG85" t="n">
-        <v>14.153</v>
+        <v>14.106</v>
       </c>
       <c r="AH85" t="n">
-        <v>8.606999999999999</v>
+        <v>8.428000000000001</v>
       </c>
       <c r="AI85" t="n">
-        <v>3.329</v>
+        <v>3.31</v>
       </c>
       <c r="AJ85" t="n">
-        <v>16.853</v>
+        <v>16.756</v>
       </c>
       <c r="AK85" t="n">
-        <v>2.4</v>
+        <v>-3</v>
       </c>
       <c r="AL85" t="n">
-        <v>4.4</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="86">
@@ -12026,22 +12026,22 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F97" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G97" t="b">
         <v>1</v>
       </c>
       <c r="H97" t="n">
-        <v>1536.386</v>
+        <v>1542.857</v>
       </c>
       <c r="I97" t="n">
-        <v>0.9002</v>
+        <v>0.8197</v>
       </c>
       <c r="J97" t="n">
-        <v>1417.8</v>
+        <v>1422.2</v>
       </c>
       <c r="K97" t="n">
         <v>199</v>
@@ -12062,70 +12062,70 @@
         <v>194</v>
       </c>
       <c r="Q97" t="n">
-        <v>111.677</v>
+        <v>112.011</v>
       </c>
       <c r="R97" t="n">
-        <v>107.709</v>
+        <v>107.277</v>
       </c>
       <c r="S97" t="n">
-        <v>3.968</v>
+        <v>4.734</v>
       </c>
       <c r="T97" t="n">
-        <v>0.25628</v>
+        <v>0.25616</v>
       </c>
       <c r="U97" t="n">
-        <v>0.17153</v>
+        <v>0.17102</v>
       </c>
       <c r="V97" t="n">
-        <v>75.08</v>
+        <v>75.06999999999999</v>
       </c>
       <c r="W97" t="n">
-        <v>72.55</v>
+        <v>72.06999999999999</v>
       </c>
       <c r="X97" t="n">
-        <v>0.6034</v>
+        <v>0.616</v>
       </c>
       <c r="Y97" t="n">
-        <v>26.685</v>
+        <v>26.592</v>
       </c>
       <c r="Z97" t="n">
-        <v>56.691</v>
+        <v>56.496</v>
       </c>
       <c r="AA97" t="n">
-        <v>8.802</v>
+        <v>8.568</v>
       </c>
       <c r="AB97" t="n">
-        <v>26.576</v>
+        <v>26.208</v>
       </c>
       <c r="AC97" t="n">
-        <v>12.747</v>
+        <v>12.56</v>
       </c>
       <c r="AD97" t="n">
-        <v>18.358</v>
+        <v>18.288</v>
       </c>
       <c r="AE97" t="n">
-        <v>9.007</v>
+        <v>8.912000000000001</v>
       </c>
       <c r="AF97" t="n">
-        <v>25.246</v>
+        <v>25.008</v>
       </c>
       <c r="AG97" t="n">
-        <v>15.033</v>
+        <v>14.632</v>
       </c>
       <c r="AH97" t="n">
-        <v>4.348</v>
+        <v>4.48</v>
       </c>
       <c r="AI97" t="n">
-        <v>3.33</v>
+        <v>3.28</v>
       </c>
       <c r="AJ97" t="n">
-        <v>15.572</v>
+        <v>15.472</v>
       </c>
       <c r="AK97" t="n">
-        <v>4.4</v>
+        <v>5.6</v>
       </c>
       <c r="AL97" t="n">
-        <v>1.9</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="98">
@@ -12266,22 +12266,22 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F99" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G99" t="b">
         <v>1</v>
       </c>
       <c r="H99" t="n">
-        <v>1448.4</v>
+        <v>1444.414</v>
       </c>
       <c r="I99" t="n">
-        <v>0.7301</v>
+        <v>0.7778</v>
       </c>
       <c r="J99" t="n">
-        <v>1444.4</v>
+        <v>1449.5</v>
       </c>
       <c r="K99" t="n">
         <v>230</v>
@@ -12302,70 +12302,70 @@
         <v>219</v>
       </c>
       <c r="Q99" t="n">
-        <v>111.539</v>
+        <v>111.045</v>
       </c>
       <c r="R99" t="n">
-        <v>111.349</v>
+        <v>111.873</v>
       </c>
       <c r="S99" t="n">
-        <v>0.191</v>
+        <v>-0.827</v>
       </c>
       <c r="T99" t="n">
-        <v>0.31519</v>
+        <v>0.31381</v>
       </c>
       <c r="U99" t="n">
-        <v>0.14788</v>
+        <v>0.14918</v>
       </c>
       <c r="V99" t="n">
-        <v>80.45999999999999</v>
+        <v>79.72</v>
       </c>
       <c r="W99" t="n">
-        <v>80.42</v>
+        <v>80.31</v>
       </c>
       <c r="X99" t="n">
-        <v>0.5629</v>
+        <v>0.5381</v>
       </c>
       <c r="Y99" t="n">
-        <v>26.038</v>
+        <v>25.769</v>
       </c>
       <c r="Z99" t="n">
-        <v>60.962</v>
+        <v>60.49</v>
       </c>
       <c r="AA99" t="n">
-        <v>9.417</v>
+        <v>9.359</v>
       </c>
       <c r="AB99" t="n">
-        <v>28.855</v>
+        <v>28.85</v>
       </c>
       <c r="AC99" t="n">
-        <v>17.759</v>
+        <v>17.691</v>
       </c>
       <c r="AD99" t="n">
-        <v>24.536</v>
+        <v>24.233</v>
       </c>
       <c r="AE99" t="n">
-        <v>10.155</v>
+        <v>9.956</v>
       </c>
       <c r="AF99" t="n">
-        <v>21.786</v>
+        <v>21.44</v>
       </c>
       <c r="AG99" t="n">
-        <v>10.767</v>
+        <v>10.662</v>
       </c>
       <c r="AH99" t="n">
-        <v>7.777</v>
+        <v>7.913</v>
       </c>
       <c r="AI99" t="n">
-        <v>3.33</v>
+        <v>3.312</v>
       </c>
       <c r="AJ99" t="n">
-        <v>19.503</v>
+        <v>19.342</v>
       </c>
       <c r="AK99" t="n">
-        <v>8.800000000000001</v>
+        <v>4.8</v>
       </c>
       <c r="AL99" t="n">
-        <v>4.2</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="100">
@@ -13106,22 +13106,22 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="F106" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G106" t="b">
         <v>1</v>
       </c>
       <c r="H106" t="n">
-        <v>2061.642</v>
+        <v>2063.153</v>
       </c>
       <c r="I106" t="n">
-        <v>6.7538</v>
+        <v>6.2559</v>
       </c>
       <c r="J106" t="n">
-        <v>1597.9</v>
+        <v>1593.1</v>
       </c>
       <c r="K106" t="n">
         <v>10</v>
@@ -13142,70 +13142,70 @@
         <v>5</v>
       </c>
       <c r="Q106" t="n">
-        <v>120.347</v>
+        <v>120.058</v>
       </c>
       <c r="R106" t="n">
-        <v>93.251</v>
+        <v>92.989</v>
       </c>
       <c r="S106" t="n">
-        <v>27.097</v>
+        <v>27.069</v>
       </c>
       <c r="T106" t="n">
-        <v>0.2992</v>
+        <v>0.2963</v>
       </c>
       <c r="U106" t="n">
-        <v>0.13289</v>
+        <v>0.13371</v>
       </c>
       <c r="V106" t="n">
-        <v>85.66</v>
+        <v>85.09</v>
       </c>
       <c r="W106" t="n">
-        <v>66.3</v>
+        <v>65.83</v>
       </c>
       <c r="X106" t="n">
-        <v>0.8928</v>
+        <v>0.9073</v>
       </c>
       <c r="Y106" t="n">
-        <v>32.586</v>
+        <v>32.388</v>
       </c>
       <c r="Z106" t="n">
-        <v>63.971</v>
+        <v>63.603</v>
       </c>
       <c r="AA106" t="n">
-        <v>6.658</v>
+        <v>6.524</v>
       </c>
       <c r="AB106" t="n">
-        <v>19.614</v>
+        <v>19.41</v>
       </c>
       <c r="AC106" t="n">
-        <v>13.826</v>
+        <v>13.793</v>
       </c>
       <c r="AD106" t="n">
-        <v>19.748</v>
+        <v>19.554</v>
       </c>
       <c r="AE106" t="n">
-        <v>11.017</v>
+        <v>10.895</v>
       </c>
       <c r="AF106" t="n">
-        <v>25.919</v>
+        <v>25.96</v>
       </c>
       <c r="AG106" t="n">
-        <v>18.133</v>
+        <v>18.144</v>
       </c>
       <c r="AH106" t="n">
-        <v>8.587999999999999</v>
+        <v>8.648999999999999</v>
       </c>
       <c r="AI106" t="n">
-        <v>3.681</v>
+        <v>3.691</v>
       </c>
       <c r="AJ106" t="n">
-        <v>17.148</v>
+        <v>17.03</v>
       </c>
       <c r="AK106" t="n">
-        <v>13.6</v>
+        <v>13.8</v>
       </c>
       <c r="AL106" t="n">
-        <v>12.1</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="107">
@@ -13226,22 +13226,22 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="F107" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G107" t="b">
         <v>1</v>
       </c>
       <c r="H107" t="n">
-        <v>1310.866</v>
+        <v>1312.041</v>
       </c>
       <c r="I107" t="n">
-        <v>-0.5341</v>
+        <v>-0.5671</v>
       </c>
       <c r="J107" t="n">
-        <v>1363.2</v>
+        <v>1352.3</v>
       </c>
       <c r="K107" t="n">
         <v>298</v>
@@ -13262,70 +13262,70 @@
         <v>301</v>
       </c>
       <c r="Q107" t="n">
-        <v>99.773</v>
+        <v>100.56</v>
       </c>
       <c r="R107" t="n">
-        <v>104.045</v>
+        <v>103.092</v>
       </c>
       <c r="S107" t="n">
-        <v>-4.273</v>
+        <v>-2.532</v>
       </c>
       <c r="T107" t="n">
-        <v>0.29712</v>
+        <v>0.29737</v>
       </c>
       <c r="U107" t="n">
-        <v>0.20505</v>
+        <v>0.20438</v>
       </c>
       <c r="V107" t="n">
-        <v>68.84999999999999</v>
+        <v>69.25</v>
       </c>
       <c r="W107" t="n">
-        <v>71.93000000000001</v>
+        <v>71.16</v>
       </c>
       <c r="X107" t="n">
-        <v>0.3864</v>
+        <v>0.4063</v>
       </c>
       <c r="Y107" t="n">
-        <v>23.091</v>
+        <v>23.142</v>
       </c>
       <c r="Z107" t="n">
-        <v>54.205</v>
+        <v>54.142</v>
       </c>
       <c r="AA107" t="n">
-        <v>6.466</v>
+        <v>6.766</v>
       </c>
       <c r="AB107" t="n">
-        <v>20.83</v>
+        <v>20.867</v>
       </c>
       <c r="AC107" t="n">
-        <v>16.205</v>
+        <v>16.198</v>
       </c>
       <c r="AD107" t="n">
-        <v>22.136</v>
+        <v>22.252</v>
       </c>
       <c r="AE107" t="n">
-        <v>9.034000000000001</v>
+        <v>9.087</v>
       </c>
       <c r="AF107" t="n">
-        <v>21.341</v>
+        <v>21.438</v>
       </c>
       <c r="AG107" t="n">
-        <v>11.83</v>
+        <v>11.999</v>
       </c>
       <c r="AH107" t="n">
-        <v>7.693</v>
+        <v>7.627</v>
       </c>
       <c r="AI107" t="n">
-        <v>2.614</v>
+        <v>2.681</v>
       </c>
       <c r="AJ107" t="n">
-        <v>18.875</v>
+        <v>18.814</v>
       </c>
       <c r="AK107" t="n">
-        <v>-0.6</v>
+        <v>0.2</v>
       </c>
       <c r="AL107" t="n">
-        <v>-2.3</v>
+        <v>-0.8</v>
       </c>
     </row>
     <row r="108">
@@ -13946,22 +13946,22 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F113" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G113" t="b">
         <v>1</v>
       </c>
       <c r="H113" t="n">
-        <v>1574.472</v>
+        <v>1582.041</v>
       </c>
       <c r="I113" t="n">
-        <v>3.7174</v>
+        <v>3.5064</v>
       </c>
       <c r="J113" t="n">
-        <v>1481.7</v>
+        <v>1484.4</v>
       </c>
       <c r="K113" t="n">
         <v>84</v>
@@ -13982,70 +13982,70 @@
         <v>88</v>
       </c>
       <c r="Q113" t="n">
-        <v>113.985</v>
+        <v>113.542</v>
       </c>
       <c r="R113" t="n">
-        <v>102.458</v>
+        <v>102.659</v>
       </c>
       <c r="S113" t="n">
-        <v>11.527</v>
+        <v>10.883</v>
       </c>
       <c r="T113" t="n">
-        <v>0.30387</v>
+        <v>0.30742</v>
       </c>
       <c r="U113" t="n">
-        <v>0.15122</v>
+        <v>0.15226</v>
       </c>
       <c r="V113" t="n">
-        <v>74.88</v>
+        <v>74.42</v>
       </c>
       <c r="W113" t="n">
-        <v>67.53</v>
+        <v>67.48999999999999</v>
       </c>
       <c r="X113" t="n">
-        <v>0.6702</v>
+        <v>0.6806</v>
       </c>
       <c r="Y113" t="n">
-        <v>25.559</v>
+        <v>25.469</v>
       </c>
       <c r="Z113" t="n">
-        <v>58.273</v>
+        <v>58.432</v>
       </c>
       <c r="AA113" t="n">
-        <v>9.382</v>
+        <v>9.403</v>
       </c>
       <c r="AB113" t="n">
-        <v>25.247</v>
+        <v>25.336</v>
       </c>
       <c r="AC113" t="n">
-        <v>14.381</v>
+        <v>14.079</v>
       </c>
       <c r="AD113" t="n">
-        <v>19.049</v>
+        <v>18.603</v>
       </c>
       <c r="AE113" t="n">
-        <v>10.69</v>
+        <v>10.857</v>
       </c>
       <c r="AF113" t="n">
-        <v>24.373</v>
+        <v>24.31</v>
       </c>
       <c r="AG113" t="n">
-        <v>12.495</v>
+        <v>12.354</v>
       </c>
       <c r="AH113" t="n">
-        <v>4.813</v>
+        <v>4.683</v>
       </c>
       <c r="AI113" t="n">
-        <v>3.694</v>
+        <v>3.619</v>
       </c>
       <c r="AJ113" t="n">
-        <v>17.678</v>
+        <v>17.45</v>
       </c>
       <c r="AK113" t="n">
-        <v>20.2</v>
+        <v>13.6</v>
       </c>
       <c r="AL113" t="n">
-        <v>15.6</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="114">
@@ -21626,22 +21626,22 @@
         </is>
       </c>
       <c r="E177" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F177" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G177" t="b">
         <v>1</v>
       </c>
       <c r="H177" t="n">
-        <v>1447.398</v>
+        <v>1450.738</v>
       </c>
       <c r="I177" t="n">
-        <v>1.1918</v>
+        <v>1.2494</v>
       </c>
       <c r="J177" t="n">
-        <v>1458.5</v>
+        <v>1456.7</v>
       </c>
       <c r="K177" t="n">
         <v>181</v>
@@ -21662,70 +21662,70 @@
         <v>169</v>
       </c>
       <c r="Q177" t="n">
-        <v>106.485</v>
+        <v>106.718</v>
       </c>
       <c r="R177" t="n">
-        <v>105.001</v>
+        <v>104.796</v>
       </c>
       <c r="S177" t="n">
-        <v>1.484</v>
+        <v>1.922</v>
       </c>
       <c r="T177" t="n">
-        <v>0.30647</v>
+        <v>0.31254</v>
       </c>
       <c r="U177" t="n">
-        <v>0.16555</v>
+        <v>0.16263</v>
       </c>
       <c r="V177" t="n">
-        <v>71.93000000000001</v>
+        <v>72.08</v>
       </c>
       <c r="W177" t="n">
-        <v>70.90000000000001</v>
+        <v>70.75</v>
       </c>
       <c r="X177" t="n">
-        <v>0.5528</v>
+        <v>0.5665</v>
       </c>
       <c r="Y177" t="n">
-        <v>25.46</v>
+        <v>25.465</v>
       </c>
       <c r="Z177" t="n">
-        <v>58.114</v>
+        <v>58.266</v>
       </c>
       <c r="AA177" t="n">
-        <v>6.949</v>
+        <v>6.809</v>
       </c>
       <c r="AB177" t="n">
-        <v>19.939</v>
+        <v>19.889</v>
       </c>
       <c r="AC177" t="n">
-        <v>14.064</v>
+        <v>14.342</v>
       </c>
       <c r="AD177" t="n">
-        <v>18.831</v>
+        <v>19.045</v>
       </c>
       <c r="AE177" t="n">
-        <v>10.076</v>
+        <v>10.133</v>
       </c>
       <c r="AF177" t="n">
-        <v>22.592</v>
+        <v>22.206</v>
       </c>
       <c r="AG177" t="n">
-        <v>13.843</v>
+        <v>13.756</v>
       </c>
       <c r="AH177" t="n">
-        <v>7.508</v>
+        <v>7.705</v>
       </c>
       <c r="AI177" t="n">
-        <v>4.442</v>
+        <v>4.252</v>
       </c>
       <c r="AJ177" t="n">
-        <v>15.917</v>
+        <v>15.898</v>
       </c>
       <c r="AK177" t="n">
-        <v>6.4</v>
+        <v>10.6</v>
       </c>
       <c r="AL177" t="n">
-        <v>2.8</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="178">
@@ -21746,22 +21746,22 @@
         </is>
       </c>
       <c r="E178" t="n">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="F178" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G178" t="b">
         <v>1</v>
       </c>
       <c r="H178" t="n">
-        <v>1458.848</v>
+        <v>1464.637</v>
       </c>
       <c r="I178" t="n">
-        <v>-1.7046</v>
+        <v>-1.6217</v>
       </c>
       <c r="J178" t="n">
-        <v>1432.7</v>
+        <v>1434.8</v>
       </c>
       <c r="K178" t="n">
         <v>187</v>
@@ -21782,70 +21782,70 @@
         <v>199</v>
       </c>
       <c r="Q178" t="n">
-        <v>106.424</v>
+        <v>107.791</v>
       </c>
       <c r="R178" t="n">
-        <v>109.34</v>
+        <v>109.828</v>
       </c>
       <c r="S178" t="n">
-        <v>-2.916</v>
+        <v>-2.037</v>
       </c>
       <c r="T178" t="n">
-        <v>0.18347</v>
+        <v>0.18463</v>
       </c>
       <c r="U178" t="n">
-        <v>0.19261</v>
+        <v>0.18961</v>
       </c>
       <c r="V178" t="n">
-        <v>75.17</v>
+        <v>76.26000000000001</v>
       </c>
       <c r="W178" t="n">
-        <v>77.45</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="X178" t="n">
-        <v>0.4762</v>
+        <v>0.5051</v>
       </c>
       <c r="Y178" t="n">
-        <v>26.04</v>
+        <v>26.298</v>
       </c>
       <c r="Z178" t="n">
-        <v>54.212</v>
+        <v>54.323</v>
       </c>
       <c r="AA178" t="n">
-        <v>8.223000000000001</v>
+        <v>8.247</v>
       </c>
       <c r="AB178" t="n">
-        <v>22.476</v>
+        <v>22.414</v>
       </c>
       <c r="AC178" t="n">
-        <v>14.864</v>
+        <v>15.419</v>
       </c>
       <c r="AD178" t="n">
-        <v>19.267</v>
+        <v>19.854</v>
       </c>
       <c r="AE178" t="n">
-        <v>5.502</v>
+        <v>5.586</v>
       </c>
       <c r="AF178" t="n">
-        <v>24.604</v>
+        <v>24.758</v>
       </c>
       <c r="AG178" t="n">
-        <v>14.81</v>
+        <v>14.677</v>
       </c>
       <c r="AH178" t="n">
-        <v>5.601</v>
+        <v>5.465</v>
       </c>
       <c r="AI178" t="n">
-        <v>2.498</v>
+        <v>2.414</v>
       </c>
       <c r="AJ178" t="n">
-        <v>17.498</v>
+        <v>17.52</v>
       </c>
       <c r="AK178" t="n">
-        <v>-7.6</v>
+        <v>-5.6</v>
       </c>
       <c r="AL178" t="n">
-        <v>-5.5</v>
+        <v>-5.3</v>
       </c>
     </row>
     <row r="179">
@@ -22226,22 +22226,22 @@
         </is>
       </c>
       <c r="E182" t="n">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="F182" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G182" t="b">
         <v>1</v>
       </c>
       <c r="H182" t="n">
-        <v>1094.905</v>
+        <v>1093.731</v>
       </c>
       <c r="I182" t="n">
-        <v>-2.9612</v>
+        <v>-2.8469</v>
       </c>
       <c r="J182" t="n">
-        <v>1372.9</v>
+        <v>1371.1</v>
       </c>
       <c r="K182" t="n">
         <v>365</v>
@@ -22262,70 +22262,70 @@
         <v>365</v>
       </c>
       <c r="Q182" t="n">
-        <v>91.205</v>
+        <v>90.483</v>
       </c>
       <c r="R182" t="n">
-        <v>119.189</v>
+        <v>119.095</v>
       </c>
       <c r="S182" t="n">
-        <v>-27.984</v>
+        <v>-28.613</v>
       </c>
       <c r="T182" t="n">
-        <v>0.28556</v>
+        <v>0.291</v>
       </c>
       <c r="U182" t="n">
-        <v>0.20728</v>
+        <v>0.2104</v>
       </c>
       <c r="V182" t="n">
-        <v>63.74</v>
+        <v>63.1</v>
       </c>
       <c r="W182" t="n">
-        <v>83.92</v>
+        <v>83.62</v>
       </c>
       <c r="X182" t="n">
-        <v>0.0638</v>
+        <v>0.0618</v>
       </c>
       <c r="Y182" t="n">
-        <v>22.606</v>
+        <v>22.421</v>
       </c>
       <c r="Z182" t="n">
-        <v>55.116</v>
+        <v>55.122</v>
       </c>
       <c r="AA182" t="n">
-        <v>4.951</v>
+        <v>4.907</v>
       </c>
       <c r="AB182" t="n">
-        <v>16.725</v>
+        <v>16.638</v>
       </c>
       <c r="AC182" t="n">
-        <v>13.574</v>
+        <v>13.349</v>
       </c>
       <c r="AD182" t="n">
-        <v>18.872</v>
+        <v>18.669</v>
       </c>
       <c r="AE182" t="n">
-        <v>7.91</v>
+        <v>8.177</v>
       </c>
       <c r="AF182" t="n">
-        <v>19.672</v>
+        <v>19.743</v>
       </c>
       <c r="AG182" t="n">
-        <v>11.843</v>
+        <v>11.898</v>
       </c>
       <c r="AH182" t="n">
-        <v>6.922</v>
+        <v>7.094</v>
       </c>
       <c r="AI182" t="n">
-        <v>2.554</v>
+        <v>2.567</v>
       </c>
       <c r="AJ182" t="n">
-        <v>21.838</v>
+        <v>21.503</v>
       </c>
       <c r="AK182" t="n">
-        <v>-6</v>
+        <v>-11.2</v>
       </c>
       <c r="AL182" t="n">
-        <v>-10.8</v>
+        <v>-11.7</v>
       </c>
     </row>
     <row r="183">
@@ -22706,22 +22706,22 @@
         </is>
       </c>
       <c r="E186" t="n">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="F186" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G186" t="b">
         <v>1</v>
       </c>
       <c r="H186" t="n">
-        <v>1492.824</v>
+        <v>1487.034</v>
       </c>
       <c r="I186" t="n">
-        <v>-2.3144</v>
+        <v>-2.1857</v>
       </c>
       <c r="J186" t="n">
-        <v>1399.2</v>
+        <v>1401.2</v>
       </c>
       <c r="K186" t="n">
         <v>136</v>
@@ -22742,70 +22742,70 @@
         <v>139</v>
       </c>
       <c r="Q186" t="n">
-        <v>112.556</v>
+        <v>112.831</v>
       </c>
       <c r="R186" t="n">
-        <v>107.837</v>
+        <v>108.911</v>
       </c>
       <c r="S186" t="n">
-        <v>4.718</v>
+        <v>3.92</v>
       </c>
       <c r="T186" t="n">
-        <v>0.22</v>
+        <v>0.22488</v>
       </c>
       <c r="U186" t="n">
-        <v>0.15335</v>
+        <v>0.14965</v>
       </c>
       <c r="V186" t="n">
-        <v>80.56999999999999</v>
+        <v>80.89</v>
       </c>
       <c r="W186" t="n">
-        <v>77.3</v>
+        <v>78.19</v>
       </c>
       <c r="X186" t="n">
-        <v>0.6103</v>
+        <v>0.5818</v>
       </c>
       <c r="Y186" t="n">
-        <v>29.564</v>
+        <v>29.638</v>
       </c>
       <c r="Z186" t="n">
-        <v>60.8</v>
+        <v>61.177</v>
       </c>
       <c r="AA186" t="n">
-        <v>8.91</v>
+        <v>8.856</v>
       </c>
       <c r="AB186" t="n">
-        <v>25.359</v>
+        <v>25.35</v>
       </c>
       <c r="AC186" t="n">
-        <v>12.535</v>
+        <v>12.756</v>
       </c>
       <c r="AD186" t="n">
-        <v>16.519</v>
+        <v>16.839</v>
       </c>
       <c r="AE186" t="n">
-        <v>7.382</v>
+        <v>7.543</v>
       </c>
       <c r="AF186" t="n">
-        <v>26.108</v>
+        <v>25.909</v>
       </c>
       <c r="AG186" t="n">
-        <v>15.815</v>
+        <v>15.787</v>
       </c>
       <c r="AH186" t="n">
-        <v>4.084</v>
+        <v>3.993</v>
       </c>
       <c r="AI186" t="n">
-        <v>2.795</v>
+        <v>2.711</v>
       </c>
       <c r="AJ186" t="n">
-        <v>18.448</v>
+        <v>18.521</v>
       </c>
       <c r="AK186" t="n">
-        <v>8</v>
+        <v>4.4</v>
       </c>
       <c r="AL186" t="n">
-        <v>8.9</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="187">
@@ -23066,22 +23066,22 @@
         </is>
       </c>
       <c r="E189" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F189" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G189" t="b">
         <v>1</v>
       </c>
       <c r="H189" t="n">
-        <v>1439.016</v>
+        <v>1434.798</v>
       </c>
       <c r="I189" t="n">
-        <v>0.2239</v>
+        <v>0.1976</v>
       </c>
       <c r="J189" t="n">
-        <v>1427.9</v>
+        <v>1429.8</v>
       </c>
       <c r="K189" t="n">
         <v>172</v>
@@ -23102,70 +23102,70 @@
         <v>178</v>
       </c>
       <c r="Q189" t="n">
-        <v>113.32</v>
+        <v>113.17</v>
       </c>
       <c r="R189" t="n">
-        <v>108.95</v>
+        <v>109.867</v>
       </c>
       <c r="S189" t="n">
-        <v>4.37</v>
+        <v>3.303</v>
       </c>
       <c r="T189" t="n">
-        <v>0.31536</v>
+        <v>0.32037</v>
       </c>
       <c r="U189" t="n">
-        <v>0.15936</v>
+        <v>0.16094</v>
       </c>
       <c r="V189" t="n">
-        <v>80.73</v>
+        <v>80.98</v>
       </c>
       <c r="W189" t="n">
-        <v>77.84999999999999</v>
+        <v>78.87</v>
       </c>
       <c r="X189" t="n">
-        <v>0.5704</v>
+        <v>0.544</v>
       </c>
       <c r="Y189" t="n">
-        <v>27.694</v>
+        <v>27.752</v>
       </c>
       <c r="Z189" t="n">
-        <v>60.534</v>
+        <v>60.736</v>
       </c>
       <c r="AA189" t="n">
-        <v>8.858000000000001</v>
+        <v>8.904</v>
       </c>
       <c r="AB189" t="n">
-        <v>27.02</v>
+        <v>26.968</v>
       </c>
       <c r="AC189" t="n">
-        <v>15.654</v>
+        <v>15.928</v>
       </c>
       <c r="AD189" t="n">
-        <v>21.578</v>
+        <v>21.936</v>
       </c>
       <c r="AE189" t="n">
-        <v>9.891</v>
+        <v>10.136</v>
       </c>
       <c r="AF189" t="n">
-        <v>21.553</v>
+        <v>21.544</v>
       </c>
       <c r="AG189" t="n">
-        <v>15.356</v>
+        <v>15.36</v>
       </c>
       <c r="AH189" t="n">
-        <v>8.170999999999999</v>
+        <v>8.144</v>
       </c>
       <c r="AI189" t="n">
-        <v>3.562</v>
+        <v>3.584</v>
       </c>
       <c r="AJ189" t="n">
-        <v>18.511</v>
+        <v>18.712</v>
       </c>
       <c r="AK189" t="n">
-        <v>5</v>
+        <v>3.6</v>
       </c>
       <c r="AL189" t="n">
-        <v>3.5</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="190">
@@ -24386,22 +24386,22 @@
         </is>
       </c>
       <c r="E200" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F200" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G200" t="b">
         <v>1</v>
       </c>
       <c r="H200" t="n">
-        <v>1341.993</v>
+        <v>1339.625</v>
       </c>
       <c r="I200" t="n">
-        <v>0.5805</v>
+        <v>0.6274</v>
       </c>
       <c r="J200" t="n">
-        <v>1453</v>
+        <v>1451.6</v>
       </c>
       <c r="K200" t="n">
         <v>182</v>
@@ -24422,70 +24422,70 @@
         <v>208</v>
       </c>
       <c r="Q200" t="n">
-        <v>106.165</v>
+        <v>106.272</v>
       </c>
       <c r="R200" t="n">
-        <v>110.071</v>
+        <v>111.114</v>
       </c>
       <c r="S200" t="n">
-        <v>-3.906</v>
+        <v>-4.843</v>
       </c>
       <c r="T200" t="n">
-        <v>0.29265</v>
+        <v>0.30559</v>
       </c>
       <c r="U200" t="n">
-        <v>0.19673</v>
+        <v>0.1946</v>
       </c>
       <c r="V200" t="n">
-        <v>74.92</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="W200" t="n">
-        <v>77.62</v>
+        <v>77.64</v>
       </c>
       <c r="X200" t="n">
-        <v>0.4735</v>
+        <v>0.4507</v>
       </c>
       <c r="Y200" t="n">
-        <v>24.876</v>
+        <v>24.611</v>
       </c>
       <c r="Z200" t="n">
-        <v>55.805</v>
+        <v>55.704</v>
       </c>
       <c r="AA200" t="n">
-        <v>6.022</v>
+        <v>5.953</v>
       </c>
       <c r="AB200" t="n">
-        <v>18.689</v>
+        <v>18.798</v>
       </c>
       <c r="AC200" t="n">
-        <v>19.146</v>
+        <v>19.227</v>
       </c>
       <c r="AD200" t="n">
-        <v>25.73</v>
+        <v>25.883</v>
       </c>
       <c r="AE200" t="n">
-        <v>10.35</v>
+        <v>10.638</v>
       </c>
       <c r="AF200" t="n">
-        <v>24.846</v>
+        <v>24.251</v>
       </c>
       <c r="AG200" t="n">
-        <v>13.031</v>
+        <v>12.915</v>
       </c>
       <c r="AH200" t="n">
-        <v>5.69</v>
+        <v>5.815</v>
       </c>
       <c r="AI200" t="n">
-        <v>3.805</v>
+        <v>3.743</v>
       </c>
       <c r="AJ200" t="n">
-        <v>19.712</v>
+        <v>19.576</v>
       </c>
       <c r="AK200" t="n">
-        <v>3.2</v>
+        <v>-0.6</v>
       </c>
       <c r="AL200" t="n">
-        <v>2.5</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="201">
@@ -24626,22 +24626,22 @@
         </is>
       </c>
       <c r="E202" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F202" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G202" t="b">
         <v>1</v>
       </c>
       <c r="H202" t="n">
-        <v>1364.252</v>
+        <v>1361.859</v>
       </c>
       <c r="I202" t="n">
-        <v>-1.4633</v>
+        <v>-1.4014</v>
       </c>
       <c r="J202" t="n">
-        <v>1425.9</v>
+        <v>1426</v>
       </c>
       <c r="K202" t="n">
         <v>232</v>
@@ -24662,70 +24662,70 @@
         <v>246</v>
       </c>
       <c r="Q202" t="n">
-        <v>104.332</v>
+        <v>104.281</v>
       </c>
       <c r="R202" t="n">
-        <v>109.702</v>
+        <v>110.789</v>
       </c>
       <c r="S202" t="n">
-        <v>-5.371</v>
+        <v>-6.508</v>
       </c>
       <c r="T202" t="n">
-        <v>0.32196</v>
+        <v>0.32388</v>
       </c>
       <c r="U202" t="n">
-        <v>0.16798</v>
+        <v>0.16939</v>
       </c>
       <c r="V202" t="n">
-        <v>70.97</v>
+        <v>70.94</v>
       </c>
       <c r="W202" t="n">
-        <v>75.08</v>
+        <v>75.78</v>
       </c>
       <c r="X202" t="n">
-        <v>0.425</v>
+        <v>0.4026</v>
       </c>
       <c r="Y202" t="n">
-        <v>24.808</v>
+        <v>24.774</v>
       </c>
       <c r="Z202" t="n">
-        <v>57.236</v>
+        <v>57.168</v>
       </c>
       <c r="AA202" t="n">
-        <v>8.417999999999999</v>
+        <v>8.314</v>
       </c>
       <c r="AB202" t="n">
-        <v>25.197</v>
+        <v>25.048</v>
       </c>
       <c r="AC202" t="n">
-        <v>12.932</v>
+        <v>13.08</v>
       </c>
       <c r="AD202" t="n">
-        <v>19.711</v>
+        <v>19.694</v>
       </c>
       <c r="AE202" t="n">
-        <v>9.179</v>
+        <v>9.195</v>
       </c>
       <c r="AF202" t="n">
-        <v>19.262</v>
+        <v>19.137</v>
       </c>
       <c r="AG202" t="n">
-        <v>12.987</v>
+        <v>12.889</v>
       </c>
       <c r="AH202" t="n">
-        <v>8.699999999999999</v>
+        <v>8.65</v>
       </c>
       <c r="AI202" t="n">
-        <v>2.796</v>
+        <v>2.743</v>
       </c>
       <c r="AJ202" t="n">
-        <v>18.067</v>
+        <v>17.973</v>
       </c>
       <c r="AK202" t="n">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="AL202" t="n">
-        <v>-1</v>
+        <v>-3.1</v>
       </c>
     </row>
     <row r="203">
@@ -27146,22 +27146,22 @@
         </is>
       </c>
       <c r="E223" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F223" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G223" t="b">
         <v>1</v>
       </c>
       <c r="H223" t="n">
-        <v>1551.535</v>
+        <v>1550.024</v>
       </c>
       <c r="I223" t="n">
-        <v>-2.8876</v>
+        <v>-2.6712</v>
       </c>
       <c r="J223" t="n">
-        <v>1538.2</v>
+        <v>1558.8</v>
       </c>
       <c r="K223" t="n">
         <v>179</v>
@@ -27182,70 +27182,70 @@
         <v>171</v>
       </c>
       <c r="Q223" t="n">
-        <v>107.333</v>
+        <v>106.457</v>
       </c>
       <c r="R223" t="n">
-        <v>111.753</v>
+        <v>111.328</v>
       </c>
       <c r="S223" t="n">
-        <v>-4.42</v>
+        <v>-4.871</v>
       </c>
       <c r="T223" t="n">
-        <v>0.24647</v>
+        <v>0.24935</v>
       </c>
       <c r="U223" t="n">
-        <v>0.17043</v>
+        <v>0.17074</v>
       </c>
       <c r="V223" t="n">
-        <v>71.66</v>
+        <v>70.97</v>
       </c>
       <c r="W223" t="n">
-        <v>74.47</v>
+        <v>74.06</v>
       </c>
       <c r="X223" t="n">
-        <v>0.5363</v>
+        <v>0.51</v>
       </c>
       <c r="Y223" t="n">
-        <v>22.785</v>
+        <v>22.6</v>
       </c>
       <c r="Z223" t="n">
-        <v>52.929</v>
+        <v>53.03</v>
       </c>
       <c r="AA223" t="n">
-        <v>8.31</v>
+        <v>8.19</v>
       </c>
       <c r="AB223" t="n">
-        <v>23.413</v>
+        <v>23.47</v>
       </c>
       <c r="AC223" t="n">
-        <v>17.782</v>
+        <v>17.58</v>
       </c>
       <c r="AD223" t="n">
-        <v>23.028</v>
+        <v>22.77</v>
       </c>
       <c r="AE223" t="n">
-        <v>7.558</v>
+        <v>7.67</v>
       </c>
       <c r="AF223" t="n">
-        <v>22.907</v>
+        <v>22.87</v>
       </c>
       <c r="AG223" t="n">
-        <v>14.012</v>
+        <v>13.81</v>
       </c>
       <c r="AH223" t="n">
-        <v>5.566</v>
+        <v>5.49</v>
       </c>
       <c r="AI223" t="n">
-        <v>3.681</v>
+        <v>3.67</v>
       </c>
       <c r="AJ223" t="n">
-        <v>17.835</v>
+        <v>17.73</v>
       </c>
       <c r="AK223" t="n">
-        <v>-2</v>
+        <v>-1.8</v>
       </c>
       <c r="AL223" t="n">
-        <v>1.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="224">
@@ -29426,22 +29426,22 @@
         </is>
       </c>
       <c r="E242" t="n">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="F242" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G242" t="b">
         <v>1</v>
       </c>
       <c r="H242" t="n">
-        <v>1538.807</v>
+        <v>1532.735</v>
       </c>
       <c r="I242" t="n">
-        <v>-1.3441</v>
+        <v>-1.224</v>
       </c>
       <c r="J242" t="n">
-        <v>1429.2</v>
+        <v>1424.9</v>
       </c>
       <c r="K242" t="n">
         <v>139</v>
@@ -29462,70 +29462,70 @@
         <v>135</v>
       </c>
       <c r="Q242" t="n">
-        <v>115.297</v>
+        <v>114.922</v>
       </c>
       <c r="R242" t="n">
-        <v>108.919</v>
+        <v>109.407</v>
       </c>
       <c r="S242" t="n">
-        <v>6.378</v>
+        <v>5.514</v>
       </c>
       <c r="T242" t="n">
-        <v>0.33378</v>
+        <v>0.33745</v>
       </c>
       <c r="U242" t="n">
-        <v>0.17483</v>
+        <v>0.1723</v>
       </c>
       <c r="V242" t="n">
-        <v>77.14</v>
+        <v>76.68000000000001</v>
       </c>
       <c r="W242" t="n">
-        <v>73.28</v>
+        <v>73.34999999999999</v>
       </c>
       <c r="X242" t="n">
-        <v>0.6702</v>
+        <v>0.6389</v>
       </c>
       <c r="Y242" t="n">
-        <v>28.1</v>
+        <v>27.961</v>
       </c>
       <c r="Z242" t="n">
-        <v>59.52</v>
+        <v>59.492</v>
       </c>
       <c r="AA242" t="n">
-        <v>9.34</v>
+        <v>9.153</v>
       </c>
       <c r="AB242" t="n">
-        <v>24.232</v>
+        <v>23.881</v>
       </c>
       <c r="AC242" t="n">
-        <v>11.595</v>
+        <v>11.857</v>
       </c>
       <c r="AD242" t="n">
-        <v>16.628</v>
+        <v>16.889</v>
       </c>
       <c r="AE242" t="n">
-        <v>11.505</v>
+        <v>11.604</v>
       </c>
       <c r="AF242" t="n">
-        <v>23.426</v>
+        <v>23.226</v>
       </c>
       <c r="AG242" t="n">
-        <v>17.661</v>
+        <v>17.379</v>
       </c>
       <c r="AH242" t="n">
-        <v>5.549</v>
+        <v>5.678</v>
       </c>
       <c r="AI242" t="n">
-        <v>2.483</v>
+        <v>2.447</v>
       </c>
       <c r="AJ242" t="n">
-        <v>18.234</v>
+        <v>18.204</v>
       </c>
       <c r="AK242" t="n">
-        <v>16.4</v>
+        <v>10.4</v>
       </c>
       <c r="AL242" t="n">
-        <v>11.5</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="243">
@@ -30986,22 +30986,22 @@
         </is>
       </c>
       <c r="E255" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F255" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G255" t="b">
         <v>1</v>
       </c>
       <c r="H255" t="n">
-        <v>1768.33</v>
+        <v>1787.889</v>
       </c>
       <c r="I255" t="n">
-        <v>-0.4727</v>
+        <v>-0.2548</v>
       </c>
       <c r="J255" t="n">
-        <v>1566.6</v>
+        <v>1580.2</v>
       </c>
       <c r="K255" t="n">
         <v>37</v>
@@ -31022,70 +31022,70 @@
         <v>42</v>
       </c>
       <c r="Q255" t="n">
-        <v>117.67</v>
+        <v>117.903</v>
       </c>
       <c r="R255" t="n">
-        <v>102.695</v>
+        <v>103.181</v>
       </c>
       <c r="S255" t="n">
-        <v>14.975</v>
+        <v>14.722</v>
       </c>
       <c r="T255" t="n">
-        <v>0.34723</v>
+        <v>0.34454</v>
       </c>
       <c r="U255" t="n">
-        <v>0.14938</v>
+        <v>0.15002</v>
       </c>
       <c r="V255" t="n">
-        <v>83.47</v>
+        <v>83.25</v>
       </c>
       <c r="W255" t="n">
-        <v>72.86</v>
+        <v>72.83</v>
       </c>
       <c r="X255" t="n">
-        <v>0.7764</v>
+        <v>0.7832</v>
       </c>
       <c r="Y255" t="n">
-        <v>30.322</v>
+        <v>30.101</v>
       </c>
       <c r="Z255" t="n">
-        <v>64.524</v>
+        <v>64.126</v>
       </c>
       <c r="AA255" t="n">
-        <v>10.176</v>
+        <v>9.964</v>
       </c>
       <c r="AB255" t="n">
-        <v>29.068</v>
+        <v>28.64</v>
       </c>
       <c r="AC255" t="n">
-        <v>12.654</v>
+        <v>12.881</v>
       </c>
       <c r="AD255" t="n">
-        <v>16.932</v>
+        <v>17.08</v>
       </c>
       <c r="AE255" t="n">
-        <v>11.656</v>
+        <v>11.628</v>
       </c>
       <c r="AF255" t="n">
-        <v>21.319</v>
+        <v>21.59</v>
       </c>
       <c r="AG255" t="n">
-        <v>16.943</v>
+        <v>16.747</v>
       </c>
       <c r="AH255" t="n">
-        <v>8.919</v>
+        <v>8.648999999999999</v>
       </c>
       <c r="AI255" t="n">
-        <v>3.703</v>
+        <v>3.721</v>
       </c>
       <c r="AJ255" t="n">
-        <v>19.539</v>
+        <v>19.468</v>
       </c>
       <c r="AK255" t="n">
-        <v>4.6</v>
+        <v>7.2</v>
       </c>
       <c r="AL255" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="256">
@@ -33506,22 +33506,22 @@
         </is>
       </c>
       <c r="E276" t="n">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="F276" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G276" t="b">
         <v>1</v>
       </c>
       <c r="H276" t="n">
-        <v>1877.369</v>
+        <v>1857.81</v>
       </c>
       <c r="I276" t="n">
-        <v>-0.5286</v>
+        <v>-0.2818</v>
       </c>
       <c r="J276" t="n">
-        <v>1595.3</v>
+        <v>1596.9</v>
       </c>
       <c r="K276" t="n">
         <v>22</v>
@@ -33542,70 +33542,70 @@
         <v>20</v>
       </c>
       <c r="Q276" t="n">
-        <v>118.867</v>
+        <v>118.734</v>
       </c>
       <c r="R276" t="n">
-        <v>98.821</v>
+        <v>99.88200000000001</v>
       </c>
       <c r="S276" t="n">
-        <v>20.046</v>
+        <v>18.852</v>
       </c>
       <c r="T276" t="n">
-        <v>0.29664</v>
+        <v>0.2975</v>
       </c>
       <c r="U276" t="n">
-        <v>0.15573</v>
+        <v>0.15247</v>
       </c>
       <c r="V276" t="n">
-        <v>77.73999999999999</v>
+        <v>77.54000000000001</v>
       </c>
       <c r="W276" t="n">
-        <v>64.86</v>
+        <v>65.41</v>
       </c>
       <c r="X276" t="n">
-        <v>0.8683</v>
+        <v>0.829</v>
       </c>
       <c r="Y276" t="n">
-        <v>26.489</v>
+        <v>26.684</v>
       </c>
       <c r="Z276" t="n">
-        <v>57.738</v>
+        <v>57.823</v>
       </c>
       <c r="AA276" t="n">
-        <v>8.166</v>
+        <v>8.194000000000001</v>
       </c>
       <c r="AB276" t="n">
-        <v>20.92</v>
+        <v>20.951</v>
       </c>
       <c r="AC276" t="n">
-        <v>16.591</v>
+        <v>16.191</v>
       </c>
       <c r="AD276" t="n">
-        <v>20.545</v>
+        <v>20.377</v>
       </c>
       <c r="AE276" t="n">
-        <v>11.478</v>
+        <v>11.371</v>
       </c>
       <c r="AF276" t="n">
-        <v>26.44</v>
+        <v>26.154</v>
       </c>
       <c r="AG276" t="n">
-        <v>15.428</v>
+        <v>15.241</v>
       </c>
       <c r="AH276" t="n">
-        <v>5.625</v>
+        <v>5.562</v>
       </c>
       <c r="AI276" t="n">
-        <v>3.572</v>
+        <v>3.586</v>
       </c>
       <c r="AJ276" t="n">
-        <v>15.502</v>
+        <v>15.771</v>
       </c>
       <c r="AK276" t="n">
-        <v>11.8</v>
+        <v>8.6</v>
       </c>
       <c r="AL276" t="n">
-        <v>13.7</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="277">
@@ -34226,22 +34226,22 @@
         </is>
       </c>
       <c r="E282" t="n">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="F282" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G282" t="b">
         <v>1</v>
       </c>
       <c r="H282" t="n">
-        <v>1376.177</v>
+        <v>1378.544</v>
       </c>
       <c r="I282" t="n">
-        <v>-0.451</v>
+        <v>-0.4106</v>
       </c>
       <c r="J282" t="n">
-        <v>1426.5</v>
+        <v>1424</v>
       </c>
       <c r="K282" t="n">
         <v>180</v>
@@ -34262,70 +34262,70 @@
         <v>196</v>
       </c>
       <c r="Q282" t="n">
-        <v>102.165</v>
+        <v>103.004</v>
       </c>
       <c r="R282" t="n">
-        <v>103.54</v>
+        <v>103.532</v>
       </c>
       <c r="S282" t="n">
-        <v>-1.375</v>
+        <v>-0.528</v>
       </c>
       <c r="T282" t="n">
-        <v>0.29116</v>
+        <v>0.29593</v>
       </c>
       <c r="U282" t="n">
-        <v>0.18053</v>
+        <v>0.18515</v>
       </c>
       <c r="V282" t="n">
-        <v>68.84</v>
+        <v>68.93000000000001</v>
       </c>
       <c r="W282" t="n">
-        <v>70.05</v>
+        <v>69.64</v>
       </c>
       <c r="X282" t="n">
-        <v>0.486</v>
+        <v>0.504</v>
       </c>
       <c r="Y282" t="n">
-        <v>23.759</v>
+        <v>23.89</v>
       </c>
       <c r="Z282" t="n">
-        <v>54.512</v>
+        <v>54.417</v>
       </c>
       <c r="AA282" t="n">
-        <v>5.76</v>
+        <v>5.926</v>
       </c>
       <c r="AB282" t="n">
-        <v>17.007</v>
+        <v>17.052</v>
       </c>
       <c r="AC282" t="n">
-        <v>15.559</v>
+        <v>15.227</v>
       </c>
       <c r="AD282" t="n">
-        <v>23.01</v>
+        <v>22.601</v>
       </c>
       <c r="AE282" t="n">
-        <v>9.182</v>
+        <v>9.49</v>
       </c>
       <c r="AF282" t="n">
-        <v>21.678</v>
+        <v>21.768</v>
       </c>
       <c r="AG282" t="n">
-        <v>11.871</v>
+        <v>12.032</v>
       </c>
       <c r="AH282" t="n">
-        <v>7.21</v>
+        <v>7.09</v>
       </c>
       <c r="AI282" t="n">
-        <v>2.642</v>
+        <v>2.646</v>
       </c>
       <c r="AJ282" t="n">
-        <v>20.708</v>
+        <v>20.882</v>
       </c>
       <c r="AK282" t="n">
-        <v>0.8</v>
+        <v>5.4</v>
       </c>
       <c r="AL282" t="n">
-        <v>1.8</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="283">
@@ -35666,22 +35666,22 @@
         </is>
       </c>
       <c r="E294" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F294" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G294" t="b">
         <v>1</v>
       </c>
       <c r="H294" t="n">
-        <v>1556.938</v>
+        <v>1549.369</v>
       </c>
       <c r="I294" t="n">
-        <v>-2.7806</v>
+        <v>-2.6439</v>
       </c>
       <c r="J294" t="n">
-        <v>1524.4</v>
+        <v>1525.9</v>
       </c>
       <c r="K294" t="n">
         <v>157</v>
@@ -35702,70 +35702,70 @@
         <v>160</v>
       </c>
       <c r="Q294" t="n">
-        <v>104.063</v>
+        <v>103.887</v>
       </c>
       <c r="R294" t="n">
-        <v>102.391</v>
+        <v>102.852</v>
       </c>
       <c r="S294" t="n">
-        <v>1.672</v>
+        <v>1.034</v>
       </c>
       <c r="T294" t="n">
-        <v>0.33571</v>
+        <v>0.33827</v>
       </c>
       <c r="U294" t="n">
-        <v>0.15173</v>
+        <v>0.14979</v>
       </c>
       <c r="V294" t="n">
-        <v>67.26000000000001</v>
+        <v>67.04000000000001</v>
       </c>
       <c r="W294" t="n">
-        <v>66.29000000000001</v>
+        <v>66.45</v>
       </c>
       <c r="X294" t="n">
-        <v>0.5528</v>
+        <v>0.5265</v>
       </c>
       <c r="Y294" t="n">
-        <v>24.044</v>
+        <v>24.022</v>
       </c>
       <c r="Z294" t="n">
-        <v>58.428</v>
+        <v>58.594</v>
       </c>
       <c r="AA294" t="n">
-        <v>5.811</v>
+        <v>5.805</v>
       </c>
       <c r="AB294" t="n">
-        <v>20.69</v>
+        <v>20.49</v>
       </c>
       <c r="AC294" t="n">
-        <v>12.322</v>
+        <v>12.421</v>
       </c>
       <c r="AD294" t="n">
-        <v>18.182</v>
+        <v>18.186</v>
       </c>
       <c r="AE294" t="n">
-        <v>11.543</v>
+        <v>11.686</v>
       </c>
       <c r="AF294" t="n">
-        <v>23.028</v>
+        <v>23.013</v>
       </c>
       <c r="AG294" t="n">
-        <v>9.592000000000001</v>
+        <v>9.406000000000001</v>
       </c>
       <c r="AH294" t="n">
-        <v>5.801</v>
+        <v>5.725</v>
       </c>
       <c r="AI294" t="n">
-        <v>3.403</v>
+        <v>3.412</v>
       </c>
       <c r="AJ294" t="n">
-        <v>15.949</v>
+        <v>15.889</v>
       </c>
       <c r="AK294" t="n">
-        <v>9.800000000000001</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="AL294" t="n">
-        <v>6.4</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="295">
@@ -35786,22 +35786,22 @@
         </is>
       </c>
       <c r="E295" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F295" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G295" t="b">
         <v>1</v>
       </c>
       <c r="H295" t="n">
-        <v>1596.975</v>
+        <v>1600.961</v>
       </c>
       <c r="I295" t="n">
-        <v>1.2134</v>
+        <v>1.1284</v>
       </c>
       <c r="J295" t="n">
-        <v>1466.1</v>
+        <v>1466</v>
       </c>
       <c r="K295" t="n">
         <v>153</v>
@@ -35822,70 +35822,70 @@
         <v>132</v>
       </c>
       <c r="Q295" t="n">
-        <v>111.849</v>
+        <v>112.278</v>
       </c>
       <c r="R295" t="n">
-        <v>106.582</v>
+        <v>106.193</v>
       </c>
       <c r="S295" t="n">
-        <v>5.267</v>
+        <v>6.085</v>
       </c>
       <c r="T295" t="n">
-        <v>0.31634</v>
+        <v>0.316</v>
       </c>
       <c r="U295" t="n">
-        <v>0.16365</v>
+        <v>0.16673</v>
       </c>
       <c r="V295" t="n">
-        <v>78.33</v>
+        <v>78.27</v>
       </c>
       <c r="W295" t="n">
-        <v>74.86</v>
+        <v>74.3</v>
       </c>
       <c r="X295" t="n">
-        <v>0.6388</v>
+        <v>0.65</v>
       </c>
       <c r="Y295" t="n">
-        <v>26.401</v>
+        <v>26.627</v>
       </c>
       <c r="Z295" t="n">
-        <v>60.115</v>
+        <v>59.845</v>
       </c>
       <c r="AA295" t="n">
-        <v>9.108000000000001</v>
+        <v>9.009</v>
       </c>
       <c r="AB295" t="n">
-        <v>27.509</v>
+        <v>27.182</v>
       </c>
       <c r="AC295" t="n">
-        <v>16.419</v>
+        <v>16.009</v>
       </c>
       <c r="AD295" t="n">
-        <v>22.171</v>
+        <v>21.709</v>
       </c>
       <c r="AE295" t="n">
-        <v>11.194</v>
+        <v>11.159</v>
       </c>
       <c r="AF295" t="n">
-        <v>24.062</v>
+        <v>24.032</v>
       </c>
       <c r="AG295" t="n">
-        <v>15.054</v>
+        <v>15.186</v>
       </c>
       <c r="AH295" t="n">
-        <v>7.278</v>
+        <v>7.255</v>
       </c>
       <c r="AI295" t="n">
-        <v>3.567</v>
+        <v>3.341</v>
       </c>
       <c r="AJ295" t="n">
-        <v>16.865</v>
+        <v>16.75</v>
       </c>
       <c r="AK295" t="n">
-        <v>6.4</v>
+        <v>9.4</v>
       </c>
       <c r="AL295" t="n">
-        <v>1.5</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="296">
@@ -36146,22 +36146,22 @@
         </is>
       </c>
       <c r="E298" t="n">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="F298" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G298" t="b">
         <v>1</v>
       </c>
       <c r="H298" t="n">
-        <v>1394.986</v>
+        <v>1397.379</v>
       </c>
       <c r="I298" t="n">
-        <v>1.606</v>
+        <v>1.648</v>
       </c>
       <c r="J298" t="n">
-        <v>1426.5</v>
+        <v>1425</v>
       </c>
       <c r="K298" t="n">
         <v>124</v>
@@ -36182,70 +36182,70 @@
         <v>134</v>
       </c>
       <c r="Q298" t="n">
-        <v>109.771</v>
+        <v>110.546</v>
       </c>
       <c r="R298" t="n">
-        <v>105.084</v>
+        <v>105.058</v>
       </c>
       <c r="S298" t="n">
-        <v>4.687</v>
+        <v>5.488</v>
       </c>
       <c r="T298" t="n">
-        <v>0.24194</v>
+        <v>0.23978</v>
       </c>
       <c r="U298" t="n">
-        <v>0.17004</v>
+        <v>0.17131</v>
       </c>
       <c r="V298" t="n">
-        <v>73.11</v>
+        <v>73.62</v>
       </c>
       <c r="W298" t="n">
-        <v>70.18000000000001</v>
+        <v>70.15000000000001</v>
       </c>
       <c r="X298" t="n">
-        <v>0.5551</v>
+        <v>0.5697</v>
       </c>
       <c r="Y298" t="n">
-        <v>26.057</v>
+        <v>26.233</v>
       </c>
       <c r="Z298" t="n">
-        <v>56.057</v>
+        <v>55.913</v>
       </c>
       <c r="AA298" t="n">
-        <v>8.863</v>
+        <v>8.988</v>
       </c>
       <c r="AB298" t="n">
-        <v>24.301</v>
+        <v>24.298</v>
       </c>
       <c r="AC298" t="n">
-        <v>12.134</v>
+        <v>12.166</v>
       </c>
       <c r="AD298" t="n">
-        <v>16.058</v>
+        <v>15.939</v>
       </c>
       <c r="AE298" t="n">
-        <v>7.89</v>
+        <v>7.781</v>
       </c>
       <c r="AF298" t="n">
-        <v>23.418</v>
+        <v>23.357</v>
       </c>
       <c r="AG298" t="n">
-        <v>15.624</v>
+        <v>15.796</v>
       </c>
       <c r="AH298" t="n">
-        <v>5.871</v>
+        <v>5.868</v>
       </c>
       <c r="AI298" t="n">
-        <v>2.787</v>
+        <v>2.801</v>
       </c>
       <c r="AJ298" t="n">
-        <v>18.315</v>
+        <v>18.218</v>
       </c>
       <c r="AK298" t="n">
-        <v>7.8</v>
+        <v>10.4</v>
       </c>
       <c r="AL298" t="n">
-        <v>9.9</v>
+        <v>10.4</v>
       </c>
     </row>
     <row r="299">
@@ -40706,22 +40706,22 @@
         </is>
       </c>
       <c r="E336" t="n">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="F336" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G336" t="b">
         <v>1</v>
       </c>
       <c r="H336" t="n">
-        <v>1362.868</v>
+        <v>1359.891</v>
       </c>
       <c r="I336" t="n">
-        <v>-0.0298</v>
+        <v>-0.0016</v>
       </c>
       <c r="J336" t="n">
-        <v>1423.8</v>
+        <v>1419</v>
       </c>
       <c r="K336" t="n">
         <v>193</v>
@@ -40742,70 +40742,70 @@
         <v>197</v>
       </c>
       <c r="Q336" t="n">
-        <v>111.294</v>
+        <v>111.687</v>
       </c>
       <c r="R336" t="n">
-        <v>111.437</v>
+        <v>111.82</v>
       </c>
       <c r="S336" t="n">
-        <v>-0.143</v>
+        <v>-0.132</v>
       </c>
       <c r="T336" t="n">
-        <v>0.3076</v>
+        <v>0.30496</v>
       </c>
       <c r="U336" t="n">
-        <v>0.15521</v>
+        <v>0.15381</v>
       </c>
       <c r="V336" t="n">
-        <v>78.65000000000001</v>
+        <v>78.83</v>
       </c>
       <c r="W336" t="n">
-        <v>78.94</v>
+        <v>79.11</v>
       </c>
       <c r="X336" t="n">
-        <v>0.4783</v>
+        <v>0.4626</v>
       </c>
       <c r="Y336" t="n">
-        <v>27.484</v>
+        <v>27.496</v>
       </c>
       <c r="Z336" t="n">
-        <v>59.916</v>
+        <v>59.734</v>
       </c>
       <c r="AA336" t="n">
-        <v>6.811</v>
+        <v>6.751</v>
       </c>
       <c r="AB336" t="n">
-        <v>19.634</v>
+        <v>19.595</v>
       </c>
       <c r="AC336" t="n">
-        <v>16.873</v>
+        <v>17.092</v>
       </c>
       <c r="AD336" t="n">
-        <v>23.264</v>
+        <v>23.405</v>
       </c>
       <c r="AE336" t="n">
-        <v>10.248</v>
+        <v>10.106</v>
       </c>
       <c r="AF336" t="n">
-        <v>23.332</v>
+        <v>23.247</v>
       </c>
       <c r="AG336" t="n">
-        <v>12.783</v>
+        <v>12.585</v>
       </c>
       <c r="AH336" t="n">
-        <v>6.947</v>
+        <v>6.925</v>
       </c>
       <c r="AI336" t="n">
-        <v>1.503</v>
+        <v>1.537</v>
       </c>
       <c r="AJ336" t="n">
-        <v>18.339</v>
+        <v>18.697</v>
       </c>
       <c r="AK336" t="n">
-        <v>-1.8</v>
+        <v>0.8</v>
       </c>
       <c r="AL336" t="n">
-        <v>-0.5</v>
+        <v>-1.2</v>
       </c>
     </row>
     <row r="337">
@@ -41786,22 +41786,22 @@
         </is>
       </c>
       <c r="E345" t="n">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="F345" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G345" t="b">
         <v>1</v>
       </c>
       <c r="H345" t="n">
-        <v>1464.47</v>
+        <v>1468.688</v>
       </c>
       <c r="I345" t="n">
-        <v>2.7711</v>
+        <v>2.7502</v>
       </c>
       <c r="J345" t="n">
-        <v>1435.1</v>
+        <v>1435.9</v>
       </c>
       <c r="K345" t="n">
         <v>144</v>
@@ -41822,70 +41822,70 @@
         <v>133</v>
       </c>
       <c r="Q345" t="n">
-        <v>115.653</v>
+        <v>116.218</v>
       </c>
       <c r="R345" t="n">
-        <v>109.069</v>
+        <v>109.523</v>
       </c>
       <c r="S345" t="n">
-        <v>6.584</v>
+        <v>6.695</v>
       </c>
       <c r="T345" t="n">
-        <v>0.29919</v>
+        <v>0.29519</v>
       </c>
       <c r="U345" t="n">
-        <v>0.15797</v>
+        <v>0.15692</v>
       </c>
       <c r="V345" t="n">
-        <v>79.76000000000001</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="W345" t="n">
-        <v>75.20999999999999</v>
+        <v>75.92</v>
       </c>
       <c r="X345" t="n">
-        <v>0.6365</v>
+        <v>0.648</v>
       </c>
       <c r="Y345" t="n">
-        <v>28.241</v>
+        <v>28.392</v>
       </c>
       <c r="Z345" t="n">
-        <v>58.315</v>
+        <v>58.328</v>
       </c>
       <c r="AA345" t="n">
-        <v>7.106</v>
+        <v>7.208</v>
       </c>
       <c r="AB345" t="n">
-        <v>19.626</v>
+        <v>19.72</v>
       </c>
       <c r="AC345" t="n">
-        <v>16.167</v>
+        <v>16.608</v>
       </c>
       <c r="AD345" t="n">
-        <v>21.695</v>
+        <v>22.12</v>
       </c>
       <c r="AE345" t="n">
-        <v>9.753</v>
+        <v>9.584</v>
       </c>
       <c r="AF345" t="n">
-        <v>22.384</v>
+        <v>22.408</v>
       </c>
       <c r="AG345" t="n">
-        <v>13.224</v>
+        <v>13.352</v>
       </c>
       <c r="AH345" t="n">
-        <v>7.073</v>
+        <v>7.216</v>
       </c>
       <c r="AI345" t="n">
-        <v>4.322</v>
+        <v>4.32</v>
       </c>
       <c r="AJ345" t="n">
-        <v>17.289</v>
+        <v>17.528</v>
       </c>
       <c r="AK345" t="n">
-        <v>6.6</v>
+        <v>6.8</v>
       </c>
       <c r="AL345" t="n">
-        <v>4.9</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="346">

</xml_diff>

<commit_message>
Update team snapshot (2026-03-16)
</commit_message>
<xml_diff>
--- a/team_snapshot_2026.xlsx
+++ b/team_snapshot_2026.xlsx
@@ -2306,22 +2306,22 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F16" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G16" t="b">
         <v>1</v>
       </c>
       <c r="H16" t="n">
-        <v>1961.738</v>
+        <v>1977.002</v>
       </c>
       <c r="I16" t="n">
-        <v>5.2535</v>
+        <v>5.1479</v>
       </c>
       <c r="J16" t="n">
-        <v>1726.7</v>
+        <v>1736</v>
       </c>
       <c r="K16" t="n">
         <v>18</v>
@@ -2342,70 +2342,70 @@
         <v>18</v>
       </c>
       <c r="Q16" t="n">
-        <v>122.845</v>
+        <v>122.871</v>
       </c>
       <c r="R16" t="n">
-        <v>109.473</v>
+        <v>109.332</v>
       </c>
       <c r="S16" t="n">
-        <v>13.372</v>
+        <v>13.539</v>
       </c>
       <c r="T16" t="n">
-        <v>0.30449</v>
+        <v>0.29787</v>
       </c>
       <c r="U16" t="n">
-        <v>0.11969</v>
+        <v>0.12058</v>
       </c>
       <c r="V16" t="n">
-        <v>90.09</v>
+        <v>89.91</v>
       </c>
       <c r="W16" t="n">
-        <v>80.31999999999999</v>
+        <v>80.05</v>
       </c>
       <c r="X16" t="n">
-        <v>0.7596000000000001</v>
+        <v>0.7665999999999999</v>
       </c>
       <c r="Y16" t="n">
-        <v>32.15</v>
+        <v>32.072</v>
       </c>
       <c r="Z16" t="n">
-        <v>64.40300000000001</v>
+        <v>64.128</v>
       </c>
       <c r="AA16" t="n">
-        <v>8.103</v>
+        <v>8.375999999999999</v>
       </c>
       <c r="AB16" t="n">
-        <v>21.314</v>
+        <v>21.432</v>
       </c>
       <c r="AC16" t="n">
-        <v>17.681</v>
+        <v>17.391</v>
       </c>
       <c r="AD16" t="n">
-        <v>23.668</v>
+        <v>23.287</v>
       </c>
       <c r="AE16" t="n">
-        <v>10.231</v>
+        <v>9.99</v>
       </c>
       <c r="AF16" t="n">
-        <v>23.343</v>
+        <v>23.588</v>
       </c>
       <c r="AG16" t="n">
-        <v>16.863</v>
+        <v>17.031</v>
       </c>
       <c r="AH16" t="n">
-        <v>7.377</v>
+        <v>7.239</v>
       </c>
       <c r="AI16" t="n">
-        <v>5.087</v>
+        <v>5.117</v>
       </c>
       <c r="AJ16" t="n">
-        <v>16.971</v>
+        <v>16.881</v>
       </c>
       <c r="AK16" t="n">
-        <v>-0.8</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="AL16" t="n">
-        <v>5.9</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="17">
@@ -8546,22 +8546,22 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F68" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G68" t="b">
         <v>1</v>
       </c>
       <c r="H68" t="n">
-        <v>1688.075</v>
+        <v>1677.744</v>
       </c>
       <c r="I68" t="n">
-        <v>-2.1851</v>
+        <v>-1.9174</v>
       </c>
       <c r="J68" t="n">
-        <v>1570.2</v>
+        <v>1574.7</v>
       </c>
       <c r="K68" t="n">
         <v>79</v>
@@ -8582,70 +8582,70 @@
         <v>75</v>
       </c>
       <c r="Q68" t="n">
-        <v>109.548</v>
+        <v>109.173</v>
       </c>
       <c r="R68" t="n">
-        <v>101.885</v>
+        <v>102.25</v>
       </c>
       <c r="S68" t="n">
-        <v>7.662</v>
+        <v>6.923</v>
       </c>
       <c r="T68" t="n">
-        <v>0.25276</v>
+        <v>0.25145</v>
       </c>
       <c r="U68" t="n">
-        <v>0.1736</v>
+        <v>0.17261</v>
       </c>
       <c r="V68" t="n">
-        <v>74.67</v>
+        <v>74.22</v>
       </c>
       <c r="W68" t="n">
-        <v>69.87</v>
+        <v>69.88</v>
       </c>
       <c r="X68" t="n">
-        <v>0.7005</v>
+        <v>0.6691</v>
       </c>
       <c r="Y68" t="n">
-        <v>24.007</v>
+        <v>23.989</v>
       </c>
       <c r="Z68" t="n">
-        <v>53.456</v>
+        <v>53.465</v>
       </c>
       <c r="AA68" t="n">
-        <v>7.694</v>
+        <v>7.64</v>
       </c>
       <c r="AB68" t="n">
-        <v>22.46</v>
+        <v>22.338</v>
       </c>
       <c r="AC68" t="n">
-        <v>18.923</v>
+        <v>18.571</v>
       </c>
       <c r="AD68" t="n">
-        <v>25.026</v>
+        <v>24.796</v>
       </c>
       <c r="AE68" t="n">
-        <v>7.928</v>
+        <v>7.942</v>
       </c>
       <c r="AF68" t="n">
-        <v>22.969</v>
+        <v>23.233</v>
       </c>
       <c r="AG68" t="n">
-        <v>14.341</v>
+        <v>14.4</v>
       </c>
       <c r="AH68" t="n">
-        <v>8.311999999999999</v>
+        <v>8.148999999999999</v>
       </c>
       <c r="AI68" t="n">
-        <v>4.173</v>
+        <v>4.145</v>
       </c>
       <c r="AJ68" t="n">
-        <v>16.891</v>
+        <v>16.865</v>
       </c>
       <c r="AK68" t="n">
-        <v>1.4</v>
+        <v>-0.6</v>
       </c>
       <c r="AL68" t="n">
-        <v>3.4</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="69">
@@ -20666,22 +20666,22 @@
         </is>
       </c>
       <c r="E169" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F169" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G169" t="b">
         <v>1</v>
       </c>
       <c r="H169" t="n">
-        <v>2196.807</v>
+        <v>2173.708</v>
       </c>
       <c r="I169" t="n">
-        <v>6.739</v>
+        <v>6.5185</v>
       </c>
       <c r="J169" t="n">
-        <v>1772.9</v>
+        <v>1779.9</v>
       </c>
       <c r="K169" t="n">
         <v>2</v>
@@ -20702,70 +20702,70 @@
         <v>2</v>
       </c>
       <c r="Q169" t="n">
-        <v>120.645</v>
+        <v>120.66</v>
       </c>
       <c r="R169" t="n">
-        <v>95.937</v>
+        <v>97.182</v>
       </c>
       <c r="S169" t="n">
-        <v>24.707</v>
+        <v>23.477</v>
       </c>
       <c r="T169" t="n">
-        <v>0.26043</v>
+        <v>0.25981</v>
       </c>
       <c r="U169" t="n">
-        <v>0.16661</v>
+        <v>0.1613</v>
       </c>
       <c r="V169" t="n">
-        <v>87.11</v>
+        <v>86.70999999999999</v>
       </c>
       <c r="W169" t="n">
-        <v>68.84999999999999</v>
+        <v>69.29000000000001</v>
       </c>
       <c r="X169" t="n">
-        <v>0.9399</v>
+        <v>0.9046</v>
       </c>
       <c r="Y169" t="n">
-        <v>30.379</v>
+        <v>30.409</v>
       </c>
       <c r="Z169" t="n">
-        <v>60.043</v>
+        <v>59.947</v>
       </c>
       <c r="AA169" t="n">
-        <v>9.112</v>
+        <v>8.932</v>
       </c>
       <c r="AB169" t="n">
-        <v>25.18</v>
+        <v>24.768</v>
       </c>
       <c r="AC169" t="n">
-        <v>17.242</v>
+        <v>17.255</v>
       </c>
       <c r="AD169" t="n">
-        <v>23.088</v>
+        <v>23.138</v>
       </c>
       <c r="AE169" t="n">
-        <v>10.03</v>
+        <v>9.917999999999999</v>
       </c>
       <c r="AF169" t="n">
-        <v>28.197</v>
+        <v>27.953</v>
       </c>
       <c r="AG169" t="n">
-        <v>18.529</v>
+        <v>18.666</v>
       </c>
       <c r="AH169" t="n">
-        <v>5.811</v>
+        <v>5.751</v>
       </c>
       <c r="AI169" t="n">
-        <v>5.987</v>
+        <v>5.934</v>
       </c>
       <c r="AJ169" t="n">
-        <v>15.482</v>
+        <v>15.451</v>
       </c>
       <c r="AK169" t="n">
-        <v>6.8</v>
+        <v>2.4</v>
       </c>
       <c r="AL169" t="n">
-        <v>9.199999999999999</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="170">
@@ -27386,22 +27386,22 @@
         </is>
       </c>
       <c r="E225" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F225" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G225" t="b">
         <v>1</v>
       </c>
       <c r="H225" t="n">
-        <v>1431.706</v>
+        <v>1458.418</v>
       </c>
       <c r="I225" t="n">
-        <v>1.1135</v>
+        <v>1.2024</v>
       </c>
       <c r="J225" t="n">
-        <v>1482.7</v>
+        <v>1493.7</v>
       </c>
       <c r="K225" t="n">
         <v>163</v>
@@ -27422,70 +27422,70 @@
         <v>148</v>
       </c>
       <c r="Q225" t="n">
-        <v>107.489</v>
+        <v>108.543</v>
       </c>
       <c r="R225" t="n">
-        <v>105.825</v>
+        <v>106.705</v>
       </c>
       <c r="S225" t="n">
-        <v>1.663</v>
+        <v>1.838</v>
       </c>
       <c r="T225" t="n">
-        <v>0.30844</v>
+        <v>0.31426</v>
       </c>
       <c r="U225" t="n">
-        <v>0.15432</v>
+        <v>0.15185</v>
       </c>
       <c r="V225" t="n">
-        <v>73.91</v>
+        <v>74.73999999999999</v>
       </c>
       <c r="W225" t="n">
-        <v>72.79000000000001</v>
+        <v>73.48999999999999</v>
       </c>
       <c r="X225" t="n">
-        <v>0.5981</v>
+        <v>0.612</v>
       </c>
       <c r="Y225" t="n">
-        <v>25.84</v>
+        <v>26.097</v>
       </c>
       <c r="Z225" t="n">
-        <v>59.369</v>
+        <v>59.889</v>
       </c>
       <c r="AA225" t="n">
-        <v>7.89</v>
+        <v>7.942</v>
       </c>
       <c r="AB225" t="n">
-        <v>21.135</v>
+        <v>21.143</v>
       </c>
       <c r="AC225" t="n">
-        <v>14.24</v>
+        <v>14.34</v>
       </c>
       <c r="AD225" t="n">
-        <v>20.671</v>
+        <v>20.739</v>
       </c>
       <c r="AE225" t="n">
-        <v>10.306</v>
+        <v>10.616</v>
       </c>
       <c r="AF225" t="n">
-        <v>23.427</v>
+        <v>23.33</v>
       </c>
       <c r="AG225" t="n">
-        <v>13.662</v>
+        <v>14.076</v>
       </c>
       <c r="AH225" t="n">
-        <v>6.435</v>
+        <v>6.601</v>
       </c>
       <c r="AI225" t="n">
-        <v>3.223</v>
+        <v>3.224</v>
       </c>
       <c r="AJ225" t="n">
-        <v>16.763</v>
+        <v>16.776</v>
       </c>
       <c r="AK225" t="n">
-        <v>6.2</v>
+        <v>7.8</v>
       </c>
       <c r="AL225" t="n">
-        <v>5.2</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="226">
@@ -28586,22 +28586,22 @@
         </is>
       </c>
       <c r="E235" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F235" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G235" t="b">
         <v>1</v>
       </c>
       <c r="H235" t="n">
-        <v>1986.929</v>
+        <v>2010.028</v>
       </c>
       <c r="I235" t="n">
-        <v>-0.5973000000000001</v>
+        <v>-0.7024</v>
       </c>
       <c r="J235" t="n">
-        <v>1754.6</v>
+        <v>1769.7</v>
       </c>
       <c r="K235" t="n">
         <v>8</v>
@@ -28622,70 +28622,70 @@
         <v>10</v>
       </c>
       <c r="Q235" t="n">
-        <v>124.757</v>
+        <v>124.873</v>
       </c>
       <c r="R235" t="n">
-        <v>107.247</v>
+        <v>107.488</v>
       </c>
       <c r="S235" t="n">
-        <v>17.51</v>
+        <v>17.385</v>
       </c>
       <c r="T235" t="n">
-        <v>0.31049</v>
+        <v>0.31102</v>
       </c>
       <c r="U235" t="n">
-        <v>0.13425</v>
+        <v>0.13371</v>
       </c>
       <c r="V235" t="n">
-        <v>81.62</v>
+        <v>81.64</v>
       </c>
       <c r="W235" t="n">
-        <v>70.05</v>
+        <v>70.16</v>
       </c>
       <c r="X235" t="n">
-        <v>0.7669</v>
+        <v>0.7734</v>
       </c>
       <c r="Y235" t="n">
-        <v>29.662</v>
+        <v>29.717</v>
       </c>
       <c r="Z235" t="n">
-        <v>59.914</v>
+        <v>60.092</v>
       </c>
       <c r="AA235" t="n">
-        <v>9.331</v>
+        <v>9.266</v>
       </c>
       <c r="AB235" t="n">
-        <v>24.516</v>
+        <v>24.538</v>
       </c>
       <c r="AC235" t="n">
-        <v>12.234</v>
+        <v>11.996</v>
       </c>
       <c r="AD235" t="n">
-        <v>16.536</v>
+        <v>16.196</v>
       </c>
       <c r="AE235" t="n">
-        <v>10.515</v>
+        <v>10.547</v>
       </c>
       <c r="AF235" t="n">
-        <v>22.944</v>
+        <v>22.963</v>
       </c>
       <c r="AG235" t="n">
-        <v>19.632</v>
+        <v>19.475</v>
       </c>
       <c r="AH235" t="n">
-        <v>5.64</v>
+        <v>5.484</v>
       </c>
       <c r="AI235" t="n">
-        <v>2.632</v>
+        <v>2.66</v>
       </c>
       <c r="AJ235" t="n">
-        <v>14.883</v>
+        <v>14.998</v>
       </c>
       <c r="AK235" t="n">
-        <v>7.2</v>
+        <v>8</v>
       </c>
       <c r="AL235" t="n">
-        <v>6.5</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="236">
@@ -32426,22 +32426,22 @@
         </is>
       </c>
       <c r="E267" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F267" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G267" t="b">
         <v>1</v>
       </c>
       <c r="H267" t="n">
-        <v>1714.878</v>
+        <v>1723.482</v>
       </c>
       <c r="I267" t="n">
-        <v>9.035</v>
+        <v>8.857799999999999</v>
       </c>
       <c r="J267" t="n">
-        <v>1550.3</v>
+        <v>1554.8</v>
       </c>
       <c r="K267" t="n">
         <v>51</v>
@@ -32462,70 +32462,70 @@
         <v>49</v>
       </c>
       <c r="Q267" t="n">
-        <v>116.325</v>
+        <v>115.66</v>
       </c>
       <c r="R267" t="n">
-        <v>101.484</v>
+        <v>100.714</v>
       </c>
       <c r="S267" t="n">
-        <v>14.84</v>
+        <v>14.946</v>
       </c>
       <c r="T267" t="n">
-        <v>0.34115</v>
+        <v>0.33977</v>
       </c>
       <c r="U267" t="n">
-        <v>0.14659</v>
+        <v>0.14645</v>
       </c>
       <c r="V267" t="n">
-        <v>87.53</v>
+        <v>86.81999999999999</v>
       </c>
       <c r="W267" t="n">
-        <v>76.84999999999999</v>
+        <v>76.08</v>
       </c>
       <c r="X267" t="n">
-        <v>0.7449</v>
+        <v>0.7527</v>
       </c>
       <c r="Y267" t="n">
-        <v>28.907</v>
+        <v>28.626</v>
       </c>
       <c r="Z267" t="n">
-        <v>65.907</v>
+        <v>65.66800000000001</v>
       </c>
       <c r="AA267" t="n">
-        <v>9.672000000000001</v>
+        <v>9.493</v>
       </c>
       <c r="AB267" t="n">
-        <v>29</v>
+        <v>28.708</v>
       </c>
       <c r="AC267" t="n">
-        <v>20.043</v>
+        <v>20.071</v>
       </c>
       <c r="AD267" t="n">
-        <v>26.997</v>
+        <v>26.988</v>
       </c>
       <c r="AE267" t="n">
-        <v>13.397</v>
+        <v>13.34</v>
       </c>
       <c r="AF267" t="n">
-        <v>25.67</v>
+        <v>25.733</v>
       </c>
       <c r="AG267" t="n">
-        <v>16.988</v>
+        <v>16.833</v>
       </c>
       <c r="AH267" t="n">
-        <v>8.843</v>
+        <v>8.856</v>
       </c>
       <c r="AI267" t="n">
-        <v>4.072</v>
+        <v>4.051</v>
       </c>
       <c r="AJ267" t="n">
-        <v>19.71</v>
+        <v>19.753</v>
       </c>
       <c r="AK267" t="n">
-        <v>19.8</v>
+        <v>19</v>
       </c>
       <c r="AL267" t="n">
-        <v>15.7</v>
+        <v>15.1</v>
       </c>
     </row>
     <row r="268">
@@ -38786,22 +38786,22 @@
         </is>
       </c>
       <c r="E320" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F320" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G320" t="b">
         <v>1</v>
       </c>
       <c r="H320" t="n">
-        <v>1751.007</v>
+        <v>1761.339</v>
       </c>
       <c r="I320" t="n">
-        <v>3.1884</v>
+        <v>3.2921</v>
       </c>
       <c r="J320" t="n">
-        <v>1553.9</v>
+        <v>1558.4</v>
       </c>
       <c r="K320" t="n">
         <v>45</v>
@@ -38822,70 +38822,70 @@
         <v>44</v>
       </c>
       <c r="Q320" t="n">
-        <v>118.302</v>
+        <v>117.937</v>
       </c>
       <c r="R320" t="n">
-        <v>103.549</v>
+        <v>103.323</v>
       </c>
       <c r="S320" t="n">
-        <v>14.753</v>
+        <v>14.613</v>
       </c>
       <c r="T320" t="n">
-        <v>0.29877</v>
+        <v>0.29406</v>
       </c>
       <c r="U320" t="n">
-        <v>0.1491</v>
+        <v>0.14675</v>
       </c>
       <c r="V320" t="n">
-        <v>81.86</v>
+        <v>81.45</v>
       </c>
       <c r="W320" t="n">
-        <v>71.68000000000001</v>
+        <v>71.38</v>
       </c>
       <c r="X320" t="n">
-        <v>0.79</v>
+        <v>0.796</v>
       </c>
       <c r="Y320" t="n">
-        <v>26.87</v>
+        <v>26.7</v>
       </c>
       <c r="Z320" t="n">
-        <v>58.15</v>
+        <v>58.049</v>
       </c>
       <c r="AA320" t="n">
-        <v>9.26</v>
+        <v>9.339</v>
       </c>
       <c r="AB320" t="n">
-        <v>25.44</v>
+        <v>25.399</v>
       </c>
       <c r="AC320" t="n">
-        <v>18.86</v>
+        <v>18.711</v>
       </c>
       <c r="AD320" t="n">
-        <v>25.46</v>
+        <v>25.323</v>
       </c>
       <c r="AE320" t="n">
-        <v>10.38</v>
+        <v>10.196</v>
       </c>
       <c r="AF320" t="n">
-        <v>24.16</v>
+        <v>24.27</v>
       </c>
       <c r="AG320" t="n">
-        <v>14.17</v>
+        <v>14.069</v>
       </c>
       <c r="AH320" t="n">
-        <v>7.33</v>
+        <v>7.397</v>
       </c>
       <c r="AI320" t="n">
         <v>4.35</v>
       </c>
       <c r="AJ320" t="n">
-        <v>17.21</v>
+        <v>17.301</v>
       </c>
       <c r="AK320" t="n">
-        <v>9.6</v>
+        <v>7.4</v>
       </c>
       <c r="AL320" t="n">
-        <v>9.5</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="321">
@@ -39026,22 +39026,22 @@
         </is>
       </c>
       <c r="E322" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F322" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G322" t="b">
         <v>1</v>
       </c>
       <c r="H322" t="n">
-        <v>1967.845</v>
+        <v>1952.581</v>
       </c>
       <c r="I322" t="n">
-        <v>1.6985</v>
+        <v>1.6305</v>
       </c>
       <c r="J322" t="n">
-        <v>1712.2</v>
+        <v>1718.8</v>
       </c>
       <c r="K322" t="n">
         <v>13</v>
@@ -39062,70 +39062,70 @@
         <v>16</v>
       </c>
       <c r="Q322" t="n">
-        <v>122.917</v>
+        <v>122.082</v>
       </c>
       <c r="R322" t="n">
-        <v>106.352</v>
+        <v>106.871</v>
       </c>
       <c r="S322" t="n">
-        <v>16.565</v>
+        <v>15.211</v>
       </c>
       <c r="T322" t="n">
-        <v>0.29372</v>
+        <v>0.29148</v>
       </c>
       <c r="U322" t="n">
-        <v>0.13022</v>
+        <v>0.12812</v>
       </c>
       <c r="V322" t="n">
-        <v>86.73999999999999</v>
+        <v>86.25</v>
       </c>
       <c r="W322" t="n">
-        <v>74.87</v>
+        <v>75.31</v>
       </c>
       <c r="X322" t="n">
-        <v>0.79</v>
+        <v>0.7576000000000001</v>
       </c>
       <c r="Y322" t="n">
-        <v>29.12</v>
+        <v>28.992</v>
       </c>
       <c r="Z322" t="n">
-        <v>61.2</v>
+        <v>61.425</v>
       </c>
       <c r="AA322" t="n">
-        <v>9.289999999999999</v>
+        <v>9.359</v>
       </c>
       <c r="AB322" t="n">
-        <v>26.6</v>
+        <v>26.593</v>
       </c>
       <c r="AC322" t="n">
-        <v>18.53</v>
+        <v>18.409</v>
       </c>
       <c r="AD322" t="n">
-        <v>23.66</v>
+        <v>23.333</v>
       </c>
       <c r="AE322" t="n">
-        <v>10.07</v>
+        <v>9.971</v>
       </c>
       <c r="AF322" t="n">
-        <v>23.64</v>
+        <v>23.709</v>
       </c>
       <c r="AG322" t="n">
-        <v>16.18</v>
+        <v>16.127</v>
       </c>
       <c r="AH322" t="n">
-        <v>8.06</v>
+        <v>8.048999999999999</v>
       </c>
       <c r="AI322" t="n">
-        <v>4.68</v>
+        <v>4.555</v>
       </c>
       <c r="AJ322" t="n">
-        <v>19.59</v>
+        <v>19.323</v>
       </c>
       <c r="AK322" t="n">
-        <v>3.4</v>
+        <v>4</v>
       </c>
       <c r="AL322" t="n">
-        <v>4.1</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="323">
@@ -41186,22 +41186,22 @@
         </is>
       </c>
       <c r="E340" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F340" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G340" t="b">
         <v>1</v>
       </c>
       <c r="H340" t="n">
-        <v>1632.575</v>
+        <v>1623.971</v>
       </c>
       <c r="I340" t="n">
-        <v>1.6748</v>
+        <v>1.8722</v>
       </c>
       <c r="J340" t="n">
-        <v>1540.9</v>
+        <v>1546.5</v>
       </c>
       <c r="K340" t="n">
         <v>88</v>
@@ -41222,70 +41222,70 @@
         <v>80</v>
       </c>
       <c r="Q340" t="n">
-        <v>113.009</v>
+        <v>111.577</v>
       </c>
       <c r="R340" t="n">
-        <v>102.222</v>
+        <v>102.283</v>
       </c>
       <c r="S340" t="n">
-        <v>10.787</v>
+        <v>9.295</v>
       </c>
       <c r="T340" t="n">
-        <v>0.34609</v>
+        <v>0.34458</v>
       </c>
       <c r="U340" t="n">
-        <v>0.14266</v>
+        <v>0.14529</v>
       </c>
       <c r="V340" t="n">
-        <v>77.84</v>
+        <v>76.86</v>
       </c>
       <c r="W340" t="n">
         <v>70.45999999999999</v>
       </c>
       <c r="X340" t="n">
-        <v>0.6812</v>
+        <v>0.6492</v>
       </c>
       <c r="Y340" t="n">
-        <v>27.522</v>
+        <v>27.161</v>
       </c>
       <c r="Z340" t="n">
-        <v>62.443</v>
+        <v>62.214</v>
       </c>
       <c r="AA340" t="n">
-        <v>7.281</v>
+        <v>7.091</v>
       </c>
       <c r="AB340" t="n">
-        <v>21.377</v>
+        <v>21.226</v>
       </c>
       <c r="AC340" t="n">
-        <v>15.519</v>
+        <v>15.442</v>
       </c>
       <c r="AD340" t="n">
-        <v>22.528</v>
+        <v>22.473</v>
       </c>
       <c r="AE340" t="n">
-        <v>13.319</v>
+        <v>13.267</v>
       </c>
       <c r="AF340" t="n">
-        <v>25.11</v>
+        <v>25.187</v>
       </c>
       <c r="AG340" t="n">
-        <v>11.588</v>
+        <v>11.401</v>
       </c>
       <c r="AH340" t="n">
-        <v>6.041</v>
+        <v>6.103</v>
       </c>
       <c r="AI340" t="n">
-        <v>3.881</v>
+        <v>4.032</v>
       </c>
       <c r="AJ340" t="n">
-        <v>17.475</v>
+        <v>17.578</v>
       </c>
       <c r="AK340" t="n">
-        <v>13.2</v>
+        <v>7.8</v>
       </c>
       <c r="AL340" t="n">
-        <v>8.9</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="341">
@@ -42146,22 +42146,22 @@
         </is>
       </c>
       <c r="E348" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F348" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G348" t="b">
         <v>1</v>
       </c>
       <c r="H348" t="n">
-        <v>1727.414</v>
+        <v>1684.172</v>
       </c>
       <c r="I348" t="n">
-        <v>1.0257</v>
+        <v>0.9762999999999999</v>
       </c>
       <c r="J348" t="n">
-        <v>1459.8</v>
+        <v>1457.5</v>
       </c>
       <c r="K348" t="n">
         <v>78</v>
@@ -42182,70 +42182,70 @@
         <v>66</v>
       </c>
       <c r="Q348" t="n">
-        <v>122.206</v>
+        <v>121.507</v>
       </c>
       <c r="R348" t="n">
-        <v>108.541</v>
+        <v>108.892</v>
       </c>
       <c r="S348" t="n">
-        <v>13.665</v>
+        <v>12.615</v>
       </c>
       <c r="T348" t="n">
-        <v>0.29232</v>
+        <v>0.29055</v>
       </c>
       <c r="U348" t="n">
-        <v>0.13558</v>
+        <v>0.13803</v>
       </c>
       <c r="V348" t="n">
-        <v>80.59999999999999</v>
+        <v>80.66</v>
       </c>
       <c r="W348" t="n">
-        <v>71.45</v>
+        <v>72.2</v>
       </c>
       <c r="X348" t="n">
-        <v>0.8178</v>
+        <v>0.7741</v>
       </c>
       <c r="Y348" t="n">
-        <v>28.405</v>
+        <v>28.331</v>
       </c>
       <c r="Z348" t="n">
-        <v>57.623</v>
+        <v>57.843</v>
       </c>
       <c r="AA348" t="n">
-        <v>8.324</v>
+        <v>8.581</v>
       </c>
       <c r="AB348" t="n">
-        <v>20.81</v>
+        <v>21.104</v>
       </c>
       <c r="AC348" t="n">
-        <v>15.47</v>
+        <v>15.613</v>
       </c>
       <c r="AD348" t="n">
-        <v>20.449</v>
+        <v>20.328</v>
       </c>
       <c r="AE348" t="n">
-        <v>9.587</v>
+        <v>9.557</v>
       </c>
       <c r="AF348" t="n">
-        <v>22.984</v>
+        <v>23.15</v>
       </c>
       <c r="AG348" t="n">
-        <v>15.644</v>
+        <v>15.628</v>
       </c>
       <c r="AH348" t="n">
-        <v>5.202</v>
+        <v>5.211</v>
       </c>
       <c r="AI348" t="n">
-        <v>3.121</v>
+        <v>3.12</v>
       </c>
       <c r="AJ348" t="n">
-        <v>16.028</v>
+        <v>16.106</v>
       </c>
       <c r="AK348" t="n">
-        <v>8.800000000000001</v>
+        <v>7.2</v>
       </c>
       <c r="AL348" t="n">
-        <v>7.4</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="349">

</xml_diff>

<commit_message>
Update team snapshot (2026-03-18)
</commit_message>
<xml_diff>
--- a/team_snapshot_2026.xlsx
+++ b/team_snapshot_2026.xlsx
@@ -2666,22 +2666,22 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="F19" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G19" t="b">
         <v>1</v>
       </c>
       <c r="H19" t="n">
-        <v>1825.157</v>
+        <v>1830.518</v>
       </c>
       <c r="I19" t="n">
-        <v>-7.4529</v>
+        <v>-7.3446</v>
       </c>
       <c r="J19" t="n">
-        <v>1757.6</v>
+        <v>1748.1</v>
       </c>
       <c r="K19" t="n">
         <v>38</v>
@@ -2702,70 +2702,70 @@
         <v>38</v>
       </c>
       <c r="Q19" t="n">
-        <v>118.016</v>
+        <v>118.347</v>
       </c>
       <c r="R19" t="n">
-        <v>113.691</v>
+        <v>113.34</v>
       </c>
       <c r="S19" t="n">
-        <v>4.325</v>
+        <v>5.007</v>
       </c>
       <c r="T19" t="n">
-        <v>0.34924</v>
+        <v>0.34722</v>
       </c>
       <c r="U19" t="n">
-        <v>0.14565</v>
+        <v>0.14503</v>
       </c>
       <c r="V19" t="n">
-        <v>82.52</v>
+        <v>82.55</v>
       </c>
       <c r="W19" t="n">
-        <v>79.31999999999999</v>
+        <v>78.92</v>
       </c>
       <c r="X19" t="n">
-        <v>0.51</v>
+        <v>0.5338000000000001</v>
       </c>
       <c r="Y19" t="n">
-        <v>27.36</v>
+        <v>27.293</v>
       </c>
       <c r="Z19" t="n">
-        <v>60.03</v>
+        <v>60.068</v>
       </c>
       <c r="AA19" t="n">
-        <v>7.93</v>
+        <v>8.249000000000001</v>
       </c>
       <c r="AB19" t="n">
-        <v>23.54</v>
+        <v>24.303</v>
       </c>
       <c r="AC19" t="n">
-        <v>19.87</v>
+        <v>19.711</v>
       </c>
       <c r="AD19" t="n">
-        <v>26.75</v>
+        <v>26.441</v>
       </c>
       <c r="AE19" t="n">
-        <v>12.07</v>
+        <v>12.068</v>
       </c>
       <c r="AF19" t="n">
-        <v>22.05</v>
+        <v>22.298</v>
       </c>
       <c r="AG19" t="n">
-        <v>12.6</v>
+        <v>12.872</v>
       </c>
       <c r="AH19" t="n">
-        <v>7.4</v>
+        <v>7.322</v>
       </c>
       <c r="AI19" t="n">
-        <v>4.17</v>
+        <v>4.213</v>
       </c>
       <c r="AJ19" t="n">
-        <v>17.59</v>
+        <v>17.303</v>
       </c>
       <c r="AK19" t="n">
-        <v>0.8</v>
+        <v>4.2</v>
       </c>
       <c r="AL19" t="n">
-        <v>-3.4</v>
+        <v>-1.5</v>
       </c>
     </row>
     <row r="20">
@@ -8426,22 +8426,22 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="F67" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G67" t="b">
         <v>1</v>
       </c>
       <c r="H67" t="n">
-        <v>1527.507</v>
+        <v>1520.481</v>
       </c>
       <c r="I67" t="n">
-        <v>-2.3908</v>
+        <v>-2.2791</v>
       </c>
       <c r="J67" t="n">
-        <v>1539.4</v>
+        <v>1545.3</v>
       </c>
       <c r="K67" t="n">
         <v>114</v>
@@ -8462,70 +8462,70 @@
         <v>115</v>
       </c>
       <c r="Q67" t="n">
-        <v>107.992</v>
+        <v>108.143</v>
       </c>
       <c r="R67" t="n">
-        <v>105.223</v>
+        <v>105.516</v>
       </c>
       <c r="S67" t="n">
-        <v>2.769</v>
+        <v>2.627</v>
       </c>
       <c r="T67" t="n">
-        <v>0.2874</v>
+        <v>0.28302</v>
       </c>
       <c r="U67" t="n">
-        <v>0.15602</v>
+        <v>0.15297</v>
       </c>
       <c r="V67" t="n">
-        <v>69.45999999999999</v>
+        <v>69.95</v>
       </c>
       <c r="W67" t="n">
-        <v>68.05</v>
+        <v>68.65000000000001</v>
       </c>
       <c r="X67" t="n">
-        <v>0.576</v>
+        <v>0.5583</v>
       </c>
       <c r="Y67" t="n">
-        <v>24.824</v>
+        <v>25.037</v>
       </c>
       <c r="Z67" t="n">
-        <v>55.456</v>
+        <v>56.011</v>
       </c>
       <c r="AA67" t="n">
-        <v>8.608000000000001</v>
+        <v>8.859</v>
       </c>
       <c r="AB67" t="n">
-        <v>24.456</v>
+        <v>25.019</v>
       </c>
       <c r="AC67" t="n">
-        <v>11.2</v>
+        <v>11.017</v>
       </c>
       <c r="AD67" t="n">
-        <v>17.568</v>
+        <v>17.236</v>
       </c>
       <c r="AE67" t="n">
-        <v>8.848000000000001</v>
+        <v>8.73</v>
       </c>
       <c r="AF67" t="n">
-        <v>21.552</v>
+        <v>21.751</v>
       </c>
       <c r="AG67" t="n">
-        <v>13.232</v>
+        <v>13.448</v>
       </c>
       <c r="AH67" t="n">
-        <v>6.344</v>
+        <v>6.38</v>
       </c>
       <c r="AI67" t="n">
-        <v>4.032</v>
+        <v>4.108</v>
       </c>
       <c r="AJ67" t="n">
-        <v>16.88</v>
+        <v>16.991</v>
       </c>
       <c r="AK67" t="n">
-        <v>0.4</v>
+        <v>-1.8</v>
       </c>
       <c r="AL67" t="n">
-        <v>2</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="68">
@@ -12506,22 +12506,22 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="F101" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G101" t="b">
         <v>1</v>
       </c>
       <c r="H101" t="n">
-        <v>1709.338</v>
+        <v>1685.089</v>
       </c>
       <c r="I101" t="n">
-        <v>-1.2025</v>
+        <v>-1.4337</v>
       </c>
       <c r="J101" t="n">
-        <v>1514.4</v>
+        <v>1522.7</v>
       </c>
       <c r="K101" t="n">
         <v>96</v>
@@ -12542,67 +12542,67 @@
         <v>92</v>
       </c>
       <c r="Q101" t="n">
-        <v>111.945</v>
+        <v>112.217</v>
       </c>
       <c r="R101" t="n">
-        <v>104.412</v>
+        <v>105.202</v>
       </c>
       <c r="S101" t="n">
-        <v>7.533</v>
+        <v>7.015</v>
       </c>
       <c r="T101" t="n">
-        <v>0.26281</v>
+        <v>0.26936</v>
       </c>
       <c r="U101" t="n">
-        <v>0.15292</v>
+        <v>0.1523</v>
       </c>
       <c r="V101" t="n">
-        <v>72.75</v>
+        <v>72.84999999999999</v>
       </c>
       <c r="W101" t="n">
-        <v>67.62</v>
+        <v>68.06999999999999</v>
       </c>
       <c r="X101" t="n">
-        <v>0.7014</v>
+        <v>0.6801</v>
       </c>
       <c r="Y101" t="n">
-        <v>25.177</v>
+        <v>25.133</v>
       </c>
       <c r="Z101" t="n">
-        <v>53.487</v>
+        <v>53.745</v>
       </c>
       <c r="AA101" t="n">
-        <v>6.22</v>
+        <v>6.206</v>
       </c>
       <c r="AB101" t="n">
-        <v>18.525</v>
+        <v>18.546</v>
       </c>
       <c r="AC101" t="n">
-        <v>16.438</v>
+        <v>16.569</v>
       </c>
       <c r="AD101" t="n">
-        <v>22.736</v>
+        <v>22.763</v>
       </c>
       <c r="AE101" t="n">
-        <v>8.606</v>
+        <v>8.879</v>
       </c>
       <c r="AF101" t="n">
-        <v>23.745</v>
+        <v>23.628</v>
       </c>
       <c r="AG101" t="n">
-        <v>12.87</v>
+        <v>12.657</v>
       </c>
       <c r="AH101" t="n">
-        <v>5.142</v>
+        <v>5.093</v>
       </c>
       <c r="AI101" t="n">
-        <v>3.023</v>
+        <v>3.042</v>
       </c>
       <c r="AJ101" t="n">
-        <v>15.371</v>
+        <v>15.413</v>
       </c>
       <c r="AK101" t="n">
-        <v>2.6</v>
+        <v>5</v>
       </c>
       <c r="AL101" t="n">
         <v>-3.1</v>
@@ -14426,22 +14426,22 @@
         </is>
       </c>
       <c r="E117" t="n">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="F117" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G117" t="b">
         <v>1</v>
       </c>
       <c r="H117" t="n">
-        <v>1407.766</v>
+        <v>1413.012</v>
       </c>
       <c r="I117" t="n">
-        <v>2.9318</v>
+        <v>2.8128</v>
       </c>
       <c r="J117" t="n">
-        <v>1372.4</v>
+        <v>1374.4</v>
       </c>
       <c r="K117" t="n">
         <v>207</v>
@@ -14462,70 +14462,70 @@
         <v>203</v>
       </c>
       <c r="Q117" t="n">
-        <v>109.065</v>
+        <v>109.768</v>
       </c>
       <c r="R117" t="n">
-        <v>98.31699999999999</v>
+        <v>99.30200000000001</v>
       </c>
       <c r="S117" t="n">
-        <v>10.748</v>
+        <v>10.466</v>
       </c>
       <c r="T117" t="n">
-        <v>0.31905</v>
+        <v>0.31778</v>
       </c>
       <c r="U117" t="n">
-        <v>0.18558</v>
+        <v>0.18288</v>
       </c>
       <c r="V117" t="n">
-        <v>74.94</v>
+        <v>75.48</v>
       </c>
       <c r="W117" t="n">
-        <v>67.73999999999999</v>
+        <v>68.45</v>
       </c>
       <c r="X117" t="n">
-        <v>0.6591</v>
+        <v>0.6702</v>
       </c>
       <c r="Y117" t="n">
-        <v>24.932</v>
+        <v>25.174</v>
       </c>
       <c r="Z117" t="n">
-        <v>55.92</v>
+        <v>56.184</v>
       </c>
       <c r="AA117" t="n">
-        <v>6.636</v>
+        <v>6.801</v>
       </c>
       <c r="AB117" t="n">
-        <v>19.17</v>
+        <v>19.252</v>
       </c>
       <c r="AC117" t="n">
-        <v>18.443</v>
+        <v>18.33</v>
       </c>
       <c r="AD117" t="n">
-        <v>24.841</v>
+        <v>24.736</v>
       </c>
       <c r="AE117" t="n">
-        <v>10.716</v>
+        <v>10.714</v>
       </c>
       <c r="AF117" t="n">
-        <v>22.682</v>
+        <v>22.834</v>
       </c>
       <c r="AG117" t="n">
-        <v>15.227</v>
+        <v>15.22</v>
       </c>
       <c r="AH117" t="n">
-        <v>8.625</v>
+        <v>8.375999999999999</v>
       </c>
       <c r="AI117" t="n">
-        <v>3.898</v>
+        <v>3.771</v>
       </c>
       <c r="AJ117" t="n">
-        <v>18.636</v>
+        <v>18.714</v>
       </c>
       <c r="AK117" t="n">
-        <v>15.4</v>
+        <v>11</v>
       </c>
       <c r="AL117" t="n">
-        <v>19</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="118">
@@ -17666,22 +17666,22 @@
         </is>
       </c>
       <c r="E144" t="n">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="F144" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G144" t="b">
         <v>1</v>
       </c>
       <c r="H144" t="n">
-        <v>1719.236</v>
+        <v>1743.485</v>
       </c>
       <c r="I144" t="n">
-        <v>2.9746</v>
+        <v>2.673</v>
       </c>
       <c r="J144" t="n">
-        <v>1481.5</v>
+        <v>1491.2</v>
       </c>
       <c r="K144" t="n">
         <v>125</v>
@@ -17702,70 +17702,70 @@
         <v>106</v>
       </c>
       <c r="Q144" t="n">
-        <v>117.433</v>
+        <v>117.773</v>
       </c>
       <c r="R144" t="n">
-        <v>111.215</v>
+        <v>111.278</v>
       </c>
       <c r="S144" t="n">
-        <v>6.218</v>
+        <v>6.495</v>
       </c>
       <c r="T144" t="n">
-        <v>0.17119</v>
+        <v>0.17409</v>
       </c>
       <c r="U144" t="n">
-        <v>0.1328</v>
+        <v>0.13118</v>
       </c>
       <c r="V144" t="n">
-        <v>76.15000000000001</v>
+        <v>76.23999999999999</v>
       </c>
       <c r="W144" t="n">
-        <v>72.20999999999999</v>
+        <v>72.13</v>
       </c>
       <c r="X144" t="n">
-        <v>0.753</v>
+        <v>0.7683</v>
       </c>
       <c r="Y144" t="n">
-        <v>27.076</v>
+        <v>27.066</v>
       </c>
       <c r="Z144" t="n">
-        <v>53.286</v>
+        <v>53.378</v>
       </c>
       <c r="AA144" t="n">
-        <v>10.19</v>
+        <v>10.039</v>
       </c>
       <c r="AB144" t="n">
-        <v>25.549</v>
+        <v>25.276</v>
       </c>
       <c r="AC144" t="n">
-        <v>12.144</v>
+        <v>12.332</v>
       </c>
       <c r="AD144" t="n">
-        <v>17.311</v>
+        <v>17.385</v>
       </c>
       <c r="AE144" t="n">
-        <v>4.673</v>
+        <v>4.789</v>
       </c>
       <c r="AF144" t="n">
-        <v>21.626</v>
+        <v>21.683</v>
       </c>
       <c r="AG144" t="n">
-        <v>16.533</v>
+        <v>16.53</v>
       </c>
       <c r="AH144" t="n">
-        <v>5.978</v>
+        <v>6.04</v>
       </c>
       <c r="AI144" t="n">
-        <v>3.308</v>
+        <v>3.298</v>
       </c>
       <c r="AJ144" t="n">
-        <v>14.335</v>
+        <v>14.451</v>
       </c>
       <c r="AK144" t="n">
-        <v>-2.4</v>
+        <v>0.6</v>
       </c>
       <c r="AL144" t="n">
-        <v>-1.8</v>
+        <v>-1.5</v>
       </c>
     </row>
     <row r="145">
@@ -23546,19 +23546,19 @@
         </is>
       </c>
       <c r="E193" t="n">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="F193" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G193" t="b">
         <v>1</v>
       </c>
       <c r="H193" t="n">
-        <v>1734.013</v>
+        <v>1711.533</v>
       </c>
       <c r="I193" t="n">
-        <v>6.962</v>
+        <v>6.597</v>
       </c>
       <c r="J193" t="n">
         <v>1681.7</v>
@@ -23582,70 +23582,70 @@
         <v>36</v>
       </c>
       <c r="Q193" t="n">
-        <v>119.356</v>
+        <v>118.677</v>
       </c>
       <c r="R193" t="n">
-        <v>109.318</v>
+        <v>108.955</v>
       </c>
       <c r="S193" t="n">
-        <v>10.038</v>
+        <v>9.722</v>
       </c>
       <c r="T193" t="n">
-        <v>0.2802</v>
+        <v>0.28198</v>
       </c>
       <c r="U193" t="n">
-        <v>0.12879</v>
+        <v>0.13052</v>
       </c>
       <c r="V193" t="n">
-        <v>83.62</v>
+        <v>83.04000000000001</v>
       </c>
       <c r="W193" t="n">
-        <v>76.55</v>
+        <v>76.2</v>
       </c>
       <c r="X193" t="n">
-        <v>0.601</v>
+        <v>0.5836</v>
       </c>
       <c r="Y193" t="n">
-        <v>28.392</v>
+        <v>28.178</v>
       </c>
       <c r="Z193" t="n">
-        <v>60.756</v>
+        <v>60.648</v>
       </c>
       <c r="AA193" t="n">
-        <v>10.369</v>
+        <v>10.165</v>
       </c>
       <c r="AB193" t="n">
-        <v>26.657</v>
+        <v>26.338</v>
       </c>
       <c r="AC193" t="n">
-        <v>16.463</v>
+        <v>16.594</v>
       </c>
       <c r="AD193" t="n">
-        <v>21.416</v>
+        <v>21.676</v>
       </c>
       <c r="AE193" t="n">
-        <v>9.129</v>
+        <v>9.339</v>
       </c>
       <c r="AF193" t="n">
-        <v>23.21</v>
+        <v>23.464</v>
       </c>
       <c r="AG193" t="n">
-        <v>15.576</v>
+        <v>15.398</v>
       </c>
       <c r="AH193" t="n">
-        <v>8.035</v>
+        <v>8.021000000000001</v>
       </c>
       <c r="AI193" t="n">
-        <v>3.394</v>
+        <v>3.424</v>
       </c>
       <c r="AJ193" t="n">
-        <v>18.117</v>
+        <v>18.072</v>
       </c>
       <c r="AK193" t="n">
-        <v>-6.6</v>
+        <v>-5.8</v>
       </c>
       <c r="AL193" t="n">
-        <v>-7.1</v>
+        <v>-8.199999999999999</v>
       </c>
     </row>
     <row r="194">
@@ -26666,22 +26666,22 @@
         </is>
       </c>
       <c r="E219" t="n">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="F219" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G219" t="b">
         <v>1</v>
       </c>
       <c r="H219" t="n">
-        <v>1706.568</v>
+        <v>1713.594</v>
       </c>
       <c r="I219" t="n">
-        <v>-1.149</v>
+        <v>-1.1886</v>
       </c>
       <c r="J219" t="n">
-        <v>1692.8</v>
+        <v>1685</v>
       </c>
       <c r="K219" t="n">
         <v>66</v>
@@ -26702,70 +26702,70 @@
         <v>74</v>
       </c>
       <c r="Q219" t="n">
-        <v>111.498</v>
+        <v>111.537</v>
       </c>
       <c r="R219" t="n">
-        <v>110.641</v>
+        <v>110.394</v>
       </c>
       <c r="S219" t="n">
-        <v>0.857</v>
+        <v>1.144</v>
       </c>
       <c r="T219" t="n">
-        <v>0.28469</v>
+        <v>0.27727</v>
       </c>
       <c r="U219" t="n">
-        <v>0.15383</v>
+        <v>0.15255</v>
       </c>
       <c r="V219" t="n">
-        <v>84.31</v>
+        <v>84.26000000000001</v>
       </c>
       <c r="W219" t="n">
-        <v>83.03</v>
+        <v>82.8</v>
       </c>
       <c r="X219" t="n">
-        <v>0.57</v>
+        <v>0.5921</v>
       </c>
       <c r="Y219" t="n">
-        <v>29.14</v>
+        <v>29.049</v>
       </c>
       <c r="Z219" t="n">
-        <v>63.21</v>
+        <v>62.876</v>
       </c>
       <c r="AA219" t="n">
-        <v>7.75</v>
+        <v>7.758</v>
       </c>
       <c r="AB219" t="n">
-        <v>22.93</v>
+        <v>22.663</v>
       </c>
       <c r="AC219" t="n">
-        <v>18.01</v>
+        <v>18.145</v>
       </c>
       <c r="AD219" t="n">
-        <v>24.17</v>
+        <v>24.464</v>
       </c>
       <c r="AE219" t="n">
-        <v>10.02</v>
+        <v>9.779</v>
       </c>
       <c r="AF219" t="n">
-        <v>25.01</v>
+        <v>25.404</v>
       </c>
       <c r="AG219" t="n">
-        <v>14.8</v>
+        <v>14.748</v>
       </c>
       <c r="AH219" t="n">
-        <v>7.16</v>
+        <v>7.098</v>
       </c>
       <c r="AI219" t="n">
-        <v>2.6</v>
+        <v>2.544</v>
       </c>
       <c r="AJ219" t="n">
-        <v>17.39</v>
+        <v>17.08</v>
       </c>
       <c r="AK219" t="n">
-        <v>-4.2</v>
+        <v>1.2</v>
       </c>
       <c r="AL219" t="n">
-        <v>-5.2</v>
+        <v>-3.9</v>
       </c>
     </row>
     <row r="220">
@@ -27395,7 +27395,7 @@
         <v>1</v>
       </c>
       <c r="H225" t="n">
-        <v>1458.418</v>
+        <v>1435.396</v>
       </c>
       <c r="I225" t="n">
         <v>1.2024</v>
@@ -31466,22 +31466,22 @@
         </is>
       </c>
       <c r="E259" t="n">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="F259" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G259" t="b">
         <v>1</v>
       </c>
       <c r="H259" t="n">
-        <v>1548.014</v>
+        <v>1560.056</v>
       </c>
       <c r="I259" t="n">
-        <v>2.3807</v>
+        <v>2.1732</v>
       </c>
       <c r="J259" t="n">
-        <v>1521.6</v>
+        <v>1524.1</v>
       </c>
       <c r="K259" t="n">
         <v>119</v>
@@ -31502,70 +31502,70 @@
         <v>122</v>
       </c>
       <c r="Q259" t="n">
-        <v>100.946</v>
+        <v>100.859</v>
       </c>
       <c r="R259" t="n">
-        <v>98.42700000000001</v>
+        <v>97.512</v>
       </c>
       <c r="S259" t="n">
-        <v>2.519</v>
+        <v>3.347</v>
       </c>
       <c r="T259" t="n">
-        <v>0.2559</v>
+        <v>0.25248</v>
       </c>
       <c r="U259" t="n">
-        <v>0.16862</v>
+        <v>0.16788</v>
       </c>
       <c r="V259" t="n">
         <v>69.59999999999999</v>
       </c>
       <c r="W259" t="n">
-        <v>67.93000000000001</v>
+        <v>67.36</v>
       </c>
       <c r="X259" t="n">
-        <v>0.575</v>
+        <v>0.5974</v>
       </c>
       <c r="Y259" t="n">
-        <v>24.315</v>
+        <v>24.212</v>
       </c>
       <c r="Z259" t="n">
-        <v>56.549</v>
+        <v>56.508</v>
       </c>
       <c r="AA259" t="n">
-        <v>7.192</v>
+        <v>7.266</v>
       </c>
       <c r="AB259" t="n">
-        <v>22.044</v>
+        <v>22.022</v>
       </c>
       <c r="AC259" t="n">
-        <v>13.774</v>
+        <v>13.912</v>
       </c>
       <c r="AD259" t="n">
-        <v>19.592</v>
+        <v>19.646</v>
       </c>
       <c r="AE259" t="n">
-        <v>7.786</v>
+        <v>7.663</v>
       </c>
       <c r="AF259" t="n">
-        <v>21.997</v>
+        <v>22.049</v>
       </c>
       <c r="AG259" t="n">
-        <v>12.894</v>
+        <v>12.987</v>
       </c>
       <c r="AH259" t="n">
-        <v>7.767</v>
+        <v>7.823</v>
       </c>
       <c r="AI259" t="n">
-        <v>4.786</v>
+        <v>4.863</v>
       </c>
       <c r="AJ259" t="n">
-        <v>16.769</v>
+        <v>16.574</v>
       </c>
       <c r="AK259" t="n">
-        <v>4.6</v>
+        <v>5.2</v>
       </c>
       <c r="AL259" t="n">
-        <v>2</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="260">
@@ -31706,22 +31706,22 @@
         </is>
       </c>
       <c r="E261" t="n">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="F261" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G261" t="b">
         <v>1</v>
       </c>
       <c r="H261" t="n">
-        <v>1559.844</v>
+        <v>1550.507</v>
       </c>
       <c r="I261" t="n">
-        <v>3.1865</v>
+        <v>3.0971</v>
       </c>
       <c r="J261" t="n">
-        <v>1397.1</v>
+        <v>1405.2</v>
       </c>
       <c r="K261" t="n">
         <v>91</v>
@@ -31742,70 +31742,70 @@
         <v>89</v>
       </c>
       <c r="Q261" t="n">
-        <v>112.195</v>
+        <v>112.155</v>
       </c>
       <c r="R261" t="n">
-        <v>99.51000000000001</v>
+        <v>99.89400000000001</v>
       </c>
       <c r="S261" t="n">
-        <v>12.685</v>
+        <v>12.261</v>
       </c>
       <c r="T261" t="n">
-        <v>0.3073</v>
+        <v>0.30966</v>
       </c>
       <c r="U261" t="n">
-        <v>0.13545</v>
+        <v>0.13657</v>
       </c>
       <c r="V261" t="n">
-        <v>74.52</v>
+        <v>75</v>
       </c>
       <c r="W261" t="n">
-        <v>66.05</v>
+        <v>66.84999999999999</v>
       </c>
       <c r="X261" t="n">
-        <v>0.832</v>
+        <v>0.8065</v>
       </c>
       <c r="Y261" t="n">
-        <v>27.072</v>
+        <v>27.254</v>
       </c>
       <c r="Z261" t="n">
-        <v>60.144</v>
+        <v>60.571</v>
       </c>
       <c r="AA261" t="n">
-        <v>8.68</v>
+        <v>8.728</v>
       </c>
       <c r="AB261" t="n">
-        <v>23.632</v>
+        <v>23.998</v>
       </c>
       <c r="AC261" t="n">
-        <v>12.376</v>
+        <v>12.295</v>
       </c>
       <c r="AD261" t="n">
-        <v>17.984</v>
+        <v>17.954</v>
       </c>
       <c r="AE261" t="n">
-        <v>10.576</v>
+        <v>10.674</v>
       </c>
       <c r="AF261" t="n">
-        <v>23.48</v>
+        <v>23.434</v>
       </c>
       <c r="AG261" t="n">
-        <v>13.232</v>
+        <v>13.179</v>
       </c>
       <c r="AH261" t="n">
-        <v>6.824</v>
+        <v>7.045</v>
       </c>
       <c r="AI261" t="n">
-        <v>3.736</v>
+        <v>3.798</v>
       </c>
       <c r="AJ261" t="n">
-        <v>15.784</v>
+        <v>16.045</v>
       </c>
       <c r="AK261" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="AL261" t="n">
-        <v>4.6</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="262">
@@ -32066,22 +32066,22 @@
         </is>
       </c>
       <c r="E264" t="n">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="F264" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G264" t="b">
         <v>1</v>
       </c>
       <c r="H264" t="n">
-        <v>1548.072</v>
+        <v>1542.711</v>
       </c>
       <c r="I264" t="n">
-        <v>0.0533</v>
+        <v>-0.006</v>
       </c>
       <c r="J264" t="n">
-        <v>1442.8</v>
+        <v>1459.5</v>
       </c>
       <c r="K264" t="n">
         <v>205</v>
@@ -32102,70 +32102,70 @@
         <v>187</v>
       </c>
       <c r="Q264" t="n">
-        <v>109.756</v>
+        <v>109.4</v>
       </c>
       <c r="R264" t="n">
-        <v>106.668</v>
+        <v>107.005</v>
       </c>
       <c r="S264" t="n">
-        <v>3.088</v>
+        <v>2.395</v>
       </c>
       <c r="T264" t="n">
-        <v>0.21373</v>
+        <v>0.21434</v>
       </c>
       <c r="U264" t="n">
-        <v>0.12862</v>
+        <v>0.12568</v>
       </c>
       <c r="V264" t="n">
-        <v>73.58</v>
+        <v>73.15000000000001</v>
       </c>
       <c r="W264" t="n">
-        <v>71.34999999999999</v>
+        <v>71.37</v>
       </c>
       <c r="X264" t="n">
-        <v>0.6254</v>
+        <v>0.6058</v>
       </c>
       <c r="Y264" t="n">
-        <v>26.005</v>
+        <v>26.012</v>
       </c>
       <c r="Z264" t="n">
-        <v>55.621</v>
+        <v>55.855</v>
       </c>
       <c r="AA264" t="n">
-        <v>7.694</v>
+        <v>7.478</v>
       </c>
       <c r="AB264" t="n">
-        <v>21.618</v>
+        <v>21.275</v>
       </c>
       <c r="AC264" t="n">
-        <v>14.284</v>
+        <v>13.939</v>
       </c>
       <c r="AD264" t="n">
-        <v>21.542</v>
+        <v>21.139</v>
       </c>
       <c r="AE264" t="n">
-        <v>6.922</v>
+        <v>6.936</v>
       </c>
       <c r="AF264" t="n">
-        <v>24.613</v>
+        <v>24.606</v>
       </c>
       <c r="AG264" t="n">
-        <v>12.191</v>
+        <v>12.194</v>
       </c>
       <c r="AH264" t="n">
-        <v>7.81</v>
+        <v>7.797</v>
       </c>
       <c r="AI264" t="n">
-        <v>2.354</v>
+        <v>2.319</v>
       </c>
       <c r="AJ264" t="n">
-        <v>13.26</v>
+        <v>13.148</v>
       </c>
       <c r="AK264" t="n">
-        <v>3.2</v>
+        <v>2.6</v>
       </c>
       <c r="AL264" t="n">
-        <v>2.6</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="265">
@@ -34946,22 +34946,22 @@
         </is>
       </c>
       <c r="E288" t="n">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="F288" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G288" t="b">
         <v>1</v>
       </c>
       <c r="H288" t="n">
-        <v>1741.68</v>
+        <v>1764.159</v>
       </c>
       <c r="I288" t="n">
-        <v>2.8164</v>
+        <v>2.6628</v>
       </c>
       <c r="J288" t="n">
-        <v>1696.4</v>
+        <v>1698.6</v>
       </c>
       <c r="K288" t="n">
         <v>37</v>
@@ -34982,70 +34982,70 @@
         <v>42</v>
       </c>
       <c r="Q288" t="n">
-        <v>119.505</v>
+        <v>118.998</v>
       </c>
       <c r="R288" t="n">
-        <v>111.341</v>
+        <v>110.826</v>
       </c>
       <c r="S288" t="n">
-        <v>8.164</v>
+        <v>8.173</v>
       </c>
       <c r="T288" t="n">
-        <v>0.30721</v>
+        <v>0.30408</v>
       </c>
       <c r="U288" t="n">
-        <v>0.145</v>
+        <v>0.14433</v>
       </c>
       <c r="V288" t="n">
-        <v>82.48</v>
+        <v>82.06</v>
       </c>
       <c r="W288" t="n">
-        <v>76.77</v>
+        <v>76.34</v>
       </c>
       <c r="X288" t="n">
-        <v>0.5431</v>
+        <v>0.5665</v>
       </c>
       <c r="Y288" t="n">
-        <v>28.019</v>
+        <v>27.8</v>
       </c>
       <c r="Z288" t="n">
-        <v>58.09</v>
+        <v>58.071</v>
       </c>
       <c r="AA288" t="n">
-        <v>7.038</v>
+        <v>7.053</v>
       </c>
       <c r="AB288" t="n">
-        <v>20.446</v>
+        <v>20.366</v>
       </c>
       <c r="AC288" t="n">
-        <v>19.824</v>
+        <v>19.636</v>
       </c>
       <c r="AD288" t="n">
-        <v>26.421</v>
+        <v>26.145</v>
       </c>
       <c r="AE288" t="n">
-        <v>10.651</v>
+        <v>10.53</v>
       </c>
       <c r="AF288" t="n">
-        <v>24.115</v>
+        <v>24.173</v>
       </c>
       <c r="AG288" t="n">
-        <v>11.779</v>
+        <v>11.734</v>
       </c>
       <c r="AH288" t="n">
-        <v>5.994</v>
+        <v>6.018</v>
       </c>
       <c r="AI288" t="n">
-        <v>2.901</v>
+        <v>2.956</v>
       </c>
       <c r="AJ288" t="n">
-        <v>18.853</v>
+        <v>18.996</v>
       </c>
       <c r="AK288" t="n">
-        <v>-8</v>
+        <v>-5</v>
       </c>
       <c r="AL288" t="n">
-        <v>-1.1</v>
+        <v>-1.8</v>
       </c>
     </row>
     <row r="289">
@@ -36026,22 +36026,22 @@
         </is>
       </c>
       <c r="E297" t="n">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="F297" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G297" t="b">
         <v>1</v>
       </c>
       <c r="H297" t="n">
-        <v>1673.101</v>
+        <v>1682.437</v>
       </c>
       <c r="I297" t="n">
-        <v>8.4628</v>
+        <v>8.0585</v>
       </c>
       <c r="J297" t="n">
-        <v>1509.4</v>
+        <v>1510.5</v>
       </c>
       <c r="K297" t="n">
         <v>63</v>
@@ -36062,70 +36062,70 @@
         <v>52</v>
       </c>
       <c r="Q297" t="n">
-        <v>121.126</v>
+        <v>121.034</v>
       </c>
       <c r="R297" t="n">
-        <v>106.46</v>
+        <v>106.412</v>
       </c>
       <c r="S297" t="n">
-        <v>14.667</v>
+        <v>14.622</v>
       </c>
       <c r="T297" t="n">
-        <v>0.27526</v>
+        <v>0.28053</v>
       </c>
       <c r="U297" t="n">
-        <v>0.14728</v>
+        <v>0.14866</v>
       </c>
       <c r="V297" t="n">
-        <v>84.16</v>
+        <v>84.47</v>
       </c>
       <c r="W297" t="n">
-        <v>73.98999999999999</v>
+        <v>74.31999999999999</v>
       </c>
       <c r="X297" t="n">
-        <v>0.768</v>
+        <v>0.7829</v>
       </c>
       <c r="Y297" t="n">
-        <v>27.48</v>
+        <v>27.381</v>
       </c>
       <c r="Z297" t="n">
-        <v>58.136</v>
+        <v>58.439</v>
       </c>
       <c r="AA297" t="n">
-        <v>10.656</v>
+        <v>10.582</v>
       </c>
       <c r="AB297" t="n">
-        <v>27.032</v>
+        <v>27.231</v>
       </c>
       <c r="AC297" t="n">
-        <v>18.544</v>
+        <v>19.128</v>
       </c>
       <c r="AD297" t="n">
-        <v>23.704</v>
+        <v>24.437</v>
       </c>
       <c r="AE297" t="n">
-        <v>9.295999999999999</v>
+        <v>9.747999999999999</v>
       </c>
       <c r="AF297" t="n">
-        <v>24.224</v>
+        <v>24.402</v>
       </c>
       <c r="AG297" t="n">
-        <v>15.336</v>
+        <v>15.226</v>
       </c>
       <c r="AH297" t="n">
-        <v>6.44</v>
+        <v>6.665</v>
       </c>
       <c r="AI297" t="n">
-        <v>2.312</v>
+        <v>2.387</v>
       </c>
       <c r="AJ297" t="n">
-        <v>16.32</v>
+        <v>16.156</v>
       </c>
       <c r="AK297" t="n">
-        <v>11.2</v>
+        <v>5.4</v>
       </c>
       <c r="AL297" t="n">
-        <v>7.2</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="298">
@@ -36626,22 +36626,22 @@
         </is>
       </c>
       <c r="E302" t="n">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="F302" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G302" t="b">
         <v>1</v>
       </c>
       <c r="H302" t="n">
-        <v>1609.971</v>
+        <v>1592.022</v>
       </c>
       <c r="I302" t="n">
-        <v>2.2217</v>
+        <v>2.1658</v>
       </c>
       <c r="J302" t="n">
-        <v>1475.3</v>
+        <v>1481.2</v>
       </c>
       <c r="K302" t="n">
         <v>104</v>
@@ -36662,70 +36662,70 @@
         <v>117</v>
       </c>
       <c r="Q302" t="n">
-        <v>103.957</v>
+        <v>103.857</v>
       </c>
       <c r="R302" t="n">
-        <v>97.05800000000001</v>
+        <v>97.233</v>
       </c>
       <c r="S302" t="n">
-        <v>6.899</v>
+        <v>6.624</v>
       </c>
       <c r="T302" t="n">
-        <v>0.27524</v>
+        <v>0.27504</v>
       </c>
       <c r="U302" t="n">
-        <v>0.17235</v>
+        <v>0.17126</v>
       </c>
       <c r="V302" t="n">
         <v>74.19</v>
       </c>
       <c r="W302" t="n">
-        <v>69.23</v>
+        <v>69.44</v>
       </c>
       <c r="X302" t="n">
-        <v>0.6503</v>
+        <v>0.631</v>
       </c>
       <c r="Y302" t="n">
-        <v>27</v>
+        <v>26.923</v>
       </c>
       <c r="Z302" t="n">
-        <v>59.992</v>
+        <v>60.017</v>
       </c>
       <c r="AA302" t="n">
-        <v>5.832</v>
+        <v>5.704</v>
       </c>
       <c r="AB302" t="n">
-        <v>17.422</v>
+        <v>17.177</v>
       </c>
       <c r="AC302" t="n">
-        <v>14.636</v>
+        <v>14.853</v>
       </c>
       <c r="AD302" t="n">
-        <v>21.286</v>
+        <v>21.484</v>
       </c>
       <c r="AE302" t="n">
-        <v>10.28</v>
+        <v>10.249</v>
       </c>
       <c r="AF302" t="n">
-        <v>27.053</v>
+        <v>27.022</v>
       </c>
       <c r="AG302" t="n">
-        <v>15.049</v>
+        <v>14.992</v>
       </c>
       <c r="AH302" t="n">
-        <v>7.526</v>
+        <v>7.819</v>
       </c>
       <c r="AI302" t="n">
-        <v>6.036</v>
+        <v>5.885</v>
       </c>
       <c r="AJ302" t="n">
-        <v>15.818</v>
+        <v>15.927</v>
       </c>
       <c r="AK302" t="n">
-        <v>8.800000000000001</v>
+        <v>7.4</v>
       </c>
       <c r="AL302" t="n">
-        <v>6.9</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="303">
@@ -37346,22 +37346,22 @@
         </is>
       </c>
       <c r="E308" t="n">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="F308" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G308" t="b">
         <v>1</v>
       </c>
       <c r="H308" t="n">
-        <v>1397.919</v>
+        <v>1392.673</v>
       </c>
       <c r="I308" t="n">
-        <v>1.3468</v>
+        <v>1.415</v>
       </c>
       <c r="J308" t="n">
-        <v>1369.1</v>
+        <v>1369.9</v>
       </c>
       <c r="K308" t="n">
         <v>185</v>
@@ -37382,70 +37382,70 @@
         <v>196</v>
       </c>
       <c r="Q308" t="n">
-        <v>113.392</v>
+        <v>113.599</v>
       </c>
       <c r="R308" t="n">
-        <v>101.925</v>
+        <v>102.819</v>
       </c>
       <c r="S308" t="n">
-        <v>11.468</v>
+        <v>10.78</v>
       </c>
       <c r="T308" t="n">
-        <v>0.21757</v>
+        <v>0.21619</v>
       </c>
       <c r="U308" t="n">
-        <v>0.13504</v>
+        <v>0.13477</v>
       </c>
       <c r="V308" t="n">
-        <v>75.42</v>
+        <v>75.72</v>
       </c>
       <c r="W308" t="n">
-        <v>67.90000000000001</v>
+        <v>68.66</v>
       </c>
       <c r="X308" t="n">
-        <v>0.7352</v>
+        <v>0.7050999999999999</v>
       </c>
       <c r="Y308" t="n">
-        <v>26.462</v>
+        <v>26.596</v>
       </c>
       <c r="Z308" t="n">
-        <v>56.396</v>
+        <v>56.417</v>
       </c>
       <c r="AA308" t="n">
-        <v>7.881</v>
+        <v>7.91</v>
       </c>
       <c r="AB308" t="n">
-        <v>21.928</v>
+        <v>21.904</v>
       </c>
       <c r="AC308" t="n">
-        <v>14.618</v>
+        <v>14.622</v>
       </c>
       <c r="AD308" t="n">
-        <v>19.114</v>
+        <v>19.256</v>
       </c>
       <c r="AE308" t="n">
-        <v>7.272</v>
+        <v>7.218</v>
       </c>
       <c r="AF308" t="n">
-        <v>25.589</v>
+        <v>25.615</v>
       </c>
       <c r="AG308" t="n">
-        <v>11.892</v>
+        <v>11.897</v>
       </c>
       <c r="AH308" t="n">
-        <v>4.821</v>
+        <v>4.878</v>
       </c>
       <c r="AI308" t="n">
-        <v>2.404</v>
+        <v>2.385</v>
       </c>
       <c r="AJ308" t="n">
-        <v>13.462</v>
+        <v>13.75</v>
       </c>
       <c r="AK308" t="n">
-        <v>23</v>
+        <v>17.6</v>
       </c>
       <c r="AL308" t="n">
-        <v>18.2</v>
+        <v>16.3</v>
       </c>
     </row>
     <row r="309">
@@ -37706,22 +37706,22 @@
         </is>
       </c>
       <c r="E311" t="n">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="F311" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G311" t="b">
         <v>1</v>
       </c>
       <c r="H311" t="n">
-        <v>1669.074</v>
+        <v>1694.511</v>
       </c>
       <c r="I311" t="n">
-        <v>1.9449</v>
+        <v>1.7793</v>
       </c>
       <c r="J311" t="n">
-        <v>1427</v>
+        <v>1439.1</v>
       </c>
       <c r="K311" t="n">
         <v>110</v>
@@ -37742,70 +37742,70 @@
         <v>96</v>
       </c>
       <c r="Q311" t="n">
-        <v>114.725</v>
+        <v>114.505</v>
       </c>
       <c r="R311" t="n">
-        <v>103.357</v>
+        <v>103.212</v>
       </c>
       <c r="S311" t="n">
-        <v>11.368</v>
+        <v>11.293</v>
       </c>
       <c r="T311" t="n">
-        <v>0.31301</v>
+        <v>0.31717</v>
       </c>
       <c r="U311" t="n">
-        <v>0.13936</v>
+        <v>0.139</v>
       </c>
       <c r="V311" t="n">
-        <v>75.23999999999999</v>
+        <v>75</v>
       </c>
       <c r="W311" t="n">
-        <v>67.95</v>
+        <v>67.73</v>
       </c>
       <c r="X311" t="n">
-        <v>0.7916</v>
+        <v>0.8083</v>
       </c>
       <c r="Y311" t="n">
-        <v>25.373</v>
+        <v>25.351</v>
       </c>
       <c r="Z311" t="n">
-        <v>57.363</v>
+        <v>57.851</v>
       </c>
       <c r="AA311" t="n">
-        <v>8.121</v>
+        <v>8.211</v>
       </c>
       <c r="AB311" t="n">
-        <v>22.594</v>
+        <v>22.742</v>
       </c>
       <c r="AC311" t="n">
-        <v>17.028</v>
+        <v>16.561</v>
       </c>
       <c r="AD311" t="n">
-        <v>24.403</v>
+        <v>23.903</v>
       </c>
       <c r="AE311" t="n">
-        <v>11.606</v>
+        <v>11.94</v>
       </c>
       <c r="AF311" t="n">
-        <v>25.031</v>
+        <v>25.167</v>
       </c>
       <c r="AG311" t="n">
-        <v>13.34</v>
+        <v>13.403</v>
       </c>
       <c r="AH311" t="n">
-        <v>5.109</v>
+        <v>5.054</v>
       </c>
       <c r="AI311" t="n">
-        <v>2.363</v>
+        <v>2.351</v>
       </c>
       <c r="AJ311" t="n">
-        <v>17.097</v>
+        <v>17.106</v>
       </c>
       <c r="AK311" t="n">
-        <v>5.8</v>
+        <v>5</v>
       </c>
       <c r="AL311" t="n">
-        <v>5.9</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="312">
@@ -37826,22 +37826,22 @@
         </is>
       </c>
       <c r="E312" t="n">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="F312" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G312" t="b">
         <v>1</v>
       </c>
       <c r="H312" t="n">
-        <v>1644.282</v>
+        <v>1662.23</v>
       </c>
       <c r="I312" t="n">
-        <v>1.7904</v>
+        <v>1.8215</v>
       </c>
       <c r="J312" t="n">
-        <v>1628.6</v>
+        <v>1625.4</v>
       </c>
       <c r="K312" t="n">
         <v>107</v>
@@ -37862,70 +37862,70 @@
         <v>111</v>
       </c>
       <c r="Q312" t="n">
-        <v>111.008</v>
+        <v>110.869</v>
       </c>
       <c r="R312" t="n">
-        <v>111.624</v>
+        <v>110.996</v>
       </c>
       <c r="S312" t="n">
-        <v>-0.616</v>
+        <v>-0.126</v>
       </c>
       <c r="T312" t="n">
-        <v>0.29551</v>
+        <v>0.29015</v>
       </c>
       <c r="U312" t="n">
-        <v>0.16541</v>
+        <v>0.16844</v>
       </c>
       <c r="V312" t="n">
-        <v>78.89</v>
+        <v>78.93000000000001</v>
       </c>
       <c r="W312" t="n">
-        <v>79.56999999999999</v>
+        <v>79.26000000000001</v>
       </c>
       <c r="X312" t="n">
-        <v>0.4946</v>
+        <v>0.52</v>
       </c>
       <c r="Y312" t="n">
-        <v>27.441</v>
+        <v>27.56</v>
       </c>
       <c r="Z312" t="n">
-        <v>58.452</v>
+        <v>58.32</v>
       </c>
       <c r="AA312" t="n">
-        <v>7.413</v>
+        <v>7.55</v>
       </c>
       <c r="AB312" t="n">
-        <v>21.022</v>
+        <v>21.12</v>
       </c>
       <c r="AC312" t="n">
-        <v>16.594</v>
+        <v>16.26</v>
       </c>
       <c r="AD312" t="n">
-        <v>24.305</v>
+        <v>23.95</v>
       </c>
       <c r="AE312" t="n">
-        <v>9.743</v>
+        <v>9.57</v>
       </c>
       <c r="AF312" t="n">
-        <v>22.794</v>
+        <v>23.03</v>
       </c>
       <c r="AG312" t="n">
-        <v>14.081</v>
+        <v>14.24</v>
       </c>
       <c r="AH312" t="n">
-        <v>7.257</v>
+        <v>7.23</v>
       </c>
       <c r="AI312" t="n">
-        <v>4.567</v>
+        <v>4.7</v>
       </c>
       <c r="AJ312" t="n">
-        <v>21.671</v>
+        <v>21.55</v>
       </c>
       <c r="AK312" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="AL312" t="n">
-        <v>2.6</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="313">
@@ -41186,22 +41186,22 @@
         </is>
       </c>
       <c r="E340" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F340" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G340" t="b">
         <v>1</v>
       </c>
       <c r="H340" t="n">
-        <v>1623.971</v>
+        <v>1632.359</v>
       </c>
       <c r="I340" t="n">
-        <v>1.8722</v>
+        <v>1.9753</v>
       </c>
       <c r="J340" t="n">
-        <v>1546.5</v>
+        <v>1543.7</v>
       </c>
       <c r="K340" t="n">
         <v>82</v>
@@ -41222,70 +41222,70 @@
         <v>78</v>
       </c>
       <c r="Q340" t="n">
-        <v>111.577</v>
+        <v>111.467</v>
       </c>
       <c r="R340" t="n">
-        <v>102.283</v>
+        <v>101.995</v>
       </c>
       <c r="S340" t="n">
-        <v>9.295</v>
+        <v>9.473000000000001</v>
       </c>
       <c r="T340" t="n">
-        <v>0.34458</v>
+        <v>0.34362</v>
       </c>
       <c r="U340" t="n">
-        <v>0.14529</v>
+        <v>0.14702</v>
       </c>
       <c r="V340" t="n">
-        <v>76.86</v>
+        <v>76.97</v>
       </c>
       <c r="W340" t="n">
-        <v>70.45999999999999</v>
+        <v>70.45</v>
       </c>
       <c r="X340" t="n">
-        <v>0.6492</v>
+        <v>0.67</v>
       </c>
       <c r="Y340" t="n">
-        <v>27.161</v>
+        <v>27.28</v>
       </c>
       <c r="Z340" t="n">
-        <v>62.214</v>
+        <v>62.39</v>
       </c>
       <c r="AA340" t="n">
-        <v>7.091</v>
+        <v>7.04</v>
       </c>
       <c r="AB340" t="n">
-        <v>21.226</v>
+        <v>21.12</v>
       </c>
       <c r="AC340" t="n">
-        <v>15.442</v>
+        <v>15.37</v>
       </c>
       <c r="AD340" t="n">
-        <v>22.473</v>
+        <v>22.52</v>
       </c>
       <c r="AE340" t="n">
-        <v>13.267</v>
+        <v>13.43</v>
       </c>
       <c r="AF340" t="n">
-        <v>25.187</v>
+        <v>25.67</v>
       </c>
       <c r="AG340" t="n">
-        <v>11.401</v>
+        <v>11.42</v>
       </c>
       <c r="AH340" t="n">
-        <v>6.103</v>
+        <v>6.01</v>
       </c>
       <c r="AI340" t="n">
-        <v>4.032</v>
+        <v>3.92</v>
       </c>
       <c r="AJ340" t="n">
-        <v>17.578</v>
+        <v>17.46</v>
       </c>
       <c r="AK340" t="n">
-        <v>7.8</v>
+        <v>7.4</v>
       </c>
       <c r="AL340" t="n">
-        <v>6.4</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="341">
@@ -41906,22 +41906,22 @@
         </is>
       </c>
       <c r="E346" t="n">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="F346" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G346" t="b">
         <v>1</v>
       </c>
       <c r="H346" t="n">
-        <v>1521.064</v>
+        <v>1512.677</v>
       </c>
       <c r="I346" t="n">
-        <v>-0.1434</v>
+        <v>-0.07820000000000001</v>
       </c>
       <c r="J346" t="n">
-        <v>1563.6</v>
+        <v>1565.2</v>
       </c>
       <c r="K346" t="n">
         <v>98</v>
@@ -41942,70 +41942,70 @@
         <v>99</v>
       </c>
       <c r="Q346" t="n">
-        <v>113.423</v>
+        <v>112.648</v>
       </c>
       <c r="R346" t="n">
-        <v>109.184</v>
+        <v>108.708</v>
       </c>
       <c r="S346" t="n">
-        <v>4.239</v>
+        <v>3.94</v>
       </c>
       <c r="T346" t="n">
-        <v>0.32866</v>
+        <v>0.3246</v>
       </c>
       <c r="U346" t="n">
-        <v>0.15531</v>
+        <v>0.15516</v>
       </c>
       <c r="V346" t="n">
-        <v>76.33</v>
+        <v>76.13</v>
       </c>
       <c r="W346" t="n">
-        <v>72.90000000000001</v>
+        <v>72.95</v>
       </c>
       <c r="X346" t="n">
-        <v>0.5431</v>
+        <v>0.5265</v>
       </c>
       <c r="Y346" t="n">
-        <v>26.256</v>
+        <v>26.208</v>
       </c>
       <c r="Z346" t="n">
-        <v>58.532</v>
+        <v>58.683</v>
       </c>
       <c r="AA346" t="n">
-        <v>8.207000000000001</v>
+        <v>8.327999999999999</v>
       </c>
       <c r="AB346" t="n">
-        <v>25.089</v>
+        <v>25.244</v>
       </c>
       <c r="AC346" t="n">
-        <v>15.607</v>
+        <v>15.388</v>
       </c>
       <c r="AD346" t="n">
-        <v>20.799</v>
+        <v>20.774</v>
       </c>
       <c r="AE346" t="n">
-        <v>10.874</v>
+        <v>10.703</v>
       </c>
       <c r="AF346" t="n">
-        <v>22.287</v>
+        <v>22.399</v>
       </c>
       <c r="AG346" t="n">
-        <v>13.939</v>
+        <v>14.129</v>
       </c>
       <c r="AH346" t="n">
-        <v>6.376</v>
+        <v>6.603</v>
       </c>
       <c r="AI346" t="n">
-        <v>2.351</v>
+        <v>2.381</v>
       </c>
       <c r="AJ346" t="n">
-        <v>21.096</v>
+        <v>21.173</v>
       </c>
       <c r="AK346" t="n">
-        <v>2.2</v>
+        <v>3.4</v>
       </c>
       <c r="AL346" t="n">
-        <v>0.4</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="347">
@@ -42146,22 +42146,22 @@
         </is>
       </c>
       <c r="E348" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F348" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G348" t="b">
         <v>1</v>
       </c>
       <c r="H348" t="n">
-        <v>1684.172</v>
+        <v>1681.756</v>
       </c>
       <c r="I348" t="n">
-        <v>0.9762999999999999</v>
+        <v>0.8274</v>
       </c>
       <c r="J348" t="n">
-        <v>1457.5</v>
+        <v>1468</v>
       </c>
       <c r="K348" t="n">
         <v>81</v>
@@ -42182,70 +42182,70 @@
         <v>68</v>
       </c>
       <c r="Q348" t="n">
-        <v>121.507</v>
+        <v>120.747</v>
       </c>
       <c r="R348" t="n">
-        <v>108.892</v>
+        <v>108.547</v>
       </c>
       <c r="S348" t="n">
-        <v>12.615</v>
+        <v>12.199</v>
       </c>
       <c r="T348" t="n">
-        <v>0.29055</v>
+        <v>0.29606</v>
       </c>
       <c r="U348" t="n">
-        <v>0.13803</v>
+        <v>0.13678</v>
       </c>
       <c r="V348" t="n">
-        <v>80.66</v>
+        <v>79.95999999999999</v>
       </c>
       <c r="W348" t="n">
-        <v>72.2</v>
+        <v>71.78</v>
       </c>
       <c r="X348" t="n">
-        <v>0.7741</v>
+        <v>0.7483</v>
       </c>
       <c r="Y348" t="n">
-        <v>28.331</v>
+        <v>28.163</v>
       </c>
       <c r="Z348" t="n">
-        <v>57.843</v>
+        <v>58.19</v>
       </c>
       <c r="AA348" t="n">
-        <v>8.581</v>
+        <v>8.476000000000001</v>
       </c>
       <c r="AB348" t="n">
-        <v>21.104</v>
+        <v>21.286</v>
       </c>
       <c r="AC348" t="n">
-        <v>15.613</v>
+        <v>15.293</v>
       </c>
       <c r="AD348" t="n">
-        <v>20.328</v>
+        <v>20.469</v>
       </c>
       <c r="AE348" t="n">
-        <v>9.557</v>
+        <v>10.034</v>
       </c>
       <c r="AF348" t="n">
-        <v>23.15</v>
+        <v>23.388</v>
       </c>
       <c r="AG348" t="n">
-        <v>15.628</v>
+        <v>15.626</v>
       </c>
       <c r="AH348" t="n">
-        <v>5.211</v>
+        <v>5.204</v>
       </c>
       <c r="AI348" t="n">
-        <v>3.12</v>
+        <v>3.197</v>
       </c>
       <c r="AJ348" t="n">
-        <v>16.106</v>
+        <v>16.054</v>
       </c>
       <c r="AK348" t="n">
-        <v>7.2</v>
+        <v>7.6</v>
       </c>
       <c r="AL348" t="n">
-        <v>7.2</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="349">
@@ -43226,22 +43226,22 @@
         </is>
       </c>
       <c r="E357" t="n">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="F357" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G357" t="b">
         <v>1</v>
       </c>
       <c r="H357" t="n">
-        <v>1562.594</v>
+        <v>1550.552</v>
       </c>
       <c r="I357" t="n">
-        <v>2.9745</v>
+        <v>2.8057</v>
       </c>
       <c r="J357" t="n">
-        <v>1395</v>
+        <v>1402</v>
       </c>
       <c r="K357" t="n">
         <v>109</v>
@@ -43262,70 +43262,70 @@
         <v>103</v>
       </c>
       <c r="Q357" t="n">
-        <v>117.765</v>
+        <v>116.064</v>
       </c>
       <c r="R357" t="n">
-        <v>105.683</v>
+        <v>105.279</v>
       </c>
       <c r="S357" t="n">
-        <v>12.082</v>
+        <v>10.785</v>
       </c>
       <c r="T357" t="n">
-        <v>0.17386</v>
+        <v>0.17931</v>
       </c>
       <c r="U357" t="n">
-        <v>0.13275</v>
+        <v>0.14</v>
       </c>
       <c r="V357" t="n">
-        <v>81.67</v>
+        <v>80.56999999999999</v>
       </c>
       <c r="W357" t="n">
-        <v>73.22</v>
+        <v>73.03</v>
       </c>
       <c r="X357" t="n">
-        <v>0.6912</v>
+        <v>0.6696</v>
       </c>
       <c r="Y357" t="n">
-        <v>29.077</v>
+        <v>28.812</v>
       </c>
       <c r="Z357" t="n">
-        <v>56.738</v>
+        <v>56.861</v>
       </c>
       <c r="AA357" t="n">
-        <v>9.798</v>
+        <v>9.622999999999999</v>
       </c>
       <c r="AB357" t="n">
-        <v>26.472</v>
+        <v>26.368</v>
       </c>
       <c r="AC357" t="n">
-        <v>13.762</v>
+        <v>13.354</v>
       </c>
       <c r="AD357" t="n">
-        <v>20.042</v>
+        <v>19.446</v>
       </c>
       <c r="AE357" t="n">
-        <v>5.476</v>
+        <v>5.771</v>
       </c>
       <c r="AF357" t="n">
-        <v>24.165</v>
+        <v>24.464</v>
       </c>
       <c r="AG357" t="n">
-        <v>16.406</v>
+        <v>16.13</v>
       </c>
       <c r="AH357" t="n">
-        <v>7.436</v>
+        <v>7.403</v>
       </c>
       <c r="AI357" t="n">
-        <v>2.613</v>
+        <v>2.606</v>
       </c>
       <c r="AJ357" t="n">
-        <v>16.149</v>
+        <v>16.183</v>
       </c>
       <c r="AK357" t="n">
-        <v>9.4</v>
+        <v>6.8</v>
       </c>
       <c r="AL357" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="358">

</xml_diff>

<commit_message>
Update team snapshot (2026-03-19)
</commit_message>
<xml_diff>
--- a/team_snapshot_2026.xlsx
+++ b/team_snapshot_2026.xlsx
@@ -3986,22 +3986,22 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="F30" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G30" t="b">
         <v>1</v>
       </c>
       <c r="H30" t="n">
-        <v>1617.146</v>
+        <v>1599.461</v>
       </c>
       <c r="I30" t="n">
-        <v>1.2181</v>
+        <v>1.0977</v>
       </c>
       <c r="J30" t="n">
-        <v>1524.5</v>
+        <v>1530.5</v>
       </c>
       <c r="K30" t="n">
         <v>123</v>
@@ -4022,70 +4022,70 @@
         <v>113</v>
       </c>
       <c r="Q30" t="n">
-        <v>110.424</v>
+        <v>110.575</v>
       </c>
       <c r="R30" t="n">
-        <v>106.062</v>
+        <v>107.267</v>
       </c>
       <c r="S30" t="n">
-        <v>4.362</v>
+        <v>3.308</v>
       </c>
       <c r="T30" t="n">
-        <v>0.26313</v>
+        <v>0.26698</v>
       </c>
       <c r="U30" t="n">
-        <v>0.13661</v>
+        <v>0.13706</v>
       </c>
       <c r="V30" t="n">
-        <v>77.20999999999999</v>
+        <v>76.84</v>
       </c>
       <c r="W30" t="n">
-        <v>74.02</v>
+        <v>74.28</v>
       </c>
       <c r="X30" t="n">
-        <v>0.6171</v>
+        <v>0.599</v>
       </c>
       <c r="Y30" t="n">
-        <v>26.501</v>
+        <v>26.324</v>
       </c>
       <c r="Z30" t="n">
-        <v>59.551</v>
+        <v>59.385</v>
       </c>
       <c r="AA30" t="n">
-        <v>8.592000000000001</v>
+        <v>8.682</v>
       </c>
       <c r="AB30" t="n">
-        <v>23.687</v>
+        <v>23.797</v>
       </c>
       <c r="AC30" t="n">
-        <v>15.788</v>
+        <v>15.63</v>
       </c>
       <c r="AD30" t="n">
-        <v>21.511</v>
+        <v>21.277</v>
       </c>
       <c r="AE30" t="n">
-        <v>8.497999999999999</v>
+        <v>8.611000000000001</v>
       </c>
       <c r="AF30" t="n">
-        <v>23.401</v>
+        <v>23.348</v>
       </c>
       <c r="AG30" t="n">
-        <v>13.377</v>
+        <v>13.329</v>
       </c>
       <c r="AH30" t="n">
-        <v>7.617</v>
+        <v>7.307</v>
       </c>
       <c r="AI30" t="n">
-        <v>3.16</v>
+        <v>3.18</v>
       </c>
       <c r="AJ30" t="n">
-        <v>18.864</v>
+        <v>18.88</v>
       </c>
       <c r="AK30" t="n">
-        <v>3.6</v>
+        <v>-2</v>
       </c>
       <c r="AL30" t="n">
-        <v>2.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="31">
@@ -5066,22 +5066,22 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="F39" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G39" t="b">
         <v>1</v>
       </c>
       <c r="H39" t="n">
-        <v>1703.272</v>
+        <v>1710.414</v>
       </c>
       <c r="I39" t="n">
-        <v>7.292</v>
+        <v>6.8262</v>
       </c>
       <c r="J39" t="n">
-        <v>1603.7</v>
+        <v>1600.4</v>
       </c>
       <c r="K39" t="n">
         <v>73</v>
@@ -5102,70 +5102,70 @@
         <v>67</v>
       </c>
       <c r="Q39" t="n">
-        <v>110.159</v>
+        <v>110.668</v>
       </c>
       <c r="R39" t="n">
-        <v>104.763</v>
+        <v>104.285</v>
       </c>
       <c r="S39" t="n">
-        <v>5.396</v>
+        <v>6.383</v>
       </c>
       <c r="T39" t="n">
-        <v>0.23512</v>
+        <v>0.23394</v>
       </c>
       <c r="U39" t="n">
-        <v>0.14496</v>
+        <v>0.14794</v>
       </c>
       <c r="V39" t="n">
-        <v>77.52</v>
+        <v>77.95</v>
       </c>
       <c r="W39" t="n">
-        <v>73.56999999999999</v>
+        <v>73.31</v>
       </c>
       <c r="X39" t="n">
-        <v>0.6377</v>
+        <v>0.6599</v>
       </c>
       <c r="Y39" t="n">
-        <v>25.867</v>
+        <v>26.065</v>
       </c>
       <c r="Z39" t="n">
-        <v>58.099</v>
+        <v>58.02</v>
       </c>
       <c r="AA39" t="n">
-        <v>9.023</v>
+        <v>9.25</v>
       </c>
       <c r="AB39" t="n">
-        <v>24.832</v>
+        <v>24.94</v>
       </c>
       <c r="AC39" t="n">
-        <v>16.765</v>
+        <v>16.575</v>
       </c>
       <c r="AD39" t="n">
-        <v>21.704</v>
+        <v>21.274</v>
       </c>
       <c r="AE39" t="n">
-        <v>7.603</v>
+        <v>7.495</v>
       </c>
       <c r="AF39" t="n">
-        <v>24.339</v>
+        <v>24.215</v>
       </c>
       <c r="AG39" t="n">
-        <v>13.838</v>
+        <v>14.168</v>
       </c>
       <c r="AH39" t="n">
-        <v>5.678</v>
+        <v>5.888</v>
       </c>
       <c r="AI39" t="n">
-        <v>3.128</v>
+        <v>2.999</v>
       </c>
       <c r="AJ39" t="n">
-        <v>19.009</v>
+        <v>18.864</v>
       </c>
       <c r="AK39" t="n">
-        <v>-2.8</v>
+        <v>0</v>
       </c>
       <c r="AL39" t="n">
-        <v>-2.1</v>
+        <v>-0.8</v>
       </c>
     </row>
     <row r="40">
@@ -7106,22 +7106,22 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="F56" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G56" t="b">
         <v>1</v>
       </c>
       <c r="H56" t="n">
-        <v>1655.821</v>
+        <v>1633.654</v>
       </c>
       <c r="I56" t="n">
-        <v>-4.6276</v>
+        <v>-4.3855</v>
       </c>
       <c r="J56" t="n">
-        <v>1564.6</v>
+        <v>1564.1</v>
       </c>
       <c r="K56" t="n">
         <v>88</v>
@@ -7142,70 +7142,70 @@
         <v>87</v>
       </c>
       <c r="Q56" t="n">
-        <v>117.701</v>
+        <v>117.184</v>
       </c>
       <c r="R56" t="n">
-        <v>112.562</v>
+        <v>112.366</v>
       </c>
       <c r="S56" t="n">
-        <v>5.14</v>
+        <v>4.819</v>
       </c>
       <c r="T56" t="n">
-        <v>0.26372</v>
+        <v>0.26623</v>
       </c>
       <c r="U56" t="n">
-        <v>0.17614</v>
+        <v>0.17522</v>
       </c>
       <c r="V56" t="n">
-        <v>75.05</v>
+        <v>74.73999999999999</v>
       </c>
       <c r="W56" t="n">
-        <v>71.65000000000001</v>
+        <v>71.55</v>
       </c>
       <c r="X56" t="n">
-        <v>0.6183</v>
+        <v>0.6</v>
       </c>
       <c r="Y56" t="n">
-        <v>24.781</v>
+        <v>24.69</v>
       </c>
       <c r="Z56" t="n">
-        <v>51.374</v>
+        <v>51.58</v>
       </c>
       <c r="AA56" t="n">
-        <v>9.878</v>
+        <v>9.73</v>
       </c>
       <c r="AB56" t="n">
-        <v>25.251</v>
+        <v>25.35</v>
       </c>
       <c r="AC56" t="n">
-        <v>15.606</v>
+        <v>15.63</v>
       </c>
       <c r="AD56" t="n">
-        <v>20.234</v>
+        <v>20.3</v>
       </c>
       <c r="AE56" t="n">
-        <v>7.763</v>
+        <v>7.92</v>
       </c>
       <c r="AF56" t="n">
-        <v>22.124</v>
+        <v>22.2</v>
       </c>
       <c r="AG56" t="n">
-        <v>15.595</v>
+        <v>15.51</v>
       </c>
       <c r="AH56" t="n">
-        <v>5.185</v>
+        <v>5.22</v>
       </c>
       <c r="AI56" t="n">
-        <v>2.155</v>
+        <v>2.15</v>
       </c>
       <c r="AJ56" t="n">
-        <v>16.984</v>
+        <v>16.92</v>
       </c>
       <c r="AK56" t="n">
-        <v>0.8</v>
+        <v>-2.6</v>
       </c>
       <c r="AL56" t="n">
-        <v>5</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="57">
@@ -8546,22 +8546,22 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="F68" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G68" t="b">
         <v>1</v>
       </c>
       <c r="H68" t="n">
-        <v>1677.744</v>
+        <v>1695.429</v>
       </c>
       <c r="I68" t="n">
-        <v>-1.9174</v>
+        <v>-1.7367</v>
       </c>
       <c r="J68" t="n">
-        <v>1574.7</v>
+        <v>1574.5</v>
       </c>
       <c r="K68" t="n">
         <v>78</v>
@@ -8582,70 +8582,70 @@
         <v>69</v>
       </c>
       <c r="Q68" t="n">
-        <v>109.173</v>
+        <v>110.224</v>
       </c>
       <c r="R68" t="n">
-        <v>102.25</v>
+        <v>102.463</v>
       </c>
       <c r="S68" t="n">
-        <v>6.923</v>
+        <v>7.761</v>
       </c>
       <c r="T68" t="n">
-        <v>0.25145</v>
+        <v>0.24689</v>
       </c>
       <c r="U68" t="n">
-        <v>0.17261</v>
+        <v>0.16853</v>
       </c>
       <c r="V68" t="n">
-        <v>74.22</v>
+        <v>74.56999999999999</v>
       </c>
       <c r="W68" t="n">
-        <v>69.88</v>
+        <v>69.73</v>
       </c>
       <c r="X68" t="n">
-        <v>0.6691</v>
+        <v>0.6889</v>
       </c>
       <c r="Y68" t="n">
-        <v>23.989</v>
+        <v>24.038</v>
       </c>
       <c r="Z68" t="n">
-        <v>53.465</v>
+        <v>53.26</v>
       </c>
       <c r="AA68" t="n">
-        <v>7.64</v>
+        <v>7.699</v>
       </c>
       <c r="AB68" t="n">
-        <v>22.338</v>
+        <v>22.186</v>
       </c>
       <c r="AC68" t="n">
-        <v>18.571</v>
+        <v>18.766</v>
       </c>
       <c r="AD68" t="n">
-        <v>24.796</v>
+        <v>24.887</v>
       </c>
       <c r="AE68" t="n">
-        <v>7.942</v>
+        <v>7.751</v>
       </c>
       <c r="AF68" t="n">
-        <v>23.233</v>
+        <v>23.103</v>
       </c>
       <c r="AG68" t="n">
-        <v>14.4</v>
+        <v>14.291</v>
       </c>
       <c r="AH68" t="n">
-        <v>8.148999999999999</v>
+        <v>8.083</v>
       </c>
       <c r="AI68" t="n">
-        <v>4.145</v>
+        <v>4.064</v>
       </c>
       <c r="AJ68" t="n">
-        <v>16.865</v>
+        <v>16.82</v>
       </c>
       <c r="AK68" t="n">
-        <v>-0.6</v>
+        <v>1.2</v>
       </c>
       <c r="AL68" t="n">
-        <v>5.2</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="69">
@@ -12146,22 +12146,22 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="F98" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G98" t="b">
         <v>1</v>
       </c>
       <c r="H98" t="n">
-        <v>1525.82</v>
+        <v>1546.505</v>
       </c>
       <c r="I98" t="n">
-        <v>-3.7537</v>
+        <v>-3.6146</v>
       </c>
       <c r="J98" t="n">
-        <v>1543.4</v>
+        <v>1543.8</v>
       </c>
       <c r="K98" t="n">
         <v>85</v>
@@ -12185,67 +12185,67 @@
         <v>114.986</v>
       </c>
       <c r="R98" t="n">
-        <v>105.766</v>
+        <v>105.859</v>
       </c>
       <c r="S98" t="n">
-        <v>9.220000000000001</v>
+        <v>9.127000000000001</v>
       </c>
       <c r="T98" t="n">
-        <v>0.32427</v>
+        <v>0.32167</v>
       </c>
       <c r="U98" t="n">
-        <v>0.17282</v>
+        <v>0.17626</v>
       </c>
       <c r="V98" t="n">
-        <v>81.59</v>
+        <v>81.48999999999999</v>
       </c>
       <c r="W98" t="n">
-        <v>74.95</v>
+        <v>74.92</v>
       </c>
       <c r="X98" t="n">
-        <v>0.5245</v>
+        <v>0.5508</v>
       </c>
       <c r="Y98" t="n">
-        <v>28.123</v>
+        <v>28.036</v>
       </c>
       <c r="Z98" t="n">
-        <v>60.651</v>
+        <v>60.217</v>
       </c>
       <c r="AA98" t="n">
-        <v>9.914</v>
+        <v>9.922000000000001</v>
       </c>
       <c r="AB98" t="n">
-        <v>28.262</v>
+        <v>27.995</v>
       </c>
       <c r="AC98" t="n">
-        <v>15.302</v>
+        <v>15.371</v>
       </c>
       <c r="AD98" t="n">
-        <v>21.327</v>
+        <v>21.246</v>
       </c>
       <c r="AE98" t="n">
-        <v>11.433</v>
+        <v>11.276</v>
       </c>
       <c r="AF98" t="n">
-        <v>23.488</v>
+        <v>23.449</v>
       </c>
       <c r="AG98" t="n">
-        <v>15.309</v>
+        <v>15.424</v>
       </c>
       <c r="AH98" t="n">
-        <v>7.407</v>
+        <v>7.461</v>
       </c>
       <c r="AI98" t="n">
-        <v>3.203</v>
+        <v>3.335</v>
       </c>
       <c r="AJ98" t="n">
         <v>18.161</v>
       </c>
       <c r="AK98" t="n">
-        <v>-0.4</v>
+        <v>0.2</v>
       </c>
       <c r="AL98" t="n">
-        <v>3.3</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="99">
@@ -14786,22 +14786,22 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="F120" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G120" t="b">
         <v>1</v>
       </c>
       <c r="H120" t="n">
-        <v>1528.61</v>
+        <v>1521.468</v>
       </c>
       <c r="I120" t="n">
-        <v>2.2588</v>
+        <v>2.3348</v>
       </c>
       <c r="J120" t="n">
-        <v>1508.7</v>
+        <v>1515.5</v>
       </c>
       <c r="K120" t="n">
         <v>105</v>
@@ -14822,70 +14822,70 @@
         <v>110</v>
       </c>
       <c r="Q120" t="n">
-        <v>108.828</v>
+        <v>108.58</v>
       </c>
       <c r="R120" t="n">
-        <v>104.272</v>
+        <v>104.924</v>
       </c>
       <c r="S120" t="n">
-        <v>4.556</v>
+        <v>3.656</v>
       </c>
       <c r="T120" t="n">
-        <v>0.34057</v>
+        <v>0.33986</v>
       </c>
       <c r="U120" t="n">
-        <v>0.16472</v>
+        <v>0.16596</v>
       </c>
       <c r="V120" t="n">
         <v>73.93000000000001</v>
       </c>
       <c r="W120" t="n">
-        <v>70.72</v>
+        <v>71.38</v>
       </c>
       <c r="X120" t="n">
-        <v>0.5273</v>
+        <v>0.5116000000000001</v>
       </c>
       <c r="Y120" t="n">
-        <v>25.944</v>
+        <v>26.021</v>
       </c>
       <c r="Z120" t="n">
-        <v>58.305</v>
+        <v>58.324</v>
       </c>
       <c r="AA120" t="n">
-        <v>6.448</v>
+        <v>6.317</v>
       </c>
       <c r="AB120" t="n">
-        <v>19.867</v>
+        <v>19.664</v>
       </c>
       <c r="AC120" t="n">
-        <v>15.769</v>
+        <v>15.634</v>
       </c>
       <c r="AD120" t="n">
-        <v>21.778</v>
+        <v>21.627</v>
       </c>
       <c r="AE120" t="n">
-        <v>11.125</v>
+        <v>11.039</v>
       </c>
       <c r="AF120" t="n">
-        <v>21.947</v>
+        <v>21.822</v>
       </c>
       <c r="AG120" t="n">
-        <v>14.175</v>
+        <v>14.35</v>
       </c>
       <c r="AH120" t="n">
-        <v>7.622</v>
+        <v>7.558</v>
       </c>
       <c r="AI120" t="n">
-        <v>3.79</v>
+        <v>3.826</v>
       </c>
       <c r="AJ120" t="n">
-        <v>17.04</v>
+        <v>16.949</v>
       </c>
       <c r="AK120" t="n">
-        <v>2</v>
+        <v>-3</v>
       </c>
       <c r="AL120" t="n">
-        <v>7.5</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="121">
@@ -15026,22 +15026,22 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>123</v>
+        <v>135</v>
       </c>
       <c r="F122" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G122" t="b">
         <v>1</v>
       </c>
       <c r="H122" t="n">
-        <v>1580.626</v>
+        <v>1594.577</v>
       </c>
       <c r="I122" t="n">
-        <v>2.2563</v>
+        <v>2.1793</v>
       </c>
       <c r="J122" t="n">
-        <v>1504.8</v>
+        <v>1508.2</v>
       </c>
       <c r="K122" t="n">
         <v>103</v>
@@ -15062,70 +15062,70 @@
         <v>95</v>
       </c>
       <c r="Q122" t="n">
-        <v>109.572</v>
+        <v>110.094</v>
       </c>
       <c r="R122" t="n">
-        <v>102.175</v>
+        <v>101.357</v>
       </c>
       <c r="S122" t="n">
-        <v>7.397</v>
+        <v>8.738</v>
       </c>
       <c r="T122" t="n">
-        <v>0.25789</v>
+        <v>0.25529</v>
       </c>
       <c r="U122" t="n">
-        <v>0.16388</v>
+        <v>0.15942</v>
       </c>
       <c r="V122" t="n">
-        <v>74.33</v>
+        <v>74.73</v>
       </c>
       <c r="W122" t="n">
-        <v>69.14</v>
+        <v>68.65000000000001</v>
       </c>
       <c r="X122" t="n">
-        <v>0.6069</v>
+        <v>0.6284</v>
       </c>
       <c r="Y122" t="n">
-        <v>27.019</v>
+        <v>27</v>
       </c>
       <c r="Z122" t="n">
-        <v>57.674</v>
+        <v>57.961</v>
       </c>
       <c r="AA122" t="n">
-        <v>8.638999999999999</v>
+        <v>8.819000000000001</v>
       </c>
       <c r="AB122" t="n">
-        <v>24.303</v>
+        <v>24.781</v>
       </c>
       <c r="AC122" t="n">
-        <v>12.568</v>
+        <v>12.588</v>
       </c>
       <c r="AD122" t="n">
-        <v>17.676</v>
+        <v>17.752</v>
       </c>
       <c r="AE122" t="n">
-        <v>8.638999999999999</v>
+        <v>8.619</v>
       </c>
       <c r="AF122" t="n">
-        <v>25.051</v>
+        <v>25.431</v>
       </c>
       <c r="AG122" t="n">
-        <v>13.812</v>
+        <v>14.032</v>
       </c>
       <c r="AH122" t="n">
-        <v>5.565</v>
+        <v>5.637</v>
       </c>
       <c r="AI122" t="n">
-        <v>2.233</v>
+        <v>2.257</v>
       </c>
       <c r="AJ122" t="n">
-        <v>17.429</v>
+        <v>17.221</v>
       </c>
       <c r="AK122" t="n">
-        <v>-2</v>
+        <v>-1.2</v>
       </c>
       <c r="AL122" t="n">
-        <v>-1.7</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="123">
@@ -16946,22 +16946,22 @@
         </is>
       </c>
       <c r="E138" t="n">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="F138" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G138" t="b">
         <v>1</v>
       </c>
       <c r="H138" t="n">
-        <v>1600.738</v>
+        <v>1586.787</v>
       </c>
       <c r="I138" t="n">
-        <v>0.115</v>
+        <v>0.0072</v>
       </c>
       <c r="J138" t="n">
-        <v>1479</v>
+        <v>1481</v>
       </c>
       <c r="K138" t="n">
         <v>148</v>
@@ -16982,70 +16982,70 @@
         <v>141</v>
       </c>
       <c r="Q138" t="n">
-        <v>112.171</v>
+        <v>111.134</v>
       </c>
       <c r="R138" t="n">
-        <v>109.176</v>
+        <v>109.344</v>
       </c>
       <c r="S138" t="n">
-        <v>2.995</v>
+        <v>1.79</v>
       </c>
       <c r="T138" t="n">
-        <v>0.32353</v>
+        <v>0.31864</v>
       </c>
       <c r="U138" t="n">
-        <v>0.17631</v>
+        <v>0.17543</v>
       </c>
       <c r="V138" t="n">
-        <v>82.89</v>
+        <v>82.03</v>
       </c>
       <c r="W138" t="n">
-        <v>80.62</v>
+        <v>80.61</v>
       </c>
       <c r="X138" t="n">
-        <v>0.7028</v>
+        <v>0.6813</v>
       </c>
       <c r="Y138" t="n">
-        <v>26.612</v>
+        <v>26.45</v>
       </c>
       <c r="Z138" t="n">
-        <v>60.812</v>
+        <v>60.872</v>
       </c>
       <c r="AA138" t="n">
-        <v>9.619</v>
+        <v>9.539</v>
       </c>
       <c r="AB138" t="n">
-        <v>27.319</v>
+        <v>27.35</v>
       </c>
       <c r="AC138" t="n">
-        <v>20.042</v>
+        <v>19.591</v>
       </c>
       <c r="AD138" t="n">
-        <v>26.917</v>
+        <v>26.338</v>
       </c>
       <c r="AE138" t="n">
-        <v>11.864</v>
+        <v>11.703</v>
       </c>
       <c r="AF138" t="n">
-        <v>24.425</v>
+        <v>24.763</v>
       </c>
       <c r="AG138" t="n">
-        <v>14.999</v>
+        <v>15.133</v>
       </c>
       <c r="AH138" t="n">
-        <v>6.671</v>
+        <v>6.49</v>
       </c>
       <c r="AI138" t="n">
-        <v>3.268</v>
+        <v>3.239</v>
       </c>
       <c r="AJ138" t="n">
-        <v>20.135</v>
+        <v>19.933</v>
       </c>
       <c r="AK138" t="n">
-        <v>3.2</v>
+        <v>3.4</v>
       </c>
       <c r="AL138" t="n">
-        <v>3.5</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="139">
@@ -17546,22 +17546,22 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="F143" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G143" t="b">
         <v>1</v>
       </c>
       <c r="H143" t="n">
-        <v>1325.524</v>
+        <v>1320.16</v>
       </c>
       <c r="I143" t="n">
-        <v>-0.465</v>
+        <v>-0.3498</v>
       </c>
       <c r="J143" t="n">
-        <v>1399</v>
+        <v>1394.1</v>
       </c>
       <c r="K143" t="n">
         <v>284</v>
@@ -17582,70 +17582,70 @@
         <v>275</v>
       </c>
       <c r="Q143" t="n">
-        <v>105.584</v>
+        <v>104.495</v>
       </c>
       <c r="R143" t="n">
-        <v>108.389</v>
+        <v>108.288</v>
       </c>
       <c r="S143" t="n">
-        <v>-2.804</v>
+        <v>-3.793</v>
       </c>
       <c r="T143" t="n">
-        <v>0.22286</v>
+        <v>0.22012</v>
       </c>
       <c r="U143" t="n">
-        <v>0.17072</v>
+        <v>0.17007</v>
       </c>
       <c r="V143" t="n">
-        <v>72.40000000000001</v>
+        <v>71.65000000000001</v>
       </c>
       <c r="W143" t="n">
-        <v>74.47</v>
+        <v>74.34</v>
       </c>
       <c r="X143" t="n">
-        <v>0.5063</v>
+        <v>0.4792</v>
       </c>
       <c r="Y143" t="n">
-        <v>25.759</v>
+        <v>25.832</v>
       </c>
       <c r="Z143" t="n">
-        <v>55.648</v>
+        <v>55.712</v>
       </c>
       <c r="AA143" t="n">
-        <v>7.766</v>
+        <v>7.552</v>
       </c>
       <c r="AB143" t="n">
-        <v>21.222</v>
+        <v>20.74</v>
       </c>
       <c r="AC143" t="n">
-        <v>13.112</v>
+        <v>12.935</v>
       </c>
       <c r="AD143" t="n">
-        <v>17.983</v>
+        <v>17.66</v>
       </c>
       <c r="AE143" t="n">
-        <v>6.564</v>
+        <v>6.491</v>
       </c>
       <c r="AF143" t="n">
-        <v>22.432</v>
+        <v>22.628</v>
       </c>
       <c r="AG143" t="n">
-        <v>13.987</v>
+        <v>13.625</v>
       </c>
       <c r="AH143" t="n">
-        <v>6.635</v>
+        <v>6.879</v>
       </c>
       <c r="AI143" t="n">
-        <v>3.161</v>
+        <v>3.37</v>
       </c>
       <c r="AJ143" t="n">
-        <v>16.136</v>
+        <v>15.911</v>
       </c>
       <c r="AK143" t="n">
-        <v>7.8</v>
+        <v>4.4</v>
       </c>
       <c r="AL143" t="n">
-        <v>2.7</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="144">
@@ -20546,22 +20546,22 @@
         </is>
       </c>
       <c r="E168" t="n">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="F168" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G168" t="b">
         <v>1</v>
       </c>
       <c r="H168" t="n">
-        <v>1758.619</v>
+        <v>1780.382</v>
       </c>
       <c r="I168" t="n">
-        <v>9.362500000000001</v>
+        <v>8.9497</v>
       </c>
       <c r="J168" t="n">
-        <v>1416.9</v>
+        <v>1429.2</v>
       </c>
       <c r="K168" t="n">
         <v>93</v>
@@ -20582,70 +20582,70 @@
         <v>64</v>
       </c>
       <c r="Q168" t="n">
-        <v>120.742</v>
+        <v>121.342</v>
       </c>
       <c r="R168" t="n">
-        <v>105.875</v>
+        <v>106.311</v>
       </c>
       <c r="S168" t="n">
-        <v>14.867</v>
+        <v>15.031</v>
       </c>
       <c r="T168" t="n">
-        <v>0.21861</v>
+        <v>0.22217</v>
       </c>
       <c r="U168" t="n">
-        <v>0.14132</v>
+        <v>0.1392</v>
       </c>
       <c r="V168" t="n">
-        <v>87.18000000000001</v>
+        <v>87.28</v>
       </c>
       <c r="W168" t="n">
-        <v>76.42</v>
+        <v>76.45</v>
       </c>
       <c r="X168" t="n">
-        <v>0.9583</v>
+        <v>0.9669</v>
       </c>
       <c r="Y168" t="n">
-        <v>30.071</v>
+        <v>30.073</v>
       </c>
       <c r="Z168" t="n">
-        <v>59.025</v>
+        <v>59.207</v>
       </c>
       <c r="AA168" t="n">
-        <v>9.468999999999999</v>
+        <v>9.337</v>
       </c>
       <c r="AB168" t="n">
-        <v>25.507</v>
+        <v>25.403</v>
       </c>
       <c r="AC168" t="n">
-        <v>17.731</v>
+        <v>17.528</v>
       </c>
       <c r="AD168" t="n">
-        <v>23.579</v>
+        <v>23.276</v>
       </c>
       <c r="AE168" t="n">
-        <v>7.485</v>
+        <v>7.597</v>
       </c>
       <c r="AF168" t="n">
-        <v>25.746</v>
+        <v>25.648</v>
       </c>
       <c r="AG168" t="n">
-        <v>15.068</v>
+        <v>15.066</v>
       </c>
       <c r="AH168" t="n">
-        <v>7.012</v>
+        <v>6.913</v>
       </c>
       <c r="AI168" t="n">
-        <v>3.088</v>
+        <v>2.979</v>
       </c>
       <c r="AJ168" t="n">
-        <v>16.665</v>
+        <v>16.709</v>
       </c>
       <c r="AK168" t="n">
         <v>2.4</v>
       </c>
       <c r="AL168" t="n">
-        <v>6.9</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="169">
@@ -22586,22 +22586,22 @@
         </is>
       </c>
       <c r="E185" t="n">
-        <v>123</v>
+        <v>135</v>
       </c>
       <c r="F185" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G185" t="b">
         <v>1</v>
       </c>
       <c r="H185" t="n">
-        <v>1572.866</v>
+        <v>1564.521</v>
       </c>
       <c r="I185" t="n">
-        <v>4.2807</v>
+        <v>3.8582</v>
       </c>
       <c r="J185" t="n">
-        <v>1504.1</v>
+        <v>1513.7</v>
       </c>
       <c r="K185" t="n">
         <v>122</v>
@@ -22622,70 +22622,70 @@
         <v>105</v>
       </c>
       <c r="Q185" t="n">
-        <v>115.54</v>
+        <v>115.201</v>
       </c>
       <c r="R185" t="n">
-        <v>111.296</v>
+        <v>111.68</v>
       </c>
       <c r="S185" t="n">
-        <v>4.244</v>
+        <v>3.521</v>
       </c>
       <c r="T185" t="n">
-        <v>0.30887</v>
+        <v>0.30569</v>
       </c>
       <c r="U185" t="n">
-        <v>0.16111</v>
+        <v>0.16293</v>
       </c>
       <c r="V185" t="n">
-        <v>83.29000000000001</v>
+        <v>83</v>
       </c>
       <c r="W185" t="n">
-        <v>80.09</v>
+        <v>80.31999999999999</v>
       </c>
       <c r="X185" t="n">
-        <v>0.6171</v>
+        <v>0.599</v>
       </c>
       <c r="Y185" t="n">
-        <v>28.353</v>
+        <v>28.27</v>
       </c>
       <c r="Z185" t="n">
-        <v>60.809</v>
+        <v>60.707</v>
       </c>
       <c r="AA185" t="n">
-        <v>9.337999999999999</v>
+        <v>9.473000000000001</v>
       </c>
       <c r="AB185" t="n">
-        <v>26.792</v>
+        <v>26.97</v>
       </c>
       <c r="AC185" t="n">
-        <v>17.809</v>
+        <v>17.374</v>
       </c>
       <c r="AD185" t="n">
-        <v>23.582</v>
+        <v>23.062</v>
       </c>
       <c r="AE185" t="n">
-        <v>10.753</v>
+        <v>10.594</v>
       </c>
       <c r="AF185" t="n">
-        <v>24.15</v>
+        <v>24.102</v>
       </c>
       <c r="AG185" t="n">
-        <v>13.945</v>
+        <v>13.827</v>
       </c>
       <c r="AH185" t="n">
-        <v>5.926</v>
+        <v>5.815</v>
       </c>
       <c r="AI185" t="n">
-        <v>3.926</v>
+        <v>3.982</v>
       </c>
       <c r="AJ185" t="n">
-        <v>18.736</v>
+        <v>18.296</v>
       </c>
       <c r="AK185" t="n">
-        <v>-8.6</v>
+        <v>-8</v>
       </c>
       <c r="AL185" t="n">
-        <v>-7</v>
+        <v>-6.7</v>
       </c>
     </row>
     <row r="186">
@@ -23186,22 +23186,22 @@
         </is>
       </c>
       <c r="E190" t="n">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="F190" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G190" t="b">
         <v>1</v>
       </c>
       <c r="H190" t="n">
-        <v>1426.747</v>
+        <v>1422.529</v>
       </c>
       <c r="I190" t="n">
-        <v>3.2284</v>
+        <v>3.1653</v>
       </c>
       <c r="J190" t="n">
-        <v>1374.6</v>
+        <v>1386.7</v>
       </c>
       <c r="K190" t="n">
         <v>142</v>
@@ -23222,70 +23222,70 @@
         <v>137</v>
       </c>
       <c r="Q190" t="n">
-        <v>113.402</v>
+        <v>113.124</v>
       </c>
       <c r="R190" t="n">
-        <v>99.34099999999999</v>
+        <v>100.097</v>
       </c>
       <c r="S190" t="n">
-        <v>14.061</v>
+        <v>13.027</v>
       </c>
       <c r="T190" t="n">
-        <v>0.27695</v>
+        <v>0.28323</v>
       </c>
       <c r="U190" t="n">
-        <v>0.16236</v>
+        <v>0.16355</v>
       </c>
       <c r="V190" t="n">
-        <v>74.09999999999999</v>
+        <v>74.04000000000001</v>
       </c>
       <c r="W190" t="n">
-        <v>65.19</v>
+        <v>65.8</v>
       </c>
       <c r="X190" t="n">
-        <v>0.7652</v>
+        <v>0.7419</v>
       </c>
       <c r="Y190" t="n">
-        <v>25.852</v>
+        <v>25.929</v>
       </c>
       <c r="Z190" t="n">
-        <v>54.742</v>
+        <v>55.077</v>
       </c>
       <c r="AA190" t="n">
-        <v>6.464</v>
+        <v>6.536</v>
       </c>
       <c r="AB190" t="n">
-        <v>18.038</v>
+        <v>18.259</v>
       </c>
       <c r="AC190" t="n">
-        <v>15.936</v>
+        <v>15.647</v>
       </c>
       <c r="AD190" t="n">
-        <v>21.629</v>
+        <v>21.254</v>
       </c>
       <c r="AE190" t="n">
-        <v>9.432</v>
+        <v>9.59</v>
       </c>
       <c r="AF190" t="n">
-        <v>24.62</v>
+        <v>24.347</v>
       </c>
       <c r="AG190" t="n">
-        <v>15.945</v>
+        <v>15.802</v>
       </c>
       <c r="AH190" t="n">
-        <v>7.577</v>
+        <v>7.442</v>
       </c>
       <c r="AI190" t="n">
-        <v>3.287</v>
+        <v>3.237</v>
       </c>
       <c r="AJ190" t="n">
-        <v>14.316</v>
+        <v>14.423</v>
       </c>
       <c r="AK190" t="n">
-        <v>13</v>
+        <v>7.4</v>
       </c>
       <c r="AL190" t="n">
-        <v>13.2</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="191">
@@ -23906,22 +23906,22 @@
         </is>
       </c>
       <c r="E196" t="n">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="F196" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G196" t="b">
         <v>1</v>
       </c>
       <c r="H196" t="n">
-        <v>1739.629</v>
+        <v>1747.974</v>
       </c>
       <c r="I196" t="n">
-        <v>5.6949</v>
+        <v>5.3805</v>
       </c>
       <c r="J196" t="n">
-        <v>1607.1</v>
+        <v>1602.9</v>
       </c>
       <c r="K196" t="n">
         <v>75</v>
@@ -23942,70 +23942,70 @@
         <v>70</v>
       </c>
       <c r="Q196" t="n">
-        <v>112.247</v>
+        <v>112.996</v>
       </c>
       <c r="R196" t="n">
-        <v>105.648</v>
+        <v>105.635</v>
       </c>
       <c r="S196" t="n">
-        <v>6.599</v>
+        <v>7.361</v>
       </c>
       <c r="T196" t="n">
-        <v>0.30122</v>
+        <v>0.30095</v>
       </c>
       <c r="U196" t="n">
-        <v>0.14585</v>
+        <v>0.14234</v>
       </c>
       <c r="V196" t="n">
-        <v>75.83</v>
+        <v>76.44</v>
       </c>
       <c r="W196" t="n">
-        <v>71.67</v>
+        <v>71.72</v>
       </c>
       <c r="X196" t="n">
-        <v>0.64</v>
+        <v>0.6606</v>
       </c>
       <c r="Y196" t="n">
-        <v>24.785</v>
+        <v>25.264</v>
       </c>
       <c r="Z196" t="n">
-        <v>56.585</v>
+        <v>57.191</v>
       </c>
       <c r="AA196" t="n">
-        <v>6.687</v>
+        <v>6.717</v>
       </c>
       <c r="AB196" t="n">
-        <v>18.447</v>
+        <v>18.54</v>
       </c>
       <c r="AC196" t="n">
-        <v>19.458</v>
+        <v>19.086</v>
       </c>
       <c r="AD196" t="n">
-        <v>26.138</v>
+        <v>25.544</v>
       </c>
       <c r="AE196" t="n">
-        <v>10.135</v>
+        <v>10.18</v>
       </c>
       <c r="AF196" t="n">
-        <v>23.382</v>
+        <v>23.532</v>
       </c>
       <c r="AG196" t="n">
-        <v>14.265</v>
+        <v>14.457</v>
       </c>
       <c r="AH196" t="n">
-        <v>6.662</v>
+        <v>6.738</v>
       </c>
       <c r="AI196" t="n">
-        <v>3.735</v>
+        <v>3.697</v>
       </c>
       <c r="AJ196" t="n">
-        <v>18.324</v>
+        <v>18.052</v>
       </c>
       <c r="AK196" t="n">
-        <v>6.2</v>
+        <v>11</v>
       </c>
       <c r="AL196" t="n">
-        <v>0.9</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="197">
@@ -24146,22 +24146,22 @@
         </is>
       </c>
       <c r="E198" t="n">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="F198" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G198" t="b">
         <v>1</v>
       </c>
       <c r="H198" t="n">
-        <v>1796.871</v>
+        <v>1802.429</v>
       </c>
       <c r="I198" t="n">
-        <v>2.7628</v>
+        <v>2.3893</v>
       </c>
       <c r="J198" t="n">
-        <v>1597.3</v>
+        <v>1593.2</v>
       </c>
       <c r="K198" t="n">
         <v>50</v>
@@ -24182,70 +24182,70 @@
         <v>46</v>
       </c>
       <c r="Q198" t="n">
-        <v>114.935</v>
+        <v>116.178</v>
       </c>
       <c r="R198" t="n">
-        <v>102.867</v>
+        <v>103.208</v>
       </c>
       <c r="S198" t="n">
-        <v>12.068</v>
+        <v>12.971</v>
       </c>
       <c r="T198" t="n">
-        <v>0.28396</v>
+        <v>0.28453</v>
       </c>
       <c r="U198" t="n">
-        <v>0.14539</v>
+        <v>0.14214</v>
       </c>
       <c r="V198" t="n">
-        <v>79.87</v>
+        <v>81.06999999999999</v>
       </c>
       <c r="W198" t="n">
-        <v>71.48999999999999</v>
+        <v>72</v>
       </c>
       <c r="X198" t="n">
-        <v>0.6813</v>
+        <v>0.6995</v>
       </c>
       <c r="Y198" t="n">
-        <v>27.556</v>
+        <v>28.062</v>
       </c>
       <c r="Z198" t="n">
-        <v>59.947</v>
+        <v>60.478</v>
       </c>
       <c r="AA198" t="n">
-        <v>9.013</v>
+        <v>9.183999999999999</v>
       </c>
       <c r="AB198" t="n">
-        <v>24.995</v>
+        <v>25.376</v>
       </c>
       <c r="AC198" t="n">
-        <v>15.743</v>
+        <v>15.76</v>
       </c>
       <c r="AD198" t="n">
-        <v>21.775</v>
+        <v>21.653</v>
       </c>
       <c r="AE198" t="n">
-        <v>9.965999999999999</v>
+        <v>9.994999999999999</v>
       </c>
       <c r="AF198" t="n">
-        <v>24.575</v>
+        <v>24.618</v>
       </c>
       <c r="AG198" t="n">
-        <v>14.508</v>
+        <v>14.78</v>
       </c>
       <c r="AH198" t="n">
-        <v>7.823</v>
+        <v>7.935</v>
       </c>
       <c r="AI198" t="n">
-        <v>2.69</v>
+        <v>2.776</v>
       </c>
       <c r="AJ198" t="n">
-        <v>17.703</v>
+        <v>17.614</v>
       </c>
       <c r="AK198" t="n">
-        <v>1.4</v>
+        <v>5.2</v>
       </c>
       <c r="AL198" t="n">
-        <v>4.4</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="199">
@@ -28106,22 +28106,22 @@
         </is>
       </c>
       <c r="E231" t="n">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="F231" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G231" t="b">
         <v>1</v>
       </c>
       <c r="H231" t="n">
-        <v>1266.708</v>
+        <v>1272.073</v>
       </c>
       <c r="I231" t="n">
-        <v>-0.5639999999999999</v>
+        <v>-0.4587</v>
       </c>
       <c r="J231" t="n">
-        <v>1383.4</v>
+        <v>1381.2</v>
       </c>
       <c r="K231" t="n">
         <v>288</v>
@@ -28142,70 +28142,70 @@
         <v>300</v>
       </c>
       <c r="Q231" t="n">
-        <v>104.378</v>
+        <v>104.266</v>
       </c>
       <c r="R231" t="n">
-        <v>107.109</v>
+        <v>106.277</v>
       </c>
       <c r="S231" t="n">
-        <v>-2.731</v>
+        <v>-2.011</v>
       </c>
       <c r="T231" t="n">
-        <v>0.28778</v>
+        <v>0.28965</v>
       </c>
       <c r="U231" t="n">
-        <v>0.15507</v>
+        <v>0.15843</v>
       </c>
       <c r="V231" t="n">
-        <v>75.70999999999999</v>
+        <v>75.41</v>
       </c>
       <c r="W231" t="n">
-        <v>78.45</v>
+        <v>77.64</v>
       </c>
       <c r="X231" t="n">
-        <v>0.456</v>
+        <v>0.4727</v>
       </c>
       <c r="Y231" t="n">
-        <v>24.92</v>
+        <v>24.784</v>
       </c>
       <c r="Z231" t="n">
-        <v>59.6</v>
+        <v>59.52</v>
       </c>
       <c r="AA231" t="n">
-        <v>5.864</v>
+        <v>5.876</v>
       </c>
       <c r="AB231" t="n">
-        <v>18.264</v>
+        <v>18.479</v>
       </c>
       <c r="AC231" t="n">
-        <v>19.032</v>
+        <v>18.6</v>
       </c>
       <c r="AD231" t="n">
-        <v>25.432</v>
+        <v>24.965</v>
       </c>
       <c r="AE231" t="n">
-        <v>9.375999999999999</v>
+        <v>9.502000000000001</v>
       </c>
       <c r="AF231" t="n">
-        <v>22.176</v>
+        <v>22.27</v>
       </c>
       <c r="AG231" t="n">
-        <v>11.136</v>
+        <v>11.124</v>
       </c>
       <c r="AH231" t="n">
-        <v>7.016</v>
+        <v>6.954</v>
       </c>
       <c r="AI231" t="n">
-        <v>4.816</v>
+        <v>4.66</v>
       </c>
       <c r="AJ231" t="n">
-        <v>19.696</v>
+        <v>19.406</v>
       </c>
       <c r="AK231" t="n">
-        <v>9.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="AL231" t="n">
-        <v>9.199999999999999</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="232">
@@ -30146,22 +30146,22 @@
         </is>
       </c>
       <c r="E248" t="n">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="F248" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G248" t="b">
         <v>1</v>
       </c>
       <c r="H248" t="n">
-        <v>1537.451</v>
+        <v>1531.893</v>
       </c>
       <c r="I248" t="n">
-        <v>4.2853</v>
+        <v>4.0919</v>
       </c>
       <c r="J248" t="n">
-        <v>1500.3</v>
+        <v>1512.1</v>
       </c>
       <c r="K248" t="n">
         <v>111</v>
@@ -30182,70 +30182,70 @@
         <v>107</v>
       </c>
       <c r="Q248" t="n">
-        <v>112.785</v>
+        <v>112.703</v>
       </c>
       <c r="R248" t="n">
-        <v>106.917</v>
+        <v>108.213</v>
       </c>
       <c r="S248" t="n">
-        <v>5.867</v>
+        <v>4.49</v>
       </c>
       <c r="T248" t="n">
-        <v>0.31269</v>
+        <v>0.31466</v>
       </c>
       <c r="U248" t="n">
-        <v>0.16204</v>
+        <v>0.16234</v>
       </c>
       <c r="V248" t="n">
-        <v>79.84</v>
+        <v>80.02</v>
       </c>
       <c r="W248" t="n">
-        <v>75.93000000000001</v>
+        <v>77.14</v>
       </c>
       <c r="X248" t="n">
-        <v>0.6279</v>
+        <v>0.608</v>
       </c>
       <c r="Y248" t="n">
-        <v>28.04</v>
+        <v>28.264</v>
       </c>
       <c r="Z248" t="n">
-        <v>61.154</v>
+        <v>61.504</v>
       </c>
       <c r="AA248" t="n">
-        <v>8.372</v>
+        <v>8.311999999999999</v>
       </c>
       <c r="AB248" t="n">
-        <v>22.033</v>
+        <v>22.032</v>
       </c>
       <c r="AC248" t="n">
-        <v>15.638</v>
+        <v>15.376</v>
       </c>
       <c r="AD248" t="n">
-        <v>21.614</v>
+        <v>21.424</v>
       </c>
       <c r="AE248" t="n">
-        <v>11.165</v>
+        <v>11.28</v>
       </c>
       <c r="AF248" t="n">
-        <v>24.437</v>
+        <v>24.448</v>
       </c>
       <c r="AG248" t="n">
-        <v>14.536</v>
+        <v>14.824</v>
       </c>
       <c r="AH248" t="n">
-        <v>6.943</v>
+        <v>6.816</v>
       </c>
       <c r="AI248" t="n">
-        <v>2.694</v>
+        <v>2.712</v>
       </c>
       <c r="AJ248" t="n">
-        <v>17.586</v>
+        <v>17.536</v>
       </c>
       <c r="AK248" t="n">
-        <v>-0.6</v>
+        <v>-6.4</v>
       </c>
       <c r="AL248" t="n">
-        <v>3.7</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="249">
@@ -31946,22 +31946,22 @@
         </is>
       </c>
       <c r="E263" t="n">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="F263" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G263" t="b">
         <v>1</v>
       </c>
       <c r="H263" t="n">
-        <v>1733.884</v>
+        <v>1712.121</v>
       </c>
       <c r="I263" t="n">
-        <v>0.2411</v>
+        <v>-0.0531</v>
       </c>
       <c r="J263" t="n">
-        <v>1649.8</v>
+        <v>1652.1</v>
       </c>
       <c r="K263" t="n">
         <v>42</v>
@@ -31982,70 +31982,70 @@
         <v>37</v>
       </c>
       <c r="Q263" t="n">
-        <v>117.96</v>
+        <v>118.261</v>
       </c>
       <c r="R263" t="n">
-        <v>109.764</v>
+        <v>110.821</v>
       </c>
       <c r="S263" t="n">
-        <v>8.196</v>
+        <v>7.44</v>
       </c>
       <c r="T263" t="n">
-        <v>0.30979</v>
+        <v>0.31093</v>
       </c>
       <c r="U263" t="n">
-        <v>0.15421</v>
+        <v>0.14986</v>
       </c>
       <c r="V263" t="n">
-        <v>83.95</v>
+        <v>84.01000000000001</v>
       </c>
       <c r="W263" t="n">
-        <v>77.45</v>
+        <v>78.04000000000001</v>
       </c>
       <c r="X263" t="n">
-        <v>0.6</v>
+        <v>0.5828</v>
       </c>
       <c r="Y263" t="n">
         <v>30.69</v>
       </c>
       <c r="Z263" t="n">
-        <v>62.69</v>
+        <v>62.805</v>
       </c>
       <c r="AA263" t="n">
-        <v>8.460000000000001</v>
+        <v>8.744999999999999</v>
       </c>
       <c r="AB263" t="n">
-        <v>22.62</v>
+        <v>23.284</v>
       </c>
       <c r="AC263" t="n">
-        <v>14.11</v>
+        <v>14.272</v>
       </c>
       <c r="AD263" t="n">
-        <v>19.05</v>
+        <v>19.319</v>
       </c>
       <c r="AE263" t="n">
-        <v>10.94</v>
+        <v>10.98</v>
       </c>
       <c r="AF263" t="n">
-        <v>24.47</v>
+        <v>24.428</v>
       </c>
       <c r="AG263" t="n">
-        <v>16.87</v>
+        <v>17.057</v>
       </c>
       <c r="AH263" t="n">
-        <v>7.07</v>
+        <v>6.972</v>
       </c>
       <c r="AI263" t="n">
-        <v>3.65</v>
+        <v>3.573</v>
       </c>
       <c r="AJ263" t="n">
-        <v>16.96</v>
+        <v>16.971</v>
       </c>
       <c r="AK263" t="n">
-        <v>-5.6</v>
+        <v>-3.6</v>
       </c>
       <c r="AL263" t="n">
-        <v>0.9</v>
+        <v>-0.9</v>
       </c>
     </row>
     <row r="264">
@@ -33266,22 +33266,22 @@
         </is>
       </c>
       <c r="E274" t="n">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="F274" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G274" t="b">
         <v>1</v>
       </c>
       <c r="H274" t="n">
-        <v>1610.925</v>
+        <v>1633.092</v>
       </c>
       <c r="I274" t="n">
-        <v>1.549</v>
+        <v>1.7131</v>
       </c>
       <c r="J274" t="n">
-        <v>1518.1</v>
+        <v>1521.6</v>
       </c>
       <c r="K274" t="n">
         <v>116</v>
@@ -33302,70 +33302,70 @@
         <v>121</v>
       </c>
       <c r="Q274" t="n">
-        <v>105.807</v>
+        <v>105.758</v>
       </c>
       <c r="R274" t="n">
-        <v>103.141</v>
+        <v>102.729</v>
       </c>
       <c r="S274" t="n">
-        <v>2.666</v>
+        <v>3.029</v>
       </c>
       <c r="T274" t="n">
-        <v>0.287</v>
+        <v>0.28861</v>
       </c>
       <c r="U274" t="n">
-        <v>0.16199</v>
+        <v>0.16399</v>
       </c>
       <c r="V274" t="n">
-        <v>71.94</v>
+        <v>71.88</v>
       </c>
       <c r="W274" t="n">
-        <v>70.38</v>
+        <v>70.08</v>
       </c>
       <c r="X274" t="n">
-        <v>0.64</v>
+        <v>0.6588000000000001</v>
       </c>
       <c r="Y274" t="n">
-        <v>25.168</v>
+        <v>25.078</v>
       </c>
       <c r="Z274" t="n">
-        <v>59.512</v>
+        <v>59.396</v>
       </c>
       <c r="AA274" t="n">
-        <v>8.304</v>
+        <v>8.241</v>
       </c>
       <c r="AB274" t="n">
-        <v>26.944</v>
+        <v>26.784</v>
       </c>
       <c r="AC274" t="n">
-        <v>13.296</v>
+        <v>13.488</v>
       </c>
       <c r="AD274" t="n">
-        <v>17.96</v>
+        <v>18.139</v>
       </c>
       <c r="AE274" t="n">
-        <v>10.352</v>
+        <v>10.464</v>
       </c>
       <c r="AF274" t="n">
-        <v>25.552</v>
+        <v>25.604</v>
       </c>
       <c r="AG274" t="n">
-        <v>15.256</v>
+        <v>15.025</v>
       </c>
       <c r="AH274" t="n">
-        <v>5.4</v>
+        <v>5.519</v>
       </c>
       <c r="AI274" t="n">
-        <v>4.624</v>
+        <v>4.659</v>
       </c>
       <c r="AJ274" t="n">
-        <v>14.144</v>
+        <v>14.232</v>
       </c>
       <c r="AK274" t="n">
-        <v>4</v>
+        <v>3.8</v>
       </c>
       <c r="AL274" t="n">
-        <v>4.6</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="275">
@@ -38546,22 +38546,22 @@
         </is>
       </c>
       <c r="E318" t="n">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="F318" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G318" t="b">
         <v>1</v>
       </c>
       <c r="H318" t="n">
-        <v>1630.19</v>
+        <v>1609.505</v>
       </c>
       <c r="I318" t="n">
-        <v>2.9069</v>
+        <v>2.7323</v>
       </c>
       <c r="J318" t="n">
-        <v>1461.8</v>
+        <v>1463.4</v>
       </c>
       <c r="K318" t="n">
         <v>90</v>
@@ -38582,70 +38582,70 @@
         <v>85</v>
       </c>
       <c r="Q318" t="n">
-        <v>110.639</v>
+        <v>110.974</v>
       </c>
       <c r="R318" t="n">
-        <v>100.286</v>
+        <v>100.987</v>
       </c>
       <c r="S318" t="n">
-        <v>10.353</v>
+        <v>9.987</v>
       </c>
       <c r="T318" t="n">
-        <v>0.30348</v>
+        <v>0.30707</v>
       </c>
       <c r="U318" t="n">
-        <v>0.19698</v>
+        <v>0.19627</v>
       </c>
       <c r="V318" t="n">
-        <v>77.55</v>
+        <v>77.68000000000001</v>
       </c>
       <c r="W318" t="n">
-        <v>70.48</v>
+        <v>70.86</v>
       </c>
       <c r="X318" t="n">
-        <v>0.7282999999999999</v>
+        <v>0.7050999999999999</v>
       </c>
       <c r="Y318" t="n">
-        <v>28.19</v>
+        <v>28.147</v>
       </c>
       <c r="Z318" t="n">
-        <v>57.305</v>
+        <v>57.327</v>
       </c>
       <c r="AA318" t="n">
-        <v>6.55</v>
+        <v>6.59</v>
       </c>
       <c r="AB318" t="n">
-        <v>19.313</v>
+        <v>19.372</v>
       </c>
       <c r="AC318" t="n">
-        <v>14.701</v>
+        <v>14.859</v>
       </c>
       <c r="AD318" t="n">
-        <v>21.262</v>
+        <v>21.397</v>
       </c>
       <c r="AE318" t="n">
-        <v>10.298</v>
+        <v>10.404</v>
       </c>
       <c r="AF318" t="n">
-        <v>23.014</v>
+        <v>22.885</v>
       </c>
       <c r="AG318" t="n">
-        <v>17.21</v>
+        <v>17.449</v>
       </c>
       <c r="AH318" t="n">
-        <v>9.317</v>
+        <v>9.359</v>
       </c>
       <c r="AI318" t="n">
-        <v>5.145</v>
+        <v>5.006</v>
       </c>
       <c r="AJ318" t="n">
-        <v>19.04</v>
+        <v>18.917</v>
       </c>
       <c r="AK318" t="n">
-        <v>2.8</v>
+        <v>1.2</v>
       </c>
       <c r="AL318" t="n">
-        <v>6.9</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="319">
@@ -40346,22 +40346,22 @@
         </is>
       </c>
       <c r="E333" t="n">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="F333" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G333" t="b">
         <v>1</v>
       </c>
       <c r="H333" t="n">
-        <v>1657.02</v>
+        <v>1661.239</v>
       </c>
       <c r="I333" t="n">
-        <v>-2.5969</v>
+        <v>-2.4181</v>
       </c>
       <c r="J333" t="n">
-        <v>1677.2</v>
+        <v>1665.4</v>
       </c>
       <c r="K333" t="n">
         <v>74</v>
@@ -40382,70 +40382,70 @@
         <v>66</v>
       </c>
       <c r="Q333" t="n">
-        <v>112.23</v>
+        <v>112.962</v>
       </c>
       <c r="R333" t="n">
         <v>110.155</v>
       </c>
       <c r="S333" t="n">
-        <v>2.075</v>
+        <v>2.807</v>
       </c>
       <c r="T333" t="n">
-        <v>0.29346</v>
+        <v>0.2982</v>
       </c>
       <c r="U333" t="n">
-        <v>0.15144</v>
+        <v>0.15295</v>
       </c>
       <c r="V333" t="n">
-        <v>78.65000000000001</v>
+        <v>78.97</v>
       </c>
       <c r="W333" t="n">
-        <v>76.98999999999999</v>
+        <v>76.86</v>
       </c>
       <c r="X333" t="n">
-        <v>0.5091</v>
+        <v>0.5345</v>
       </c>
       <c r="Y333" t="n">
-        <v>26.762</v>
+        <v>26.825</v>
       </c>
       <c r="Z333" t="n">
-        <v>59.823</v>
+        <v>59.782</v>
       </c>
       <c r="AA333" t="n">
-        <v>8.981999999999999</v>
+        <v>8.930999999999999</v>
       </c>
       <c r="AB333" t="n">
-        <v>26.073</v>
+        <v>26.276</v>
       </c>
       <c r="AC333" t="n">
-        <v>15.966</v>
+        <v>16.218</v>
       </c>
       <c r="AD333" t="n">
-        <v>20.727</v>
+        <v>20.825</v>
       </c>
       <c r="AE333" t="n">
-        <v>9.336</v>
+        <v>9.548999999999999</v>
       </c>
       <c r="AF333" t="n">
-        <v>22.197</v>
+        <v>22.145</v>
       </c>
       <c r="AG333" t="n">
-        <v>14.216</v>
+        <v>14.353</v>
       </c>
       <c r="AH333" t="n">
-        <v>7.63</v>
+        <v>7.589</v>
       </c>
       <c r="AI333" t="n">
-        <v>3.438</v>
+        <v>3.516</v>
       </c>
       <c r="AJ333" t="n">
-        <v>18.672</v>
+        <v>18.578</v>
       </c>
       <c r="AK333" t="n">
-        <v>0.8</v>
+        <v>1.8</v>
       </c>
       <c r="AL333" t="n">
-        <v>1.3</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="334">

</xml_diff>

<commit_message>
Update team snapshot (2026-03-20)
</commit_message>
<xml_diff>
--- a/team_snapshot_2026.xlsx
+++ b/team_snapshot_2026.xlsx
@@ -2306,22 +2306,22 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="F16" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G16" t="b">
         <v>1</v>
       </c>
       <c r="H16" t="n">
-        <v>1977.002</v>
+        <v>1980.818</v>
       </c>
       <c r="I16" t="n">
-        <v>5.1479</v>
+        <v>5.1109</v>
       </c>
       <c r="J16" t="n">
-        <v>1736</v>
+        <v>1727.5</v>
       </c>
       <c r="K16" t="n">
         <v>15</v>
@@ -2342,70 +2342,70 @@
         <v>15</v>
       </c>
       <c r="Q16" t="n">
-        <v>122.871</v>
+        <v>122.949</v>
       </c>
       <c r="R16" t="n">
-        <v>109.332</v>
+        <v>109.035</v>
       </c>
       <c r="S16" t="n">
-        <v>13.539</v>
+        <v>13.914</v>
       </c>
       <c r="T16" t="n">
-        <v>0.29787</v>
+        <v>0.2989</v>
       </c>
       <c r="U16" t="n">
-        <v>0.12058</v>
+        <v>0.12071</v>
       </c>
       <c r="V16" t="n">
-        <v>89.91</v>
+        <v>90.19</v>
       </c>
       <c r="W16" t="n">
-        <v>80.05</v>
+        <v>80.01000000000001</v>
       </c>
       <c r="X16" t="n">
-        <v>0.7665999999999999</v>
+        <v>0.7731</v>
       </c>
       <c r="Y16" t="n">
-        <v>32.072</v>
+        <v>32.335</v>
       </c>
       <c r="Z16" t="n">
-        <v>64.128</v>
+        <v>64.456</v>
       </c>
       <c r="AA16" t="n">
-        <v>8.375999999999999</v>
+        <v>8.169</v>
       </c>
       <c r="AB16" t="n">
-        <v>21.432</v>
+        <v>21.397</v>
       </c>
       <c r="AC16" t="n">
-        <v>17.391</v>
+        <v>17.354</v>
       </c>
       <c r="AD16" t="n">
-        <v>23.287</v>
+        <v>23.126</v>
       </c>
       <c r="AE16" t="n">
-        <v>9.99</v>
+        <v>10.1</v>
       </c>
       <c r="AF16" t="n">
-        <v>23.588</v>
+        <v>23.725</v>
       </c>
       <c r="AG16" t="n">
-        <v>17.031</v>
+        <v>17.321</v>
       </c>
       <c r="AH16" t="n">
-        <v>7.239</v>
+        <v>7.291</v>
       </c>
       <c r="AI16" t="n">
-        <v>5.117</v>
+        <v>5.113</v>
       </c>
       <c r="AJ16" t="n">
-        <v>16.881</v>
+        <v>16.665</v>
       </c>
       <c r="AK16" t="n">
-        <v>8.199999999999999</v>
+        <v>8</v>
       </c>
       <c r="AL16" t="n">
-        <v>4.1</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="17">
@@ -4706,22 +4706,22 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="F36" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G36" t="b">
         <v>1</v>
       </c>
       <c r="H36" t="n">
-        <v>1926.176</v>
+        <v>1888.501</v>
       </c>
       <c r="I36" t="n">
-        <v>0.632</v>
+        <v>0.3813</v>
       </c>
       <c r="J36" t="n">
-        <v>1733.2</v>
+        <v>1731.5</v>
       </c>
       <c r="K36" t="n">
         <v>23</v>
@@ -4742,70 +4742,70 @@
         <v>23</v>
       </c>
       <c r="Q36" t="n">
-        <v>117.675</v>
+        <v>117.423</v>
       </c>
       <c r="R36" t="n">
-        <v>106.1</v>
+        <v>106.522</v>
       </c>
       <c r="S36" t="n">
-        <v>11.575</v>
+        <v>10.901</v>
       </c>
       <c r="T36" t="n">
-        <v>0.30384</v>
+        <v>0.30731</v>
       </c>
       <c r="U36" t="n">
-        <v>0.15342</v>
+        <v>0.1519</v>
       </c>
       <c r="V36" t="n">
-        <v>83.77</v>
+        <v>83.45</v>
       </c>
       <c r="W36" t="n">
-        <v>75.31</v>
+        <v>75.45</v>
       </c>
       <c r="X36" t="n">
-        <v>0.6712</v>
+        <v>0.6523</v>
       </c>
       <c r="Y36" t="n">
-        <v>29.287</v>
+        <v>29.412</v>
       </c>
       <c r="Z36" t="n">
-        <v>61.622</v>
+        <v>61.859</v>
       </c>
       <c r="AA36" t="n">
-        <v>8.613</v>
+        <v>8.596</v>
       </c>
       <c r="AB36" t="n">
-        <v>24.733</v>
+        <v>24.694</v>
       </c>
       <c r="AC36" t="n">
-        <v>16</v>
+        <v>15.75</v>
       </c>
       <c r="AD36" t="n">
-        <v>21.48</v>
+        <v>21.375</v>
       </c>
       <c r="AE36" t="n">
-        <v>10.897</v>
+        <v>11.093</v>
       </c>
       <c r="AF36" t="n">
-        <v>24.881</v>
+        <v>24.879</v>
       </c>
       <c r="AG36" t="n">
-        <v>13.398</v>
+        <v>13.461</v>
       </c>
       <c r="AH36" t="n">
-        <v>7.138</v>
+        <v>7.106</v>
       </c>
       <c r="AI36" t="n">
-        <v>4.438</v>
+        <v>4.461</v>
       </c>
       <c r="AJ36" t="n">
-        <v>15.798</v>
+        <v>15.88</v>
       </c>
       <c r="AK36" t="n">
-        <v>2.2</v>
+        <v>5</v>
       </c>
       <c r="AL36" t="n">
-        <v>-0.3</v>
+        <v>-1.5</v>
       </c>
     </row>
     <row r="37">
@@ -9506,22 +9506,22 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="F76" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G76" t="b">
         <v>1</v>
       </c>
       <c r="H76" t="n">
-        <v>2195.855</v>
+        <v>2196.684</v>
       </c>
       <c r="I76" t="n">
-        <v>3.7176</v>
+        <v>3.7365</v>
       </c>
       <c r="J76" t="n">
-        <v>1712.3</v>
+        <v>1700.6</v>
       </c>
       <c r="K76" t="n">
         <v>1</v>
@@ -9542,70 +9542,70 @@
         <v>1</v>
       </c>
       <c r="Q76" t="n">
-        <v>122.742</v>
+        <v>122.606</v>
       </c>
       <c r="R76" t="n">
-        <v>94.669</v>
+        <v>94.999</v>
       </c>
       <c r="S76" t="n">
-        <v>28.073</v>
+        <v>27.607</v>
       </c>
       <c r="T76" t="n">
-        <v>0.29815</v>
+        <v>0.29898</v>
       </c>
       <c r="U76" t="n">
-        <v>0.15408</v>
+        <v>0.15337</v>
       </c>
       <c r="V76" t="n">
-        <v>82.2</v>
+        <v>81.86</v>
       </c>
       <c r="W76" t="n">
         <v>63.22</v>
       </c>
       <c r="X76" t="n">
-        <v>0.9418</v>
+        <v>0.9434</v>
       </c>
       <c r="Y76" t="n">
-        <v>28.578</v>
+        <v>28.44</v>
       </c>
       <c r="Z76" t="n">
-        <v>58.484</v>
+        <v>58.434</v>
       </c>
       <c r="AA76" t="n">
-        <v>9.076000000000001</v>
+        <v>8.930999999999999</v>
       </c>
       <c r="AB76" t="n">
-        <v>25.902</v>
+        <v>25.915</v>
       </c>
       <c r="AC76" t="n">
-        <v>15.971</v>
+        <v>16.049</v>
       </c>
       <c r="AD76" t="n">
-        <v>22.036</v>
+        <v>22.018</v>
       </c>
       <c r="AE76" t="n">
-        <v>11.622</v>
+        <v>11.701</v>
       </c>
       <c r="AF76" t="n">
-        <v>26.964</v>
+        <v>27.028</v>
       </c>
       <c r="AG76" t="n">
-        <v>16.92</v>
+        <v>16.713</v>
       </c>
       <c r="AH76" t="n">
-        <v>7.775</v>
+        <v>7.61</v>
       </c>
       <c r="AI76" t="n">
-        <v>3.24</v>
+        <v>3.255</v>
       </c>
       <c r="AJ76" t="n">
-        <v>15.676</v>
+        <v>15.486</v>
       </c>
       <c r="AK76" t="n">
-        <v>12.2</v>
+        <v>7.6</v>
       </c>
       <c r="AL76" t="n">
-        <v>18.6</v>
+        <v>17.9</v>
       </c>
     </row>
     <row r="77">
@@ -12746,22 +12746,22 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="F103" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G103" t="b">
         <v>1</v>
       </c>
       <c r="H103" t="n">
-        <v>1798.055</v>
+        <v>1771.672</v>
       </c>
       <c r="I103" t="n">
-        <v>0.2861</v>
+        <v>0.2428</v>
       </c>
       <c r="J103" t="n">
-        <v>1643.1</v>
+        <v>1649.4</v>
       </c>
       <c r="K103" t="n">
         <v>32</v>
@@ -12782,70 +12782,70 @@
         <v>33</v>
       </c>
       <c r="Q103" t="n">
-        <v>119.916</v>
+        <v>119.281</v>
       </c>
       <c r="R103" t="n">
-        <v>106.588</v>
+        <v>107.6</v>
       </c>
       <c r="S103" t="n">
-        <v>13.328</v>
+        <v>11.68</v>
       </c>
       <c r="T103" t="n">
-        <v>0.31812</v>
+        <v>0.31594</v>
       </c>
       <c r="U103" t="n">
-        <v>0.14104</v>
+        <v>0.14131</v>
       </c>
       <c r="V103" t="n">
-        <v>89.59</v>
+        <v>89.28</v>
       </c>
       <c r="W103" t="n">
-        <v>79.12</v>
+        <v>80.11</v>
       </c>
       <c r="X103" t="n">
-        <v>0.6788</v>
+        <v>0.6589</v>
       </c>
       <c r="Y103" t="n">
-        <v>30.919</v>
+        <v>31.428</v>
       </c>
       <c r="Z103" t="n">
-        <v>65.276</v>
+        <v>65.621</v>
       </c>
       <c r="AA103" t="n">
-        <v>9.802</v>
+        <v>9.779</v>
       </c>
       <c r="AB103" t="n">
-        <v>28.115</v>
+        <v>28.21</v>
       </c>
       <c r="AC103" t="n">
-        <v>18.122</v>
+        <v>17.805</v>
       </c>
       <c r="AD103" t="n">
-        <v>23.924</v>
+        <v>23.458</v>
       </c>
       <c r="AE103" t="n">
-        <v>11.579</v>
+        <v>11.599</v>
       </c>
       <c r="AF103" t="n">
-        <v>24.446</v>
+        <v>24.859</v>
       </c>
       <c r="AG103" t="n">
-        <v>14.813</v>
+        <v>15.38</v>
       </c>
       <c r="AH103" t="n">
-        <v>8.278</v>
+        <v>8.27</v>
       </c>
       <c r="AI103" t="n">
-        <v>6.098</v>
+        <v>6.12</v>
       </c>
       <c r="AJ103" t="n">
-        <v>17.192</v>
+        <v>17.275</v>
       </c>
       <c r="AK103" t="n">
-        <v>4.6</v>
+        <v>1.2</v>
       </c>
       <c r="AL103" t="n">
-        <v>1.8</v>
+        <v>-1.9</v>
       </c>
     </row>
     <row r="104">
@@ -13106,22 +13106,22 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="F106" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G106" t="b">
         <v>1</v>
       </c>
       <c r="H106" t="n">
-        <v>2068.259</v>
+        <v>2070.396</v>
       </c>
       <c r="I106" t="n">
-        <v>5.8188</v>
+        <v>5.4527</v>
       </c>
       <c r="J106" t="n">
-        <v>1601.3</v>
+        <v>1596.4</v>
       </c>
       <c r="K106" t="n">
         <v>10</v>
@@ -13142,70 +13142,70 @@
         <v>7</v>
       </c>
       <c r="Q106" t="n">
-        <v>120.754</v>
+        <v>120.168</v>
       </c>
       <c r="R106" t="n">
-        <v>93.89400000000001</v>
+        <v>93.744</v>
       </c>
       <c r="S106" t="n">
-        <v>26.861</v>
+        <v>26.424</v>
       </c>
       <c r="T106" t="n">
-        <v>0.29917</v>
+        <v>0.30091</v>
       </c>
       <c r="U106" t="n">
-        <v>0.13348</v>
+        <v>0.13405</v>
       </c>
       <c r="V106" t="n">
-        <v>85.06</v>
+        <v>84.66</v>
       </c>
       <c r="W106" t="n">
-        <v>66.02</v>
+        <v>65.92</v>
       </c>
       <c r="X106" t="n">
-        <v>0.91</v>
+        <v>0.9126</v>
       </c>
       <c r="Y106" t="n">
-        <v>32.29</v>
+        <v>32.051</v>
       </c>
       <c r="Z106" t="n">
-        <v>63.29</v>
+        <v>63.379</v>
       </c>
       <c r="AA106" t="n">
-        <v>6.7</v>
+        <v>6.526</v>
       </c>
       <c r="AB106" t="n">
-        <v>19.69</v>
+        <v>19.573</v>
       </c>
       <c r="AC106" t="n">
-        <v>13.78</v>
+        <v>14.027</v>
       </c>
       <c r="AD106" t="n">
-        <v>19.76</v>
+        <v>19.853</v>
       </c>
       <c r="AE106" t="n">
-        <v>10.98</v>
+        <v>11.163</v>
       </c>
       <c r="AF106" t="n">
-        <v>25.82</v>
+        <v>25.97</v>
       </c>
       <c r="AG106" t="n">
-        <v>18.39</v>
+        <v>18.282</v>
       </c>
       <c r="AH106" t="n">
-        <v>8.470000000000001</v>
+        <v>8.457000000000001</v>
       </c>
       <c r="AI106" t="n">
-        <v>3.7</v>
+        <v>3.747</v>
       </c>
       <c r="AJ106" t="n">
-        <v>16.74</v>
+        <v>16.902</v>
       </c>
       <c r="AK106" t="n">
         <v>11.8</v>
       </c>
       <c r="AL106" t="n">
-        <v>13.1</v>
+        <v>14.7</v>
       </c>
     </row>
     <row r="107">
@@ -13595,7 +13595,7 @@
         <v>1</v>
       </c>
       <c r="H110" t="n">
-        <v>1490.535</v>
+        <v>1500.659</v>
       </c>
       <c r="I110" t="n">
         <v>2.799</v>
@@ -13706,22 +13706,22 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="F111" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G111" t="b">
         <v>1</v>
       </c>
       <c r="H111" t="n">
-        <v>1549.123</v>
+        <v>1545.307</v>
       </c>
       <c r="I111" t="n">
-        <v>2.9832</v>
+        <v>2.9403</v>
       </c>
       <c r="J111" t="n">
-        <v>1452.3</v>
+        <v>1472.5</v>
       </c>
       <c r="K111" t="n">
         <v>108</v>
@@ -13742,70 +13742,70 @@
         <v>101</v>
       </c>
       <c r="Q111" t="n">
-        <v>108.144</v>
+        <v>108.056</v>
       </c>
       <c r="R111" t="n">
-        <v>96.693</v>
+        <v>98.124</v>
       </c>
       <c r="S111" t="n">
-        <v>11.451</v>
+        <v>9.932</v>
       </c>
       <c r="T111" t="n">
-        <v>0.25834</v>
+        <v>0.2616</v>
       </c>
       <c r="U111" t="n">
-        <v>0.18506</v>
+        <v>0.18375</v>
       </c>
       <c r="V111" t="n">
-        <v>78.65000000000001</v>
+        <v>78.7</v>
       </c>
       <c r="W111" t="n">
-        <v>70.23</v>
+        <v>71.41</v>
       </c>
       <c r="X111" t="n">
-        <v>0.7361</v>
+        <v>0.7028</v>
       </c>
       <c r="Y111" t="n">
-        <v>26.387</v>
+        <v>26.624</v>
       </c>
       <c r="Z111" t="n">
-        <v>58.064</v>
+        <v>58.49</v>
       </c>
       <c r="AA111" t="n">
-        <v>7.177</v>
+        <v>7.317</v>
       </c>
       <c r="AB111" t="n">
-        <v>22.478</v>
+        <v>22.908</v>
       </c>
       <c r="AC111" t="n">
-        <v>18.397</v>
+        <v>17.915</v>
       </c>
       <c r="AD111" t="n">
-        <v>24.685</v>
+        <v>24.193</v>
       </c>
       <c r="AE111" t="n">
-        <v>9.537000000000001</v>
+        <v>9.561999999999999</v>
       </c>
       <c r="AF111" t="n">
-        <v>26.693</v>
+        <v>26.421</v>
       </c>
       <c r="AG111" t="n">
-        <v>12.958</v>
+        <v>13.083</v>
       </c>
       <c r="AH111" t="n">
-        <v>6.658</v>
+        <v>6.565</v>
       </c>
       <c r="AI111" t="n">
-        <v>3.955</v>
+        <v>3.853</v>
       </c>
       <c r="AJ111" t="n">
-        <v>18.001</v>
+        <v>17.824</v>
       </c>
       <c r="AK111" t="n">
-        <v>6.8</v>
+        <v>2.6</v>
       </c>
       <c r="AL111" t="n">
-        <v>2.1</v>
+        <v>-1.3</v>
       </c>
     </row>
     <row r="112">
@@ -13826,22 +13826,22 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="F112" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G112" t="b">
         <v>1</v>
       </c>
       <c r="H112" t="n">
-        <v>1625.523</v>
+        <v>1664.344</v>
       </c>
       <c r="I112" t="n">
-        <v>-0.8564000000000001</v>
+        <v>-0.6842</v>
       </c>
       <c r="J112" t="n">
-        <v>1382.5</v>
+        <v>1401.4</v>
       </c>
       <c r="K112" t="n">
         <v>92</v>
@@ -13862,70 +13862,70 @@
         <v>75</v>
       </c>
       <c r="Q112" t="n">
-        <v>121.161</v>
+        <v>120.784</v>
       </c>
       <c r="R112" t="n">
-        <v>100.188</v>
+        <v>100.586</v>
       </c>
       <c r="S112" t="n">
-        <v>20.973</v>
+        <v>20.197</v>
       </c>
       <c r="T112" t="n">
-        <v>0.30613</v>
+        <v>0.30161</v>
       </c>
       <c r="U112" t="n">
-        <v>0.12761</v>
+        <v>0.12796</v>
       </c>
       <c r="V112" t="n">
-        <v>86.5</v>
+        <v>86.31</v>
       </c>
       <c r="W112" t="n">
-        <v>71.84999999999999</v>
+        <v>72.20999999999999</v>
       </c>
       <c r="X112" t="n">
-        <v>0.8722</v>
+        <v>0.8761</v>
       </c>
       <c r="Y112" t="n">
-        <v>28.949</v>
+        <v>29.049</v>
       </c>
       <c r="Z112" t="n">
-        <v>61.172</v>
+        <v>61.346</v>
       </c>
       <c r="AA112" t="n">
-        <v>9.042</v>
+        <v>9.031000000000001</v>
       </c>
       <c r="AB112" t="n">
-        <v>26.217</v>
+        <v>26.128</v>
       </c>
       <c r="AC112" t="n">
-        <v>19.557</v>
+        <v>19.145</v>
       </c>
       <c r="AD112" t="n">
-        <v>26.314</v>
+        <v>25.688</v>
       </c>
       <c r="AE112" t="n">
-        <v>10.258</v>
+        <v>10.119</v>
       </c>
       <c r="AF112" t="n">
-        <v>22.906</v>
+        <v>23.134</v>
       </c>
       <c r="AG112" t="n">
-        <v>15.246</v>
+        <v>15.328</v>
       </c>
       <c r="AH112" t="n">
-        <v>10.364</v>
+        <v>10.052</v>
       </c>
       <c r="AI112" t="n">
-        <v>3.681</v>
+        <v>3.69</v>
       </c>
       <c r="AJ112" t="n">
-        <v>18.867</v>
+        <v>18.534</v>
       </c>
       <c r="AK112" t="n">
-        <v>9.800000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="AL112" t="n">
-        <v>15.9</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="113">
@@ -14186,22 +14186,22 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="F115" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G115" t="b">
         <v>1</v>
       </c>
       <c r="H115" t="n">
-        <v>2111.715</v>
+        <v>2112.552</v>
       </c>
       <c r="I115" t="n">
-        <v>1.2196</v>
+        <v>1.1096</v>
       </c>
       <c r="J115" t="n">
-        <v>1742.7</v>
+        <v>1725.6</v>
       </c>
       <c r="K115" t="n">
         <v>5</v>
@@ -14222,70 +14222,70 @@
         <v>5</v>
       </c>
       <c r="Q115" t="n">
-        <v>117.346</v>
+        <v>117.422</v>
       </c>
       <c r="R115" t="n">
-        <v>95.8</v>
+        <v>94.66500000000001</v>
       </c>
       <c r="S115" t="n">
-        <v>21.546</v>
+        <v>22.757</v>
       </c>
       <c r="T115" t="n">
-        <v>0.33855</v>
+        <v>0.33192</v>
       </c>
       <c r="U115" t="n">
-        <v>0.12356</v>
+        <v>0.12292</v>
       </c>
       <c r="V115" t="n">
-        <v>77.12</v>
+        <v>77.18000000000001</v>
       </c>
       <c r="W115" t="n">
-        <v>63</v>
+        <v>62.27</v>
       </c>
       <c r="X115" t="n">
-        <v>0.8159</v>
+        <v>0.8300999999999999</v>
       </c>
       <c r="Y115" t="n">
-        <v>27.767</v>
+        <v>27.885</v>
       </c>
       <c r="Z115" t="n">
-        <v>61.756</v>
+        <v>61.745</v>
       </c>
       <c r="AA115" t="n">
-        <v>8.787000000000001</v>
+        <v>8.765000000000001</v>
       </c>
       <c r="AB115" t="n">
-        <v>25.138</v>
+        <v>24.8</v>
       </c>
       <c r="AC115" t="n">
-        <v>12.797</v>
+        <v>12.645</v>
       </c>
       <c r="AD115" t="n">
-        <v>16.593</v>
+        <v>16.41</v>
       </c>
       <c r="AE115" t="n">
-        <v>11.514</v>
+        <v>11.37</v>
       </c>
       <c r="AF115" t="n">
-        <v>22.544</v>
+        <v>23.168</v>
       </c>
       <c r="AG115" t="n">
-        <v>14.661</v>
+        <v>14.503</v>
       </c>
       <c r="AH115" t="n">
-        <v>7.7</v>
+        <v>7.745</v>
       </c>
       <c r="AI115" t="n">
-        <v>3.845</v>
+        <v>3.747</v>
       </c>
       <c r="AJ115" t="n">
-        <v>18.057</v>
+        <v>17.917</v>
       </c>
       <c r="AK115" t="n">
-        <v>8.800000000000001</v>
+        <v>12.4</v>
       </c>
       <c r="AL115" t="n">
-        <v>7.5</v>
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="116">
@@ -14426,22 +14426,22 @@
         </is>
       </c>
       <c r="E117" t="n">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F117" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G117" t="b">
         <v>1</v>
       </c>
       <c r="H117" t="n">
-        <v>1413.012</v>
+        <v>1412.371</v>
       </c>
       <c r="I117" t="n">
-        <v>2.8128</v>
+        <v>2.7318</v>
       </c>
       <c r="J117" t="n">
-        <v>1374.4</v>
+        <v>1406.7</v>
       </c>
       <c r="K117" t="n">
         <v>207</v>
@@ -14462,70 +14462,70 @@
         <v>203</v>
       </c>
       <c r="Q117" t="n">
-        <v>109.768</v>
+        <v>109.688</v>
       </c>
       <c r="R117" t="n">
-        <v>99.30200000000001</v>
+        <v>100.821</v>
       </c>
       <c r="S117" t="n">
-        <v>10.466</v>
+        <v>8.867000000000001</v>
       </c>
       <c r="T117" t="n">
-        <v>0.31778</v>
+        <v>0.31724</v>
       </c>
       <c r="U117" t="n">
-        <v>0.18288</v>
+        <v>0.18058</v>
       </c>
       <c r="V117" t="n">
-        <v>75.48</v>
+        <v>75.56</v>
       </c>
       <c r="W117" t="n">
-        <v>68.45</v>
+        <v>69.66</v>
       </c>
       <c r="X117" t="n">
-        <v>0.6702</v>
+        <v>0.6389</v>
       </c>
       <c r="Y117" t="n">
-        <v>25.174</v>
+        <v>25.211</v>
       </c>
       <c r="Z117" t="n">
-        <v>56.184</v>
+        <v>56.419</v>
       </c>
       <c r="AA117" t="n">
-        <v>6.801</v>
+        <v>7.068</v>
       </c>
       <c r="AB117" t="n">
-        <v>19.252</v>
+        <v>19.64</v>
       </c>
       <c r="AC117" t="n">
-        <v>18.33</v>
+        <v>18.069</v>
       </c>
       <c r="AD117" t="n">
-        <v>24.736</v>
+        <v>24.411</v>
       </c>
       <c r="AE117" t="n">
-        <v>10.714</v>
+        <v>10.546</v>
       </c>
       <c r="AF117" t="n">
-        <v>22.834</v>
+        <v>22.517</v>
       </c>
       <c r="AG117" t="n">
-        <v>15.22</v>
+        <v>15.182</v>
       </c>
       <c r="AH117" t="n">
-        <v>8.375999999999999</v>
+        <v>8.207000000000001</v>
       </c>
       <c r="AI117" t="n">
-        <v>3.771</v>
+        <v>3.642</v>
       </c>
       <c r="AJ117" t="n">
-        <v>18.714</v>
+        <v>18.546</v>
       </c>
       <c r="AK117" t="n">
-        <v>11</v>
+        <v>2.8</v>
       </c>
       <c r="AL117" t="n">
-        <v>16.5</v>
+        <v>15</v>
       </c>
     </row>
     <row r="118">
@@ -14546,22 +14546,22 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="F118" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G118" t="b">
         <v>1</v>
       </c>
       <c r="H118" t="n">
-        <v>1409.955</v>
+        <v>1409.118</v>
       </c>
       <c r="I118" t="n">
-        <v>-0.3498</v>
+        <v>-0.2978</v>
       </c>
       <c r="J118" t="n">
-        <v>1415.2</v>
+        <v>1439.8</v>
       </c>
       <c r="K118" t="n">
         <v>145</v>
@@ -14582,70 +14582,70 @@
         <v>145</v>
       </c>
       <c r="Q118" t="n">
-        <v>110.278</v>
+        <v>108.976</v>
       </c>
       <c r="R118" t="n">
-        <v>106.528</v>
+        <v>107.138</v>
       </c>
       <c r="S118" t="n">
-        <v>3.75</v>
+        <v>1.838</v>
       </c>
       <c r="T118" t="n">
-        <v>0.26932</v>
+        <v>0.26845</v>
       </c>
       <c r="U118" t="n">
-        <v>0.14751</v>
+        <v>0.14698</v>
       </c>
       <c r="V118" t="n">
-        <v>76.66</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="W118" t="n">
-        <v>73.95</v>
+        <v>74.14</v>
       </c>
       <c r="X118" t="n">
-        <v>0.5651</v>
+        <v>0.5424</v>
       </c>
       <c r="Y118" t="n">
-        <v>25.728</v>
+        <v>25.402</v>
       </c>
       <c r="Z118" t="n">
-        <v>59.747</v>
+        <v>59.646</v>
       </c>
       <c r="AA118" t="n">
-        <v>9.696999999999999</v>
+        <v>9.586</v>
       </c>
       <c r="AB118" t="n">
-        <v>28.106</v>
+        <v>28.192</v>
       </c>
       <c r="AC118" t="n">
-        <v>14.571</v>
+        <v>14.364</v>
       </c>
       <c r="AD118" t="n">
-        <v>20.006</v>
+        <v>19.821</v>
       </c>
       <c r="AE118" t="n">
-        <v>9.212999999999999</v>
+        <v>9.17</v>
       </c>
       <c r="AF118" t="n">
-        <v>24.379</v>
+        <v>24.397</v>
       </c>
       <c r="AG118" t="n">
-        <v>11.722</v>
+        <v>11.616</v>
       </c>
       <c r="AH118" t="n">
-        <v>5.534</v>
+        <v>5.512</v>
       </c>
       <c r="AI118" t="n">
-        <v>2.379</v>
+        <v>2.469</v>
       </c>
       <c r="AJ118" t="n">
-        <v>19.111</v>
+        <v>18.876</v>
       </c>
       <c r="AK118" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="AL118" t="n">
-        <v>9.199999999999999</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="119">
@@ -14906,22 +14906,22 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="F121" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G121" t="b">
         <v>1</v>
       </c>
       <c r="H121" t="n">
-        <v>1982.683</v>
+        <v>1984.447</v>
       </c>
       <c r="I121" t="n">
-        <v>7.8712</v>
+        <v>7.3951</v>
       </c>
       <c r="J121" t="n">
-        <v>1717.2</v>
+        <v>1704.4</v>
       </c>
       <c r="K121" t="n">
         <v>7</v>
@@ -14942,70 +14942,70 @@
         <v>8</v>
       </c>
       <c r="Q121" t="n">
-        <v>125.113</v>
+        <v>126.534</v>
       </c>
       <c r="R121" t="n">
-        <v>103.663</v>
+        <v>103.563</v>
       </c>
       <c r="S121" t="n">
-        <v>21.45</v>
+        <v>22.971</v>
       </c>
       <c r="T121" t="n">
-        <v>0.32225</v>
+        <v>0.32629</v>
       </c>
       <c r="U121" t="n">
-        <v>0.12812</v>
+        <v>0.12517</v>
       </c>
       <c r="V121" t="n">
-        <v>84.41</v>
+        <v>85.2</v>
       </c>
       <c r="W121" t="n">
-        <v>70.04000000000001</v>
+        <v>69.81999999999999</v>
       </c>
       <c r="X121" t="n">
-        <v>0.7419</v>
+        <v>0.76</v>
       </c>
       <c r="Y121" t="n">
-        <v>28.464</v>
+        <v>28.81</v>
       </c>
       <c r="Z121" t="n">
-        <v>61.919</v>
+        <v>62.36</v>
       </c>
       <c r="AA121" t="n">
-        <v>10.927</v>
+        <v>11.1</v>
       </c>
       <c r="AB121" t="n">
-        <v>31.849</v>
+        <v>31.92</v>
       </c>
       <c r="AC121" t="n">
-        <v>16.684</v>
+        <v>16.57</v>
       </c>
       <c r="AD121" t="n">
-        <v>20.973</v>
+        <v>20.88</v>
       </c>
       <c r="AE121" t="n">
-        <v>12.329</v>
+        <v>12.65</v>
       </c>
       <c r="AF121" t="n">
-        <v>26.185</v>
+        <v>26.26</v>
       </c>
       <c r="AG121" t="n">
-        <v>14.743</v>
+        <v>14.73</v>
       </c>
       <c r="AH121" t="n">
-        <v>3.887</v>
+        <v>3.8</v>
       </c>
       <c r="AI121" t="n">
-        <v>4.597</v>
+        <v>4.52</v>
       </c>
       <c r="AJ121" t="n">
-        <v>13.312</v>
+        <v>13.12</v>
       </c>
       <c r="AK121" t="n">
-        <v>2.8</v>
+        <v>10</v>
       </c>
       <c r="AL121" t="n">
-        <v>10.5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="122">
@@ -16826,22 +16826,22 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="F137" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G137" t="b">
         <v>1</v>
       </c>
       <c r="H137" t="n">
-        <v>1521.308</v>
+        <v>1519.171</v>
       </c>
       <c r="I137" t="n">
-        <v>-0.1615</v>
+        <v>-0.0429</v>
       </c>
       <c r="J137" t="n">
-        <v>1474.6</v>
+        <v>1497.2</v>
       </c>
       <c r="K137" t="n">
         <v>163</v>
@@ -16862,70 +16862,70 @@
         <v>155</v>
       </c>
       <c r="Q137" t="n">
-        <v>111.121</v>
+        <v>110.411</v>
       </c>
       <c r="R137" t="n">
-        <v>108.097</v>
+        <v>108.109</v>
       </c>
       <c r="S137" t="n">
-        <v>3.024</v>
+        <v>2.302</v>
       </c>
       <c r="T137" t="n">
-        <v>0.34498</v>
+        <v>0.34286</v>
       </c>
       <c r="U137" t="n">
-        <v>0.16501</v>
+        <v>0.16508</v>
       </c>
       <c r="V137" t="n">
-        <v>80.47</v>
+        <v>79.91</v>
       </c>
       <c r="W137" t="n">
-        <v>78.27</v>
+        <v>78.20999999999999</v>
       </c>
       <c r="X137" t="n">
-        <v>0.584</v>
+        <v>0.5583</v>
       </c>
       <c r="Y137" t="n">
-        <v>26.064</v>
+        <v>25.901</v>
       </c>
       <c r="Z137" t="n">
-        <v>61.28</v>
+        <v>61.071</v>
       </c>
       <c r="AA137" t="n">
-        <v>8.688000000000001</v>
+        <v>8.521000000000001</v>
       </c>
       <c r="AB137" t="n">
-        <v>26.592</v>
+        <v>26.212</v>
       </c>
       <c r="AC137" t="n">
-        <v>18.736</v>
+        <v>18.783</v>
       </c>
       <c r="AD137" t="n">
-        <v>26.712</v>
+        <v>26.744</v>
       </c>
       <c r="AE137" t="n">
-        <v>12.632</v>
+        <v>12.489</v>
       </c>
       <c r="AF137" t="n">
-        <v>23.856</v>
+        <v>23.837</v>
       </c>
       <c r="AG137" t="n">
-        <v>13.6</v>
+        <v>13.359</v>
       </c>
       <c r="AH137" t="n">
-        <v>6.632</v>
+        <v>6.736</v>
       </c>
       <c r="AI137" t="n">
-        <v>5.128</v>
+        <v>5.086</v>
       </c>
       <c r="AJ137" t="n">
-        <v>20.912</v>
+        <v>20.823</v>
       </c>
       <c r="AK137" t="n">
-        <v>3.2</v>
+        <v>2.8</v>
       </c>
       <c r="AL137" t="n">
-        <v>3.6</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="138">
@@ -18386,22 +18386,22 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="F150" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G150" t="b">
         <v>1</v>
       </c>
       <c r="H150" t="n">
-        <v>1836.881</v>
+        <v>1854.143</v>
       </c>
       <c r="I150" t="n">
-        <v>-2.5958</v>
+        <v>-2.5004</v>
       </c>
       <c r="J150" t="n">
-        <v>1686.1</v>
+        <v>1686.9</v>
       </c>
       <c r="K150" t="n">
         <v>19</v>
@@ -18422,70 +18422,70 @@
         <v>17</v>
       </c>
       <c r="Q150" t="n">
-        <v>118.896</v>
+        <v>118.734</v>
       </c>
       <c r="R150" t="n">
-        <v>101.876</v>
+        <v>101.945</v>
       </c>
       <c r="S150" t="n">
-        <v>17.02</v>
+        <v>16.789</v>
       </c>
       <c r="T150" t="n">
-        <v>0.28905</v>
+        <v>0.2886</v>
       </c>
       <c r="U150" t="n">
-        <v>0.15971</v>
+        <v>0.16453</v>
       </c>
       <c r="V150" t="n">
-        <v>84.66</v>
+        <v>84.69</v>
       </c>
       <c r="W150" t="n">
-        <v>72.23</v>
+        <v>72.43000000000001</v>
       </c>
       <c r="X150" t="n">
-        <v>0.6911</v>
+        <v>0.7082000000000001</v>
       </c>
       <c r="Y150" t="n">
-        <v>28.532</v>
+        <v>28.525</v>
       </c>
       <c r="Z150" t="n">
-        <v>61.349</v>
+        <v>61.046</v>
       </c>
       <c r="AA150" t="n">
-        <v>11.288</v>
+        <v>11.395</v>
       </c>
       <c r="AB150" t="n">
-        <v>32.323</v>
+        <v>32.12</v>
       </c>
       <c r="AC150" t="n">
-        <v>15.915</v>
+        <v>15.868</v>
       </c>
       <c r="AD150" t="n">
-        <v>20.726</v>
+        <v>20.915</v>
       </c>
       <c r="AE150" t="n">
-        <v>10.713</v>
+        <v>10.737</v>
       </c>
       <c r="AF150" t="n">
-        <v>26.159</v>
+        <v>26.294</v>
       </c>
       <c r="AG150" t="n">
-        <v>16.841</v>
+        <v>16.854</v>
       </c>
       <c r="AH150" t="n">
-        <v>6.893</v>
+        <v>6.838</v>
       </c>
       <c r="AI150" t="n">
-        <v>3.394</v>
+        <v>3.35</v>
       </c>
       <c r="AJ150" t="n">
-        <v>18.347</v>
+        <v>18.284</v>
       </c>
       <c r="AK150" t="n">
-        <v>2.4</v>
+        <v>4.2</v>
       </c>
       <c r="AL150" t="n">
-        <v>6.8</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="151">
@@ -19946,22 +19946,22 @@
         </is>
       </c>
       <c r="E163" t="n">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="F163" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G163" t="b">
         <v>1</v>
       </c>
       <c r="H163" t="n">
-        <v>1726.811</v>
+        <v>1715.565</v>
       </c>
       <c r="I163" t="n">
-        <v>2.6895</v>
+        <v>2.6075</v>
       </c>
       <c r="J163" t="n">
-        <v>1428.4</v>
+        <v>1447.5</v>
       </c>
       <c r="K163" t="n">
         <v>68</v>
@@ -19982,70 +19982,70 @@
         <v>56</v>
       </c>
       <c r="Q163" t="n">
-        <v>115.07</v>
+        <v>114.775</v>
       </c>
       <c r="R163" t="n">
-        <v>100.006</v>
+        <v>100.989</v>
       </c>
       <c r="S163" t="n">
-        <v>15.064</v>
+        <v>13.786</v>
       </c>
       <c r="T163" t="n">
-        <v>0.34832</v>
+        <v>0.35346</v>
       </c>
       <c r="U163" t="n">
-        <v>0.13903</v>
+        <v>0.13698</v>
       </c>
       <c r="V163" t="n">
-        <v>76.83</v>
+        <v>76.5</v>
       </c>
       <c r="W163" t="n">
-        <v>66.97</v>
+        <v>67.45</v>
       </c>
       <c r="X163" t="n">
-        <v>0.84</v>
+        <v>0.8065</v>
       </c>
       <c r="Y163" t="n">
-        <v>26.424</v>
+        <v>26.427</v>
       </c>
       <c r="Z163" t="n">
-        <v>58.808</v>
+        <v>59.261</v>
       </c>
       <c r="AA163" t="n">
-        <v>6.408</v>
+        <v>6.519</v>
       </c>
       <c r="AB163" t="n">
-        <v>20.808</v>
+        <v>21.006</v>
       </c>
       <c r="AC163" t="n">
-        <v>16.896</v>
+        <v>16.599</v>
       </c>
       <c r="AD163" t="n">
-        <v>22.808</v>
+        <v>22.306</v>
       </c>
       <c r="AE163" t="n">
-        <v>11.096</v>
+        <v>11.316</v>
       </c>
       <c r="AF163" t="n">
-        <v>20.68</v>
+        <v>20.605</v>
       </c>
       <c r="AG163" t="n">
-        <v>13.008</v>
+        <v>12.954</v>
       </c>
       <c r="AH163" t="n">
-        <v>10.12</v>
+        <v>10.117</v>
       </c>
       <c r="AI163" t="n">
-        <v>4.248</v>
+        <v>4.287</v>
       </c>
       <c r="AJ163" t="n">
-        <v>19.064</v>
+        <v>19.047</v>
       </c>
       <c r="AK163" t="n">
-        <v>8.199999999999999</v>
+        <v>4.8</v>
       </c>
       <c r="AL163" t="n">
-        <v>13.2</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="164">
@@ -20666,22 +20666,22 @@
         </is>
       </c>
       <c r="E169" t="n">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="F169" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G169" t="b">
         <v>1</v>
       </c>
       <c r="H169" t="n">
-        <v>2173.708</v>
+        <v>2174.35</v>
       </c>
       <c r="I169" t="n">
-        <v>6.5185</v>
+        <v>6.1854</v>
       </c>
       <c r="J169" t="n">
-        <v>1779.9</v>
+        <v>1765.3</v>
       </c>
       <c r="K169" t="n">
         <v>3</v>
@@ -20702,70 +20702,70 @@
         <v>2</v>
       </c>
       <c r="Q169" t="n">
-        <v>120.66</v>
+        <v>121.548</v>
       </c>
       <c r="R169" t="n">
-        <v>97.182</v>
+        <v>97.557</v>
       </c>
       <c r="S169" t="n">
-        <v>23.477</v>
+        <v>23.992</v>
       </c>
       <c r="T169" t="n">
-        <v>0.25981</v>
+        <v>0.25476</v>
       </c>
       <c r="U169" t="n">
-        <v>0.1613</v>
+        <v>0.16164</v>
       </c>
       <c r="V169" t="n">
-        <v>86.70999999999999</v>
+        <v>87.33</v>
       </c>
       <c r="W169" t="n">
-        <v>69.29000000000001</v>
+        <v>69.59</v>
       </c>
       <c r="X169" t="n">
-        <v>0.9046</v>
+        <v>0.9149</v>
       </c>
       <c r="Y169" t="n">
-        <v>30.409</v>
+        <v>30.647</v>
       </c>
       <c r="Z169" t="n">
-        <v>59.947</v>
+        <v>59.793</v>
       </c>
       <c r="AA169" t="n">
-        <v>8.932</v>
+        <v>9.042999999999999</v>
       </c>
       <c r="AB169" t="n">
-        <v>24.768</v>
+        <v>24.822</v>
       </c>
       <c r="AC169" t="n">
-        <v>17.255</v>
+        <v>17.22</v>
       </c>
       <c r="AD169" t="n">
-        <v>23.138</v>
+        <v>23.035</v>
       </c>
       <c r="AE169" t="n">
-        <v>9.917999999999999</v>
+        <v>9.728999999999999</v>
       </c>
       <c r="AF169" t="n">
-        <v>27.953</v>
+        <v>28.107</v>
       </c>
       <c r="AG169" t="n">
-        <v>18.666</v>
+        <v>18.945</v>
       </c>
       <c r="AH169" t="n">
-        <v>5.751</v>
+        <v>5.702</v>
       </c>
       <c r="AI169" t="n">
-        <v>5.934</v>
+        <v>6.015</v>
       </c>
       <c r="AJ169" t="n">
-        <v>15.451</v>
+        <v>15.382</v>
       </c>
       <c r="AK169" t="n">
-        <v>2.4</v>
+        <v>6</v>
       </c>
       <c r="AL169" t="n">
-        <v>7.2</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="170">
@@ -20786,22 +20786,22 @@
         </is>
       </c>
       <c r="E170" t="n">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="F170" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G170" t="b">
         <v>1</v>
       </c>
       <c r="H170" t="n">
-        <v>2027.394</v>
+        <v>2031.39</v>
       </c>
       <c r="I170" t="n">
-        <v>0.218</v>
+        <v>0.0735</v>
       </c>
       <c r="J170" t="n">
-        <v>1730.1</v>
+        <v>1723.2</v>
       </c>
       <c r="K170" t="n">
         <v>9</v>
@@ -20822,70 +20822,70 @@
         <v>11</v>
       </c>
       <c r="Q170" t="n">
-        <v>117.657</v>
+        <v>117.934</v>
       </c>
       <c r="R170" t="n">
-        <v>102.118</v>
+        <v>101.399</v>
       </c>
       <c r="S170" t="n">
-        <v>15.539</v>
+        <v>16.535</v>
       </c>
       <c r="T170" t="n">
-        <v>0.29627</v>
+        <v>0.28968</v>
       </c>
       <c r="U170" t="n">
-        <v>0.16068</v>
+        <v>0.1613</v>
       </c>
       <c r="V170" t="n">
-        <v>78.98999999999999</v>
+        <v>79.45999999999999</v>
       </c>
       <c r="W170" t="n">
-        <v>68.62</v>
+        <v>68.34999999999999</v>
       </c>
       <c r="X170" t="n">
-        <v>0.7728</v>
+        <v>0.79</v>
       </c>
       <c r="Y170" t="n">
-        <v>27.651</v>
+        <v>27.84</v>
       </c>
       <c r="Z170" t="n">
-        <v>58.266</v>
+        <v>58.22</v>
       </c>
       <c r="AA170" t="n">
-        <v>7.776</v>
+        <v>7.81</v>
       </c>
       <c r="AB170" t="n">
-        <v>21.497</v>
+        <v>21.38</v>
       </c>
       <c r="AC170" t="n">
-        <v>16.082</v>
+        <v>16.09</v>
       </c>
       <c r="AD170" t="n">
-        <v>21.071</v>
+        <v>20.97</v>
       </c>
       <c r="AE170" t="n">
-        <v>11.194</v>
+        <v>10.96</v>
       </c>
       <c r="AF170" t="n">
-        <v>26.152</v>
+        <v>26.41</v>
       </c>
       <c r="AG170" t="n">
-        <v>18.362</v>
+        <v>18.65</v>
       </c>
       <c r="AH170" t="n">
-        <v>5.477</v>
+        <v>5.39</v>
       </c>
       <c r="AI170" t="n">
-        <v>4.113</v>
+        <v>4.2</v>
       </c>
       <c r="AJ170" t="n">
-        <v>16.456</v>
+        <v>16.31</v>
       </c>
       <c r="AK170" t="n">
-        <v>1</v>
+        <v>5.6</v>
       </c>
       <c r="AL170" t="n">
-        <v>1.3</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="171">
@@ -22826,22 +22826,22 @@
         </is>
       </c>
       <c r="E187" t="n">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="F187" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G187" t="b">
         <v>1</v>
       </c>
       <c r="H187" t="n">
-        <v>1593.755</v>
+        <v>1589.758</v>
       </c>
       <c r="I187" t="n">
-        <v>3.5257</v>
+        <v>3.408</v>
       </c>
       <c r="J187" t="n">
-        <v>1410.6</v>
+        <v>1434.7</v>
       </c>
       <c r="K187" t="n">
         <v>113</v>
@@ -22862,70 +22862,70 @@
         <v>114</v>
       </c>
       <c r="Q187" t="n">
-        <v>114.28</v>
+        <v>113.469</v>
       </c>
       <c r="R187" t="n">
-        <v>102.18</v>
+        <v>103.166</v>
       </c>
       <c r="S187" t="n">
-        <v>12.099</v>
+        <v>10.303</v>
       </c>
       <c r="T187" t="n">
-        <v>0.31044</v>
+        <v>0.30533</v>
       </c>
       <c r="U187" t="n">
-        <v>0.15061</v>
+        <v>0.15101</v>
       </c>
       <c r="V187" t="n">
-        <v>78.98999999999999</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="W187" t="n">
-        <v>70.7</v>
+        <v>71.59</v>
       </c>
       <c r="X187" t="n">
-        <v>0.776</v>
+        <v>0.7444</v>
       </c>
       <c r="Y187" t="n">
-        <v>28.072</v>
+        <v>27.978</v>
       </c>
       <c r="Z187" t="n">
-        <v>61.408</v>
+        <v>61.28</v>
       </c>
       <c r="AA187" t="n">
-        <v>9.391999999999999</v>
+        <v>9.257</v>
       </c>
       <c r="AB187" t="n">
-        <v>26.232</v>
+        <v>26.21</v>
       </c>
       <c r="AC187" t="n">
-        <v>13.456</v>
+        <v>13.388</v>
       </c>
       <c r="AD187" t="n">
-        <v>18.84</v>
+        <v>18.768</v>
       </c>
       <c r="AE187" t="n">
-        <v>10.912</v>
+        <v>10.638</v>
       </c>
       <c r="AF187" t="n">
-        <v>23.688</v>
+        <v>23.467</v>
       </c>
       <c r="AG187" t="n">
-        <v>14.88</v>
+        <v>14.83</v>
       </c>
       <c r="AH187" t="n">
-        <v>7.712</v>
+        <v>7.675</v>
       </c>
       <c r="AI187" t="n">
-        <v>2.832</v>
+        <v>2.768</v>
       </c>
       <c r="AJ187" t="n">
-        <v>15.152</v>
+        <v>15.232</v>
       </c>
       <c r="AK187" t="n">
-        <v>10.8</v>
+        <v>10.2</v>
       </c>
       <c r="AL187" t="n">
-        <v>11.6</v>
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="188">
@@ -23786,22 +23786,22 @@
         </is>
       </c>
       <c r="E195" t="n">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="F195" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G195" t="b">
         <v>1</v>
       </c>
       <c r="H195" t="n">
-        <v>1982.884</v>
+        <v>1988.043</v>
       </c>
       <c r="I195" t="n">
-        <v>9.932399999999999</v>
+        <v>9.170199999999999</v>
       </c>
       <c r="J195" t="n">
-        <v>1675.8</v>
+        <v>1669.8</v>
       </c>
       <c r="K195" t="n">
         <v>14</v>
@@ -23822,70 +23822,70 @@
         <v>14</v>
       </c>
       <c r="Q195" t="n">
-        <v>114.614</v>
+        <v>115.233</v>
       </c>
       <c r="R195" t="n">
-        <v>98.94199999999999</v>
+        <v>97.834</v>
       </c>
       <c r="S195" t="n">
-        <v>15.672</v>
+        <v>17.399</v>
       </c>
       <c r="T195" t="n">
-        <v>0.24333</v>
+        <v>0.24652</v>
       </c>
       <c r="U195" t="n">
-        <v>0.1403</v>
+        <v>0.13855</v>
       </c>
       <c r="V195" t="n">
-        <v>77.06999999999999</v>
+        <v>77.23</v>
       </c>
       <c r="W195" t="n">
-        <v>66.3</v>
+        <v>65.45</v>
       </c>
       <c r="X195" t="n">
-        <v>0.8038</v>
+        <v>0.82</v>
       </c>
       <c r="Y195" t="n">
-        <v>27.484</v>
+        <v>27.52</v>
       </c>
       <c r="Z195" t="n">
-        <v>58.927</v>
+        <v>59.18</v>
       </c>
       <c r="AA195" t="n">
-        <v>10.526</v>
+        <v>10.67</v>
       </c>
       <c r="AB195" t="n">
-        <v>29.887</v>
+        <v>30.24</v>
       </c>
       <c r="AC195" t="n">
-        <v>12.247</v>
+        <v>12</v>
       </c>
       <c r="AD195" t="n">
-        <v>16.133</v>
+        <v>15.75</v>
       </c>
       <c r="AE195" t="n">
-        <v>8.332000000000001</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="AF195" t="n">
-        <v>25.329</v>
+        <v>25.29</v>
       </c>
       <c r="AG195" t="n">
-        <v>18.145</v>
+        <v>18.2</v>
       </c>
       <c r="AH195" t="n">
-        <v>7.298</v>
+        <v>7.42</v>
       </c>
       <c r="AI195" t="n">
-        <v>2.556</v>
+        <v>2.5</v>
       </c>
       <c r="AJ195" t="n">
-        <v>14.226</v>
+        <v>14.12</v>
       </c>
       <c r="AK195" t="n">
-        <v>0.2</v>
+        <v>3.4</v>
       </c>
       <c r="AL195" t="n">
-        <v>4.7</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="196">
@@ -24986,22 +24986,22 @@
         </is>
       </c>
       <c r="E205" t="n">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="F205" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G205" t="b">
         <v>1</v>
       </c>
       <c r="H205" t="n">
-        <v>1899.484</v>
+        <v>1863.313</v>
       </c>
       <c r="I205" t="n">
-        <v>2.2848</v>
+        <v>2.0961</v>
       </c>
       <c r="J205" t="n">
-        <v>1677.4</v>
+        <v>1679</v>
       </c>
       <c r="K205" t="n">
         <v>29</v>
@@ -25022,70 +25022,70 @@
         <v>24</v>
       </c>
       <c r="Q205" t="n">
-        <v>115.28</v>
+        <v>114.782</v>
       </c>
       <c r="R205" t="n">
-        <v>103.723</v>
+        <v>103.763</v>
       </c>
       <c r="S205" t="n">
-        <v>11.556</v>
+        <v>11.019</v>
       </c>
       <c r="T205" t="n">
-        <v>0.25957</v>
+        <v>0.258</v>
       </c>
       <c r="U205" t="n">
-        <v>0.13749</v>
+        <v>0.13763</v>
       </c>
       <c r="V205" t="n">
-        <v>79.77</v>
+        <v>79.70999999999999</v>
       </c>
       <c r="W205" t="n">
-        <v>71.41</v>
+        <v>71.73999999999999</v>
       </c>
       <c r="X205" t="n">
-        <v>0.7419</v>
+        <v>0.72</v>
       </c>
       <c r="Y205" t="n">
-        <v>27.927</v>
+        <v>28.02</v>
       </c>
       <c r="Z205" t="n">
-        <v>58.988</v>
+        <v>59.31</v>
       </c>
       <c r="AA205" t="n">
-        <v>8.567</v>
+        <v>8.66</v>
       </c>
       <c r="AB205" t="n">
-        <v>24.626</v>
+        <v>24.74</v>
       </c>
       <c r="AC205" t="n">
-        <v>15.392</v>
+        <v>15.2</v>
       </c>
       <c r="AD205" t="n">
-        <v>22.351</v>
+        <v>22.09</v>
       </c>
       <c r="AE205" t="n">
-        <v>9.214</v>
+        <v>9.19</v>
       </c>
       <c r="AF205" t="n">
-        <v>26.155</v>
+        <v>26.39</v>
       </c>
       <c r="AG205" t="n">
-        <v>15.792</v>
+        <v>15.69</v>
       </c>
       <c r="AH205" t="n">
-        <v>5.444</v>
+        <v>5.42</v>
       </c>
       <c r="AI205" t="n">
-        <v>3.402</v>
+        <v>3.47</v>
       </c>
       <c r="AJ205" t="n">
-        <v>14.578</v>
+        <v>14.66</v>
       </c>
       <c r="AK205" t="n">
-        <v>-0.4</v>
+        <v>-1.8</v>
       </c>
       <c r="AL205" t="n">
-        <v>-0.5</v>
+        <v>-1.2</v>
       </c>
     </row>
     <row r="206">
@@ -26426,22 +26426,22 @@
         </is>
       </c>
       <c r="E217" t="n">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="F217" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G217" t="b">
         <v>1</v>
       </c>
       <c r="H217" t="n">
-        <v>1813.861</v>
+        <v>1789.287</v>
       </c>
       <c r="I217" t="n">
-        <v>1.9487</v>
+        <v>2.1115</v>
       </c>
       <c r="J217" t="n">
-        <v>1722.9</v>
+        <v>1723.3</v>
       </c>
       <c r="K217" t="n">
         <v>26</v>
@@ -26462,70 +26462,70 @@
         <v>29</v>
       </c>
       <c r="Q217" t="n">
-        <v>118</v>
+        <v>117.639</v>
       </c>
       <c r="R217" t="n">
-        <v>108.071</v>
+        <v>108.068</v>
       </c>
       <c r="S217" t="n">
-        <v>9.929</v>
+        <v>9.571</v>
       </c>
       <c r="T217" t="n">
-        <v>0.25505</v>
+        <v>0.25683</v>
       </c>
       <c r="U217" t="n">
-        <v>0.15026</v>
+        <v>0.14892</v>
       </c>
       <c r="V217" t="n">
-        <v>79.68000000000001</v>
+        <v>79.2</v>
       </c>
       <c r="W217" t="n">
-        <v>72.77</v>
+        <v>72.54000000000001</v>
       </c>
       <c r="X217" t="n">
-        <v>0.631</v>
+        <v>0.6128</v>
       </c>
       <c r="Y217" t="n">
-        <v>27.409</v>
+        <v>27.327</v>
       </c>
       <c r="Z217" t="n">
-        <v>55.776</v>
+        <v>55.915</v>
       </c>
       <c r="AA217" t="n">
-        <v>8.09</v>
+        <v>8.125</v>
       </c>
       <c r="AB217" t="n">
-        <v>22.588</v>
+        <v>22.591</v>
       </c>
       <c r="AC217" t="n">
-        <v>16.893</v>
+        <v>16.616</v>
       </c>
       <c r="AD217" t="n">
-        <v>21.846</v>
+        <v>21.587</v>
       </c>
       <c r="AE217" t="n">
-        <v>8.106999999999999</v>
+        <v>8.236000000000001</v>
       </c>
       <c r="AF217" t="n">
-        <v>23.082</v>
+        <v>23.199</v>
       </c>
       <c r="AG217" t="n">
-        <v>14.335</v>
+        <v>14.276</v>
       </c>
       <c r="AH217" t="n">
-        <v>4.828</v>
+        <v>4.788</v>
       </c>
       <c r="AI217" t="n">
-        <v>2.498</v>
+        <v>2.541</v>
       </c>
       <c r="AJ217" t="n">
-        <v>17.391</v>
+        <v>17.231</v>
       </c>
       <c r="AK217" t="n">
-        <v>10.4</v>
+        <v>8.4</v>
       </c>
       <c r="AL217" t="n">
-        <v>4.9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="218">
@@ -27386,22 +27386,22 @@
         </is>
       </c>
       <c r="E225" t="n">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="F225" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G225" t="b">
         <v>1</v>
       </c>
       <c r="H225" t="n">
-        <v>1435.396</v>
+        <v>1433.632</v>
       </c>
       <c r="I225" t="n">
-        <v>1.2024</v>
+        <v>1.3668</v>
       </c>
       <c r="J225" t="n">
-        <v>1493.7</v>
+        <v>1513.2</v>
       </c>
       <c r="K225" t="n">
         <v>150</v>
@@ -27422,70 +27422,70 @@
         <v>139</v>
       </c>
       <c r="Q225" t="n">
-        <v>108.543</v>
+        <v>108.034</v>
       </c>
       <c r="R225" t="n">
-        <v>106.705</v>
+        <v>108.635</v>
       </c>
       <c r="S225" t="n">
-        <v>1.838</v>
+        <v>-0.601</v>
       </c>
       <c r="T225" t="n">
-        <v>0.31426</v>
+        <v>0.3115</v>
       </c>
       <c r="U225" t="n">
-        <v>0.15185</v>
+        <v>0.15052</v>
       </c>
       <c r="V225" t="n">
-        <v>74.73999999999999</v>
+        <v>74.36</v>
       </c>
       <c r="W225" t="n">
-        <v>73.48999999999999</v>
+        <v>74.8</v>
       </c>
       <c r="X225" t="n">
-        <v>0.612</v>
+        <v>0.5795</v>
       </c>
       <c r="Y225" t="n">
-        <v>26.097</v>
+        <v>26.216</v>
       </c>
       <c r="Z225" t="n">
-        <v>59.889</v>
+        <v>60.08</v>
       </c>
       <c r="AA225" t="n">
-        <v>7.942</v>
+        <v>7.977</v>
       </c>
       <c r="AB225" t="n">
-        <v>21.143</v>
+        <v>21.511</v>
       </c>
       <c r="AC225" t="n">
-        <v>14.34</v>
+        <v>13.75</v>
       </c>
       <c r="AD225" t="n">
-        <v>20.739</v>
+        <v>19.932</v>
       </c>
       <c r="AE225" t="n">
-        <v>10.616</v>
+        <v>10.375</v>
       </c>
       <c r="AF225" t="n">
-        <v>23.33</v>
+        <v>23.08</v>
       </c>
       <c r="AG225" t="n">
-        <v>14.076</v>
+        <v>13.92</v>
       </c>
       <c r="AH225" t="n">
-        <v>6.601</v>
+        <v>6.364</v>
       </c>
       <c r="AI225" t="n">
-        <v>3.224</v>
+        <v>3.205</v>
       </c>
       <c r="AJ225" t="n">
-        <v>16.776</v>
+        <v>17.023</v>
       </c>
       <c r="AK225" t="n">
-        <v>7.8</v>
+        <v>-1</v>
       </c>
       <c r="AL225" t="n">
-        <v>6.1</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="226">
@@ -31826,22 +31826,22 @@
         </is>
       </c>
       <c r="E262" t="n">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="F262" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G262" t="b">
         <v>1</v>
       </c>
       <c r="H262" t="n">
-        <v>1478.017</v>
+        <v>1477.189</v>
       </c>
       <c r="I262" t="n">
-        <v>0.9489</v>
+        <v>0.9855</v>
       </c>
       <c r="J262" t="n">
-        <v>1430.3</v>
+        <v>1458.8</v>
       </c>
       <c r="K262" t="n">
         <v>192</v>
@@ -31862,70 +31862,70 @@
         <v>183</v>
       </c>
       <c r="Q262" t="n">
-        <v>109.727</v>
+        <v>109.579</v>
       </c>
       <c r="R262" t="n">
-        <v>101.773</v>
+        <v>102.384</v>
       </c>
       <c r="S262" t="n">
-        <v>7.954</v>
+        <v>7.195</v>
       </c>
       <c r="T262" t="n">
-        <v>0.27993</v>
+        <v>0.28293</v>
       </c>
       <c r="U262" t="n">
-        <v>0.1508</v>
+        <v>0.14927</v>
       </c>
       <c r="V262" t="n">
-        <v>70.45999999999999</v>
+        <v>70.31999999999999</v>
       </c>
       <c r="W262" t="n">
-        <v>65.55</v>
+        <v>65.88</v>
       </c>
       <c r="X262" t="n">
-        <v>0.68</v>
+        <v>0.6505</v>
       </c>
       <c r="Y262" t="n">
-        <v>25.087</v>
+        <v>25.17</v>
       </c>
       <c r="Z262" t="n">
-        <v>55.469</v>
+        <v>55.809</v>
       </c>
       <c r="AA262" t="n">
-        <v>5.607</v>
+        <v>5.691</v>
       </c>
       <c r="AB262" t="n">
-        <v>18.258</v>
+        <v>18.421</v>
       </c>
       <c r="AC262" t="n">
-        <v>14.276</v>
+        <v>14.003</v>
       </c>
       <c r="AD262" t="n">
-        <v>18.644</v>
+        <v>18.217</v>
       </c>
       <c r="AE262" t="n">
-        <v>8.92</v>
+        <v>9.02</v>
       </c>
       <c r="AF262" t="n">
-        <v>22.491</v>
+        <v>22.432</v>
       </c>
       <c r="AG262" t="n">
-        <v>13.247</v>
+        <v>13.36</v>
       </c>
       <c r="AH262" t="n">
-        <v>5.993</v>
+        <v>5.933</v>
       </c>
       <c r="AI262" t="n">
-        <v>3.233</v>
+        <v>3.103</v>
       </c>
       <c r="AJ262" t="n">
-        <v>13.935</v>
+        <v>13.992</v>
       </c>
       <c r="AK262" t="n">
-        <v>6.2</v>
+        <v>7.8</v>
       </c>
       <c r="AL262" t="n">
-        <v>2</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="263">
@@ -32426,22 +32426,22 @@
         </is>
       </c>
       <c r="E267" t="n">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="F267" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G267" t="b">
         <v>1</v>
       </c>
       <c r="H267" t="n">
-        <v>1723.482</v>
+        <v>1706.22</v>
       </c>
       <c r="I267" t="n">
-        <v>8.857799999999999</v>
+        <v>8.7103</v>
       </c>
       <c r="J267" t="n">
-        <v>1554.8</v>
+        <v>1565.3</v>
       </c>
       <c r="K267" t="n">
         <v>47</v>
@@ -32462,70 +32462,70 @@
         <v>45</v>
       </c>
       <c r="Q267" t="n">
-        <v>115.66</v>
+        <v>115.379</v>
       </c>
       <c r="R267" t="n">
-        <v>100.714</v>
+        <v>101.318</v>
       </c>
       <c r="S267" t="n">
-        <v>14.946</v>
+        <v>14.062</v>
       </c>
       <c r="T267" t="n">
-        <v>0.33977</v>
+        <v>0.34579</v>
       </c>
       <c r="U267" t="n">
-        <v>0.14645</v>
+        <v>0.14539</v>
       </c>
       <c r="V267" t="n">
-        <v>86.81999999999999</v>
+        <v>86.68000000000001</v>
       </c>
       <c r="W267" t="n">
-        <v>76.08</v>
+        <v>76.58</v>
       </c>
       <c r="X267" t="n">
-        <v>0.7527</v>
+        <v>0.72</v>
       </c>
       <c r="Y267" t="n">
-        <v>28.626</v>
+        <v>28.74</v>
       </c>
       <c r="Z267" t="n">
-        <v>65.66800000000001</v>
+        <v>66.17</v>
       </c>
       <c r="AA267" t="n">
-        <v>9.493</v>
+        <v>9.35</v>
       </c>
       <c r="AB267" t="n">
-        <v>28.708</v>
+        <v>28.95</v>
       </c>
       <c r="AC267" t="n">
-        <v>20.071</v>
+        <v>19.85</v>
       </c>
       <c r="AD267" t="n">
-        <v>26.988</v>
+        <v>26.59</v>
       </c>
       <c r="AE267" t="n">
-        <v>13.34</v>
+        <v>13.53</v>
       </c>
       <c r="AF267" t="n">
-        <v>25.733</v>
+        <v>25.45</v>
       </c>
       <c r="AG267" t="n">
-        <v>16.833</v>
+        <v>16.76</v>
       </c>
       <c r="AH267" t="n">
-        <v>8.856</v>
+        <v>9.09</v>
       </c>
       <c r="AI267" t="n">
-        <v>4.051</v>
+        <v>4.02</v>
       </c>
       <c r="AJ267" t="n">
-        <v>19.753</v>
+        <v>19.8</v>
       </c>
       <c r="AK267" t="n">
-        <v>19</v>
+        <v>12.6</v>
       </c>
       <c r="AL267" t="n">
-        <v>15.1</v>
+        <v>14.1</v>
       </c>
     </row>
     <row r="268">
@@ -33386,22 +33386,22 @@
         </is>
       </c>
       <c r="E275" t="n">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="F275" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G275" t="b">
         <v>1</v>
       </c>
       <c r="H275" t="n">
-        <v>1793.214</v>
+        <v>1819.597</v>
       </c>
       <c r="I275" t="n">
-        <v>8.666399999999999</v>
+        <v>8.063000000000001</v>
       </c>
       <c r="J275" t="n">
-        <v>1516.9</v>
+        <v>1526.5</v>
       </c>
       <c r="K275" t="n">
         <v>41</v>
@@ -33422,70 +33422,70 @@
         <v>31</v>
       </c>
       <c r="Q275" t="n">
-        <v>120.005</v>
+        <v>120.498</v>
       </c>
       <c r="R275" t="n">
-        <v>98.72799999999999</v>
+        <v>98.57599999999999</v>
       </c>
       <c r="S275" t="n">
-        <v>21.276</v>
+        <v>21.922</v>
       </c>
       <c r="T275" t="n">
-        <v>0.24179</v>
+        <v>0.24815</v>
       </c>
       <c r="U275" t="n">
-        <v>0.1658</v>
+        <v>0.16516</v>
       </c>
       <c r="V275" t="n">
-        <v>86.22</v>
+        <v>87.03</v>
       </c>
       <c r="W275" t="n">
-        <v>70.65000000000001</v>
+        <v>70.91</v>
       </c>
       <c r="X275" t="n">
-        <v>0.8347</v>
+        <v>0.85</v>
       </c>
       <c r="Y275" t="n">
-        <v>29.882</v>
+        <v>29.8</v>
       </c>
       <c r="Z275" t="n">
-        <v>59.544</v>
+        <v>60.09</v>
       </c>
       <c r="AA275" t="n">
-        <v>10.782</v>
+        <v>10.78</v>
       </c>
       <c r="AB275" t="n">
-        <v>26.69</v>
+        <v>27.21</v>
       </c>
       <c r="AC275" t="n">
-        <v>15.715</v>
+        <v>15.68</v>
       </c>
       <c r="AD275" t="n">
-        <v>21.086</v>
+        <v>21.2</v>
       </c>
       <c r="AE275" t="n">
-        <v>8.917999999999999</v>
+        <v>9.15</v>
       </c>
       <c r="AF275" t="n">
-        <v>27.823</v>
+        <v>27.6</v>
       </c>
       <c r="AG275" t="n">
-        <v>17.977</v>
+        <v>17.67</v>
       </c>
       <c r="AH275" t="n">
-        <v>7.238</v>
+        <v>7.29</v>
       </c>
       <c r="AI275" t="n">
-        <v>3.206</v>
+        <v>3.25</v>
       </c>
       <c r="AJ275" t="n">
-        <v>18.267</v>
+        <v>18.11</v>
       </c>
       <c r="AK275" t="n">
-        <v>1.2</v>
+        <v>3.2</v>
       </c>
       <c r="AL275" t="n">
-        <v>5</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="276">
@@ -33506,22 +33506,22 @@
         </is>
       </c>
       <c r="E276" t="n">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="F276" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G276" t="b">
         <v>1</v>
       </c>
       <c r="H276" t="n">
-        <v>1857.81</v>
+        <v>1829.011</v>
       </c>
       <c r="I276" t="n">
-        <v>-0.2818</v>
+        <v>-0.1963</v>
       </c>
       <c r="J276" t="n">
-        <v>1596.9</v>
+        <v>1604.4</v>
       </c>
       <c r="K276" t="n">
         <v>24</v>
@@ -33542,70 +33542,70 @@
         <v>22</v>
       </c>
       <c r="Q276" t="n">
-        <v>118.734</v>
+        <v>117.386</v>
       </c>
       <c r="R276" t="n">
-        <v>99.88200000000001</v>
+        <v>99.93899999999999</v>
       </c>
       <c r="S276" t="n">
-        <v>18.852</v>
+        <v>17.447</v>
       </c>
       <c r="T276" t="n">
-        <v>0.2975</v>
+        <v>0.2968</v>
       </c>
       <c r="U276" t="n">
-        <v>0.15247</v>
+        <v>0.1542</v>
       </c>
       <c r="V276" t="n">
-        <v>77.54000000000001</v>
+        <v>76.45999999999999</v>
       </c>
       <c r="W276" t="n">
-        <v>65.41</v>
+        <v>65.19</v>
       </c>
       <c r="X276" t="n">
-        <v>0.829</v>
+        <v>0.8038</v>
       </c>
       <c r="Y276" t="n">
-        <v>26.684</v>
+        <v>26.493</v>
       </c>
       <c r="Z276" t="n">
-        <v>57.823</v>
+        <v>57.534</v>
       </c>
       <c r="AA276" t="n">
-        <v>8.194000000000001</v>
+        <v>8.154999999999999</v>
       </c>
       <c r="AB276" t="n">
-        <v>20.951</v>
+        <v>20.991</v>
       </c>
       <c r="AC276" t="n">
-        <v>16.191</v>
+        <v>16.017</v>
       </c>
       <c r="AD276" t="n">
-        <v>20.377</v>
+        <v>20.141</v>
       </c>
       <c r="AE276" t="n">
-        <v>11.371</v>
+        <v>11.288</v>
       </c>
       <c r="AF276" t="n">
-        <v>26.154</v>
+        <v>26.05</v>
       </c>
       <c r="AG276" t="n">
-        <v>15.241</v>
+        <v>15.278</v>
       </c>
       <c r="AH276" t="n">
-        <v>5.562</v>
+        <v>5.848</v>
       </c>
       <c r="AI276" t="n">
-        <v>3.586</v>
+        <v>3.473</v>
       </c>
       <c r="AJ276" t="n">
-        <v>15.771</v>
+        <v>15.722</v>
       </c>
       <c r="AK276" t="n">
-        <v>8.6</v>
+        <v>5.6</v>
       </c>
       <c r="AL276" t="n">
-        <v>12.6</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="277">
@@ -34346,22 +34346,22 @@
         </is>
       </c>
       <c r="E283" t="n">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="F283" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G283" t="b">
         <v>1</v>
       </c>
       <c r="H283" t="n">
-        <v>1836.074</v>
+        <v>1860.648</v>
       </c>
       <c r="I283" t="n">
-        <v>6.9164</v>
+        <v>6.8435</v>
       </c>
       <c r="J283" t="n">
-        <v>1691.3</v>
+        <v>1693.5</v>
       </c>
       <c r="K283" t="n">
         <v>43</v>
@@ -34382,70 +34382,70 @@
         <v>39</v>
       </c>
       <c r="Q283" t="n">
-        <v>111.157</v>
+        <v>111.032</v>
       </c>
       <c r="R283" t="n">
-        <v>102.345</v>
+        <v>102.3</v>
       </c>
       <c r="S283" t="n">
-        <v>8.813000000000001</v>
+        <v>8.731</v>
       </c>
       <c r="T283" t="n">
-        <v>0.32311</v>
+        <v>0.31828</v>
       </c>
       <c r="U283" t="n">
-        <v>0.15137</v>
+        <v>0.14957</v>
       </c>
       <c r="V283" t="n">
-        <v>78.26000000000001</v>
+        <v>77.84999999999999</v>
       </c>
       <c r="W283" t="n">
-        <v>72.11</v>
+        <v>71.76000000000001</v>
       </c>
       <c r="X283" t="n">
-        <v>0.6611</v>
+        <v>0.679</v>
       </c>
       <c r="Y283" t="n">
-        <v>27.133</v>
+        <v>27.035</v>
       </c>
       <c r="Z283" t="n">
-        <v>60.635</v>
+        <v>60.473</v>
       </c>
       <c r="AA283" t="n">
-        <v>7.407</v>
+        <v>7.342</v>
       </c>
       <c r="AB283" t="n">
-        <v>22.356</v>
+        <v>22.358</v>
       </c>
       <c r="AC283" t="n">
-        <v>16.584</v>
+        <v>16.361</v>
       </c>
       <c r="AD283" t="n">
-        <v>23.409</v>
+        <v>22.993</v>
       </c>
       <c r="AE283" t="n">
-        <v>11.219</v>
+        <v>11.019</v>
       </c>
       <c r="AF283" t="n">
-        <v>22.651</v>
+        <v>22.732</v>
       </c>
       <c r="AG283" t="n">
-        <v>15.589</v>
+        <v>15.724</v>
       </c>
       <c r="AH283" t="n">
-        <v>7.666</v>
+        <v>7.56</v>
       </c>
       <c r="AI283" t="n">
-        <v>4.541</v>
+        <v>4.488</v>
       </c>
       <c r="AJ283" t="n">
-        <v>16.359</v>
+        <v>16.07</v>
       </c>
       <c r="AK283" t="n">
-        <v>5.8</v>
+        <v>4.4</v>
       </c>
       <c r="AL283" t="n">
-        <v>4.6</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="284">
@@ -34946,22 +34946,22 @@
         </is>
       </c>
       <c r="E288" t="n">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F288" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G288" t="b">
         <v>1</v>
       </c>
       <c r="H288" t="n">
-        <v>1764.159</v>
+        <v>1801.834</v>
       </c>
       <c r="I288" t="n">
-        <v>2.6628</v>
+        <v>2.6488</v>
       </c>
       <c r="J288" t="n">
-        <v>1698.6</v>
+        <v>1706</v>
       </c>
       <c r="K288" t="n">
         <v>37</v>
@@ -34982,70 +34982,70 @@
         <v>42</v>
       </c>
       <c r="Q288" t="n">
-        <v>118.998</v>
+        <v>119.208</v>
       </c>
       <c r="R288" t="n">
-        <v>110.826</v>
+        <v>110.835</v>
       </c>
       <c r="S288" t="n">
-        <v>8.173</v>
+        <v>8.372999999999999</v>
       </c>
       <c r="T288" t="n">
-        <v>0.30408</v>
+        <v>0.30312</v>
       </c>
       <c r="U288" t="n">
-        <v>0.14433</v>
+        <v>0.14324</v>
       </c>
       <c r="V288" t="n">
         <v>82.06</v>
       </c>
       <c r="W288" t="n">
-        <v>76.34</v>
+        <v>76.23</v>
       </c>
       <c r="X288" t="n">
-        <v>0.5665</v>
+        <v>0.5793</v>
       </c>
       <c r="Y288" t="n">
-        <v>27.8</v>
+        <v>27.696</v>
       </c>
       <c r="Z288" t="n">
-        <v>58.071</v>
+        <v>57.983</v>
       </c>
       <c r="AA288" t="n">
-        <v>7.053</v>
+        <v>6.945</v>
       </c>
       <c r="AB288" t="n">
-        <v>20.366</v>
+        <v>20.468</v>
       </c>
       <c r="AC288" t="n">
-        <v>19.636</v>
+        <v>19.661</v>
       </c>
       <c r="AD288" t="n">
-        <v>26.145</v>
+        <v>26.133</v>
       </c>
       <c r="AE288" t="n">
-        <v>10.53</v>
+        <v>10.464</v>
       </c>
       <c r="AF288" t="n">
-        <v>24.173</v>
+        <v>24.112</v>
       </c>
       <c r="AG288" t="n">
-        <v>11.734</v>
+        <v>11.529</v>
       </c>
       <c r="AH288" t="n">
-        <v>6.018</v>
+        <v>6</v>
       </c>
       <c r="AI288" t="n">
-        <v>2.956</v>
+        <v>2.978</v>
       </c>
       <c r="AJ288" t="n">
-        <v>18.996</v>
+        <v>18.97</v>
       </c>
       <c r="AK288" t="n">
-        <v>-5</v>
+        <v>-4.6</v>
       </c>
       <c r="AL288" t="n">
-        <v>-1.8</v>
+        <v>-2.1</v>
       </c>
     </row>
     <row r="289">
@@ -35066,22 +35066,22 @@
         </is>
       </c>
       <c r="E289" t="n">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="F289" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G289" t="b">
         <v>1</v>
       </c>
       <c r="H289" t="n">
-        <v>1823.96</v>
+        <v>1852.759</v>
       </c>
       <c r="I289" t="n">
-        <v>4.3608</v>
+        <v>4.0806</v>
       </c>
       <c r="J289" t="n">
-        <v>1653.7</v>
+        <v>1661.5</v>
       </c>
       <c r="K289" t="n">
         <v>39</v>
@@ -35102,70 +35102,70 @@
         <v>44</v>
       </c>
       <c r="Q289" t="n">
-        <v>117.135</v>
+        <v>116.943</v>
       </c>
       <c r="R289" t="n">
-        <v>107.431</v>
+        <v>106.221</v>
       </c>
       <c r="S289" t="n">
-        <v>9.702999999999999</v>
+        <v>10.722</v>
       </c>
       <c r="T289" t="n">
-        <v>0.30978</v>
+        <v>0.31014</v>
       </c>
       <c r="U289" t="n">
-        <v>0.13892</v>
+        <v>0.14624</v>
       </c>
       <c r="V289" t="n">
-        <v>87.41</v>
+        <v>86.69</v>
       </c>
       <c r="W289" t="n">
-        <v>79.61</v>
+        <v>78.33</v>
       </c>
       <c r="X289" t="n">
-        <v>0.648</v>
+        <v>0.6706</v>
       </c>
       <c r="Y289" t="n">
-        <v>29.827</v>
+        <v>29.32</v>
       </c>
       <c r="Z289" t="n">
-        <v>64.822</v>
+        <v>64.04000000000001</v>
       </c>
       <c r="AA289" t="n">
-        <v>10.777</v>
+        <v>10.779</v>
       </c>
       <c r="AB289" t="n">
-        <v>29.846</v>
+        <v>29.559</v>
       </c>
       <c r="AC289" t="n">
-        <v>17.844</v>
+        <v>17.327</v>
       </c>
       <c r="AD289" t="n">
-        <v>24.14</v>
+        <v>23.668</v>
       </c>
       <c r="AE289" t="n">
-        <v>11.317</v>
+        <v>11.21</v>
       </c>
       <c r="AF289" t="n">
-        <v>24.495</v>
+        <v>24.294</v>
       </c>
       <c r="AG289" t="n">
-        <v>18.222</v>
+        <v>17.823</v>
       </c>
       <c r="AH289" t="n">
-        <v>8.129</v>
+        <v>8.025</v>
       </c>
       <c r="AI289" t="n">
-        <v>3.365</v>
+        <v>3.329</v>
       </c>
       <c r="AJ289" t="n">
-        <v>19.233</v>
+        <v>18.924</v>
       </c>
       <c r="AK289" t="n">
-        <v>-5.4</v>
+        <v>0.2</v>
       </c>
       <c r="AL289" t="n">
-        <v>-5.3</v>
+        <v>-2.1</v>
       </c>
     </row>
     <row r="290">
@@ -35786,22 +35786,22 @@
         </is>
       </c>
       <c r="E295" t="n">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="F295" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G295" t="b">
         <v>1</v>
       </c>
       <c r="H295" t="n">
-        <v>1600.961</v>
+        <v>1595.802</v>
       </c>
       <c r="I295" t="n">
-        <v>1.1284</v>
+        <v>1.0762</v>
       </c>
       <c r="J295" t="n">
-        <v>1466</v>
+        <v>1488.7</v>
       </c>
       <c r="K295" t="n">
         <v>143</v>
@@ -35822,70 +35822,70 @@
         <v>125</v>
       </c>
       <c r="Q295" t="n">
-        <v>112.278</v>
+        <v>110.674</v>
       </c>
       <c r="R295" t="n">
-        <v>106.193</v>
+        <v>107.202</v>
       </c>
       <c r="S295" t="n">
-        <v>6.085</v>
+        <v>3.471</v>
       </c>
       <c r="T295" t="n">
-        <v>0.316</v>
+        <v>0.31414</v>
       </c>
       <c r="U295" t="n">
-        <v>0.16673</v>
+        <v>0.17064</v>
       </c>
       <c r="V295" t="n">
-        <v>78.27</v>
+        <v>76.93000000000001</v>
       </c>
       <c r="W295" t="n">
-        <v>74.3</v>
+        <v>74.55</v>
       </c>
       <c r="X295" t="n">
-        <v>0.65</v>
+        <v>0.6171</v>
       </c>
       <c r="Y295" t="n">
-        <v>26.627</v>
+        <v>25.99</v>
       </c>
       <c r="Z295" t="n">
-        <v>59.845</v>
+        <v>59.36</v>
       </c>
       <c r="AA295" t="n">
-        <v>9.009</v>
+        <v>9.018000000000001</v>
       </c>
       <c r="AB295" t="n">
-        <v>27.182</v>
+        <v>27.352</v>
       </c>
       <c r="AC295" t="n">
-        <v>16.009</v>
+        <v>15.931</v>
       </c>
       <c r="AD295" t="n">
-        <v>21.709</v>
+        <v>21.436</v>
       </c>
       <c r="AE295" t="n">
-        <v>11.159</v>
+        <v>11.067</v>
       </c>
       <c r="AF295" t="n">
-        <v>24.032</v>
+        <v>24.031</v>
       </c>
       <c r="AG295" t="n">
-        <v>15.186</v>
+        <v>14.98</v>
       </c>
       <c r="AH295" t="n">
-        <v>7.255</v>
+        <v>7.16</v>
       </c>
       <c r="AI295" t="n">
-        <v>3.341</v>
+        <v>3.327</v>
       </c>
       <c r="AJ295" t="n">
-        <v>16.75</v>
+        <v>16.567</v>
       </c>
       <c r="AK295" t="n">
-        <v>9.4</v>
+        <v>5.8</v>
       </c>
       <c r="AL295" t="n">
-        <v>5.3</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="296">
@@ -38786,22 +38786,22 @@
         </is>
       </c>
       <c r="E320" t="n">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="F320" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G320" t="b">
         <v>1</v>
       </c>
       <c r="H320" t="n">
-        <v>1761.339</v>
+        <v>1797.509</v>
       </c>
       <c r="I320" t="n">
-        <v>3.2921</v>
+        <v>3.4141</v>
       </c>
       <c r="J320" t="n">
-        <v>1558.4</v>
+        <v>1569.9</v>
       </c>
       <c r="K320" t="n">
         <v>45</v>
@@ -38822,70 +38822,70 @@
         <v>43</v>
       </c>
       <c r="Q320" t="n">
-        <v>117.937</v>
+        <v>117.658</v>
       </c>
       <c r="R320" t="n">
-        <v>103.323</v>
+        <v>103.371</v>
       </c>
       <c r="S320" t="n">
-        <v>14.613</v>
+        <v>14.287</v>
       </c>
       <c r="T320" t="n">
-        <v>0.29406</v>
+        <v>0.29349</v>
       </c>
       <c r="U320" t="n">
-        <v>0.14675</v>
+        <v>0.14585</v>
       </c>
       <c r="V320" t="n">
-        <v>81.45</v>
+        <v>81.58</v>
       </c>
       <c r="W320" t="n">
-        <v>71.38</v>
+        <v>71.70999999999999</v>
       </c>
       <c r="X320" t="n">
-        <v>0.796</v>
+        <v>0.8017</v>
       </c>
       <c r="Y320" t="n">
-        <v>26.7</v>
+        <v>26.819</v>
       </c>
       <c r="Z320" t="n">
-        <v>58.049</v>
+        <v>58.501</v>
       </c>
       <c r="AA320" t="n">
-        <v>9.339</v>
+        <v>9.275</v>
       </c>
       <c r="AB320" t="n">
-        <v>25.399</v>
+        <v>25.545</v>
       </c>
       <c r="AC320" t="n">
-        <v>18.711</v>
+        <v>18.514</v>
       </c>
       <c r="AD320" t="n">
-        <v>25.323</v>
+        <v>25.183</v>
       </c>
       <c r="AE320" t="n">
-        <v>10.196</v>
+        <v>10.264</v>
       </c>
       <c r="AF320" t="n">
-        <v>24.27</v>
+        <v>24.56</v>
       </c>
       <c r="AG320" t="n">
-        <v>14.069</v>
+        <v>14.233</v>
       </c>
       <c r="AH320" t="n">
-        <v>7.397</v>
+        <v>7.405</v>
       </c>
       <c r="AI320" t="n">
-        <v>4.35</v>
+        <v>4.229</v>
       </c>
       <c r="AJ320" t="n">
-        <v>17.301</v>
+        <v>17.283</v>
       </c>
       <c r="AK320" t="n">
-        <v>7.4</v>
+        <v>7.2</v>
       </c>
       <c r="AL320" t="n">
-        <v>7.7</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="321">
@@ -39026,22 +39026,22 @@
         </is>
       </c>
       <c r="E322" t="n">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="F322" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G322" t="b">
         <v>1</v>
       </c>
       <c r="H322" t="n">
-        <v>1952.581</v>
+        <v>1963.829</v>
       </c>
       <c r="I322" t="n">
-        <v>1.6305</v>
+        <v>1.4886</v>
       </c>
       <c r="J322" t="n">
-        <v>1718.8</v>
+        <v>1716.9</v>
       </c>
       <c r="K322" t="n">
         <v>12</v>
@@ -39062,70 +39062,70 @@
         <v>13</v>
       </c>
       <c r="Q322" t="n">
-        <v>122.082</v>
+        <v>122.218</v>
       </c>
       <c r="R322" t="n">
-        <v>106.871</v>
+        <v>106.709</v>
       </c>
       <c r="S322" t="n">
-        <v>15.211</v>
+        <v>15.509</v>
       </c>
       <c r="T322" t="n">
-        <v>0.29148</v>
+        <v>0.28967</v>
       </c>
       <c r="U322" t="n">
-        <v>0.12812</v>
+        <v>0.13117</v>
       </c>
       <c r="V322" t="n">
-        <v>86.25</v>
+        <v>86.04000000000001</v>
       </c>
       <c r="W322" t="n">
-        <v>75.31</v>
+        <v>74.94</v>
       </c>
       <c r="X322" t="n">
-        <v>0.7576000000000001</v>
+        <v>0.7734</v>
       </c>
       <c r="Y322" t="n">
-        <v>28.992</v>
+        <v>28.917</v>
       </c>
       <c r="Z322" t="n">
-        <v>61.425</v>
+        <v>60.998</v>
       </c>
       <c r="AA322" t="n">
-        <v>9.359</v>
+        <v>9.34</v>
       </c>
       <c r="AB322" t="n">
-        <v>26.593</v>
+        <v>26.521</v>
       </c>
       <c r="AC322" t="n">
-        <v>18.409</v>
+        <v>18.388</v>
       </c>
       <c r="AD322" t="n">
-        <v>23.333</v>
+        <v>23.285</v>
       </c>
       <c r="AE322" t="n">
-        <v>9.971</v>
+        <v>9.935</v>
       </c>
       <c r="AF322" t="n">
-        <v>23.709</v>
+        <v>23.865</v>
       </c>
       <c r="AG322" t="n">
-        <v>16.127</v>
+        <v>16.105</v>
       </c>
       <c r="AH322" t="n">
-        <v>8.048999999999999</v>
+        <v>7.871</v>
       </c>
       <c r="AI322" t="n">
-        <v>4.555</v>
+        <v>4.529</v>
       </c>
       <c r="AJ322" t="n">
-        <v>19.323</v>
+        <v>19.072</v>
       </c>
       <c r="AK322" t="n">
-        <v>4</v>
+        <v>5.4</v>
       </c>
       <c r="AL322" t="n">
-        <v>2.2</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="323">
@@ -41546,22 +41546,22 @@
         </is>
       </c>
       <c r="E343" t="n">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="F343" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G343" t="b">
         <v>1</v>
       </c>
       <c r="H343" t="n">
-        <v>1882.441</v>
+        <v>1843.62</v>
       </c>
       <c r="I343" t="n">
-        <v>2.4266</v>
+        <v>2.6405</v>
       </c>
       <c r="J343" t="n">
-        <v>1724.6</v>
+        <v>1717.5</v>
       </c>
       <c r="K343" t="n">
         <v>22</v>
@@ -41582,70 +41582,70 @@
         <v>25</v>
       </c>
       <c r="Q343" t="n">
-        <v>118.801</v>
+        <v>118.854</v>
       </c>
       <c r="R343" t="n">
-        <v>108.528</v>
+        <v>108.886</v>
       </c>
       <c r="S343" t="n">
-        <v>10.273</v>
+        <v>9.968</v>
       </c>
       <c r="T343" t="n">
-        <v>0.27758</v>
+        <v>0.27955</v>
       </c>
       <c r="U343" t="n">
-        <v>0.12395</v>
+        <v>0.12224</v>
       </c>
       <c r="V343" t="n">
-        <v>82.86</v>
+        <v>82.95999999999999</v>
       </c>
       <c r="W343" t="n">
-        <v>75.84999999999999</v>
+        <v>76.16</v>
       </c>
       <c r="X343" t="n">
-        <v>0.7003</v>
+        <v>0.6807</v>
       </c>
       <c r="Y343" t="n">
-        <v>28.019</v>
+        <v>28.164</v>
       </c>
       <c r="Z343" t="n">
-        <v>62.051</v>
+        <v>62.485</v>
       </c>
       <c r="AA343" t="n">
-        <v>11.769</v>
+        <v>11.852</v>
       </c>
       <c r="AB343" t="n">
-        <v>32.339</v>
+        <v>32.569</v>
       </c>
       <c r="AC343" t="n">
-        <v>14.964</v>
+        <v>14.735</v>
       </c>
       <c r="AD343" t="n">
-        <v>19.211</v>
+        <v>18.955</v>
       </c>
       <c r="AE343" t="n">
-        <v>9.305</v>
+        <v>9.455</v>
       </c>
       <c r="AF343" t="n">
-        <v>23.926</v>
+        <v>24.05</v>
       </c>
       <c r="AG343" t="n">
-        <v>15.926</v>
+        <v>16.015</v>
       </c>
       <c r="AH343" t="n">
-        <v>5.586</v>
+        <v>5.575</v>
       </c>
       <c r="AI343" t="n">
-        <v>3.103</v>
+        <v>3.157</v>
       </c>
       <c r="AJ343" t="n">
-        <v>17.268</v>
+        <v>17.212</v>
       </c>
       <c r="AK343" t="n">
-        <v>8</v>
+        <v>1.2</v>
       </c>
       <c r="AL343" t="n">
-        <v>6</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="344">

</xml_diff>

<commit_message>
Update team snapshot (2026-03-21)
</commit_message>
<xml_diff>
--- a/team_snapshot_2026.xlsx
+++ b/team_snapshot_2026.xlsx
@@ -866,22 +866,22 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="F4" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G4" t="b">
         <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>1707.887</v>
+        <v>1700.07</v>
       </c>
       <c r="I4" t="n">
-        <v>1.9745</v>
+        <v>2.0575</v>
       </c>
       <c r="J4" t="n">
-        <v>1479.2</v>
+        <v>1499.8</v>
       </c>
       <c r="K4" t="n">
         <v>64</v>
@@ -902,70 +902,70 @@
         <v>54</v>
       </c>
       <c r="Q4" t="n">
-        <v>121.636</v>
+        <v>121.234</v>
       </c>
       <c r="R4" t="n">
-        <v>104.361</v>
+        <v>105.697</v>
       </c>
       <c r="S4" t="n">
-        <v>17.275</v>
+        <v>15.537</v>
       </c>
       <c r="T4" t="n">
-        <v>0.28865</v>
+        <v>0.29368</v>
       </c>
       <c r="U4" t="n">
-        <v>0.14997</v>
+        <v>0.14984</v>
       </c>
       <c r="V4" t="n">
-        <v>86.8</v>
+        <v>86.26000000000001</v>
       </c>
       <c r="W4" t="n">
-        <v>74.51000000000001</v>
+        <v>75.13</v>
       </c>
       <c r="X4" t="n">
-        <v>0.8452</v>
+        <v>0.8113</v>
       </c>
       <c r="Y4" t="n">
-        <v>31.173</v>
+        <v>30.919</v>
       </c>
       <c r="Z4" t="n">
-        <v>62.67</v>
+        <v>62.417</v>
       </c>
       <c r="AA4" t="n">
-        <v>10.867</v>
+        <v>10.649</v>
       </c>
       <c r="AB4" t="n">
-        <v>28.302</v>
+        <v>27.894</v>
       </c>
       <c r="AC4" t="n">
-        <v>13.591</v>
+        <v>13.776</v>
       </c>
       <c r="AD4" t="n">
-        <v>18.105</v>
+        <v>18.257</v>
       </c>
       <c r="AE4" t="n">
-        <v>9.974</v>
+        <v>9.978</v>
       </c>
       <c r="AF4" t="n">
-        <v>25.292</v>
+        <v>24.877</v>
       </c>
       <c r="AG4" t="n">
-        <v>17.849</v>
+        <v>17.649</v>
       </c>
       <c r="AH4" t="n">
-        <v>7.23</v>
+        <v>7.163</v>
       </c>
       <c r="AI4" t="n">
-        <v>2.885</v>
+        <v>2.918</v>
       </c>
       <c r="AJ4" t="n">
-        <v>16.243</v>
+        <v>16.155</v>
       </c>
       <c r="AK4" t="n">
-        <v>13</v>
+        <v>6.4</v>
       </c>
       <c r="AL4" t="n">
-        <v>13.8</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="5">
@@ -986,22 +986,22 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="F5" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G5" t="b">
         <v>1</v>
       </c>
       <c r="H5" t="n">
-        <v>1949.262</v>
+        <v>1954.667</v>
       </c>
       <c r="I5" t="n">
-        <v>-1.3255</v>
+        <v>-1.3316</v>
       </c>
       <c r="J5" t="n">
-        <v>1767</v>
+        <v>1760.9</v>
       </c>
       <c r="K5" t="n">
         <v>18</v>
@@ -1022,70 +1022,70 @@
         <v>18</v>
       </c>
       <c r="Q5" t="n">
-        <v>121.371</v>
+        <v>121.89</v>
       </c>
       <c r="R5" t="n">
-        <v>110.604</v>
+        <v>110.305</v>
       </c>
       <c r="S5" t="n">
-        <v>10.767</v>
+        <v>11.585</v>
       </c>
       <c r="T5" t="n">
-        <v>0.28088</v>
+        <v>0.28487</v>
       </c>
       <c r="U5" t="n">
-        <v>0.12877</v>
+        <v>0.1295</v>
       </c>
       <c r="V5" t="n">
-        <v>91.59999999999999</v>
+        <v>91.65000000000001</v>
       </c>
       <c r="W5" t="n">
-        <v>83.44</v>
+        <v>82.95</v>
       </c>
       <c r="X5" t="n">
-        <v>0.7123</v>
+        <v>0.7296</v>
       </c>
       <c r="Y5" t="n">
-        <v>30.319</v>
+        <v>30.377</v>
       </c>
       <c r="Z5" t="n">
-        <v>65.97799999999999</v>
+        <v>66.008</v>
       </c>
       <c r="AA5" t="n">
-        <v>12.583</v>
+        <v>12.601</v>
       </c>
       <c r="AB5" t="n">
-        <v>34.886</v>
+        <v>35.069</v>
       </c>
       <c r="AC5" t="n">
-        <v>18.423</v>
+        <v>18.327</v>
       </c>
       <c r="AD5" t="n">
-        <v>24.105</v>
+        <v>23.988</v>
       </c>
       <c r="AE5" t="n">
-        <v>10.858</v>
+        <v>11.111</v>
       </c>
       <c r="AF5" t="n">
-        <v>27.55</v>
+        <v>27.558</v>
       </c>
       <c r="AG5" t="n">
-        <v>16.106</v>
+        <v>16.12</v>
       </c>
       <c r="AH5" t="n">
-        <v>6.345</v>
+        <v>6.361</v>
       </c>
       <c r="AI5" t="n">
-        <v>5.093</v>
+        <v>5.129</v>
       </c>
       <c r="AJ5" t="n">
-        <v>18.752</v>
+        <v>18.529</v>
       </c>
       <c r="AK5" t="n">
-        <v>5.6</v>
+        <v>4.6</v>
       </c>
       <c r="AL5" t="n">
-        <v>7.4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -1826,22 +1826,22 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="F12" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G12" t="b">
         <v>1</v>
       </c>
       <c r="H12" t="n">
-        <v>2272.125</v>
+        <v>2272.508</v>
       </c>
       <c r="I12" t="n">
-        <v>6.8151</v>
+        <v>6.6001</v>
       </c>
       <c r="J12" t="n">
-        <v>1769.2</v>
+        <v>1753.9</v>
       </c>
       <c r="K12" t="n">
         <v>2</v>
@@ -1862,70 +1862,70 @@
         <v>3</v>
       </c>
       <c r="Q12" t="n">
-        <v>121.138</v>
+        <v>121.602</v>
       </c>
       <c r="R12" t="n">
-        <v>97.108</v>
+        <v>96.53400000000001</v>
       </c>
       <c r="S12" t="n">
-        <v>24.03</v>
+        <v>25.069</v>
       </c>
       <c r="T12" t="n">
-        <v>0.29246</v>
+        <v>0.29327</v>
       </c>
       <c r="U12" t="n">
-        <v>0.1497</v>
+        <v>0.14976</v>
       </c>
       <c r="V12" t="n">
-        <v>86.09</v>
+        <v>86.36</v>
       </c>
       <c r="W12" t="n">
-        <v>68.84</v>
+        <v>68.41</v>
       </c>
       <c r="X12" t="n">
-        <v>0.9416</v>
+        <v>0.9433</v>
       </c>
       <c r="Y12" t="n">
-        <v>30.515</v>
+        <v>30.61</v>
       </c>
       <c r="Z12" t="n">
-        <v>60.799</v>
+        <v>60.822</v>
       </c>
       <c r="AA12" t="n">
-        <v>5.883</v>
+        <v>5.887</v>
       </c>
       <c r="AB12" t="n">
-        <v>16.297</v>
+        <v>16.205</v>
       </c>
       <c r="AC12" t="n">
-        <v>19.177</v>
+        <v>19.249</v>
       </c>
       <c r="AD12" t="n">
-        <v>26.095</v>
+        <v>26.335</v>
       </c>
       <c r="AE12" t="n">
-        <v>11.976</v>
+        <v>12.143</v>
       </c>
       <c r="AF12" t="n">
-        <v>28.655</v>
+        <v>28.938</v>
       </c>
       <c r="AG12" t="n">
-        <v>16.879</v>
+        <v>16.908</v>
       </c>
       <c r="AH12" t="n">
-        <v>7.778</v>
+        <v>7.687</v>
       </c>
       <c r="AI12" t="n">
-        <v>4.218</v>
+        <v>4.441</v>
       </c>
       <c r="AJ12" t="n">
-        <v>16</v>
+        <v>15.857</v>
       </c>
       <c r="AK12" t="n">
-        <v>11</v>
+        <v>14.6</v>
       </c>
       <c r="AL12" t="n">
-        <v>9.6</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="13">
@@ -6386,22 +6386,22 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="F50" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G50" t="b">
         <v>1</v>
       </c>
       <c r="H50" t="n">
-        <v>1859.484</v>
+        <v>1831.145</v>
       </c>
       <c r="I50" t="n">
-        <v>2.557</v>
+        <v>2.3914</v>
       </c>
       <c r="J50" t="n">
-        <v>1672.9</v>
+        <v>1674.2</v>
       </c>
       <c r="K50" t="n">
         <v>36</v>
@@ -6422,70 +6422,70 @@
         <v>34</v>
       </c>
       <c r="Q50" t="n">
-        <v>112.594</v>
+        <v>112.781</v>
       </c>
       <c r="R50" t="n">
-        <v>101.684</v>
+        <v>102.417</v>
       </c>
       <c r="S50" t="n">
-        <v>10.91</v>
+        <v>10.363</v>
       </c>
       <c r="T50" t="n">
-        <v>0.25542</v>
+        <v>0.25948</v>
       </c>
       <c r="U50" t="n">
-        <v>0.13604</v>
+        <v>0.1369</v>
       </c>
       <c r="V50" t="n">
-        <v>74.02</v>
+        <v>73.66</v>
       </c>
       <c r="W50" t="n">
-        <v>66.79000000000001</v>
+        <v>66.75</v>
       </c>
       <c r="X50" t="n">
-        <v>0.6993</v>
+        <v>0.6797</v>
       </c>
       <c r="Y50" t="n">
-        <v>25.401</v>
+        <v>25.194</v>
       </c>
       <c r="Z50" t="n">
-        <v>56.224</v>
+        <v>55.893</v>
       </c>
       <c r="AA50" t="n">
-        <v>8.253</v>
+        <v>8.218</v>
       </c>
       <c r="AB50" t="n">
-        <v>24.388</v>
+        <v>24.405</v>
       </c>
       <c r="AC50" t="n">
-        <v>14.941</v>
+        <v>15.248</v>
       </c>
       <c r="AD50" t="n">
-        <v>20.669</v>
+        <v>21.031</v>
       </c>
       <c r="AE50" t="n">
-        <v>8.583</v>
+        <v>8.826000000000001</v>
       </c>
       <c r="AF50" t="n">
-        <v>23.895</v>
+        <v>23.98</v>
       </c>
       <c r="AG50" t="n">
-        <v>12.855</v>
+        <v>12.59</v>
       </c>
       <c r="AH50" t="n">
-        <v>6.242</v>
+        <v>6.115</v>
       </c>
       <c r="AI50" t="n">
-        <v>2.854</v>
+        <v>2.784</v>
       </c>
       <c r="AJ50" t="n">
-        <v>16.097</v>
+        <v>16.011</v>
       </c>
       <c r="AK50" t="n">
-        <v>-0.6</v>
+        <v>-1</v>
       </c>
       <c r="AL50" t="n">
-        <v>-3.4</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="51">
@@ -7346,22 +7346,22 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="F58" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G58" t="b">
         <v>1</v>
       </c>
       <c r="H58" t="n">
-        <v>2050.719</v>
+        <v>2053.381</v>
       </c>
       <c r="I58" t="n">
-        <v>7.1741</v>
+        <v>6.6189</v>
       </c>
       <c r="J58" t="n">
-        <v>1670.2</v>
+        <v>1662.8</v>
       </c>
       <c r="K58" t="n">
         <v>11</v>
@@ -7382,70 +7382,70 @@
         <v>10</v>
       </c>
       <c r="Q58" t="n">
-        <v>116.057</v>
+        <v>116.791</v>
       </c>
       <c r="R58" t="n">
-        <v>98.01000000000001</v>
+        <v>98.316</v>
       </c>
       <c r="S58" t="n">
-        <v>18.046</v>
+        <v>18.475</v>
       </c>
       <c r="T58" t="n">
-        <v>0.30128</v>
+        <v>0.30395</v>
       </c>
       <c r="U58" t="n">
-        <v>0.16031</v>
+        <v>0.15867</v>
       </c>
       <c r="V58" t="n">
-        <v>77.26000000000001</v>
+        <v>77.67</v>
       </c>
       <c r="W58" t="n">
-        <v>65.18000000000001</v>
+        <v>65.34</v>
       </c>
       <c r="X58" t="n">
-        <v>0.845</v>
+        <v>0.8584000000000001</v>
       </c>
       <c r="Y58" t="n">
-        <v>28.207</v>
+        <v>28.431</v>
       </c>
       <c r="Z58" t="n">
-        <v>58.622</v>
+        <v>58.882</v>
       </c>
       <c r="AA58" t="n">
-        <v>8.273999999999999</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="AB58" t="n">
-        <v>23.604</v>
+        <v>23.697</v>
       </c>
       <c r="AC58" t="n">
-        <v>12.573</v>
+        <v>12.603</v>
       </c>
       <c r="AD58" t="n">
-        <v>17.555</v>
+        <v>17.603</v>
       </c>
       <c r="AE58" t="n">
-        <v>10.473</v>
+        <v>10.693</v>
       </c>
       <c r="AF58" t="n">
-        <v>23.914</v>
+        <v>24.017</v>
       </c>
       <c r="AG58" t="n">
-        <v>18.314</v>
+        <v>18.516</v>
       </c>
       <c r="AH58" t="n">
-        <v>6.874</v>
+        <v>6.887</v>
       </c>
       <c r="AI58" t="n">
-        <v>5.234</v>
+        <v>5.107</v>
       </c>
       <c r="AJ58" t="n">
-        <v>18.069</v>
+        <v>18.048</v>
       </c>
       <c r="AK58" t="n">
-        <v>3.8</v>
+        <v>5.2</v>
       </c>
       <c r="AL58" t="n">
-        <v>6.8</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="59">
@@ -11306,22 +11306,22 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="F91" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G91" t="b">
         <v>1</v>
       </c>
       <c r="H91" t="n">
-        <v>2006.659</v>
+        <v>2007.171</v>
       </c>
       <c r="I91" t="n">
-        <v>3.4651</v>
+        <v>3.5894</v>
       </c>
       <c r="J91" t="n">
-        <v>1722.9</v>
+        <v>1703.3</v>
       </c>
       <c r="K91" t="n">
         <v>4</v>
@@ -11342,70 +11342,70 @@
         <v>4</v>
       </c>
       <c r="Q91" t="n">
-        <v>119.994</v>
+        <v>121.802</v>
       </c>
       <c r="R91" t="n">
-        <v>100.186</v>
+        <v>99.018</v>
       </c>
       <c r="S91" t="n">
-        <v>19.808</v>
+        <v>22.784</v>
       </c>
       <c r="T91" t="n">
-        <v>0.33419</v>
+        <v>0.3326</v>
       </c>
       <c r="U91" t="n">
-        <v>0.15683</v>
+        <v>0.15503</v>
       </c>
       <c r="V91" t="n">
-        <v>86.66</v>
+        <v>87.83</v>
       </c>
       <c r="W91" t="n">
-        <v>72.19</v>
+        <v>71.34999999999999</v>
       </c>
       <c r="X91" t="n">
-        <v>0.78</v>
+        <v>0.796</v>
       </c>
       <c r="Y91" t="n">
-        <v>30.9</v>
+        <v>31.451</v>
       </c>
       <c r="Z91" t="n">
-        <v>64.23999999999999</v>
+        <v>64.551</v>
       </c>
       <c r="AA91" t="n">
-        <v>7.54</v>
+        <v>7.611</v>
       </c>
       <c r="AB91" t="n">
-        <v>24</v>
+        <v>23.952</v>
       </c>
       <c r="AC91" t="n">
+        <v>17.817</v>
+      </c>
+      <c r="AD91" t="n">
+        <v>24.876</v>
+      </c>
+      <c r="AE91" t="n">
+        <v>14.572</v>
+      </c>
+      <c r="AF91" t="n">
+        <v>28.676</v>
+      </c>
+      <c r="AG91" t="n">
+        <v>17.345</v>
+      </c>
+      <c r="AH91" t="n">
+        <v>6.681</v>
+      </c>
+      <c r="AI91" t="n">
+        <v>5.135</v>
+      </c>
+      <c r="AJ91" t="n">
+        <v>17.681</v>
+      </c>
+      <c r="AK91" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="AL91" t="n">
         <v>18</v>
-      </c>
-      <c r="AD91" t="n">
-        <v>25.13</v>
-      </c>
-      <c r="AE91" t="n">
-        <v>14.45</v>
-      </c>
-      <c r="AF91" t="n">
-        <v>28.17</v>
-      </c>
-      <c r="AG91" t="n">
-        <v>16.92</v>
-      </c>
-      <c r="AH91" t="n">
-        <v>6.8</v>
-      </c>
-      <c r="AI91" t="n">
-        <v>5.04</v>
-      </c>
-      <c r="AJ91" t="n">
-        <v>17.8</v>
-      </c>
-      <c r="AK91" t="n">
-        <v>13.2</v>
-      </c>
-      <c r="AL91" t="n">
-        <v>14.1</v>
       </c>
     </row>
     <row r="92">
@@ -12026,22 +12026,22 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="F97" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G97" t="b">
         <v>1</v>
       </c>
       <c r="H97" t="n">
-        <v>1542.857</v>
+        <v>1540.197</v>
       </c>
       <c r="I97" t="n">
-        <v>0.8197</v>
+        <v>0.788</v>
       </c>
       <c r="J97" t="n">
-        <v>1422.2</v>
+        <v>1445.6</v>
       </c>
       <c r="K97" t="n">
         <v>191</v>
@@ -12062,70 +12062,70 @@
         <v>186</v>
       </c>
       <c r="Q97" t="n">
-        <v>112.011</v>
+        <v>111.793</v>
       </c>
       <c r="R97" t="n">
-        <v>107.277</v>
+        <v>108.038</v>
       </c>
       <c r="S97" t="n">
-        <v>4.734</v>
+        <v>3.754</v>
       </c>
       <c r="T97" t="n">
-        <v>0.25616</v>
+        <v>0.25304</v>
       </c>
       <c r="U97" t="n">
-        <v>0.17102</v>
+        <v>0.17098</v>
       </c>
       <c r="V97" t="n">
-        <v>75.06999999999999</v>
+        <v>74.91</v>
       </c>
       <c r="W97" t="n">
-        <v>72.06999999999999</v>
+        <v>72.54000000000001</v>
       </c>
       <c r="X97" t="n">
-        <v>0.616</v>
+        <v>0.5893</v>
       </c>
       <c r="Y97" t="n">
-        <v>26.592</v>
+        <v>26.397</v>
       </c>
       <c r="Z97" t="n">
-        <v>56.496</v>
+        <v>56.181</v>
       </c>
       <c r="AA97" t="n">
-        <v>8.568</v>
+        <v>8.628</v>
       </c>
       <c r="AB97" t="n">
-        <v>26.208</v>
+        <v>26.202</v>
       </c>
       <c r="AC97" t="n">
-        <v>12.56</v>
+        <v>12.866</v>
       </c>
       <c r="AD97" t="n">
-        <v>18.288</v>
+        <v>18.587</v>
       </c>
       <c r="AE97" t="n">
-        <v>8.912000000000001</v>
+        <v>8.746</v>
       </c>
       <c r="AF97" t="n">
-        <v>25.008</v>
+        <v>24.831</v>
       </c>
       <c r="AG97" t="n">
-        <v>14.632</v>
+        <v>14.682</v>
       </c>
       <c r="AH97" t="n">
-        <v>4.48</v>
+        <v>4.396</v>
       </c>
       <c r="AI97" t="n">
-        <v>3.28</v>
+        <v>3.279</v>
       </c>
       <c r="AJ97" t="n">
-        <v>15.472</v>
+        <v>15.465</v>
       </c>
       <c r="AK97" t="n">
-        <v>5.6</v>
+        <v>-0.8</v>
       </c>
       <c r="AL97" t="n">
-        <v>3.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="98">
@@ -13946,22 +13946,22 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="F113" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G113" t="b">
         <v>1</v>
       </c>
       <c r="H113" t="n">
-        <v>1586.191</v>
+        <v>1580.784</v>
       </c>
       <c r="I113" t="n">
-        <v>3.3583</v>
+        <v>3.2408</v>
       </c>
       <c r="J113" t="n">
-        <v>1482.3</v>
+        <v>1500.6</v>
       </c>
       <c r="K113" t="n">
         <v>87</v>
@@ -13982,70 +13982,70 @@
         <v>88</v>
       </c>
       <c r="Q113" t="n">
-        <v>113.557</v>
+        <v>113.029</v>
       </c>
       <c r="R113" t="n">
-        <v>102.691</v>
+        <v>103.66</v>
       </c>
       <c r="S113" t="n">
-        <v>10.866</v>
+        <v>9.369</v>
       </c>
       <c r="T113" t="n">
-        <v>0.30811</v>
+        <v>0.31061</v>
       </c>
       <c r="U113" t="n">
-        <v>0.15271</v>
+        <v>0.1533</v>
       </c>
       <c r="V113" t="n">
-        <v>74.5</v>
+        <v>74.33</v>
       </c>
       <c r="W113" t="n">
-        <v>67.58</v>
+        <v>68.43000000000001</v>
       </c>
       <c r="X113" t="n">
-        <v>0.6903</v>
+        <v>0.6611</v>
       </c>
       <c r="Y113" t="n">
-        <v>25.385</v>
+        <v>25.506</v>
       </c>
       <c r="Z113" t="n">
-        <v>58.372</v>
+        <v>58.784</v>
       </c>
       <c r="AA113" t="n">
-        <v>9.252000000000001</v>
+        <v>9.347</v>
       </c>
       <c r="AB113" t="n">
-        <v>25.159</v>
+        <v>25.142</v>
       </c>
       <c r="AC113" t="n">
-        <v>14.484</v>
+        <v>13.968</v>
       </c>
       <c r="AD113" t="n">
-        <v>19.05</v>
+        <v>18.431</v>
       </c>
       <c r="AE113" t="n">
-        <v>10.974</v>
+        <v>11.017</v>
       </c>
       <c r="AF113" t="n">
-        <v>24.47</v>
+        <v>24.305</v>
       </c>
       <c r="AG113" t="n">
-        <v>12.292</v>
+        <v>12.3</v>
       </c>
       <c r="AH113" t="n">
-        <v>4.801</v>
+        <v>4.828</v>
       </c>
       <c r="AI113" t="n">
-        <v>3.539</v>
+        <v>3.541</v>
       </c>
       <c r="AJ113" t="n">
-        <v>17.585</v>
+        <v>17.425</v>
       </c>
       <c r="AK113" t="n">
-        <v>12</v>
+        <v>6.2</v>
       </c>
       <c r="AL113" t="n">
-        <v>13.2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="114">
@@ -15626,22 +15626,22 @@
         </is>
       </c>
       <c r="E127" t="n">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="F127" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G127" t="b">
         <v>1</v>
       </c>
       <c r="H127" t="n">
-        <v>1831.779</v>
+        <v>1860.117</v>
       </c>
       <c r="I127" t="n">
-        <v>3.3952</v>
+        <v>3.0379</v>
       </c>
       <c r="J127" t="n">
-        <v>1712.2</v>
+        <v>1717.1</v>
       </c>
       <c r="K127" t="n">
         <v>25</v>
@@ -15662,70 +15662,70 @@
         <v>27</v>
       </c>
       <c r="Q127" t="n">
-        <v>118.924</v>
+        <v>119.224</v>
       </c>
       <c r="R127" t="n">
-        <v>104.806</v>
+        <v>105.017</v>
       </c>
       <c r="S127" t="n">
-        <v>14.118</v>
+        <v>14.206</v>
       </c>
       <c r="T127" t="n">
-        <v>0.28864</v>
+        <v>0.29176</v>
       </c>
       <c r="U127" t="n">
-        <v>0.14551</v>
+        <v>0.14178</v>
       </c>
       <c r="V127" t="n">
-        <v>75.15000000000001</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="W127" t="n">
-        <v>66.03</v>
+        <v>65.78</v>
       </c>
       <c r="X127" t="n">
-        <v>0.63</v>
+        <v>0.6503</v>
       </c>
       <c r="Y127" t="n">
-        <v>26.41</v>
+        <v>26.283</v>
       </c>
       <c r="Z127" t="n">
-        <v>53.75</v>
+        <v>53.854</v>
       </c>
       <c r="AA127" t="n">
-        <v>8.02</v>
+        <v>8.038</v>
       </c>
       <c r="AB127" t="n">
-        <v>22.38</v>
+        <v>22.533</v>
       </c>
       <c r="AC127" t="n">
-        <v>14.31</v>
+        <v>14.061</v>
       </c>
       <c r="AD127" t="n">
-        <v>18.58</v>
+        <v>18.323</v>
       </c>
       <c r="AE127" t="n">
-        <v>7.96</v>
+        <v>8.048</v>
       </c>
       <c r="AF127" t="n">
-        <v>19.58</v>
+        <v>19.506</v>
       </c>
       <c r="AG127" t="n">
-        <v>15.34</v>
+        <v>15.205</v>
       </c>
       <c r="AH127" t="n">
-        <v>7.1</v>
+        <v>7.001</v>
       </c>
       <c r="AI127" t="n">
         <v>2</v>
       </c>
       <c r="AJ127" t="n">
-        <v>17.62</v>
+        <v>17.766</v>
       </c>
       <c r="AK127" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="AL127" t="n">
         <v>-1.2</v>
-      </c>
-      <c r="AL127" t="n">
-        <v>-2.5</v>
       </c>
     </row>
     <row r="128">
@@ -15746,22 +15746,22 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="F128" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G128" t="b">
         <v>1</v>
       </c>
       <c r="H128" t="n">
-        <v>2038.996</v>
+        <v>2040.699</v>
       </c>
       <c r="I128" t="n">
-        <v>2.2111</v>
+        <v>1.9908</v>
       </c>
       <c r="J128" t="n">
-        <v>1718</v>
+        <v>1704.9</v>
       </c>
       <c r="K128" t="n">
         <v>6</v>
@@ -15782,70 +15782,70 @@
         <v>6</v>
       </c>
       <c r="Q128" t="n">
-        <v>118.901</v>
+        <v>119.647</v>
       </c>
       <c r="R128" t="n">
-        <v>95.73399999999999</v>
+        <v>95.52800000000001</v>
       </c>
       <c r="S128" t="n">
-        <v>23.167</v>
+        <v>24.119</v>
       </c>
       <c r="T128" t="n">
-        <v>0.32166</v>
+        <v>0.32421</v>
       </c>
       <c r="U128" t="n">
-        <v>0.14689</v>
+        <v>0.14659</v>
       </c>
       <c r="V128" t="n">
-        <v>81.78</v>
+        <v>82.73</v>
       </c>
       <c r="W128" t="n">
-        <v>65.28</v>
+        <v>65.45999999999999</v>
       </c>
       <c r="X128" t="n">
-        <v>0.7879</v>
+        <v>0.8015</v>
       </c>
       <c r="Y128" t="n">
-        <v>29.191</v>
+        <v>29.492</v>
       </c>
       <c r="Z128" t="n">
-        <v>60.281</v>
+        <v>60.655</v>
       </c>
       <c r="AA128" t="n">
-        <v>9.127000000000001</v>
+        <v>9.157</v>
       </c>
       <c r="AB128" t="n">
-        <v>23.734</v>
+        <v>23.688</v>
       </c>
       <c r="AC128" t="n">
-        <v>13.63</v>
+        <v>13.966</v>
       </c>
       <c r="AD128" t="n">
-        <v>20.256</v>
+        <v>20.59</v>
       </c>
       <c r="AE128" t="n">
-        <v>10.71</v>
+        <v>10.938</v>
       </c>
       <c r="AF128" t="n">
-        <v>22.618</v>
+        <v>22.731</v>
       </c>
       <c r="AG128" t="n">
-        <v>17.122</v>
+        <v>17.392</v>
       </c>
       <c r="AH128" t="n">
-        <v>8.904999999999999</v>
+        <v>8.914999999999999</v>
       </c>
       <c r="AI128" t="n">
-        <v>2.7</v>
+        <v>2.788</v>
       </c>
       <c r="AJ128" t="n">
-        <v>15.883</v>
+        <v>15.922</v>
       </c>
       <c r="AK128" t="n">
-        <v>14.8</v>
+        <v>24.8</v>
       </c>
       <c r="AL128" t="n">
-        <v>9.199999999999999</v>
+        <v>10.8</v>
       </c>
     </row>
     <row r="129">
@@ -16586,22 +16586,22 @@
         </is>
       </c>
       <c r="E135" t="n">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="F135" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G135" t="b">
         <v>1</v>
       </c>
       <c r="H135" t="n">
-        <v>1973.656</v>
+        <v>1979.25</v>
       </c>
       <c r="I135" t="n">
-        <v>10.346</v>
+        <v>9.864800000000001</v>
       </c>
       <c r="J135" t="n">
-        <v>1791.1</v>
+        <v>1780.1</v>
       </c>
       <c r="K135" t="n">
         <v>21</v>
@@ -16622,70 +16622,70 @@
         <v>21</v>
       </c>
       <c r="Q135" t="n">
-        <v>109.902</v>
+        <v>109.767</v>
       </c>
       <c r="R135" t="n">
-        <v>101.514</v>
+        <v>100.723</v>
       </c>
       <c r="S135" t="n">
-        <v>8.388999999999999</v>
+        <v>9.044</v>
       </c>
       <c r="T135" t="n">
-        <v>0.25561</v>
+        <v>0.25343</v>
       </c>
       <c r="U135" t="n">
-        <v>0.15124</v>
+        <v>0.14997</v>
       </c>
       <c r="V135" t="n">
-        <v>75.3</v>
+        <v>75.33</v>
       </c>
       <c r="W135" t="n">
-        <v>69.39</v>
+        <v>69.02</v>
       </c>
       <c r="X135" t="n">
-        <v>0.6888</v>
+        <v>0.7091</v>
       </c>
       <c r="Y135" t="n">
-        <v>26.608</v>
+        <v>26.727</v>
       </c>
       <c r="Z135" t="n">
-        <v>59.007</v>
+        <v>59.269</v>
       </c>
       <c r="AA135" t="n">
-        <v>7.359</v>
+        <v>7.229</v>
       </c>
       <c r="AB135" t="n">
-        <v>21.083</v>
+        <v>20.978</v>
       </c>
       <c r="AC135" t="n">
-        <v>14.725</v>
+        <v>14.647</v>
       </c>
       <c r="AD135" t="n">
-        <v>19.228</v>
+        <v>19.033</v>
       </c>
       <c r="AE135" t="n">
-        <v>9.49</v>
+        <v>9.446999999999999</v>
       </c>
       <c r="AF135" t="n">
-        <v>27.48</v>
+        <v>27.684</v>
       </c>
       <c r="AG135" t="n">
-        <v>14.199</v>
+        <v>14.022</v>
       </c>
       <c r="AH135" t="n">
-        <v>5.456</v>
+        <v>5.465</v>
       </c>
       <c r="AI135" t="n">
-        <v>5.684</v>
+        <v>5.658</v>
       </c>
       <c r="AJ135" t="n">
-        <v>14.414</v>
+        <v>14.436</v>
       </c>
       <c r="AK135" t="n">
-        <v>-6.2</v>
+        <v>0</v>
       </c>
       <c r="AL135" t="n">
-        <v>-3.6</v>
+        <v>-3.2</v>
       </c>
     </row>
     <row r="136">
@@ -17066,22 +17066,22 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="F139" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G139" t="b">
         <v>1</v>
       </c>
       <c r="H139" t="n">
-        <v>1886.896</v>
+        <v>1905.506</v>
       </c>
       <c r="I139" t="n">
-        <v>4.7611</v>
+        <v>4.5369</v>
       </c>
       <c r="J139" t="n">
-        <v>1734.8</v>
+        <v>1734</v>
       </c>
       <c r="K139" t="n">
         <v>28</v>
@@ -17102,70 +17102,70 @@
         <v>28</v>
       </c>
       <c r="Q139" t="n">
-        <v>115.762</v>
+        <v>116.168</v>
       </c>
       <c r="R139" t="n">
-        <v>106.053</v>
+        <v>106.38</v>
       </c>
       <c r="S139" t="n">
-        <v>9.709</v>
+        <v>9.788</v>
       </c>
       <c r="T139" t="n">
-        <v>0.31063</v>
+        <v>0.30777</v>
       </c>
       <c r="U139" t="n">
-        <v>0.14646</v>
+        <v>0.14633</v>
       </c>
       <c r="V139" t="n">
-        <v>80.59999999999999</v>
+        <v>81.06999999999999</v>
       </c>
       <c r="W139" t="n">
-        <v>73.8</v>
+        <v>74.2</v>
       </c>
       <c r="X139" t="n">
-        <v>0.6119</v>
+        <v>0.6318</v>
       </c>
       <c r="Y139" t="n">
-        <v>27.993</v>
+        <v>28.205</v>
       </c>
       <c r="Z139" t="n">
-        <v>60.486</v>
+        <v>60.593</v>
       </c>
       <c r="AA139" t="n">
-        <v>8.029999999999999</v>
+        <v>8.131</v>
       </c>
       <c r="AB139" t="n">
-        <v>23.466</v>
+        <v>23.638</v>
       </c>
       <c r="AC139" t="n">
-        <v>16.408</v>
+        <v>16.359</v>
       </c>
       <c r="AD139" t="n">
-        <v>22.652</v>
+        <v>22.614</v>
       </c>
       <c r="AE139" t="n">
-        <v>11.001</v>
+        <v>10.954</v>
       </c>
       <c r="AF139" t="n">
-        <v>24.38</v>
+        <v>24.656</v>
       </c>
       <c r="AG139" t="n">
-        <v>15.702</v>
+        <v>15.885</v>
       </c>
       <c r="AH139" t="n">
-        <v>7.106</v>
+        <v>7.011</v>
       </c>
       <c r="AI139" t="n">
-        <v>4.204</v>
+        <v>4.458</v>
       </c>
       <c r="AJ139" t="n">
-        <v>18.464</v>
+        <v>18.359</v>
       </c>
       <c r="AK139" t="n">
-        <v>-3</v>
+        <v>0.2</v>
       </c>
       <c r="AL139" t="n">
-        <v>-1</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="140">
@@ -18026,22 +18026,22 @@
         </is>
       </c>
       <c r="E147" t="n">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="F147" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G147" t="b">
         <v>1</v>
       </c>
       <c r="H147" t="n">
-        <v>1418.21</v>
+        <v>1417.828</v>
       </c>
       <c r="I147" t="n">
-        <v>2.3581</v>
+        <v>2.3176</v>
       </c>
       <c r="J147" t="n">
-        <v>1378.8</v>
+        <v>1411.9</v>
       </c>
       <c r="K147" t="n">
         <v>216</v>
@@ -18062,70 +18062,70 @@
         <v>198</v>
       </c>
       <c r="Q147" t="n">
-        <v>109.383</v>
+        <v>108.226</v>
       </c>
       <c r="R147" t="n">
-        <v>104.38</v>
+        <v>105.253</v>
       </c>
       <c r="S147" t="n">
-        <v>5.003</v>
+        <v>2.973</v>
       </c>
       <c r="T147" t="n">
-        <v>0.31186</v>
+        <v>0.31587</v>
       </c>
       <c r="U147" t="n">
-        <v>0.18305</v>
+        <v>0.18279</v>
       </c>
       <c r="V147" t="n">
-        <v>74.13</v>
+        <v>73.48999999999999</v>
       </c>
       <c r="W147" t="n">
-        <v>71.11</v>
+        <v>71.89</v>
       </c>
       <c r="X147" t="n">
-        <v>0.7086</v>
+        <v>0.6797</v>
       </c>
       <c r="Y147" t="n">
-        <v>27.456</v>
+        <v>27.24</v>
       </c>
       <c r="Z147" t="n">
-        <v>57.041</v>
+        <v>57.492</v>
       </c>
       <c r="AA147" t="n">
-        <v>5.962</v>
+        <v>6.046</v>
       </c>
       <c r="AB147" t="n">
-        <v>16.459</v>
+        <v>16.917</v>
       </c>
       <c r="AC147" t="n">
-        <v>13.261</v>
+        <v>12.967</v>
       </c>
       <c r="AD147" t="n">
-        <v>19.909</v>
+        <v>19.46</v>
       </c>
       <c r="AE147" t="n">
-        <v>10.4</v>
+        <v>10.499</v>
       </c>
       <c r="AF147" t="n">
-        <v>22.551</v>
+        <v>22.37</v>
       </c>
       <c r="AG147" t="n">
-        <v>13.669</v>
+        <v>13.697</v>
       </c>
       <c r="AH147" t="n">
-        <v>7.816</v>
+        <v>7.756</v>
       </c>
       <c r="AI147" t="n">
-        <v>5.379</v>
+        <v>5.368</v>
       </c>
       <c r="AJ147" t="n">
-        <v>17.593</v>
+        <v>17.78</v>
       </c>
       <c r="AK147" t="n">
-        <v>10.4</v>
+        <v>0.2</v>
       </c>
       <c r="AL147" t="n">
-        <v>7.1</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="148">
@@ -20426,22 +20426,22 @@
         </is>
       </c>
       <c r="E167" t="n">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="F167" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G167" t="b">
         <v>1</v>
       </c>
       <c r="H167" t="n">
-        <v>1772.273</v>
+        <v>1794.728</v>
       </c>
       <c r="I167" t="n">
-        <v>11.776</v>
+        <v>11.4257</v>
       </c>
       <c r="J167" t="n">
-        <v>1635.9</v>
+        <v>1636.7</v>
       </c>
       <c r="K167" t="n">
         <v>31</v>
@@ -20462,70 +20462,70 @@
         <v>32</v>
       </c>
       <c r="Q167" t="n">
-        <v>117.066</v>
+        <v>117.437</v>
       </c>
       <c r="R167" t="n">
-        <v>102.955</v>
+        <v>102.471</v>
       </c>
       <c r="S167" t="n">
-        <v>14.111</v>
+        <v>14.966</v>
       </c>
       <c r="T167" t="n">
-        <v>0.30957</v>
+        <v>0.31068</v>
       </c>
       <c r="U167" t="n">
-        <v>0.15694</v>
+        <v>0.15663</v>
       </c>
       <c r="V167" t="n">
-        <v>81.70999999999999</v>
+        <v>81.86</v>
       </c>
       <c r="W167" t="n">
-        <v>71.33</v>
+        <v>70.97</v>
       </c>
       <c r="X167" t="n">
-        <v>0.7487</v>
+        <v>0.7673</v>
       </c>
       <c r="Y167" t="n">
-        <v>29.906</v>
+        <v>29.84</v>
       </c>
       <c r="Z167" t="n">
-        <v>59.815</v>
+        <v>59.855</v>
       </c>
       <c r="AA167" t="n">
-        <v>6.546</v>
+        <v>6.753</v>
       </c>
       <c r="AB167" t="n">
-        <v>18.952</v>
+        <v>19.142</v>
       </c>
       <c r="AC167" t="n">
-        <v>15.348</v>
+        <v>15.429</v>
       </c>
       <c r="AD167" t="n">
-        <v>22.337</v>
+        <v>22.687</v>
       </c>
       <c r="AE167" t="n">
-        <v>10.827</v>
+        <v>11.055</v>
       </c>
       <c r="AF167" t="n">
-        <v>24.038</v>
+        <v>24.356</v>
       </c>
       <c r="AG167" t="n">
-        <v>15.973</v>
+        <v>16.207</v>
       </c>
       <c r="AH167" t="n">
-        <v>7.857</v>
+        <v>7.844</v>
       </c>
       <c r="AI167" t="n">
-        <v>3.389</v>
+        <v>3.338</v>
       </c>
       <c r="AJ167" t="n">
-        <v>15.461</v>
+        <v>15.476</v>
       </c>
       <c r="AK167" t="n">
-        <v>2</v>
+        <v>0.4</v>
       </c>
       <c r="AL167" t="n">
-        <v>2.8</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="168">
@@ -20546,22 +20546,22 @@
         </is>
       </c>
       <c r="E168" t="n">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F168" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G168" t="b">
         <v>1</v>
       </c>
       <c r="H168" t="n">
-        <v>1780.382</v>
+        <v>1762.633</v>
       </c>
       <c r="I168" t="n">
-        <v>8.9497</v>
+        <v>8.696899999999999</v>
       </c>
       <c r="J168" t="n">
-        <v>1429.2</v>
+        <v>1434.9</v>
       </c>
       <c r="K168" t="n">
         <v>93</v>
@@ -20582,70 +20582,70 @@
         <v>64</v>
       </c>
       <c r="Q168" t="n">
-        <v>121.342</v>
+        <v>119.936</v>
       </c>
       <c r="R168" t="n">
-        <v>106.311</v>
+        <v>106.804</v>
       </c>
       <c r="S168" t="n">
-        <v>15.031</v>
+        <v>13.132</v>
       </c>
       <c r="T168" t="n">
-        <v>0.22217</v>
+        <v>0.22513</v>
       </c>
       <c r="U168" t="n">
-        <v>0.1392</v>
+        <v>0.14135</v>
       </c>
       <c r="V168" t="n">
-        <v>87.28</v>
+        <v>86.06</v>
       </c>
       <c r="W168" t="n">
-        <v>76.45</v>
+        <v>76.48999999999999</v>
       </c>
       <c r="X168" t="n">
-        <v>0.9669</v>
+        <v>0.9295</v>
       </c>
       <c r="Y168" t="n">
-        <v>30.073</v>
+        <v>29.641</v>
       </c>
       <c r="Z168" t="n">
-        <v>59.207</v>
+        <v>58.968</v>
       </c>
       <c r="AA168" t="n">
-        <v>9.337</v>
+        <v>9.276</v>
       </c>
       <c r="AB168" t="n">
-        <v>25.403</v>
+        <v>25.571</v>
       </c>
       <c r="AC168" t="n">
-        <v>17.528</v>
+        <v>17.314</v>
       </c>
       <c r="AD168" t="n">
-        <v>23.276</v>
+        <v>22.974</v>
       </c>
       <c r="AE168" t="n">
-        <v>7.597</v>
+        <v>7.583</v>
       </c>
       <c r="AF168" t="n">
-        <v>25.648</v>
+        <v>25.333</v>
       </c>
       <c r="AG168" t="n">
-        <v>15.066</v>
+        <v>14.795</v>
       </c>
       <c r="AH168" t="n">
-        <v>6.913</v>
+        <v>6.974</v>
       </c>
       <c r="AI168" t="n">
-        <v>2.979</v>
+        <v>3</v>
       </c>
       <c r="AJ168" t="n">
-        <v>16.709</v>
+        <v>16.596</v>
       </c>
       <c r="AK168" t="n">
-        <v>2.4</v>
+        <v>-2.4</v>
       </c>
       <c r="AL168" t="n">
-        <v>7.7</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="169">
@@ -21266,22 +21266,22 @@
         </is>
       </c>
       <c r="E174" t="n">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="F174" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G174" t="b">
         <v>1</v>
       </c>
       <c r="H174" t="n">
-        <v>1747.812</v>
+        <v>1725.357</v>
       </c>
       <c r="I174" t="n">
-        <v>-1.7576</v>
+        <v>-1.6662</v>
       </c>
       <c r="J174" t="n">
-        <v>1658.3</v>
+        <v>1660.3</v>
       </c>
       <c r="K174" t="n">
         <v>52</v>
@@ -21302,70 +21302,70 @@
         <v>58</v>
       </c>
       <c r="Q174" t="n">
-        <v>114.923</v>
+        <v>114.338</v>
       </c>
       <c r="R174" t="n">
-        <v>109.478</v>
+        <v>109.815</v>
       </c>
       <c r="S174" t="n">
-        <v>5.446</v>
+        <v>4.523</v>
       </c>
       <c r="T174" t="n">
-        <v>0.29962</v>
+        <v>0.29735</v>
       </c>
       <c r="U174" t="n">
-        <v>0.16854</v>
+        <v>0.16754</v>
       </c>
       <c r="V174" t="n">
-        <v>79.56</v>
+        <v>79.09</v>
       </c>
       <c r="W174" t="n">
-        <v>75.38</v>
+        <v>75.54000000000001</v>
       </c>
       <c r="X174" t="n">
-        <v>0.6171</v>
+        <v>0.599</v>
       </c>
       <c r="Y174" t="n">
-        <v>27.957</v>
+        <v>27.637</v>
       </c>
       <c r="Z174" t="n">
-        <v>56.944</v>
+        <v>56.97</v>
       </c>
       <c r="AA174" t="n">
-        <v>7.203</v>
+        <v>7.335</v>
       </c>
       <c r="AB174" t="n">
-        <v>20.784</v>
+        <v>21.082</v>
       </c>
       <c r="AC174" t="n">
-        <v>16.704</v>
+        <v>16.659</v>
       </c>
       <c r="AD174" t="n">
-        <v>24.173</v>
+        <v>23.93</v>
       </c>
       <c r="AE174" t="n">
-        <v>10.116</v>
+        <v>10.025</v>
       </c>
       <c r="AF174" t="n">
-        <v>22.777</v>
+        <v>22.82</v>
       </c>
       <c r="AG174" t="n">
-        <v>14.421</v>
+        <v>14.443</v>
       </c>
       <c r="AH174" t="n">
-        <v>6.748</v>
+        <v>6.647</v>
       </c>
       <c r="AI174" t="n">
-        <v>3.755</v>
+        <v>3.742</v>
       </c>
       <c r="AJ174" t="n">
-        <v>17.742</v>
+        <v>17.826</v>
       </c>
       <c r="AK174" t="n">
-        <v>0.4</v>
+        <v>-3.2</v>
       </c>
       <c r="AL174" t="n">
-        <v>-0.2</v>
+        <v>-3.5</v>
       </c>
     </row>
     <row r="175">
@@ -25706,22 +25706,22 @@
         </is>
       </c>
       <c r="E211" t="n">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="F211" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G211" t="b">
         <v>1</v>
       </c>
       <c r="H211" t="n">
-        <v>1573.879</v>
+        <v>1569.56</v>
       </c>
       <c r="I211" t="n">
-        <v>-3.696</v>
+        <v>-3.4213</v>
       </c>
       <c r="J211" t="n">
-        <v>1515.8</v>
+        <v>1532.4</v>
       </c>
       <c r="K211" t="n">
         <v>72</v>
@@ -25742,70 +25742,70 @@
         <v>72</v>
       </c>
       <c r="Q211" t="n">
-        <v>108.741</v>
+        <v>107.639</v>
       </c>
       <c r="R211" t="n">
-        <v>97.495</v>
+        <v>98.39400000000001</v>
       </c>
       <c r="S211" t="n">
-        <v>11.246</v>
+        <v>9.244999999999999</v>
       </c>
       <c r="T211" t="n">
-        <v>0.22502</v>
+        <v>0.22193</v>
       </c>
       <c r="U211" t="n">
-        <v>0.13537</v>
+        <v>0.13436</v>
       </c>
       <c r="V211" t="n">
-        <v>69.18000000000001</v>
+        <v>68.48999999999999</v>
       </c>
       <c r="W211" t="n">
-        <v>62.11</v>
+        <v>62.66</v>
       </c>
       <c r="X211" t="n">
-        <v>0.6498</v>
+        <v>0.6239</v>
       </c>
       <c r="Y211" t="n">
-        <v>25.162</v>
+        <v>25.035</v>
       </c>
       <c r="Z211" t="n">
-        <v>55.172</v>
+        <v>55.185</v>
       </c>
       <c r="AA211" t="n">
-        <v>7.284</v>
+        <v>7.141</v>
       </c>
       <c r="AB211" t="n">
-        <v>21.815</v>
+        <v>21.572</v>
       </c>
       <c r="AC211" t="n">
-        <v>10.255</v>
+        <v>10.112</v>
       </c>
       <c r="AD211" t="n">
-        <v>14.486</v>
+        <v>14.439</v>
       </c>
       <c r="AE211" t="n">
-        <v>6.426</v>
+        <v>6.369</v>
       </c>
       <c r="AF211" t="n">
-        <v>22.431</v>
+        <v>22.546</v>
       </c>
       <c r="AG211" t="n">
-        <v>13.992</v>
+        <v>13.786</v>
       </c>
       <c r="AH211" t="n">
-        <v>6.401</v>
+        <v>6.397</v>
       </c>
       <c r="AI211" t="n">
-        <v>2.918</v>
+        <v>2.908</v>
       </c>
       <c r="AJ211" t="n">
-        <v>15.138</v>
+        <v>15.249</v>
       </c>
       <c r="AK211" t="n">
-        <v>14.4</v>
+        <v>4.8</v>
       </c>
       <c r="AL211" t="n">
-        <v>10.8</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="212">
@@ -28106,22 +28106,22 @@
         </is>
       </c>
       <c r="E231" t="n">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F231" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G231" t="b">
         <v>1</v>
       </c>
       <c r="H231" t="n">
-        <v>1272.073</v>
+        <v>1271.561</v>
       </c>
       <c r="I231" t="n">
-        <v>-0.4587</v>
+        <v>-0.3388</v>
       </c>
       <c r="J231" t="n">
-        <v>1381.2</v>
+        <v>1406.5</v>
       </c>
       <c r="K231" t="n">
         <v>288</v>
@@ -28142,70 +28142,70 @@
         <v>300</v>
       </c>
       <c r="Q231" t="n">
-        <v>104.266</v>
+        <v>103.391</v>
       </c>
       <c r="R231" t="n">
-        <v>106.277</v>
+        <v>108.666</v>
       </c>
       <c r="S231" t="n">
-        <v>-2.011</v>
+        <v>-5.275</v>
       </c>
       <c r="T231" t="n">
-        <v>0.28965</v>
+        <v>0.29509</v>
       </c>
       <c r="U231" t="n">
-        <v>0.15843</v>
+        <v>0.15573</v>
       </c>
       <c r="V231" t="n">
-        <v>75.41</v>
+        <v>74.70999999999999</v>
       </c>
       <c r="W231" t="n">
-        <v>77.64</v>
+        <v>79.15000000000001</v>
       </c>
       <c r="X231" t="n">
-        <v>0.4727</v>
+        <v>0.4514</v>
       </c>
       <c r="Y231" t="n">
-        <v>24.784</v>
+        <v>24.523</v>
       </c>
       <c r="Z231" t="n">
-        <v>59.52</v>
+        <v>59.66</v>
       </c>
       <c r="AA231" t="n">
-        <v>5.876</v>
+        <v>5.88</v>
       </c>
       <c r="AB231" t="n">
-        <v>18.479</v>
+        <v>18.569</v>
       </c>
       <c r="AC231" t="n">
-        <v>18.6</v>
+        <v>18.551</v>
       </c>
       <c r="AD231" t="n">
-        <v>24.965</v>
+        <v>24.764</v>
       </c>
       <c r="AE231" t="n">
-        <v>9.502000000000001</v>
+        <v>9.451000000000001</v>
       </c>
       <c r="AF231" t="n">
-        <v>22.27</v>
+        <v>21.833</v>
       </c>
       <c r="AG231" t="n">
-        <v>11.124</v>
+        <v>10.935</v>
       </c>
       <c r="AH231" t="n">
-        <v>6.954</v>
+        <v>6.822</v>
       </c>
       <c r="AI231" t="n">
-        <v>4.66</v>
+        <v>4.625</v>
       </c>
       <c r="AJ231" t="n">
-        <v>19.406</v>
+        <v>19.34</v>
       </c>
       <c r="AK231" t="n">
-        <v>10</v>
+        <v>-3.6</v>
       </c>
       <c r="AL231" t="n">
-        <v>9.9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="232">
@@ -28586,22 +28586,22 @@
         </is>
       </c>
       <c r="E235" t="n">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="F235" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G235" t="b">
         <v>1</v>
       </c>
       <c r="H235" t="n">
-        <v>2010.028</v>
+        <v>2011.512</v>
       </c>
       <c r="I235" t="n">
-        <v>-0.7024</v>
+        <v>-0.6772</v>
       </c>
       <c r="J235" t="n">
-        <v>1769.7</v>
+        <v>1753.9</v>
       </c>
       <c r="K235" t="n">
         <v>8</v>
@@ -28622,70 +28622,70 @@
         <v>9</v>
       </c>
       <c r="Q235" t="n">
-        <v>124.873</v>
+        <v>125.909</v>
       </c>
       <c r="R235" t="n">
-        <v>107.488</v>
+        <v>107.355</v>
       </c>
       <c r="S235" t="n">
-        <v>17.385</v>
+        <v>18.555</v>
       </c>
       <c r="T235" t="n">
-        <v>0.31102</v>
+        <v>0.31279</v>
       </c>
       <c r="U235" t="n">
-        <v>0.13371</v>
+        <v>0.13549</v>
       </c>
       <c r="V235" t="n">
-        <v>81.64</v>
+        <v>82.45999999999999</v>
       </c>
       <c r="W235" t="n">
-        <v>70.16</v>
+        <v>70.17</v>
       </c>
       <c r="X235" t="n">
-        <v>0.7734</v>
+        <v>0.7796</v>
       </c>
       <c r="Y235" t="n">
-        <v>29.717</v>
+        <v>30.117</v>
       </c>
       <c r="Z235" t="n">
-        <v>60.092</v>
+        <v>60.234</v>
       </c>
       <c r="AA235" t="n">
-        <v>9.266</v>
+        <v>9.454000000000001</v>
       </c>
       <c r="AB235" t="n">
-        <v>24.538</v>
+        <v>24.523</v>
       </c>
       <c r="AC235" t="n">
-        <v>11.996</v>
+        <v>11.912</v>
       </c>
       <c r="AD235" t="n">
-        <v>16.196</v>
+        <v>16.133</v>
       </c>
       <c r="AE235" t="n">
-        <v>10.547</v>
+        <v>10.702</v>
       </c>
       <c r="AF235" t="n">
-        <v>22.963</v>
+        <v>23.08</v>
       </c>
       <c r="AG235" t="n">
-        <v>19.475</v>
+        <v>19.674</v>
       </c>
       <c r="AH235" t="n">
-        <v>5.484</v>
+        <v>5.496</v>
       </c>
       <c r="AI235" t="n">
-        <v>2.66</v>
+        <v>2.777</v>
       </c>
       <c r="AJ235" t="n">
-        <v>14.998</v>
+        <v>14.901</v>
       </c>
       <c r="AK235" t="n">
-        <v>8</v>
+        <v>15.4</v>
       </c>
       <c r="AL235" t="n">
-        <v>5.2</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="236">
@@ -30986,22 +30986,22 @@
         </is>
       </c>
       <c r="E255" t="n">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="F255" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G255" t="b">
         <v>1</v>
       </c>
       <c r="H255" t="n">
-        <v>1782.784</v>
+        <v>1764.174</v>
       </c>
       <c r="I255" t="n">
-        <v>0.0374</v>
+        <v>0.252</v>
       </c>
       <c r="J255" t="n">
-        <v>1596.2</v>
+        <v>1603.2</v>
       </c>
       <c r="K255" t="n">
         <v>35</v>
@@ -31022,70 +31022,70 @@
         <v>40</v>
       </c>
       <c r="Q255" t="n">
-        <v>117.619</v>
+        <v>117.526</v>
       </c>
       <c r="R255" t="n">
-        <v>104.107</v>
+        <v>104.506</v>
       </c>
       <c r="S255" t="n">
-        <v>13.513</v>
+        <v>13.02</v>
       </c>
       <c r="T255" t="n">
-        <v>0.35044</v>
+        <v>0.34803</v>
       </c>
       <c r="U255" t="n">
-        <v>0.14983</v>
+        <v>0.14781</v>
       </c>
       <c r="V255" t="n">
-        <v>82.72</v>
+        <v>82.89</v>
       </c>
       <c r="W255" t="n">
-        <v>73.08</v>
+        <v>73.62</v>
       </c>
       <c r="X255" t="n">
-        <v>0.7512</v>
+        <v>0.7295</v>
       </c>
       <c r="Y255" t="n">
-        <v>29.996</v>
+        <v>30.029</v>
       </c>
       <c r="Z255" t="n">
-        <v>64.364</v>
+        <v>64.654</v>
       </c>
       <c r="AA255" t="n">
-        <v>9.962</v>
+        <v>10.045</v>
       </c>
       <c r="AB255" t="n">
-        <v>28.922</v>
+        <v>29.031</v>
       </c>
       <c r="AC255" t="n">
-        <v>12.619</v>
+        <v>12.642</v>
       </c>
       <c r="AD255" t="n">
-        <v>16.714</v>
+        <v>16.648</v>
       </c>
       <c r="AE255" t="n">
-        <v>11.947</v>
+        <v>11.883</v>
       </c>
       <c r="AF255" t="n">
-        <v>21.511</v>
+        <v>21.681</v>
       </c>
       <c r="AG255" t="n">
-        <v>16.636</v>
+        <v>16.679</v>
       </c>
       <c r="AH255" t="n">
-        <v>8.653</v>
+        <v>8.641999999999999</v>
       </c>
       <c r="AI255" t="n">
-        <v>3.614</v>
+        <v>3.576</v>
       </c>
       <c r="AJ255" t="n">
-        <v>19.519</v>
+        <v>19.533</v>
       </c>
       <c r="AK255" t="n">
-        <v>0.8</v>
+        <v>3.6</v>
       </c>
       <c r="AL255" t="n">
-        <v>4.8</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="256">
@@ -33146,22 +33146,22 @@
         </is>
       </c>
       <c r="E273" t="n">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="F273" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G273" t="b">
         <v>1</v>
       </c>
       <c r="H273" t="n">
-        <v>1984.929</v>
+        <v>1989.246</v>
       </c>
       <c r="I273" t="n">
-        <v>5.6609</v>
+        <v>5.7241</v>
       </c>
       <c r="J273" t="n">
-        <v>1691.6</v>
+        <v>1684.5</v>
       </c>
       <c r="K273" t="n">
         <v>17</v>
@@ -33182,70 +33182,70 @@
         <v>16</v>
       </c>
       <c r="Q273" t="n">
-        <v>113.974</v>
+        <v>114.409</v>
       </c>
       <c r="R273" t="n">
-        <v>98.164</v>
+        <v>97.80200000000001</v>
       </c>
       <c r="S273" t="n">
-        <v>15.81</v>
+        <v>16.607</v>
       </c>
       <c r="T273" t="n">
-        <v>0.3224</v>
+        <v>0.32084</v>
       </c>
       <c r="U273" t="n">
-        <v>0.14223</v>
+        <v>0.14183</v>
       </c>
       <c r="V273" t="n">
-        <v>81.48</v>
+        <v>81.47</v>
       </c>
       <c r="W273" t="n">
-        <v>69.83</v>
+        <v>69.36</v>
       </c>
       <c r="X273" t="n">
-        <v>0.8249</v>
+        <v>0.8298</v>
       </c>
       <c r="Y273" t="n">
-        <v>27.934</v>
+        <v>27.908</v>
       </c>
       <c r="Z273" t="n">
-        <v>61.515</v>
+        <v>61.396</v>
       </c>
       <c r="AA273" t="n">
-        <v>6.897</v>
+        <v>7.022</v>
       </c>
       <c r="AB273" t="n">
-        <v>20.788</v>
+        <v>21.087</v>
       </c>
       <c r="AC273" t="n">
-        <v>18.719</v>
+        <v>18.63</v>
       </c>
       <c r="AD273" t="n">
-        <v>25.725</v>
+        <v>25.659</v>
       </c>
       <c r="AE273" t="n">
-        <v>11.589</v>
+        <v>11.631</v>
       </c>
       <c r="AF273" t="n">
-        <v>24.568</v>
+        <v>24.889</v>
       </c>
       <c r="AG273" t="n">
-        <v>16.239</v>
+        <v>16.148</v>
       </c>
       <c r="AH273" t="n">
-        <v>7.928</v>
+        <v>7.736</v>
       </c>
       <c r="AI273" t="n">
-        <v>4.907</v>
+        <v>4.922</v>
       </c>
       <c r="AJ273" t="n">
-        <v>17.292</v>
+        <v>17.105</v>
       </c>
       <c r="AK273" t="n">
-        <v>10.6</v>
+        <v>15.2</v>
       </c>
       <c r="AL273" t="n">
-        <v>9.800000000000001</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="274">
@@ -34586,19 +34586,19 @@
         </is>
       </c>
       <c r="E285" t="n">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="F285" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G285" t="b">
         <v>1</v>
       </c>
       <c r="H285" t="n">
-        <v>1897.088</v>
+        <v>1914.838</v>
       </c>
       <c r="I285" t="n">
-        <v>-1.4465</v>
+        <v>-1.3934</v>
       </c>
       <c r="J285" t="n">
         <v>1716.9</v>
@@ -34622,70 +34622,70 @@
         <v>20</v>
       </c>
       <c r="Q285" t="n">
-        <v>116.86</v>
+        <v>116.955</v>
       </c>
       <c r="R285" t="n">
-        <v>102.568</v>
+        <v>101.617</v>
       </c>
       <c r="S285" t="n">
-        <v>14.292</v>
+        <v>15.338</v>
       </c>
       <c r="T285" t="n">
-        <v>0.36001</v>
+        <v>0.35639</v>
       </c>
       <c r="U285" t="n">
-        <v>0.16434</v>
+        <v>0.16761</v>
       </c>
       <c r="V285" t="n">
-        <v>79.31999999999999</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="W285" t="n">
-        <v>69.43000000000001</v>
+        <v>68.83</v>
       </c>
       <c r="X285" t="n">
-        <v>0.6589</v>
+        <v>0.68</v>
       </c>
       <c r="Y285" t="n">
-        <v>28.223</v>
+        <v>28.382</v>
       </c>
       <c r="Z285" t="n">
-        <v>61.155</v>
+        <v>61.036</v>
       </c>
       <c r="AA285" t="n">
-        <v>6.456</v>
+        <v>6.585</v>
       </c>
       <c r="AB285" t="n">
-        <v>19.366</v>
+        <v>19.418</v>
       </c>
       <c r="AC285" t="n">
-        <v>16.419</v>
+        <v>16.047</v>
       </c>
       <c r="AD285" t="n">
-        <v>23.694</v>
+        <v>23.12</v>
       </c>
       <c r="AE285" t="n">
-        <v>14.854</v>
+        <v>14.687</v>
       </c>
       <c r="AF285" t="n">
-        <v>25.785</v>
+        <v>25.945</v>
       </c>
       <c r="AG285" t="n">
-        <v>16.852</v>
+        <v>16.993</v>
       </c>
       <c r="AH285" t="n">
-        <v>7.474</v>
+        <v>7.415</v>
       </c>
       <c r="AI285" t="n">
-        <v>3.576</v>
+        <v>3.542</v>
       </c>
       <c r="AJ285" t="n">
-        <v>17.927</v>
+        <v>17.724</v>
       </c>
       <c r="AK285" t="n">
-        <v>3.2</v>
+        <v>8</v>
       </c>
       <c r="AL285" t="n">
-        <v>5.8</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="286">
@@ -34706,22 +34706,22 @@
         </is>
       </c>
       <c r="E286" t="n">
-        <v>124</v>
+        <v>137</v>
       </c>
       <c r="F286" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G286" t="b">
         <v>1</v>
       </c>
       <c r="H286" t="n">
-        <v>1466.924</v>
+        <v>1465.222</v>
       </c>
       <c r="I286" t="n">
-        <v>3.3618</v>
+        <v>3.2842</v>
       </c>
       <c r="J286" t="n">
-        <v>1407.8</v>
+        <v>1433</v>
       </c>
       <c r="K286" t="n">
         <v>187</v>
@@ -34742,70 +34742,70 @@
         <v>172</v>
       </c>
       <c r="Q286" t="n">
-        <v>109.904</v>
+        <v>109.103</v>
       </c>
       <c r="R286" t="n">
-        <v>103.284</v>
+        <v>104.707</v>
       </c>
       <c r="S286" t="n">
-        <v>6.621</v>
+        <v>4.396</v>
       </c>
       <c r="T286" t="n">
-        <v>0.328</v>
+        <v>0.33012</v>
       </c>
       <c r="U286" t="n">
-        <v>0.15886</v>
+        <v>0.16077</v>
       </c>
       <c r="V286" t="n">
-        <v>78.18000000000001</v>
+        <v>77.91</v>
       </c>
       <c r="W286" t="n">
-        <v>73.88</v>
+        <v>75.29000000000001</v>
       </c>
       <c r="X286" t="n">
-        <v>0.6919999999999999</v>
+        <v>0.6621</v>
       </c>
       <c r="Y286" t="n">
-        <v>27.935</v>
+        <v>27.901</v>
       </c>
       <c r="Z286" t="n">
-        <v>62.106</v>
+        <v>62.186</v>
       </c>
       <c r="AA286" t="n">
-        <v>6.485</v>
+        <v>6.357</v>
       </c>
       <c r="AB286" t="n">
-        <v>19.086</v>
+        <v>19.113</v>
       </c>
       <c r="AC286" t="n">
-        <v>15.826</v>
+        <v>15.748</v>
       </c>
       <c r="AD286" t="n">
-        <v>20.735</v>
+        <v>20.721</v>
       </c>
       <c r="AE286" t="n">
-        <v>11.262</v>
+        <v>11.232</v>
       </c>
       <c r="AF286" t="n">
-        <v>22.847</v>
+        <v>22.601</v>
       </c>
       <c r="AG286" t="n">
-        <v>12.673</v>
+        <v>12.709</v>
       </c>
       <c r="AH286" t="n">
-        <v>9.012</v>
+        <v>8.993</v>
       </c>
       <c r="AI286" t="n">
-        <v>3.616</v>
+        <v>3.836</v>
       </c>
       <c r="AJ286" t="n">
-        <v>18.499</v>
+        <v>18.657</v>
       </c>
       <c r="AK286" t="n">
-        <v>19.8</v>
+        <v>7.6</v>
       </c>
       <c r="AL286" t="n">
-        <v>13.8</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="287">
@@ -35306,22 +35306,22 @@
         </is>
       </c>
       <c r="E291" t="n">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="F291" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G291" t="b">
         <v>1</v>
       </c>
       <c r="H291" t="n">
-        <v>2010.735</v>
+        <v>2018.552</v>
       </c>
       <c r="I291" t="n">
-        <v>9.579599999999999</v>
+        <v>8.9857</v>
       </c>
       <c r="J291" t="n">
-        <v>1772.3</v>
+        <v>1767</v>
       </c>
       <c r="K291" t="n">
         <v>20</v>
@@ -35342,70 +35342,70 @@
         <v>19</v>
       </c>
       <c r="Q291" t="n">
-        <v>117.198</v>
+        <v>118.539</v>
       </c>
       <c r="R291" t="n">
-        <v>106.696</v>
+        <v>106.753</v>
       </c>
       <c r="S291" t="n">
-        <v>10.501</v>
+        <v>11.786</v>
       </c>
       <c r="T291" t="n">
-        <v>0.28931</v>
+        <v>0.28763</v>
       </c>
       <c r="U291" t="n">
-        <v>0.155</v>
+        <v>0.15503</v>
       </c>
       <c r="V291" t="n">
-        <v>80.11</v>
+        <v>80.83</v>
       </c>
       <c r="W291" t="n">
-        <v>72.65000000000001</v>
+        <v>72.56</v>
       </c>
       <c r="X291" t="n">
-        <v>0.6801</v>
+        <v>0.7</v>
       </c>
       <c r="Y291" t="n">
-        <v>28.887</v>
+        <v>29.08</v>
       </c>
       <c r="Z291" t="n">
-        <v>60.977</v>
+        <v>60.71</v>
       </c>
       <c r="AA291" t="n">
-        <v>11.421</v>
+        <v>11.45</v>
       </c>
       <c r="AB291" t="n">
-        <v>28.851</v>
+        <v>28.61</v>
       </c>
       <c r="AC291" t="n">
-        <v>11.833</v>
+        <v>11.88</v>
       </c>
       <c r="AD291" t="n">
-        <v>16.628</v>
+        <v>16.75</v>
       </c>
       <c r="AE291" t="n">
-        <v>10.493</v>
+        <v>10.39</v>
       </c>
       <c r="AF291" t="n">
-        <v>24.642</v>
+        <v>24.58</v>
       </c>
       <c r="AG291" t="n">
-        <v>15.917</v>
+        <v>15.98</v>
       </c>
       <c r="AH291" t="n">
-        <v>5.867</v>
+        <v>5.97</v>
       </c>
       <c r="AI291" t="n">
-        <v>3.7</v>
+        <v>3.77</v>
       </c>
       <c r="AJ291" t="n">
-        <v>16.442</v>
+        <v>16.45</v>
       </c>
       <c r="AK291" t="n">
-        <v>-3</v>
+        <v>-1.4</v>
       </c>
       <c r="AL291" t="n">
-        <v>5.2</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="292">
@@ -36866,22 +36866,22 @@
         </is>
       </c>
       <c r="E304" t="n">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="F304" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G304" t="b">
         <v>1</v>
       </c>
       <c r="H304" t="n">
-        <v>1828.635</v>
+        <v>1805.81</v>
       </c>
       <c r="I304" t="n">
-        <v>5.8051</v>
+        <v>5.3176</v>
       </c>
       <c r="J304" t="n">
-        <v>1712.7</v>
+        <v>1713.5</v>
       </c>
       <c r="K304" t="n">
         <v>54</v>
@@ -36902,70 +36902,70 @@
         <v>51</v>
       </c>
       <c r="Q304" t="n">
-        <v>112.997</v>
+        <v>112.743</v>
       </c>
       <c r="R304" t="n">
-        <v>110.03</v>
+        <v>109.749</v>
       </c>
       <c r="S304" t="n">
-        <v>2.967</v>
+        <v>2.994</v>
       </c>
       <c r="T304" t="n">
-        <v>0.31466</v>
+        <v>0.32046</v>
       </c>
       <c r="U304" t="n">
-        <v>0.15426</v>
+        <v>0.15757</v>
       </c>
       <c r="V304" t="n">
-        <v>80.73</v>
+        <v>80.56999999999999</v>
       </c>
       <c r="W304" t="n">
-        <v>78.5</v>
+        <v>78.33</v>
       </c>
       <c r="X304" t="n">
-        <v>0.6492</v>
+        <v>0.63</v>
       </c>
       <c r="Y304" t="n">
-        <v>29.306</v>
+        <v>29.28</v>
       </c>
       <c r="Z304" t="n">
-        <v>63.031</v>
+        <v>63.39</v>
       </c>
       <c r="AA304" t="n">
-        <v>7.792</v>
+        <v>8.01</v>
       </c>
       <c r="AB304" t="n">
-        <v>21.68</v>
+        <v>22.1</v>
       </c>
       <c r="AC304" t="n">
-        <v>14.328</v>
+        <v>14</v>
       </c>
       <c r="AD304" t="n">
-        <v>19.39</v>
+        <v>19.3</v>
       </c>
       <c r="AE304" t="n">
-        <v>11.145</v>
+        <v>11.68</v>
       </c>
       <c r="AF304" t="n">
-        <v>23.526</v>
+        <v>23.71</v>
       </c>
       <c r="AG304" t="n">
-        <v>15.688</v>
+        <v>15.72</v>
       </c>
       <c r="AH304" t="n">
-        <v>5.638</v>
+        <v>5.55</v>
       </c>
       <c r="AI304" t="n">
-        <v>3</v>
+        <v>2.96</v>
       </c>
       <c r="AJ304" t="n">
-        <v>17.601</v>
+        <v>17.51</v>
       </c>
       <c r="AK304" t="n">
-        <v>-8.800000000000001</v>
+        <v>-9.4</v>
       </c>
       <c r="AL304" t="n">
-        <v>-4.5</v>
+        <v>-2.9</v>
       </c>
     </row>
     <row r="305">
@@ -36986,22 +36986,22 @@
         </is>
       </c>
       <c r="E305" t="n">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="F305" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G305" t="b">
         <v>1</v>
       </c>
       <c r="H305" t="n">
-        <v>1874.227</v>
+        <v>1897.052</v>
       </c>
       <c r="I305" t="n">
-        <v>2.8463</v>
+        <v>2.9774</v>
       </c>
       <c r="J305" t="n">
-        <v>1706.3</v>
+        <v>1708.6</v>
       </c>
       <c r="K305" t="n">
         <v>27</v>
@@ -37022,70 +37022,70 @@
         <v>30</v>
       </c>
       <c r="Q305" t="n">
-        <v>117.179</v>
+        <v>116.926</v>
       </c>
       <c r="R305" t="n">
-        <v>107.51</v>
+        <v>107.231</v>
       </c>
       <c r="S305" t="n">
-        <v>9.669</v>
+        <v>9.695</v>
       </c>
       <c r="T305" t="n">
-        <v>0.30552</v>
+        <v>0.30733</v>
       </c>
       <c r="U305" t="n">
-        <v>0.13246</v>
+        <v>0.1316</v>
       </c>
       <c r="V305" t="n">
         <v>77.64</v>
       </c>
       <c r="W305" t="n">
-        <v>71.02</v>
+        <v>71</v>
       </c>
       <c r="X305" t="n">
-        <v>0.6712</v>
+        <v>0.6879999999999999</v>
       </c>
       <c r="Y305" t="n">
-        <v>27.393</v>
+        <v>27.397</v>
       </c>
       <c r="Z305" t="n">
-        <v>58.465</v>
+        <v>58.839</v>
       </c>
       <c r="AA305" t="n">
-        <v>8.045</v>
+        <v>7.957</v>
       </c>
       <c r="AB305" t="n">
-        <v>21.113</v>
+        <v>21.057</v>
       </c>
       <c r="AC305" t="n">
-        <v>14.955</v>
+        <v>14.9</v>
       </c>
       <c r="AD305" t="n">
-        <v>19.613</v>
+        <v>19.56</v>
       </c>
       <c r="AE305" t="n">
-        <v>9.468999999999999</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="AF305" t="n">
-        <v>21.432</v>
+        <v>21.576</v>
       </c>
       <c r="AG305" t="n">
-        <v>16.565</v>
+        <v>16.332</v>
       </c>
       <c r="AH305" t="n">
-        <v>6.196</v>
+        <v>6.449</v>
       </c>
       <c r="AI305" t="n">
-        <v>2.942</v>
+        <v>3.158</v>
       </c>
       <c r="AJ305" t="n">
-        <v>16.887</v>
+        <v>16.872</v>
       </c>
       <c r="AK305" t="n">
-        <v>10.2</v>
+        <v>7</v>
       </c>
       <c r="AL305" t="n">
-        <v>1.3</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="306">
@@ -38426,22 +38426,22 @@
         </is>
       </c>
       <c r="E317" t="n">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="F317" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G317" t="b">
         <v>1</v>
       </c>
       <c r="H317" t="n">
-        <v>1897.511</v>
+        <v>1917.024</v>
       </c>
       <c r="I317" t="n">
-        <v>0.1736</v>
+        <v>0.2638</v>
       </c>
       <c r="J317" t="n">
-        <v>1611.4</v>
+        <v>1617</v>
       </c>
       <c r="K317" t="n">
         <v>30</v>
@@ -38462,70 +38462,70 @@
         <v>26</v>
       </c>
       <c r="Q317" t="n">
-        <v>119.564</v>
+        <v>119.887</v>
       </c>
       <c r="R317" t="n">
-        <v>103.487</v>
+        <v>103.861</v>
       </c>
       <c r="S317" t="n">
-        <v>16.077</v>
+        <v>16.026</v>
       </c>
       <c r="T317" t="n">
-        <v>0.30319</v>
+        <v>0.30557</v>
       </c>
       <c r="U317" t="n">
-        <v>0.14787</v>
+        <v>0.14772</v>
       </c>
       <c r="V317" t="n">
-        <v>81.64</v>
+        <v>81.84999999999999</v>
       </c>
       <c r="W317" t="n">
-        <v>70.79000000000001</v>
+        <v>71.03</v>
       </c>
       <c r="X317" t="n">
-        <v>0.8194</v>
+        <v>0.8247</v>
       </c>
       <c r="Y317" t="n">
-        <v>28.736</v>
+        <v>28.701</v>
       </c>
       <c r="Z317" t="n">
-        <v>58.139</v>
+        <v>58.266</v>
       </c>
       <c r="AA317" t="n">
-        <v>8.287000000000001</v>
+        <v>8.506</v>
       </c>
       <c r="AB317" t="n">
-        <v>23.648</v>
+        <v>23.893</v>
       </c>
       <c r="AC317" t="n">
-        <v>15.817</v>
+        <v>15.526</v>
       </c>
       <c r="AD317" t="n">
-        <v>22.419</v>
+        <v>22.146</v>
       </c>
       <c r="AE317" t="n">
-        <v>9.676</v>
+        <v>9.679</v>
       </c>
       <c r="AF317" t="n">
-        <v>22.081</v>
+        <v>21.88</v>
       </c>
       <c r="AG317" t="n">
-        <v>17.188</v>
+        <v>17.14</v>
       </c>
       <c r="AH317" t="n">
-        <v>8.669</v>
+        <v>8.571</v>
       </c>
       <c r="AI317" t="n">
-        <v>2.88</v>
+        <v>2.776</v>
       </c>
       <c r="AJ317" t="n">
-        <v>18.963</v>
+        <v>19.042</v>
       </c>
       <c r="AK317" t="n">
-        <v>4.2</v>
+        <v>11.6</v>
       </c>
       <c r="AL317" t="n">
-        <v>4.9</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="318">
@@ -39266,22 +39266,22 @@
         </is>
       </c>
       <c r="E324" t="n">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="F324" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G324" t="b">
         <v>1</v>
       </c>
       <c r="H324" t="n">
-        <v>1806.305</v>
+        <v>1786.792</v>
       </c>
       <c r="I324" t="n">
-        <v>5.8793</v>
+        <v>5.5318</v>
       </c>
       <c r="J324" t="n">
-        <v>1641.5</v>
+        <v>1652</v>
       </c>
       <c r="K324" t="n">
         <v>33</v>
@@ -39302,70 +39302,70 @@
         <v>35</v>
       </c>
       <c r="Q324" t="n">
-        <v>114.594</v>
+        <v>114.709</v>
       </c>
       <c r="R324" t="n">
-        <v>104.935</v>
+        <v>105.725</v>
       </c>
       <c r="S324" t="n">
-        <v>9.659000000000001</v>
+        <v>8.984</v>
       </c>
       <c r="T324" t="n">
-        <v>0.31301</v>
+        <v>0.31015</v>
       </c>
       <c r="U324" t="n">
-        <v>0.14469</v>
+        <v>0.1437</v>
       </c>
       <c r="V324" t="n">
-        <v>77.04000000000001</v>
+        <v>77.11</v>
       </c>
       <c r="W324" t="n">
-        <v>70.84999999999999</v>
+        <v>71.37</v>
       </c>
       <c r="X324" t="n">
-        <v>0.7432</v>
+        <v>0.7212</v>
       </c>
       <c r="Y324" t="n">
-        <v>27.523</v>
+        <v>27.519</v>
       </c>
       <c r="Z324" t="n">
-        <v>59.681</v>
+        <v>59.353</v>
       </c>
       <c r="AA324" t="n">
-        <v>9.641</v>
+        <v>9.362</v>
       </c>
       <c r="AB324" t="n">
-        <v>26.937</v>
+        <v>26.577</v>
       </c>
       <c r="AC324" t="n">
-        <v>12.911</v>
+        <v>13.517</v>
       </c>
       <c r="AD324" t="n">
-        <v>18.685</v>
+        <v>19.383</v>
       </c>
       <c r="AE324" t="n">
-        <v>10.222</v>
+        <v>10.142</v>
       </c>
       <c r="AF324" t="n">
-        <v>22.147</v>
+        <v>22.321</v>
       </c>
       <c r="AG324" t="n">
-        <v>15.495</v>
+        <v>15.635</v>
       </c>
       <c r="AH324" t="n">
-        <v>7.274</v>
+        <v>7.185</v>
       </c>
       <c r="AI324" t="n">
-        <v>2.177</v>
+        <v>2.103</v>
       </c>
       <c r="AJ324" t="n">
-        <v>15.933</v>
+        <v>15.893</v>
       </c>
       <c r="AK324" t="n">
-        <v>-1</v>
+        <v>-4.8</v>
       </c>
       <c r="AL324" t="n">
-        <v>0.9</v>
+        <v>-0.8</v>
       </c>
     </row>
     <row r="325">
@@ -39386,22 +39386,22 @@
         </is>
       </c>
       <c r="E325" t="n">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="F325" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G325" t="b">
         <v>1</v>
       </c>
       <c r="H325" t="n">
-        <v>1964.334</v>
+        <v>1966.747</v>
       </c>
       <c r="I325" t="n">
-        <v>12.2076</v>
+        <v>11.7947</v>
       </c>
       <c r="J325" t="n">
-        <v>1665.9</v>
+        <v>1654.9</v>
       </c>
       <c r="K325" t="n">
         <v>13</v>
@@ -39422,70 +39422,70 @@
         <v>12</v>
       </c>
       <c r="Q325" t="n">
-        <v>119.042</v>
+        <v>119.416</v>
       </c>
       <c r="R325" t="n">
-        <v>100.852</v>
+        <v>101.187</v>
       </c>
       <c r="S325" t="n">
-        <v>18.19</v>
+        <v>18.229</v>
       </c>
       <c r="T325" t="n">
-        <v>0.31535</v>
+        <v>0.31319</v>
       </c>
       <c r="U325" t="n">
-        <v>0.15437</v>
+        <v>0.15637</v>
       </c>
       <c r="V325" t="n">
-        <v>80.56</v>
+        <v>80.7</v>
       </c>
       <c r="W325" t="n">
-        <v>68.45999999999999</v>
+        <v>68.58</v>
       </c>
       <c r="X325" t="n">
-        <v>0.8462</v>
+        <v>0.8582</v>
       </c>
       <c r="Y325" t="n">
-        <v>28.144</v>
+        <v>28.17</v>
       </c>
       <c r="Z325" t="n">
-        <v>60.77</v>
+        <v>60.58</v>
       </c>
       <c r="AA325" t="n">
-        <v>10.101</v>
+        <v>10.221</v>
       </c>
       <c r="AB325" t="n">
-        <v>27.998</v>
+        <v>27.957</v>
       </c>
       <c r="AC325" t="n">
-        <v>14.058</v>
+        <v>14.021</v>
       </c>
       <c r="AD325" t="n">
-        <v>19.297</v>
+        <v>19.133</v>
       </c>
       <c r="AE325" t="n">
-        <v>11.868</v>
+        <v>11.815</v>
       </c>
       <c r="AF325" t="n">
-        <v>25.406</v>
+        <v>25.568</v>
       </c>
       <c r="AG325" t="n">
-        <v>16.499</v>
+        <v>16.396</v>
       </c>
       <c r="AH325" t="n">
-        <v>6.473</v>
+        <v>6.411</v>
       </c>
       <c r="AI325" t="n">
-        <v>6.426</v>
+        <v>6.333</v>
       </c>
       <c r="AJ325" t="n">
-        <v>17.854</v>
+        <v>17.572</v>
       </c>
       <c r="AK325" t="n">
-        <v>6.8</v>
+        <v>7.6</v>
       </c>
       <c r="AL325" t="n">
-        <v>7</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="326">
@@ -41786,22 +41786,22 @@
         </is>
       </c>
       <c r="E345" t="n">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="F345" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G345" t="b">
         <v>1</v>
       </c>
       <c r="H345" t="n">
-        <v>1470.5</v>
+        <v>1468.087</v>
       </c>
       <c r="I345" t="n">
-        <v>2.7419</v>
+        <v>2.7298</v>
       </c>
       <c r="J345" t="n">
-        <v>1431.7</v>
+        <v>1452.2</v>
       </c>
       <c r="K345" t="n">
         <v>140</v>
@@ -41822,70 +41822,70 @@
         <v>127</v>
       </c>
       <c r="Q345" t="n">
-        <v>115.44</v>
+        <v>115.45</v>
       </c>
       <c r="R345" t="n">
-        <v>108.906</v>
+        <v>109.658</v>
       </c>
       <c r="S345" t="n">
-        <v>6.534</v>
+        <v>5.792</v>
       </c>
       <c r="T345" t="n">
-        <v>0.29712</v>
+        <v>0.29826</v>
       </c>
       <c r="U345" t="n">
-        <v>0.15689</v>
+        <v>0.15513</v>
       </c>
       <c r="V345" t="n">
-        <v>79.86</v>
+        <v>79.70999999999999</v>
       </c>
       <c r="W345" t="n">
-        <v>75.31</v>
+        <v>75.65000000000001</v>
       </c>
       <c r="X345" t="n">
-        <v>0.6588000000000001</v>
+        <v>0.6319</v>
       </c>
       <c r="Y345" t="n">
-        <v>28.149</v>
+        <v>28.069</v>
       </c>
       <c r="Z345" t="n">
-        <v>58.31</v>
+        <v>58.412</v>
       </c>
       <c r="AA345" t="n">
-        <v>7.071</v>
+        <v>7.312</v>
       </c>
       <c r="AB345" t="n">
-        <v>19.605</v>
+        <v>20.046</v>
       </c>
       <c r="AC345" t="n">
-        <v>16.496</v>
+        <v>16.259</v>
       </c>
       <c r="AD345" t="n">
-        <v>22.185</v>
+        <v>21.743</v>
       </c>
       <c r="AE345" t="n">
-        <v>9.743</v>
+        <v>9.654999999999999</v>
       </c>
       <c r="AF345" t="n">
-        <v>22.565</v>
+        <v>22.289</v>
       </c>
       <c r="AG345" t="n">
-        <v>13.233</v>
+        <v>13.167</v>
       </c>
       <c r="AH345" t="n">
-        <v>7.071</v>
+        <v>7.127</v>
       </c>
       <c r="AI345" t="n">
-        <v>4.387</v>
+        <v>4.361</v>
       </c>
       <c r="AJ345" t="n">
-        <v>17.465</v>
+        <v>17.34</v>
       </c>
       <c r="AK345" t="n">
-        <v>10</v>
+        <v>7.4</v>
       </c>
       <c r="AL345" t="n">
-        <v>6.3</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="346">
@@ -42386,22 +42386,22 @@
         </is>
       </c>
       <c r="E350" t="n">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="F350" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G350" t="b">
         <v>1</v>
       </c>
       <c r="H350" t="n">
-        <v>1607.876</v>
+        <v>1602.282</v>
       </c>
       <c r="I350" t="n">
-        <v>1.5554</v>
+        <v>1.6245</v>
       </c>
       <c r="J350" t="n">
-        <v>1462.4</v>
+        <v>1480.3</v>
       </c>
       <c r="K350" t="n">
         <v>106</v>
@@ -42422,70 +42422,70 @@
         <v>98</v>
       </c>
       <c r="Q350" t="n">
-        <v>107.215</v>
+        <v>106.575</v>
       </c>
       <c r="R350" t="n">
-        <v>99.24299999999999</v>
+        <v>99.312</v>
       </c>
       <c r="S350" t="n">
-        <v>7.972</v>
+        <v>7.264</v>
       </c>
       <c r="T350" t="n">
-        <v>0.32874</v>
+        <v>0.32763</v>
       </c>
       <c r="U350" t="n">
-        <v>0.17351</v>
+        <v>0.17095</v>
       </c>
       <c r="V350" t="n">
-        <v>72.93000000000001</v>
+        <v>72.53</v>
       </c>
       <c r="W350" t="n">
-        <v>67.51000000000001</v>
+        <v>67.59</v>
       </c>
       <c r="X350" t="n">
-        <v>0.76</v>
+        <v>0.7284</v>
       </c>
       <c r="Y350" t="n">
-        <v>25.57</v>
+        <v>25.506</v>
       </c>
       <c r="Z350" t="n">
-        <v>58.97</v>
+        <v>59.251</v>
       </c>
       <c r="AA350" t="n">
-        <v>6.21</v>
+        <v>6.156</v>
       </c>
       <c r="AB350" t="n">
-        <v>18.41</v>
+        <v>18.457</v>
       </c>
       <c r="AC350" t="n">
-        <v>15.5</v>
+        <v>15.303</v>
       </c>
       <c r="AD350" t="n">
-        <v>21.84</v>
+        <v>21.71</v>
       </c>
       <c r="AE350" t="n">
-        <v>12.42</v>
+        <v>12.437</v>
       </c>
       <c r="AF350" t="n">
-        <v>24.78</v>
+        <v>24.988</v>
       </c>
       <c r="AG350" t="n">
-        <v>10.4</v>
+        <v>10.186</v>
       </c>
       <c r="AH350" t="n">
-        <v>5.46</v>
+        <v>5.476</v>
       </c>
       <c r="AI350" t="n">
-        <v>2.91</v>
+        <v>2.874</v>
       </c>
       <c r="AJ350" t="n">
-        <v>18.35</v>
+        <v>18.177</v>
       </c>
       <c r="AK350" t="n">
-        <v>15.4</v>
+        <v>10.8</v>
       </c>
       <c r="AL350" t="n">
-        <v>8.4</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="351">
@@ -43466,22 +43466,22 @@
         </is>
       </c>
       <c r="E359" t="n">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="F359" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G359" t="b">
         <v>1</v>
       </c>
       <c r="H359" t="n">
-        <v>1427.37</v>
+        <v>1425.887</v>
       </c>
       <c r="I359" t="n">
-        <v>1.0039</v>
+        <v>1.0261</v>
       </c>
       <c r="J359" t="n">
-        <v>1430.9</v>
+        <v>1452.8</v>
       </c>
       <c r="K359" t="n">
         <v>181</v>
@@ -43502,70 +43502,70 @@
         <v>189</v>
       </c>
       <c r="Q359" t="n">
-        <v>119.175</v>
+        <v>118.645</v>
       </c>
       <c r="R359" t="n">
-        <v>116.563</v>
+        <v>117.977</v>
       </c>
       <c r="S359" t="n">
-        <v>2.613</v>
+        <v>0.667</v>
       </c>
       <c r="T359" t="n">
-        <v>0.2859</v>
+        <v>0.28974</v>
       </c>
       <c r="U359" t="n">
-        <v>0.14407</v>
+        <v>0.14319</v>
       </c>
       <c r="V359" t="n">
-        <v>84.93000000000001</v>
+        <v>84.31</v>
       </c>
       <c r="W359" t="n">
-        <v>83.23</v>
+        <v>83.92</v>
       </c>
       <c r="X359" t="n">
-        <v>0.6094000000000001</v>
+        <v>0.5836</v>
       </c>
       <c r="Y359" t="n">
-        <v>29.025</v>
+        <v>29.037</v>
       </c>
       <c r="Z359" t="n">
-        <v>60.577</v>
+        <v>60.623</v>
       </c>
       <c r="AA359" t="n">
-        <v>9.981999999999999</v>
+        <v>9.831</v>
       </c>
       <c r="AB359" t="n">
-        <v>28.127</v>
+        <v>27.947</v>
       </c>
       <c r="AC359" t="n">
-        <v>16.494</v>
+        <v>16.052</v>
       </c>
       <c r="AD359" t="n">
-        <v>22.103</v>
+        <v>21.487</v>
       </c>
       <c r="AE359" t="n">
-        <v>9.201000000000001</v>
+        <v>9.109</v>
       </c>
       <c r="AF359" t="n">
-        <v>22.584</v>
+        <v>22.176</v>
       </c>
       <c r="AG359" t="n">
-        <v>15.768</v>
+        <v>15.915</v>
       </c>
       <c r="AH359" t="n">
-        <v>5.969</v>
+        <v>6.061</v>
       </c>
       <c r="AI359" t="n">
-        <v>2.927</v>
+        <v>2.912</v>
       </c>
       <c r="AJ359" t="n">
-        <v>19.708</v>
+        <v>19.412</v>
       </c>
       <c r="AK359" t="n">
-        <v>6.4</v>
+        <v>-3.6</v>
       </c>
       <c r="AL359" t="n">
-        <v>6.3</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="360">

</xml_diff>

<commit_message>
Update team snapshot (2026-03-22)
</commit_message>
<xml_diff>
--- a/team_snapshot_2026.xlsx
+++ b/team_snapshot_2026.xlsx
@@ -2306,22 +2306,22 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F16" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G16" t="b">
         <v>1</v>
       </c>
       <c r="H16" t="n">
-        <v>1980.818</v>
+        <v>1988.127</v>
       </c>
       <c r="I16" t="n">
-        <v>5.1109</v>
+        <v>5.0738</v>
       </c>
       <c r="J16" t="n">
-        <v>1727.5</v>
+        <v>1731.7</v>
       </c>
       <c r="K16" t="n">
         <v>15</v>
@@ -2342,70 +2342,70 @@
         <v>15</v>
       </c>
       <c r="Q16" t="n">
-        <v>122.949</v>
+        <v>122.969</v>
       </c>
       <c r="R16" t="n">
-        <v>109.035</v>
+        <v>109.338</v>
       </c>
       <c r="S16" t="n">
-        <v>13.914</v>
+        <v>13.631</v>
       </c>
       <c r="T16" t="n">
-        <v>0.2989</v>
+        <v>0.29609</v>
       </c>
       <c r="U16" t="n">
-        <v>0.12071</v>
+        <v>0.11967</v>
       </c>
       <c r="V16" t="n">
-        <v>90.19</v>
+        <v>90.28</v>
       </c>
       <c r="W16" t="n">
-        <v>80.01000000000001</v>
+        <v>80.3</v>
       </c>
       <c r="X16" t="n">
-        <v>0.7731</v>
+        <v>0.7793</v>
       </c>
       <c r="Y16" t="n">
-        <v>32.335</v>
+        <v>32.379</v>
       </c>
       <c r="Z16" t="n">
-        <v>64.456</v>
+        <v>64.524</v>
       </c>
       <c r="AA16" t="n">
-        <v>8.169</v>
+        <v>8.228</v>
       </c>
       <c r="AB16" t="n">
-        <v>21.397</v>
+        <v>21.214</v>
       </c>
       <c r="AC16" t="n">
-        <v>17.354</v>
+        <v>17.29</v>
       </c>
       <c r="AD16" t="n">
-        <v>23.126</v>
+        <v>23.062</v>
       </c>
       <c r="AE16" t="n">
-        <v>10.1</v>
+        <v>10.014</v>
       </c>
       <c r="AF16" t="n">
-        <v>23.725</v>
+        <v>23.869</v>
       </c>
       <c r="AG16" t="n">
-        <v>17.321</v>
+        <v>17.283</v>
       </c>
       <c r="AH16" t="n">
-        <v>7.291</v>
+        <v>7.31</v>
       </c>
       <c r="AI16" t="n">
-        <v>5.113</v>
+        <v>5.145</v>
       </c>
       <c r="AJ16" t="n">
-        <v>16.665</v>
+        <v>16.448</v>
       </c>
       <c r="AK16" t="n">
-        <v>8</v>
+        <v>8.4</v>
       </c>
       <c r="AL16" t="n">
-        <v>4.7</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="17">
@@ -8546,22 +8546,22 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="F68" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G68" t="b">
         <v>1</v>
       </c>
       <c r="H68" t="n">
-        <v>1695.429</v>
+        <v>1719.075</v>
       </c>
       <c r="I68" t="n">
-        <v>-1.7367</v>
+        <v>-1.4928</v>
       </c>
       <c r="J68" t="n">
-        <v>1574.5</v>
+        <v>1578.5</v>
       </c>
       <c r="K68" t="n">
         <v>78</v>
@@ -8582,70 +8582,70 @@
         <v>69</v>
       </c>
       <c r="Q68" t="n">
-        <v>110.224</v>
+        <v>110.613</v>
       </c>
       <c r="R68" t="n">
-        <v>102.463</v>
+        <v>102.177</v>
       </c>
       <c r="S68" t="n">
-        <v>7.761</v>
+        <v>8.436</v>
       </c>
       <c r="T68" t="n">
-        <v>0.24689</v>
+        <v>0.24972</v>
       </c>
       <c r="U68" t="n">
-        <v>0.16853</v>
+        <v>0.16976</v>
       </c>
       <c r="V68" t="n">
-        <v>74.56999999999999</v>
+        <v>74.72</v>
       </c>
       <c r="W68" t="n">
-        <v>69.73</v>
+        <v>69.45</v>
       </c>
       <c r="X68" t="n">
-        <v>0.6889</v>
+        <v>0.6974</v>
       </c>
       <c r="Y68" t="n">
-        <v>24.038</v>
+        <v>24.213</v>
       </c>
       <c r="Z68" t="n">
-        <v>53.26</v>
+        <v>53.414</v>
       </c>
       <c r="AA68" t="n">
-        <v>7.699</v>
+        <v>7.734</v>
       </c>
       <c r="AB68" t="n">
-        <v>22.186</v>
+        <v>22.331</v>
       </c>
       <c r="AC68" t="n">
-        <v>18.766</v>
+        <v>18.53</v>
       </c>
       <c r="AD68" t="n">
-        <v>24.887</v>
+        <v>24.557</v>
       </c>
       <c r="AE68" t="n">
-        <v>7.751</v>
+        <v>7.919</v>
       </c>
       <c r="AF68" t="n">
-        <v>23.103</v>
+        <v>23.258</v>
       </c>
       <c r="AG68" t="n">
-        <v>14.291</v>
+        <v>14.377</v>
       </c>
       <c r="AH68" t="n">
-        <v>8.083</v>
+        <v>8.073</v>
       </c>
       <c r="AI68" t="n">
-        <v>4.064</v>
+        <v>3.971</v>
       </c>
       <c r="AJ68" t="n">
-        <v>16.82</v>
+        <v>16.761</v>
       </c>
       <c r="AK68" t="n">
-        <v>1.2</v>
+        <v>6.2</v>
       </c>
       <c r="AL68" t="n">
-        <v>5.5</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="69">
@@ -9506,22 +9506,22 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F76" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G76" t="b">
         <v>1</v>
       </c>
       <c r="H76" t="n">
-        <v>2196.684</v>
+        <v>2203.313</v>
       </c>
       <c r="I76" t="n">
-        <v>3.7365</v>
+        <v>3.7385</v>
       </c>
       <c r="J76" t="n">
-        <v>1700.6</v>
+        <v>1715.1</v>
       </c>
       <c r="K76" t="n">
         <v>1</v>
@@ -9542,70 +9542,70 @@
         <v>1</v>
       </c>
       <c r="Q76" t="n">
-        <v>122.606</v>
+        <v>122.582</v>
       </c>
       <c r="R76" t="n">
-        <v>94.999</v>
+        <v>94.554</v>
       </c>
       <c r="S76" t="n">
-        <v>27.607</v>
+        <v>28.028</v>
       </c>
       <c r="T76" t="n">
-        <v>0.29898</v>
+        <v>0.29512</v>
       </c>
       <c r="U76" t="n">
-        <v>0.15337</v>
+        <v>0.15728</v>
       </c>
       <c r="V76" t="n">
-        <v>81.86</v>
+        <v>81.94</v>
       </c>
       <c r="W76" t="n">
-        <v>63.22</v>
+        <v>63.01</v>
       </c>
       <c r="X76" t="n">
-        <v>0.9434</v>
+        <v>0.945</v>
       </c>
       <c r="Y76" t="n">
-        <v>28.44</v>
+        <v>28.431</v>
       </c>
       <c r="Z76" t="n">
-        <v>58.434</v>
+        <v>58.079</v>
       </c>
       <c r="AA76" t="n">
-        <v>8.930999999999999</v>
+        <v>8.898</v>
       </c>
       <c r="AB76" t="n">
-        <v>25.915</v>
+        <v>25.732</v>
       </c>
       <c r="AC76" t="n">
-        <v>16.049</v>
+        <v>16.176</v>
       </c>
       <c r="AD76" t="n">
-        <v>22.018</v>
+        <v>22.065</v>
       </c>
       <c r="AE76" t="n">
-        <v>11.701</v>
+        <v>11.559</v>
       </c>
       <c r="AF76" t="n">
-        <v>27.028</v>
+        <v>27.25</v>
       </c>
       <c r="AG76" t="n">
-        <v>16.713</v>
+        <v>16.78</v>
       </c>
       <c r="AH76" t="n">
-        <v>7.61</v>
+        <v>7.559</v>
       </c>
       <c r="AI76" t="n">
-        <v>3.255</v>
+        <v>3.285</v>
       </c>
       <c r="AJ76" t="n">
-        <v>15.486</v>
+        <v>15.523</v>
       </c>
       <c r="AK76" t="n">
-        <v>7.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="AL76" t="n">
-        <v>17.9</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="77">
@@ -13106,22 +13106,22 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F106" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G106" t="b">
         <v>1</v>
       </c>
       <c r="H106" t="n">
-        <v>2070.396</v>
+        <v>2027.119</v>
       </c>
       <c r="I106" t="n">
-        <v>5.4527</v>
+        <v>5.1307</v>
       </c>
       <c r="J106" t="n">
-        <v>1596.4</v>
+        <v>1606.9</v>
       </c>
       <c r="K106" t="n">
         <v>10</v>
@@ -13142,70 +13142,70 @@
         <v>7</v>
       </c>
       <c r="Q106" t="n">
-        <v>120.168</v>
+        <v>119.759</v>
       </c>
       <c r="R106" t="n">
-        <v>93.744</v>
+        <v>94.54300000000001</v>
       </c>
       <c r="S106" t="n">
-        <v>26.424</v>
+        <v>25.216</v>
       </c>
       <c r="T106" t="n">
-        <v>0.30091</v>
+        <v>0.29566</v>
       </c>
       <c r="U106" t="n">
-        <v>0.13405</v>
+        <v>0.13185</v>
       </c>
       <c r="V106" t="n">
-        <v>84.66</v>
+        <v>84.14</v>
       </c>
       <c r="W106" t="n">
-        <v>65.92</v>
+        <v>66.23999999999999</v>
       </c>
       <c r="X106" t="n">
-        <v>0.9126</v>
+        <v>0.878</v>
       </c>
       <c r="Y106" t="n">
-        <v>32.051</v>
+        <v>32.076</v>
       </c>
       <c r="Z106" t="n">
-        <v>63.379</v>
+        <v>63.257</v>
       </c>
       <c r="AA106" t="n">
-        <v>6.526</v>
+        <v>6.501</v>
       </c>
       <c r="AB106" t="n">
-        <v>19.573</v>
+        <v>19.418</v>
       </c>
       <c r="AC106" t="n">
-        <v>14.027</v>
+        <v>13.712</v>
       </c>
       <c r="AD106" t="n">
-        <v>19.853</v>
+        <v>19.423</v>
       </c>
       <c r="AE106" t="n">
-        <v>11.163</v>
+        <v>10.891</v>
       </c>
       <c r="AF106" t="n">
-        <v>25.97</v>
+        <v>25.869</v>
       </c>
       <c r="AG106" t="n">
-        <v>18.282</v>
+        <v>18.357</v>
       </c>
       <c r="AH106" t="n">
-        <v>8.457000000000001</v>
+        <v>8.305</v>
       </c>
       <c r="AI106" t="n">
-        <v>3.747</v>
+        <v>3.671</v>
       </c>
       <c r="AJ106" t="n">
-        <v>16.902</v>
+        <v>16.664</v>
       </c>
       <c r="AK106" t="n">
-        <v>11.8</v>
+        <v>2.4</v>
       </c>
       <c r="AL106" t="n">
-        <v>14.7</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="107">
@@ -13826,22 +13826,22 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F112" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G112" t="b">
         <v>1</v>
       </c>
       <c r="H112" t="n">
-        <v>1664.344</v>
+        <v>1657.036</v>
       </c>
       <c r="I112" t="n">
-        <v>-0.6842</v>
+        <v>-0.3178</v>
       </c>
       <c r="J112" t="n">
-        <v>1401.4</v>
+        <v>1404.4</v>
       </c>
       <c r="K112" t="n">
         <v>92</v>
@@ -13862,70 +13862,70 @@
         <v>75</v>
       </c>
       <c r="Q112" t="n">
-        <v>120.784</v>
+        <v>120.565</v>
       </c>
       <c r="R112" t="n">
-        <v>100.586</v>
+        <v>101.276</v>
       </c>
       <c r="S112" t="n">
-        <v>20.197</v>
+        <v>19.289</v>
       </c>
       <c r="T112" t="n">
-        <v>0.30161</v>
+        <v>0.30298</v>
       </c>
       <c r="U112" t="n">
-        <v>0.12796</v>
+        <v>0.12743</v>
       </c>
       <c r="V112" t="n">
-        <v>86.31</v>
+        <v>86.41</v>
       </c>
       <c r="W112" t="n">
-        <v>72.20999999999999</v>
+        <v>72.97</v>
       </c>
       <c r="X112" t="n">
-        <v>0.8761</v>
+        <v>0.8413</v>
       </c>
       <c r="Y112" t="n">
-        <v>29.049</v>
+        <v>29.222</v>
       </c>
       <c r="Z112" t="n">
-        <v>61.346</v>
+        <v>61.839</v>
       </c>
       <c r="AA112" t="n">
-        <v>9.031000000000001</v>
+        <v>9.069000000000001</v>
       </c>
       <c r="AB112" t="n">
-        <v>26.128</v>
+        <v>26.612</v>
       </c>
       <c r="AC112" t="n">
-        <v>19.145</v>
+        <v>18.864</v>
       </c>
       <c r="AD112" t="n">
-        <v>25.688</v>
+        <v>25.243</v>
       </c>
       <c r="AE112" t="n">
-        <v>10.119</v>
+        <v>10.189</v>
       </c>
       <c r="AF112" t="n">
-        <v>23.134</v>
+        <v>23.137</v>
       </c>
       <c r="AG112" t="n">
-        <v>15.328</v>
+        <v>15.377</v>
       </c>
       <c r="AH112" t="n">
-        <v>10.052</v>
+        <v>9.928000000000001</v>
       </c>
       <c r="AI112" t="n">
-        <v>3.69</v>
+        <v>3.584</v>
       </c>
       <c r="AJ112" t="n">
-        <v>18.534</v>
+        <v>18.532</v>
       </c>
       <c r="AK112" t="n">
-        <v>9.6</v>
+        <v>7.2</v>
       </c>
       <c r="AL112" t="n">
-        <v>13.5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="113">
@@ -14186,22 +14186,22 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F115" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G115" t="b">
         <v>1</v>
       </c>
       <c r="H115" t="n">
-        <v>2112.552</v>
+        <v>2122.165</v>
       </c>
       <c r="I115" t="n">
-        <v>1.1096</v>
+        <v>1.0162</v>
       </c>
       <c r="J115" t="n">
-        <v>1725.6</v>
+        <v>1741.9</v>
       </c>
       <c r="K115" t="n">
         <v>5</v>
@@ -14222,70 +14222,70 @@
         <v>5</v>
       </c>
       <c r="Q115" t="n">
-        <v>117.422</v>
+        <v>117.91</v>
       </c>
       <c r="R115" t="n">
-        <v>94.66500000000001</v>
+        <v>94.52</v>
       </c>
       <c r="S115" t="n">
-        <v>22.757</v>
+        <v>23.39</v>
       </c>
       <c r="T115" t="n">
-        <v>0.33192</v>
+        <v>0.33619</v>
       </c>
       <c r="U115" t="n">
-        <v>0.12292</v>
+        <v>0.12241</v>
       </c>
       <c r="V115" t="n">
-        <v>77.18000000000001</v>
+        <v>77.56</v>
       </c>
       <c r="W115" t="n">
-        <v>62.27</v>
+        <v>62.21</v>
       </c>
       <c r="X115" t="n">
-        <v>0.8300999999999999</v>
+        <v>0.8347</v>
       </c>
       <c r="Y115" t="n">
-        <v>27.885</v>
+        <v>27.934</v>
       </c>
       <c r="Z115" t="n">
-        <v>61.745</v>
+        <v>61.966</v>
       </c>
       <c r="AA115" t="n">
-        <v>8.765000000000001</v>
+        <v>8.744</v>
       </c>
       <c r="AB115" t="n">
-        <v>24.8</v>
+        <v>25.104</v>
       </c>
       <c r="AC115" t="n">
-        <v>12.645</v>
+        <v>12.947</v>
       </c>
       <c r="AD115" t="n">
-        <v>16.41</v>
+        <v>16.762</v>
       </c>
       <c r="AE115" t="n">
-        <v>11.37</v>
+        <v>11.671</v>
       </c>
       <c r="AF115" t="n">
-        <v>23.168</v>
+        <v>23.17</v>
       </c>
       <c r="AG115" t="n">
-        <v>14.503</v>
+        <v>14.523</v>
       </c>
       <c r="AH115" t="n">
-        <v>7.745</v>
+        <v>7.609</v>
       </c>
       <c r="AI115" t="n">
-        <v>3.747</v>
+        <v>3.887</v>
       </c>
       <c r="AJ115" t="n">
-        <v>17.917</v>
+        <v>17.873</v>
       </c>
       <c r="AK115" t="n">
-        <v>12.4</v>
+        <v>17.2</v>
       </c>
       <c r="AL115" t="n">
-        <v>9.199999999999999</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="116">
@@ -14906,22 +14906,22 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F121" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G121" t="b">
         <v>1</v>
       </c>
       <c r="H121" t="n">
-        <v>1984.447</v>
+        <v>1997.795</v>
       </c>
       <c r="I121" t="n">
-        <v>7.3951</v>
+        <v>6.9704</v>
       </c>
       <c r="J121" t="n">
-        <v>1704.4</v>
+        <v>1718.8</v>
       </c>
       <c r="K121" t="n">
         <v>7</v>
@@ -14942,70 +14942,70 @@
         <v>8</v>
       </c>
       <c r="Q121" t="n">
-        <v>126.534</v>
+        <v>125.89</v>
       </c>
       <c r="R121" t="n">
-        <v>103.563</v>
+        <v>102.84</v>
       </c>
       <c r="S121" t="n">
-        <v>22.971</v>
+        <v>23.05</v>
       </c>
       <c r="T121" t="n">
-        <v>0.32629</v>
+        <v>0.32312</v>
       </c>
       <c r="U121" t="n">
-        <v>0.12517</v>
+        <v>0.12769</v>
       </c>
       <c r="V121" t="n">
-        <v>85.2</v>
+        <v>84.65000000000001</v>
       </c>
       <c r="W121" t="n">
-        <v>69.81999999999999</v>
+        <v>69.25</v>
       </c>
       <c r="X121" t="n">
-        <v>0.76</v>
+        <v>0.7669</v>
       </c>
       <c r="Y121" t="n">
-        <v>28.81</v>
+        <v>28.699</v>
       </c>
       <c r="Z121" t="n">
-        <v>62.36</v>
+        <v>62.079</v>
       </c>
       <c r="AA121" t="n">
-        <v>11.1</v>
+        <v>10.981</v>
       </c>
       <c r="AB121" t="n">
-        <v>31.92</v>
+        <v>31.576</v>
       </c>
       <c r="AC121" t="n">
-        <v>16.57</v>
+        <v>16.361</v>
       </c>
       <c r="AD121" t="n">
-        <v>20.88</v>
+        <v>20.73</v>
       </c>
       <c r="AE121" t="n">
-        <v>12.65</v>
+        <v>12.554</v>
       </c>
       <c r="AF121" t="n">
-        <v>26.26</v>
+        <v>26.502</v>
       </c>
       <c r="AG121" t="n">
-        <v>14.73</v>
+        <v>14.738</v>
       </c>
       <c r="AH121" t="n">
-        <v>3.8</v>
+        <v>3.864</v>
       </c>
       <c r="AI121" t="n">
-        <v>4.52</v>
+        <v>4.563</v>
       </c>
       <c r="AJ121" t="n">
-        <v>13.12</v>
+        <v>13.184</v>
       </c>
       <c r="AK121" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="AL121" t="n">
-        <v>10</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="122">
@@ -17666,22 +17666,22 @@
         </is>
       </c>
       <c r="E144" t="n">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="F144" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G144" t="b">
         <v>1</v>
       </c>
       <c r="H144" t="n">
-        <v>1743.485</v>
+        <v>1723.725</v>
       </c>
       <c r="I144" t="n">
-        <v>2.673</v>
+        <v>2.567</v>
       </c>
       <c r="J144" t="n">
-        <v>1491.2</v>
+        <v>1499.6</v>
       </c>
       <c r="K144" t="n">
         <v>125</v>
@@ -17702,70 +17702,70 @@
         <v>106</v>
       </c>
       <c r="Q144" t="n">
-        <v>117.773</v>
+        <v>117.103</v>
       </c>
       <c r="R144" t="n">
-        <v>111.278</v>
+        <v>111.5</v>
       </c>
       <c r="S144" t="n">
-        <v>6.495</v>
+        <v>5.603</v>
       </c>
       <c r="T144" t="n">
-        <v>0.17409</v>
+        <v>0.17692</v>
       </c>
       <c r="U144" t="n">
-        <v>0.13118</v>
+        <v>0.12885</v>
       </c>
       <c r="V144" t="n">
-        <v>76.23999999999999</v>
+        <v>75.72</v>
       </c>
       <c r="W144" t="n">
-        <v>72.13</v>
+        <v>72.17</v>
       </c>
       <c r="X144" t="n">
-        <v>0.7683</v>
+        <v>0.7372</v>
       </c>
       <c r="Y144" t="n">
-        <v>27.066</v>
+        <v>26.91</v>
       </c>
       <c r="Z144" t="n">
-        <v>53.378</v>
+        <v>53.506</v>
       </c>
       <c r="AA144" t="n">
-        <v>10.039</v>
+        <v>9.872</v>
       </c>
       <c r="AB144" t="n">
-        <v>25.276</v>
+        <v>25.205</v>
       </c>
       <c r="AC144" t="n">
-        <v>12.332</v>
+        <v>12.288</v>
       </c>
       <c r="AD144" t="n">
-        <v>17.385</v>
+        <v>17.314</v>
       </c>
       <c r="AE144" t="n">
-        <v>4.789</v>
+        <v>4.814</v>
       </c>
       <c r="AF144" t="n">
-        <v>21.683</v>
+        <v>21.487</v>
       </c>
       <c r="AG144" t="n">
-        <v>16.53</v>
+        <v>16.474</v>
       </c>
       <c r="AH144" t="n">
-        <v>6.04</v>
+        <v>6.032</v>
       </c>
       <c r="AI144" t="n">
-        <v>3.298</v>
+        <v>3.288</v>
       </c>
       <c r="AJ144" t="n">
-        <v>14.451</v>
+        <v>14.647</v>
       </c>
       <c r="AK144" t="n">
-        <v>0.6</v>
+        <v>-2</v>
       </c>
       <c r="AL144" t="n">
-        <v>-1.5</v>
+        <v>-2.7</v>
       </c>
     </row>
     <row r="145">
@@ -18386,22 +18386,22 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F150" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G150" t="b">
         <v>1</v>
       </c>
       <c r="H150" t="n">
-        <v>1854.143</v>
+        <v>1840.231</v>
       </c>
       <c r="I150" t="n">
-        <v>-2.5004</v>
+        <v>-2.3212</v>
       </c>
       <c r="J150" t="n">
-        <v>1686.9</v>
+        <v>1697.9</v>
       </c>
       <c r="K150" t="n">
         <v>19</v>
@@ -18422,70 +18422,70 @@
         <v>17</v>
       </c>
       <c r="Q150" t="n">
-        <v>118.734</v>
+        <v>118.298</v>
       </c>
       <c r="R150" t="n">
-        <v>101.945</v>
+        <v>102.457</v>
       </c>
       <c r="S150" t="n">
-        <v>16.789</v>
+        <v>15.841</v>
       </c>
       <c r="T150" t="n">
-        <v>0.2886</v>
+        <v>0.29073</v>
       </c>
       <c r="U150" t="n">
-        <v>0.16453</v>
+        <v>0.16363</v>
       </c>
       <c r="V150" t="n">
-        <v>84.69</v>
+        <v>84.14</v>
       </c>
       <c r="W150" t="n">
-        <v>72.43000000000001</v>
+        <v>72.55</v>
       </c>
       <c r="X150" t="n">
-        <v>0.7082000000000001</v>
+        <v>0.6807</v>
       </c>
       <c r="Y150" t="n">
-        <v>28.525</v>
+        <v>28.439</v>
       </c>
       <c r="Z150" t="n">
-        <v>61.046</v>
+        <v>61.185</v>
       </c>
       <c r="AA150" t="n">
-        <v>11.395</v>
+        <v>11.44</v>
       </c>
       <c r="AB150" t="n">
-        <v>32.12</v>
+        <v>32.349</v>
       </c>
       <c r="AC150" t="n">
-        <v>15.868</v>
+        <v>15.458</v>
       </c>
       <c r="AD150" t="n">
-        <v>20.915</v>
+        <v>20.351</v>
       </c>
       <c r="AE150" t="n">
-        <v>10.737</v>
+        <v>10.745</v>
       </c>
       <c r="AF150" t="n">
-        <v>26.294</v>
+        <v>26.077</v>
       </c>
       <c r="AG150" t="n">
-        <v>16.854</v>
+        <v>16.822</v>
       </c>
       <c r="AH150" t="n">
-        <v>6.838</v>
+        <v>6.787</v>
       </c>
       <c r="AI150" t="n">
-        <v>3.35</v>
+        <v>3.305</v>
       </c>
       <c r="AJ150" t="n">
-        <v>18.284</v>
+        <v>18.391</v>
       </c>
       <c r="AK150" t="n">
-        <v>4.2</v>
+        <v>-0.4</v>
       </c>
       <c r="AL150" t="n">
-        <v>3.1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="151">
@@ -20666,22 +20666,22 @@
         </is>
       </c>
       <c r="E169" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F169" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G169" t="b">
         <v>1</v>
       </c>
       <c r="H169" t="n">
-        <v>2174.35</v>
+        <v>2180.38</v>
       </c>
       <c r="I169" t="n">
-        <v>6.1854</v>
+        <v>5.8798</v>
       </c>
       <c r="J169" t="n">
-        <v>1765.3</v>
+        <v>1779.7</v>
       </c>
       <c r="K169" t="n">
         <v>3</v>
@@ -20702,70 +20702,70 @@
         <v>2</v>
       </c>
       <c r="Q169" t="n">
-        <v>121.548</v>
+        <v>121.931</v>
       </c>
       <c r="R169" t="n">
-        <v>97.557</v>
+        <v>97.663</v>
       </c>
       <c r="S169" t="n">
-        <v>23.992</v>
+        <v>24.268</v>
       </c>
       <c r="T169" t="n">
-        <v>0.25476</v>
+        <v>0.25601</v>
       </c>
       <c r="U169" t="n">
-        <v>0.16164</v>
+        <v>0.16069</v>
       </c>
       <c r="V169" t="n">
-        <v>87.33</v>
+        <v>87.5</v>
       </c>
       <c r="W169" t="n">
-        <v>69.59</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="X169" t="n">
-        <v>0.9149</v>
+        <v>0.9172</v>
       </c>
       <c r="Y169" t="n">
-        <v>30.647</v>
+        <v>30.717</v>
       </c>
       <c r="Z169" t="n">
-        <v>59.793</v>
+        <v>59.869</v>
       </c>
       <c r="AA169" t="n">
-        <v>9.042999999999999</v>
+        <v>9.097</v>
       </c>
       <c r="AB169" t="n">
-        <v>24.822</v>
+        <v>24.766</v>
       </c>
       <c r="AC169" t="n">
-        <v>17.22</v>
+        <v>17.186</v>
       </c>
       <c r="AD169" t="n">
-        <v>23.035</v>
+        <v>23.055</v>
       </c>
       <c r="AE169" t="n">
-        <v>9.728999999999999</v>
+        <v>9.814</v>
       </c>
       <c r="AF169" t="n">
-        <v>28.107</v>
+        <v>28.186</v>
       </c>
       <c r="AG169" t="n">
-        <v>18.945</v>
+        <v>18.924</v>
       </c>
       <c r="AH169" t="n">
-        <v>5.702</v>
+        <v>5.586</v>
       </c>
       <c r="AI169" t="n">
-        <v>6.015</v>
+        <v>6.103</v>
       </c>
       <c r="AJ169" t="n">
-        <v>15.382</v>
+        <v>15.317</v>
       </c>
       <c r="AK169" t="n">
-        <v>6</v>
+        <v>8.6</v>
       </c>
       <c r="AL169" t="n">
-        <v>6.3</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="170">
@@ -20786,22 +20786,22 @@
         </is>
       </c>
       <c r="E170" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F170" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G170" t="b">
         <v>1</v>
       </c>
       <c r="H170" t="n">
-        <v>2031.39</v>
+        <v>2045.301</v>
       </c>
       <c r="I170" t="n">
-        <v>0.0735</v>
+        <v>-0.0252</v>
       </c>
       <c r="J170" t="n">
-        <v>1723.2</v>
+        <v>1733.5</v>
       </c>
       <c r="K170" t="n">
         <v>9</v>
@@ -20822,70 +20822,70 @@
         <v>11</v>
       </c>
       <c r="Q170" t="n">
-        <v>117.934</v>
+        <v>117.697</v>
       </c>
       <c r="R170" t="n">
-        <v>101.399</v>
+        <v>101.519</v>
       </c>
       <c r="S170" t="n">
-        <v>16.535</v>
+        <v>16.178</v>
       </c>
       <c r="T170" t="n">
-        <v>0.28968</v>
+        <v>0.29109</v>
       </c>
       <c r="U170" t="n">
-        <v>0.1613</v>
+        <v>0.16361</v>
       </c>
       <c r="V170" t="n">
-        <v>79.45999999999999</v>
+        <v>79.23999999999999</v>
       </c>
       <c r="W170" t="n">
-        <v>68.34999999999999</v>
+        <v>68.39</v>
       </c>
       <c r="X170" t="n">
-        <v>0.79</v>
+        <v>0.796</v>
       </c>
       <c r="Y170" t="n">
-        <v>27.84</v>
+        <v>27.719</v>
       </c>
       <c r="Z170" t="n">
-        <v>58.22</v>
+        <v>58.118</v>
       </c>
       <c r="AA170" t="n">
-        <v>7.81</v>
+        <v>7.911</v>
       </c>
       <c r="AB170" t="n">
-        <v>21.38</v>
+        <v>21.571</v>
       </c>
       <c r="AC170" t="n">
-        <v>16.09</v>
+        <v>16.01</v>
       </c>
       <c r="AD170" t="n">
-        <v>20.97</v>
+        <v>20.923</v>
       </c>
       <c r="AE170" t="n">
-        <v>10.96</v>
+        <v>11.029</v>
       </c>
       <c r="AF170" t="n">
-        <v>26.41</v>
+        <v>26.427</v>
       </c>
       <c r="AG170" t="n">
-        <v>18.65</v>
+        <v>18.707</v>
       </c>
       <c r="AH170" t="n">
-        <v>5.39</v>
+        <v>5.34</v>
       </c>
       <c r="AI170" t="n">
-        <v>4.2</v>
+        <v>4.213</v>
       </c>
       <c r="AJ170" t="n">
-        <v>16.31</v>
+        <v>16.128</v>
       </c>
       <c r="AK170" t="n">
-        <v>5.6</v>
+        <v>4.6</v>
       </c>
       <c r="AL170" t="n">
-        <v>4.1</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="171">
@@ -23786,22 +23786,22 @@
         </is>
       </c>
       <c r="E195" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F195" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G195" t="b">
         <v>1</v>
       </c>
       <c r="H195" t="n">
-        <v>1988.043</v>
+        <v>2012.467</v>
       </c>
       <c r="I195" t="n">
-        <v>9.170199999999999</v>
+        <v>8.516999999999999</v>
       </c>
       <c r="J195" t="n">
-        <v>1669.8</v>
+        <v>1683.9</v>
       </c>
       <c r="K195" t="n">
         <v>14</v>
@@ -23822,70 +23822,70 @@
         <v>14</v>
       </c>
       <c r="Q195" t="n">
-        <v>115.233</v>
+        <v>115.192</v>
       </c>
       <c r="R195" t="n">
-        <v>97.834</v>
+        <v>98.636</v>
       </c>
       <c r="S195" t="n">
-        <v>17.399</v>
+        <v>16.556</v>
       </c>
       <c r="T195" t="n">
-        <v>0.24652</v>
+        <v>0.24223</v>
       </c>
       <c r="U195" t="n">
-        <v>0.13855</v>
+        <v>0.14089</v>
       </c>
       <c r="V195" t="n">
-        <v>77.23</v>
+        <v>77.12</v>
       </c>
       <c r="W195" t="n">
-        <v>65.45</v>
+        <v>65.88</v>
       </c>
       <c r="X195" t="n">
-        <v>0.82</v>
+        <v>0.8252</v>
       </c>
       <c r="Y195" t="n">
-        <v>27.52</v>
+        <v>27.572</v>
       </c>
       <c r="Z195" t="n">
-        <v>59.18</v>
+        <v>58.847</v>
       </c>
       <c r="AA195" t="n">
-        <v>10.67</v>
+        <v>10.573</v>
       </c>
       <c r="AB195" t="n">
-        <v>30.24</v>
+        <v>29.723</v>
       </c>
       <c r="AC195" t="n">
-        <v>12</v>
+        <v>11.866</v>
       </c>
       <c r="AD195" t="n">
-        <v>15.75</v>
+        <v>15.624</v>
       </c>
       <c r="AE195" t="n">
-        <v>8.470000000000001</v>
+        <v>8.292999999999999</v>
       </c>
       <c r="AF195" t="n">
-        <v>25.29</v>
+        <v>25.33</v>
       </c>
       <c r="AG195" t="n">
-        <v>18.2</v>
+        <v>18.098</v>
       </c>
       <c r="AH195" t="n">
-        <v>7.42</v>
+        <v>7.302</v>
       </c>
       <c r="AI195" t="n">
-        <v>2.5</v>
+        <v>2.418</v>
       </c>
       <c r="AJ195" t="n">
-        <v>14.12</v>
+        <v>14.3</v>
       </c>
       <c r="AK195" t="n">
-        <v>3.4</v>
+        <v>0.8</v>
       </c>
       <c r="AL195" t="n">
-        <v>6.4</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="196">
@@ -23906,22 +23906,22 @@
         </is>
       </c>
       <c r="E196" t="n">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="F196" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G196" t="b">
         <v>1</v>
       </c>
       <c r="H196" t="n">
-        <v>1747.974</v>
+        <v>1767.735</v>
       </c>
       <c r="I196" t="n">
-        <v>5.3805</v>
+        <v>5.1312</v>
       </c>
       <c r="J196" t="n">
-        <v>1602.9</v>
+        <v>1608.4</v>
       </c>
       <c r="K196" t="n">
         <v>75</v>
@@ -23942,70 +23942,70 @@
         <v>70</v>
       </c>
       <c r="Q196" t="n">
-        <v>112.996</v>
+        <v>113.135</v>
       </c>
       <c r="R196" t="n">
-        <v>105.635</v>
+        <v>105.56</v>
       </c>
       <c r="S196" t="n">
-        <v>7.361</v>
+        <v>7.575</v>
       </c>
       <c r="T196" t="n">
-        <v>0.30095</v>
+        <v>0.30057</v>
       </c>
       <c r="U196" t="n">
-        <v>0.14234</v>
+        <v>0.14388</v>
       </c>
       <c r="V196" t="n">
-        <v>76.44</v>
+        <v>76.19</v>
       </c>
       <c r="W196" t="n">
-        <v>71.72</v>
+        <v>71.36</v>
       </c>
       <c r="X196" t="n">
-        <v>0.6606</v>
+        <v>0.6698</v>
       </c>
       <c r="Y196" t="n">
-        <v>25.264</v>
+        <v>25.138</v>
       </c>
       <c r="Z196" t="n">
-        <v>57.191</v>
+        <v>56.916</v>
       </c>
       <c r="AA196" t="n">
-        <v>6.717</v>
+        <v>6.614</v>
       </c>
       <c r="AB196" t="n">
-        <v>18.54</v>
+        <v>18.458</v>
       </c>
       <c r="AC196" t="n">
-        <v>19.086</v>
+        <v>19.193</v>
       </c>
       <c r="AD196" t="n">
-        <v>25.544</v>
+        <v>25.503</v>
       </c>
       <c r="AE196" t="n">
-        <v>10.18</v>
+        <v>10.239</v>
       </c>
       <c r="AF196" t="n">
-        <v>23.532</v>
+        <v>23.727</v>
       </c>
       <c r="AG196" t="n">
-        <v>14.457</v>
+        <v>14.533</v>
       </c>
       <c r="AH196" t="n">
-        <v>6.738</v>
+        <v>6.577</v>
       </c>
       <c r="AI196" t="n">
-        <v>3.697</v>
+        <v>3.725</v>
       </c>
       <c r="AJ196" t="n">
-        <v>18.052</v>
+        <v>17.999</v>
       </c>
       <c r="AK196" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AL196" t="n">
-        <v>3.7</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="197">
@@ -33386,22 +33386,22 @@
         </is>
       </c>
       <c r="E275" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F275" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G275" t="b">
         <v>1</v>
       </c>
       <c r="H275" t="n">
-        <v>1819.597</v>
+        <v>1813.568</v>
       </c>
       <c r="I275" t="n">
-        <v>8.063000000000001</v>
+        <v>7.6609</v>
       </c>
       <c r="J275" t="n">
-        <v>1526.5</v>
+        <v>1540.5</v>
       </c>
       <c r="K275" t="n">
         <v>41</v>
@@ -33422,70 +33422,70 @@
         <v>31</v>
       </c>
       <c r="Q275" t="n">
-        <v>120.498</v>
+        <v>119.709</v>
       </c>
       <c r="R275" t="n">
-        <v>98.57599999999999</v>
+        <v>99.976</v>
       </c>
       <c r="S275" t="n">
-        <v>21.922</v>
+        <v>19.733</v>
       </c>
       <c r="T275" t="n">
-        <v>0.24815</v>
+        <v>0.24409</v>
       </c>
       <c r="U275" t="n">
-        <v>0.16516</v>
+        <v>0.16343</v>
       </c>
       <c r="V275" t="n">
-        <v>87.03</v>
+        <v>86.31</v>
       </c>
       <c r="W275" t="n">
-        <v>70.91</v>
+        <v>71.78</v>
       </c>
       <c r="X275" t="n">
-        <v>0.85</v>
+        <v>0.8159</v>
       </c>
       <c r="Y275" t="n">
-        <v>29.8</v>
+        <v>29.739</v>
       </c>
       <c r="Z275" t="n">
-        <v>60.09</v>
+        <v>60.009</v>
       </c>
       <c r="AA275" t="n">
-        <v>10.78</v>
+        <v>10.758</v>
       </c>
       <c r="AB275" t="n">
-        <v>27.21</v>
+        <v>27.28</v>
       </c>
       <c r="AC275" t="n">
-        <v>15.68</v>
+        <v>15.372</v>
       </c>
       <c r="AD275" t="n">
-        <v>21.2</v>
+        <v>20.915</v>
       </c>
       <c r="AE275" t="n">
-        <v>9.15</v>
+        <v>8.933999999999999</v>
       </c>
       <c r="AF275" t="n">
-        <v>27.6</v>
+        <v>27.449</v>
       </c>
       <c r="AG275" t="n">
-        <v>17.67</v>
+        <v>17.69</v>
       </c>
       <c r="AH275" t="n">
-        <v>7.29</v>
+        <v>7.262</v>
       </c>
       <c r="AI275" t="n">
-        <v>3.25</v>
+        <v>3.156</v>
       </c>
       <c r="AJ275" t="n">
-        <v>18.11</v>
+        <v>18.107</v>
       </c>
       <c r="AK275" t="n">
-        <v>3.2</v>
+        <v>-4.2</v>
       </c>
       <c r="AL275" t="n">
-        <v>5.1</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="276">
@@ -34346,22 +34346,22 @@
         </is>
       </c>
       <c r="E283" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F283" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G283" t="b">
         <v>1</v>
       </c>
       <c r="H283" t="n">
-        <v>1860.648</v>
+        <v>1854.019</v>
       </c>
       <c r="I283" t="n">
-        <v>6.8435</v>
+        <v>6.8722</v>
       </c>
       <c r="J283" t="n">
-        <v>1693.5</v>
+        <v>1707</v>
       </c>
       <c r="K283" t="n">
         <v>43</v>
@@ -34382,70 +34382,70 @@
         <v>39</v>
       </c>
       <c r="Q283" t="n">
-        <v>111.032</v>
+        <v>110.055</v>
       </c>
       <c r="R283" t="n">
-        <v>102.3</v>
+        <v>102.759</v>
       </c>
       <c r="S283" t="n">
-        <v>8.731</v>
+        <v>7.295</v>
       </c>
       <c r="T283" t="n">
-        <v>0.31828</v>
+        <v>0.32362</v>
       </c>
       <c r="U283" t="n">
-        <v>0.14957</v>
+        <v>0.14858</v>
       </c>
       <c r="V283" t="n">
-        <v>77.84999999999999</v>
+        <v>77.23</v>
       </c>
       <c r="W283" t="n">
-        <v>71.76000000000001</v>
+        <v>72.15000000000001</v>
       </c>
       <c r="X283" t="n">
-        <v>0.679</v>
+        <v>0.6523</v>
       </c>
       <c r="Y283" t="n">
-        <v>27.035</v>
+        <v>26.914</v>
       </c>
       <c r="Z283" t="n">
-        <v>60.473</v>
+        <v>60.804</v>
       </c>
       <c r="AA283" t="n">
-        <v>7.342</v>
+        <v>7.34</v>
       </c>
       <c r="AB283" t="n">
-        <v>22.358</v>
+        <v>22.412</v>
       </c>
       <c r="AC283" t="n">
-        <v>16.361</v>
+        <v>16.004</v>
       </c>
       <c r="AD283" t="n">
-        <v>22.993</v>
+        <v>22.621</v>
       </c>
       <c r="AE283" t="n">
-        <v>11.019</v>
+        <v>11.057</v>
       </c>
       <c r="AF283" t="n">
-        <v>22.732</v>
+        <v>22.395</v>
       </c>
       <c r="AG283" t="n">
-        <v>15.724</v>
+        <v>15.574</v>
       </c>
       <c r="AH283" t="n">
-        <v>7.56</v>
+        <v>7.746</v>
       </c>
       <c r="AI283" t="n">
-        <v>4.488</v>
+        <v>4.446</v>
       </c>
       <c r="AJ283" t="n">
-        <v>16.07</v>
+        <v>16.256</v>
       </c>
       <c r="AK283" t="n">
-        <v>4.4</v>
+        <v>-1.8</v>
       </c>
       <c r="AL283" t="n">
-        <v>4.1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="284">
@@ -34946,22 +34946,22 @@
         </is>
       </c>
       <c r="E288" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F288" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G288" t="b">
         <v>1</v>
       </c>
       <c r="H288" t="n">
-        <v>1801.834</v>
+        <v>1845.111</v>
       </c>
       <c r="I288" t="n">
-        <v>2.6488</v>
+        <v>2.8244</v>
       </c>
       <c r="J288" t="n">
-        <v>1706</v>
+        <v>1711</v>
       </c>
       <c r="K288" t="n">
         <v>37</v>
@@ -34982,70 +34982,70 @@
         <v>42</v>
       </c>
       <c r="Q288" t="n">
-        <v>119.208</v>
+        <v>119.114</v>
       </c>
       <c r="R288" t="n">
-        <v>110.835</v>
+        <v>110.731</v>
       </c>
       <c r="S288" t="n">
-        <v>8.372999999999999</v>
+        <v>8.382999999999999</v>
       </c>
       <c r="T288" t="n">
-        <v>0.30312</v>
+        <v>0.30206</v>
       </c>
       <c r="U288" t="n">
-        <v>0.14324</v>
+        <v>0.14233</v>
       </c>
       <c r="V288" t="n">
-        <v>82.06</v>
+        <v>81.79000000000001</v>
       </c>
       <c r="W288" t="n">
-        <v>76.23</v>
+        <v>75.97</v>
       </c>
       <c r="X288" t="n">
-        <v>0.5793</v>
+        <v>0.5915</v>
       </c>
       <c r="Y288" t="n">
-        <v>27.696</v>
+        <v>27.7</v>
       </c>
       <c r="Z288" t="n">
-        <v>57.983</v>
+        <v>58.074</v>
       </c>
       <c r="AA288" t="n">
-        <v>6.945</v>
+        <v>6.86</v>
       </c>
       <c r="AB288" t="n">
-        <v>20.468</v>
+        <v>20.29</v>
       </c>
       <c r="AC288" t="n">
-        <v>19.661</v>
+        <v>19.309</v>
       </c>
       <c r="AD288" t="n">
-        <v>26.133</v>
+        <v>25.627</v>
       </c>
       <c r="AE288" t="n">
-        <v>10.464</v>
+        <v>10.43</v>
       </c>
       <c r="AF288" t="n">
-        <v>24.112</v>
+        <v>24.154</v>
       </c>
       <c r="AG288" t="n">
-        <v>11.529</v>
+        <v>11.925</v>
       </c>
       <c r="AH288" t="n">
-        <v>6</v>
+        <v>5.963</v>
       </c>
       <c r="AI288" t="n">
-        <v>2.978</v>
+        <v>2.897</v>
       </c>
       <c r="AJ288" t="n">
-        <v>18.97</v>
+        <v>18.6</v>
       </c>
       <c r="AK288" t="n">
-        <v>-4.6</v>
+        <v>0.6</v>
       </c>
       <c r="AL288" t="n">
-        <v>-2.1</v>
+        <v>-3.2</v>
       </c>
     </row>
     <row r="289">
@@ -35066,22 +35066,22 @@
         </is>
       </c>
       <c r="E289" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F289" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G289" t="b">
         <v>1</v>
       </c>
       <c r="H289" t="n">
-        <v>1852.759</v>
+        <v>1843.146</v>
       </c>
       <c r="I289" t="n">
-        <v>4.0806</v>
+        <v>3.9805</v>
       </c>
       <c r="J289" t="n">
-        <v>1661.5</v>
+        <v>1671.3</v>
       </c>
       <c r="K289" t="n">
         <v>39</v>
@@ -35102,70 +35102,70 @@
         <v>44</v>
       </c>
       <c r="Q289" t="n">
-        <v>116.943</v>
+        <v>116.034</v>
       </c>
       <c r="R289" t="n">
-        <v>106.221</v>
+        <v>107.859</v>
       </c>
       <c r="S289" t="n">
-        <v>10.722</v>
+        <v>8.175000000000001</v>
       </c>
       <c r="T289" t="n">
-        <v>0.31014</v>
+        <v>0.30977</v>
       </c>
       <c r="U289" t="n">
-        <v>0.14624</v>
+        <v>0.14563</v>
       </c>
       <c r="V289" t="n">
-        <v>86.69</v>
+        <v>85.77</v>
       </c>
       <c r="W289" t="n">
-        <v>78.33</v>
+        <v>79.04000000000001</v>
       </c>
       <c r="X289" t="n">
-        <v>0.6706</v>
+        <v>0.64</v>
       </c>
       <c r="Y289" t="n">
-        <v>29.32</v>
+        <v>28.996</v>
       </c>
       <c r="Z289" t="n">
-        <v>64.04000000000001</v>
+        <v>63.753</v>
       </c>
       <c r="AA289" t="n">
-        <v>10.779</v>
+        <v>10.596</v>
       </c>
       <c r="AB289" t="n">
-        <v>29.559</v>
+        <v>29.411</v>
       </c>
       <c r="AC289" t="n">
-        <v>17.327</v>
+        <v>17.385</v>
       </c>
       <c r="AD289" t="n">
-        <v>23.668</v>
+        <v>23.625</v>
       </c>
       <c r="AE289" t="n">
-        <v>11.21</v>
+        <v>11.124</v>
       </c>
       <c r="AF289" t="n">
-        <v>24.294</v>
+        <v>24.16</v>
       </c>
       <c r="AG289" t="n">
-        <v>17.823</v>
+        <v>17.582</v>
       </c>
       <c r="AH289" t="n">
-        <v>8.025</v>
+        <v>7.898</v>
       </c>
       <c r="AI289" t="n">
-        <v>3.329</v>
+        <v>3.2</v>
       </c>
       <c r="AJ289" t="n">
-        <v>18.924</v>
+        <v>19.109</v>
       </c>
       <c r="AK289" t="n">
-        <v>0.2</v>
+        <v>-4.8</v>
       </c>
       <c r="AL289" t="n">
-        <v>-2.1</v>
+        <v>-5.1</v>
       </c>
     </row>
     <row r="290">
@@ -37706,22 +37706,22 @@
         </is>
       </c>
       <c r="E311" t="n">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="F311" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G311" t="b">
         <v>1</v>
       </c>
       <c r="H311" t="n">
-        <v>1694.511</v>
+        <v>1670.865</v>
       </c>
       <c r="I311" t="n">
-        <v>1.7793</v>
+        <v>1.7868</v>
       </c>
       <c r="J311" t="n">
-        <v>1439.1</v>
+        <v>1446.8</v>
       </c>
       <c r="K311" t="n">
         <v>110</v>
@@ -37742,70 +37742,70 @@
         <v>96</v>
       </c>
       <c r="Q311" t="n">
-        <v>114.505</v>
+        <v>113.876</v>
       </c>
       <c r="R311" t="n">
-        <v>103.212</v>
+        <v>104.148</v>
       </c>
       <c r="S311" t="n">
-        <v>11.293</v>
+        <v>9.728</v>
       </c>
       <c r="T311" t="n">
-        <v>0.31717</v>
+        <v>0.31802</v>
       </c>
       <c r="U311" t="n">
-        <v>0.139</v>
+        <v>0.13928</v>
       </c>
       <c r="V311" t="n">
-        <v>75</v>
+        <v>74.5</v>
       </c>
       <c r="W311" t="n">
-        <v>67.73</v>
+        <v>68.23</v>
       </c>
       <c r="X311" t="n">
-        <v>0.8083</v>
+        <v>0.7742</v>
       </c>
       <c r="Y311" t="n">
-        <v>25.351</v>
+        <v>25.301</v>
       </c>
       <c r="Z311" t="n">
-        <v>57.851</v>
+        <v>57.712</v>
       </c>
       <c r="AA311" t="n">
-        <v>8.211</v>
+        <v>7.986</v>
       </c>
       <c r="AB311" t="n">
-        <v>22.742</v>
+        <v>22.641</v>
       </c>
       <c r="AC311" t="n">
-        <v>16.561</v>
+        <v>16.379</v>
       </c>
       <c r="AD311" t="n">
-        <v>23.903</v>
+        <v>23.68</v>
       </c>
       <c r="AE311" t="n">
-        <v>11.94</v>
+        <v>11.796</v>
       </c>
       <c r="AF311" t="n">
-        <v>25.167</v>
+        <v>24.844</v>
       </c>
       <c r="AG311" t="n">
-        <v>13.403</v>
+        <v>13.132</v>
       </c>
       <c r="AH311" t="n">
-        <v>5.054</v>
+        <v>5.182</v>
       </c>
       <c r="AI311" t="n">
-        <v>2.351</v>
+        <v>2.421</v>
       </c>
       <c r="AJ311" t="n">
-        <v>17.106</v>
+        <v>17.093</v>
       </c>
       <c r="AK311" t="n">
-        <v>5</v>
+        <v>-3.4</v>
       </c>
       <c r="AL311" t="n">
-        <v>6.7</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="312">
@@ -38786,22 +38786,22 @@
         </is>
       </c>
       <c r="E320" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F320" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G320" t="b">
         <v>1</v>
       </c>
       <c r="H320" t="n">
-        <v>1797.509</v>
+        <v>1784.161</v>
       </c>
       <c r="I320" t="n">
-        <v>3.4141</v>
+        <v>3.6722</v>
       </c>
       <c r="J320" t="n">
-        <v>1569.9</v>
+        <v>1572.5</v>
       </c>
       <c r="K320" t="n">
         <v>45</v>
@@ -38822,70 +38822,70 @@
         <v>43</v>
       </c>
       <c r="Q320" t="n">
-        <v>117.658</v>
+        <v>116.484</v>
       </c>
       <c r="R320" t="n">
-        <v>103.371</v>
+        <v>103.756</v>
       </c>
       <c r="S320" t="n">
-        <v>14.287</v>
+        <v>12.728</v>
       </c>
       <c r="T320" t="n">
-        <v>0.29349</v>
+        <v>0.29816</v>
       </c>
       <c r="U320" t="n">
-        <v>0.14585</v>
+        <v>0.14635</v>
       </c>
       <c r="V320" t="n">
-        <v>81.58</v>
+        <v>80.62</v>
       </c>
       <c r="W320" t="n">
-        <v>71.70999999999999</v>
+        <v>71.81</v>
       </c>
       <c r="X320" t="n">
-        <v>0.8017</v>
+        <v>0.7714</v>
       </c>
       <c r="Y320" t="n">
-        <v>26.819</v>
+        <v>26.664</v>
       </c>
       <c r="Z320" t="n">
-        <v>58.501</v>
+        <v>58.671</v>
       </c>
       <c r="AA320" t="n">
-        <v>9.275</v>
+        <v>9.204000000000001</v>
       </c>
       <c r="AB320" t="n">
-        <v>25.545</v>
+        <v>25.746</v>
       </c>
       <c r="AC320" t="n">
-        <v>18.514</v>
+        <v>17.98</v>
       </c>
       <c r="AD320" t="n">
-        <v>25.183</v>
+        <v>24.542</v>
       </c>
       <c r="AE320" t="n">
-        <v>10.264</v>
+        <v>10.319</v>
       </c>
       <c r="AF320" t="n">
-        <v>24.56</v>
+        <v>24.218</v>
       </c>
       <c r="AG320" t="n">
-        <v>14.233</v>
+        <v>13.979</v>
       </c>
       <c r="AH320" t="n">
-        <v>7.405</v>
+        <v>7.421</v>
       </c>
       <c r="AI320" t="n">
-        <v>4.229</v>
+        <v>4.177</v>
       </c>
       <c r="AJ320" t="n">
-        <v>17.283</v>
+        <v>17.204</v>
       </c>
       <c r="AK320" t="n">
-        <v>7.2</v>
+        <v>1.8</v>
       </c>
       <c r="AL320" t="n">
-        <v>7.2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="321">
@@ -39026,22 +39026,22 @@
         </is>
       </c>
       <c r="E322" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F322" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G322" t="b">
         <v>1</v>
       </c>
       <c r="H322" t="n">
-        <v>1963.829</v>
+        <v>1939.405</v>
       </c>
       <c r="I322" t="n">
-        <v>1.4886</v>
+        <v>1.4161</v>
       </c>
       <c r="J322" t="n">
-        <v>1716.9</v>
+        <v>1726.2</v>
       </c>
       <c r="K322" t="n">
         <v>12</v>
@@ -39062,70 +39062,70 @@
         <v>13</v>
       </c>
       <c r="Q322" t="n">
-        <v>122.218</v>
+        <v>121.911</v>
       </c>
       <c r="R322" t="n">
-        <v>106.709</v>
+        <v>107.07</v>
       </c>
       <c r="S322" t="n">
-        <v>15.509</v>
+        <v>14.841</v>
       </c>
       <c r="T322" t="n">
-        <v>0.28967</v>
+        <v>0.29281</v>
       </c>
       <c r="U322" t="n">
-        <v>0.13117</v>
+        <v>0.13038</v>
       </c>
       <c r="V322" t="n">
-        <v>86.04000000000001</v>
+        <v>85.61</v>
       </c>
       <c r="W322" t="n">
-        <v>74.94</v>
+        <v>74.95999999999999</v>
       </c>
       <c r="X322" t="n">
-        <v>0.7734</v>
+        <v>0.7439</v>
       </c>
       <c r="Y322" t="n">
-        <v>28.917</v>
+        <v>28.766</v>
       </c>
       <c r="Z322" t="n">
-        <v>60.998</v>
+        <v>60.976</v>
       </c>
       <c r="AA322" t="n">
-        <v>9.34</v>
+        <v>9.473000000000001</v>
       </c>
       <c r="AB322" t="n">
-        <v>26.521</v>
+        <v>26.916</v>
       </c>
       <c r="AC322" t="n">
-        <v>18.388</v>
+        <v>18.136</v>
       </c>
       <c r="AD322" t="n">
-        <v>23.285</v>
+        <v>23.16</v>
       </c>
       <c r="AE322" t="n">
-        <v>9.935</v>
+        <v>9.981</v>
       </c>
       <c r="AF322" t="n">
-        <v>23.865</v>
+        <v>23.656</v>
       </c>
       <c r="AG322" t="n">
-        <v>16.105</v>
+        <v>16.074</v>
       </c>
       <c r="AH322" t="n">
-        <v>7.871</v>
+        <v>7.846</v>
       </c>
       <c r="AI322" t="n">
-        <v>4.529</v>
+        <v>4.523</v>
       </c>
       <c r="AJ322" t="n">
-        <v>19.072</v>
+        <v>19.031</v>
       </c>
       <c r="AK322" t="n">
-        <v>5.4</v>
+        <v>4.2</v>
       </c>
       <c r="AL322" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="323">

</xml_diff>

<commit_message>
Update team snapshot (2026-03-23)
</commit_message>
<xml_diff>
--- a/team_snapshot_2026.xlsx
+++ b/team_snapshot_2026.xlsx
@@ -986,22 +986,22 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F5" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G5" t="b">
         <v>1</v>
       </c>
       <c r="H5" t="n">
-        <v>1954.667</v>
+        <v>1985.69</v>
       </c>
       <c r="I5" t="n">
-        <v>-1.3316</v>
+        <v>-1.3006</v>
       </c>
       <c r="J5" t="n">
-        <v>1760.9</v>
+        <v>1777.2</v>
       </c>
       <c r="K5" t="n">
         <v>18</v>
@@ -1022,70 +1022,70 @@
         <v>18</v>
       </c>
       <c r="Q5" t="n">
-        <v>121.89</v>
+        <v>122.085</v>
       </c>
       <c r="R5" t="n">
-        <v>110.305</v>
+        <v>109.744</v>
       </c>
       <c r="S5" t="n">
-        <v>11.585</v>
+        <v>12.341</v>
       </c>
       <c r="T5" t="n">
-        <v>0.28487</v>
+        <v>0.28781</v>
       </c>
       <c r="U5" t="n">
-        <v>0.1295</v>
+        <v>0.13149</v>
       </c>
       <c r="V5" t="n">
-        <v>91.65000000000001</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="W5" t="n">
-        <v>82.95</v>
+        <v>82.39</v>
       </c>
       <c r="X5" t="n">
-        <v>0.7296</v>
+        <v>0.7374000000000001</v>
       </c>
       <c r="Y5" t="n">
-        <v>30.377</v>
+        <v>30.35</v>
       </c>
       <c r="Z5" t="n">
-        <v>66.008</v>
+        <v>66.074</v>
       </c>
       <c r="AA5" t="n">
-        <v>12.601</v>
+        <v>12.843</v>
       </c>
       <c r="AB5" t="n">
-        <v>35.069</v>
+        <v>35.318</v>
       </c>
       <c r="AC5" t="n">
-        <v>18.327</v>
+        <v>18.091</v>
       </c>
       <c r="AD5" t="n">
-        <v>23.988</v>
+        <v>23.696</v>
       </c>
       <c r="AE5" t="n">
-        <v>11.111</v>
+        <v>11.318</v>
       </c>
       <c r="AF5" t="n">
-        <v>27.558</v>
+        <v>27.599</v>
       </c>
       <c r="AG5" t="n">
-        <v>16.12</v>
+        <v>16.45</v>
       </c>
       <c r="AH5" t="n">
-        <v>6.361</v>
+        <v>6.424</v>
       </c>
       <c r="AI5" t="n">
-        <v>5.129</v>
+        <v>5.117</v>
       </c>
       <c r="AJ5" t="n">
-        <v>18.529</v>
+        <v>18.666</v>
       </c>
       <c r="AK5" t="n">
-        <v>4.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="AL5" t="n">
-        <v>9</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="6">
@@ -1826,22 +1826,22 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F12" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G12" t="b">
         <v>1</v>
       </c>
       <c r="H12" t="n">
-        <v>2272.508</v>
+        <v>2278.515</v>
       </c>
       <c r="I12" t="n">
-        <v>6.6001</v>
+        <v>6.3904</v>
       </c>
       <c r="J12" t="n">
-        <v>1753.9</v>
+        <v>1771.6</v>
       </c>
       <c r="K12" t="n">
         <v>2</v>
@@ -1862,70 +1862,70 @@
         <v>3</v>
       </c>
       <c r="Q12" t="n">
-        <v>121.602</v>
+        <v>121.646</v>
       </c>
       <c r="R12" t="n">
-        <v>96.53400000000001</v>
+        <v>96.95099999999999</v>
       </c>
       <c r="S12" t="n">
-        <v>25.069</v>
+        <v>24.694</v>
       </c>
       <c r="T12" t="n">
-        <v>0.29327</v>
+        <v>0.29711</v>
       </c>
       <c r="U12" t="n">
-        <v>0.14976</v>
+        <v>0.15073</v>
       </c>
       <c r="V12" t="n">
-        <v>86.36</v>
+        <v>86.03</v>
       </c>
       <c r="W12" t="n">
-        <v>68.41</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="X12" t="n">
-        <v>0.9433</v>
+        <v>0.9448</v>
       </c>
       <c r="Y12" t="n">
-        <v>30.61</v>
+        <v>30.303</v>
       </c>
       <c r="Z12" t="n">
-        <v>60.822</v>
+        <v>60.662</v>
       </c>
       <c r="AA12" t="n">
-        <v>5.887</v>
+        <v>5.924</v>
       </c>
       <c r="AB12" t="n">
-        <v>16.205</v>
+        <v>16.255</v>
       </c>
       <c r="AC12" t="n">
-        <v>19.249</v>
+        <v>19.497</v>
       </c>
       <c r="AD12" t="n">
-        <v>26.335</v>
+        <v>26.724</v>
       </c>
       <c r="AE12" t="n">
-        <v>12.143</v>
+        <v>12.455</v>
       </c>
       <c r="AF12" t="n">
-        <v>28.938</v>
+        <v>28.993</v>
       </c>
       <c r="AG12" t="n">
-        <v>16.908</v>
+        <v>16.607</v>
       </c>
       <c r="AH12" t="n">
-        <v>7.687</v>
+        <v>7.448</v>
       </c>
       <c r="AI12" t="n">
-        <v>4.441</v>
+        <v>4.421</v>
       </c>
       <c r="AJ12" t="n">
-        <v>15.857</v>
+        <v>15.821</v>
       </c>
       <c r="AK12" t="n">
-        <v>14.6</v>
+        <v>15</v>
       </c>
       <c r="AL12" t="n">
-        <v>13.3</v>
+        <v>13.8</v>
       </c>
     </row>
     <row r="13">
@@ -2666,22 +2666,22 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="F19" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G19" t="b">
         <v>1</v>
       </c>
       <c r="H19" t="n">
-        <v>1830.518</v>
+        <v>1836.183</v>
       </c>
       <c r="I19" t="n">
-        <v>-7.3446</v>
+        <v>-7.1903</v>
       </c>
       <c r="J19" t="n">
-        <v>1748.1</v>
+        <v>1743</v>
       </c>
       <c r="K19" t="n">
         <v>38</v>
@@ -2702,70 +2702,70 @@
         <v>38</v>
       </c>
       <c r="Q19" t="n">
-        <v>118.347</v>
+        <v>118.616</v>
       </c>
       <c r="R19" t="n">
-        <v>113.34</v>
+        <v>113.595</v>
       </c>
       <c r="S19" t="n">
-        <v>5.007</v>
+        <v>5.021</v>
       </c>
       <c r="T19" t="n">
-        <v>0.34722</v>
+        <v>0.34374</v>
       </c>
       <c r="U19" t="n">
-        <v>0.14503</v>
+        <v>0.14484</v>
       </c>
       <c r="V19" t="n">
-        <v>82.55</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="W19" t="n">
-        <v>78.92</v>
+        <v>79.25</v>
       </c>
       <c r="X19" t="n">
-        <v>0.5338000000000001</v>
+        <v>0.5468</v>
       </c>
       <c r="Y19" t="n">
-        <v>27.293</v>
+        <v>27.386</v>
       </c>
       <c r="Z19" t="n">
-        <v>60.068</v>
+        <v>59.983</v>
       </c>
       <c r="AA19" t="n">
-        <v>8.249000000000001</v>
+        <v>8.207000000000001</v>
       </c>
       <c r="AB19" t="n">
-        <v>24.303</v>
+        <v>24.187</v>
       </c>
       <c r="AC19" t="n">
-        <v>19.711</v>
+        <v>19.922</v>
       </c>
       <c r="AD19" t="n">
-        <v>26.441</v>
+        <v>26.732</v>
       </c>
       <c r="AE19" t="n">
-        <v>12.068</v>
+        <v>11.983</v>
       </c>
       <c r="AF19" t="n">
-        <v>22.298</v>
+        <v>22.56</v>
       </c>
       <c r="AG19" t="n">
-        <v>12.872</v>
+        <v>12.904</v>
       </c>
       <c r="AH19" t="n">
-        <v>7.322</v>
+        <v>7.229</v>
       </c>
       <c r="AI19" t="n">
-        <v>4.213</v>
+        <v>4.198</v>
       </c>
       <c r="AJ19" t="n">
-        <v>17.303</v>
+        <v>17.155</v>
       </c>
       <c r="AK19" t="n">
-        <v>4.2</v>
+        <v>2.6</v>
       </c>
       <c r="AL19" t="n">
-        <v>-1.5</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="20">
@@ -5066,22 +5066,22 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="F39" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G39" t="b">
         <v>1</v>
       </c>
       <c r="H39" t="n">
-        <v>1710.414</v>
+        <v>1684.049</v>
       </c>
       <c r="I39" t="n">
-        <v>6.8262</v>
+        <v>6.4442</v>
       </c>
       <c r="J39" t="n">
-        <v>1600.4</v>
+        <v>1602.4</v>
       </c>
       <c r="K39" t="n">
         <v>73</v>
@@ -5102,70 +5102,70 @@
         <v>67</v>
       </c>
       <c r="Q39" t="n">
-        <v>110.668</v>
+        <v>110.457</v>
       </c>
       <c r="R39" t="n">
-        <v>104.285</v>
+        <v>104.585</v>
       </c>
       <c r="S39" t="n">
-        <v>6.383</v>
+        <v>5.872</v>
       </c>
       <c r="T39" t="n">
-        <v>0.23394</v>
+        <v>0.23672</v>
       </c>
       <c r="U39" t="n">
-        <v>0.14794</v>
+        <v>0.14591</v>
       </c>
       <c r="V39" t="n">
-        <v>77.95</v>
+        <v>77.7</v>
       </c>
       <c r="W39" t="n">
-        <v>73.31</v>
+        <v>73.42</v>
       </c>
       <c r="X39" t="n">
-        <v>0.6599</v>
+        <v>0.63</v>
       </c>
       <c r="Y39" t="n">
-        <v>26.065</v>
+        <v>26.08</v>
       </c>
       <c r="Z39" t="n">
-        <v>58.02</v>
+        <v>58.39</v>
       </c>
       <c r="AA39" t="n">
-        <v>9.25</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="AB39" t="n">
-        <v>24.94</v>
+        <v>25.19</v>
       </c>
       <c r="AC39" t="n">
-        <v>16.575</v>
+        <v>16.24</v>
       </c>
       <c r="AD39" t="n">
-        <v>21.274</v>
+        <v>21</v>
       </c>
       <c r="AE39" t="n">
-        <v>7.495</v>
+        <v>7.68</v>
       </c>
       <c r="AF39" t="n">
-        <v>24.215</v>
+        <v>24.36</v>
       </c>
       <c r="AG39" t="n">
-        <v>14.168</v>
+        <v>14.09</v>
       </c>
       <c r="AH39" t="n">
-        <v>5.888</v>
+        <v>5.93</v>
       </c>
       <c r="AI39" t="n">
-        <v>2.999</v>
+        <v>3.03</v>
       </c>
       <c r="AJ39" t="n">
-        <v>18.864</v>
+        <v>18.67</v>
       </c>
       <c r="AK39" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AL39" t="n">
-        <v>-0.8</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="40">
@@ -7346,22 +7346,22 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F58" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G58" t="b">
         <v>1</v>
       </c>
       <c r="H58" t="n">
-        <v>2053.381</v>
+        <v>2068.556</v>
       </c>
       <c r="I58" t="n">
-        <v>6.6189</v>
+        <v>6.1349</v>
       </c>
       <c r="J58" t="n">
-        <v>1662.8</v>
+        <v>1675.6</v>
       </c>
       <c r="K58" t="n">
         <v>11</v>
@@ -7382,70 +7382,70 @@
         <v>10</v>
       </c>
       <c r="Q58" t="n">
-        <v>116.791</v>
+        <v>116.645</v>
       </c>
       <c r="R58" t="n">
-        <v>98.316</v>
+        <v>97.91500000000001</v>
       </c>
       <c r="S58" t="n">
-        <v>18.475</v>
+        <v>18.73</v>
       </c>
       <c r="T58" t="n">
-        <v>0.30395</v>
+        <v>0.30311</v>
       </c>
       <c r="U58" t="n">
-        <v>0.15867</v>
+        <v>0.16219</v>
       </c>
       <c r="V58" t="n">
-        <v>77.67</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="W58" t="n">
-        <v>65.34</v>
+        <v>64.98999999999999</v>
       </c>
       <c r="X58" t="n">
-        <v>0.8584000000000001</v>
+        <v>0.8622</v>
       </c>
       <c r="Y58" t="n">
-        <v>28.431</v>
+        <v>28.207</v>
       </c>
       <c r="Z58" t="n">
-        <v>58.882</v>
+        <v>58.478</v>
       </c>
       <c r="AA58" t="n">
-        <v>8.199999999999999</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="AB58" t="n">
         <v>23.697</v>
       </c>
       <c r="AC58" t="n">
-        <v>12.603</v>
+        <v>12.829</v>
       </c>
       <c r="AD58" t="n">
-        <v>17.603</v>
+        <v>17.721</v>
       </c>
       <c r="AE58" t="n">
-        <v>10.693</v>
+        <v>10.642</v>
       </c>
       <c r="AF58" t="n">
-        <v>24.017</v>
+        <v>24.036</v>
       </c>
       <c r="AG58" t="n">
-        <v>18.516</v>
+        <v>18.397</v>
       </c>
       <c r="AH58" t="n">
-        <v>6.887</v>
+        <v>6.89</v>
       </c>
       <c r="AI58" t="n">
-        <v>5.107</v>
+        <v>5.138</v>
       </c>
       <c r="AJ58" t="n">
-        <v>18.048</v>
+        <v>18.127</v>
       </c>
       <c r="AK58" t="n">
-        <v>5.2</v>
+        <v>9.6</v>
       </c>
       <c r="AL58" t="n">
-        <v>6.9</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="59">
@@ -11306,22 +11306,22 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F91" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G91" t="b">
         <v>1</v>
       </c>
       <c r="H91" t="n">
-        <v>2007.171</v>
+        <v>1970.43</v>
       </c>
       <c r="I91" t="n">
-        <v>3.5894</v>
+        <v>3.6774</v>
       </c>
       <c r="J91" t="n">
-        <v>1703.3</v>
+        <v>1725.7</v>
       </c>
       <c r="K91" t="n">
         <v>4</v>
@@ -11342,70 +11342,70 @@
         <v>4</v>
       </c>
       <c r="Q91" t="n">
-        <v>121.802</v>
+        <v>121.291</v>
       </c>
       <c r="R91" t="n">
-        <v>99.018</v>
+        <v>99.98099999999999</v>
       </c>
       <c r="S91" t="n">
-        <v>22.784</v>
+        <v>21.31</v>
       </c>
       <c r="T91" t="n">
-        <v>0.3326</v>
+        <v>0.33433</v>
       </c>
       <c r="U91" t="n">
-        <v>0.15503</v>
+        <v>0.15588</v>
       </c>
       <c r="V91" t="n">
-        <v>87.83</v>
+        <v>87.01000000000001</v>
       </c>
       <c r="W91" t="n">
-        <v>71.34999999999999</v>
+        <v>71.56</v>
       </c>
       <c r="X91" t="n">
-        <v>0.796</v>
+        <v>0.7647</v>
       </c>
       <c r="Y91" t="n">
-        <v>31.451</v>
+        <v>31.126</v>
       </c>
       <c r="Z91" t="n">
-        <v>64.551</v>
+        <v>64</v>
       </c>
       <c r="AA91" t="n">
-        <v>7.611</v>
+        <v>7.566</v>
       </c>
       <c r="AB91" t="n">
-        <v>23.952</v>
+        <v>23.972</v>
       </c>
       <c r="AC91" t="n">
-        <v>17.817</v>
+        <v>17.71</v>
       </c>
       <c r="AD91" t="n">
-        <v>24.876</v>
+        <v>24.832</v>
       </c>
       <c r="AE91" t="n">
-        <v>14.572</v>
+        <v>14.39</v>
       </c>
       <c r="AF91" t="n">
-        <v>28.676</v>
+        <v>28.159</v>
       </c>
       <c r="AG91" t="n">
-        <v>17.345</v>
+        <v>17.115</v>
       </c>
       <c r="AH91" t="n">
-        <v>6.681</v>
+        <v>6.606</v>
       </c>
       <c r="AI91" t="n">
-        <v>5.135</v>
+        <v>4.928</v>
       </c>
       <c r="AJ91" t="n">
-        <v>17.681</v>
+        <v>17.754</v>
       </c>
       <c r="AK91" t="n">
-        <v>18.2</v>
+        <v>11.2</v>
       </c>
       <c r="AL91" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="92">
@@ -12146,22 +12146,22 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="F98" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G98" t="b">
         <v>1</v>
       </c>
       <c r="H98" t="n">
-        <v>1546.505</v>
+        <v>1540.737</v>
       </c>
       <c r="I98" t="n">
-        <v>-3.6146</v>
+        <v>-3.3693</v>
       </c>
       <c r="J98" t="n">
-        <v>1543.8</v>
+        <v>1553.1</v>
       </c>
       <c r="K98" t="n">
         <v>85</v>
@@ -12182,70 +12182,70 @@
         <v>91</v>
       </c>
       <c r="Q98" t="n">
-        <v>114.986</v>
+        <v>113.989</v>
       </c>
       <c r="R98" t="n">
-        <v>105.859</v>
+        <v>106.612</v>
       </c>
       <c r="S98" t="n">
-        <v>9.127000000000001</v>
+        <v>7.378</v>
       </c>
       <c r="T98" t="n">
-        <v>0.32167</v>
+        <v>0.3226</v>
       </c>
       <c r="U98" t="n">
-        <v>0.17626</v>
+        <v>0.17667</v>
       </c>
       <c r="V98" t="n">
-        <v>81.48999999999999</v>
+        <v>80.69</v>
       </c>
       <c r="W98" t="n">
-        <v>74.92</v>
+        <v>75.31999999999999</v>
       </c>
       <c r="X98" t="n">
-        <v>0.5508</v>
+        <v>0.5236</v>
       </c>
       <c r="Y98" t="n">
-        <v>28.036</v>
+        <v>27.778</v>
       </c>
       <c r="Z98" t="n">
-        <v>60.217</v>
+        <v>60.371</v>
       </c>
       <c r="AA98" t="n">
-        <v>9.922000000000001</v>
+        <v>9.952999999999999</v>
       </c>
       <c r="AB98" t="n">
-        <v>27.995</v>
+        <v>28.309</v>
       </c>
       <c r="AC98" t="n">
-        <v>15.371</v>
+        <v>15.069</v>
       </c>
       <c r="AD98" t="n">
-        <v>21.246</v>
+        <v>20.782</v>
       </c>
       <c r="AE98" t="n">
-        <v>11.276</v>
+        <v>11.331</v>
       </c>
       <c r="AF98" t="n">
-        <v>23.449</v>
+        <v>23.476</v>
       </c>
       <c r="AG98" t="n">
-        <v>15.424</v>
+        <v>15.218</v>
       </c>
       <c r="AH98" t="n">
-        <v>7.461</v>
+        <v>7.356</v>
       </c>
       <c r="AI98" t="n">
-        <v>3.335</v>
+        <v>3.371</v>
       </c>
       <c r="AJ98" t="n">
-        <v>18.161</v>
+        <v>18.105</v>
       </c>
       <c r="AK98" t="n">
-        <v>0.2</v>
+        <v>-6.6</v>
       </c>
       <c r="AL98" t="n">
-        <v>3.6</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="99">
@@ -15026,22 +15026,22 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="F122" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G122" t="b">
         <v>1</v>
       </c>
       <c r="H122" t="n">
-        <v>1594.577</v>
+        <v>1617.365</v>
       </c>
       <c r="I122" t="n">
-        <v>2.1793</v>
+        <v>2.1828</v>
       </c>
       <c r="J122" t="n">
-        <v>1508.2</v>
+        <v>1513.3</v>
       </c>
       <c r="K122" t="n">
         <v>103</v>
@@ -15062,70 +15062,70 @@
         <v>95</v>
       </c>
       <c r="Q122" t="n">
-        <v>110.094</v>
+        <v>110.138</v>
       </c>
       <c r="R122" t="n">
-        <v>101.357</v>
+        <v>101.764</v>
       </c>
       <c r="S122" t="n">
-        <v>8.738</v>
+        <v>8.374000000000001</v>
       </c>
       <c r="T122" t="n">
-        <v>0.25529</v>
+        <v>0.25849</v>
       </c>
       <c r="U122" t="n">
-        <v>0.15942</v>
+        <v>0.15917</v>
       </c>
       <c r="V122" t="n">
-        <v>74.73</v>
+        <v>74.81</v>
       </c>
       <c r="W122" t="n">
-        <v>68.65000000000001</v>
+        <v>68.98999999999999</v>
       </c>
       <c r="X122" t="n">
-        <v>0.6284</v>
+        <v>0.6394</v>
       </c>
       <c r="Y122" t="n">
-        <v>27</v>
+        <v>26.923</v>
       </c>
       <c r="Z122" t="n">
-        <v>57.961</v>
+        <v>58.025</v>
       </c>
       <c r="AA122" t="n">
-        <v>8.819000000000001</v>
+        <v>8.827999999999999</v>
       </c>
       <c r="AB122" t="n">
-        <v>24.781</v>
+        <v>25.007</v>
       </c>
       <c r="AC122" t="n">
-        <v>12.588</v>
+        <v>12.802</v>
       </c>
       <c r="AD122" t="n">
-        <v>17.752</v>
+        <v>17.875</v>
       </c>
       <c r="AE122" t="n">
-        <v>8.619</v>
+        <v>8.678000000000001</v>
       </c>
       <c r="AF122" t="n">
-        <v>25.431</v>
+        <v>25.177</v>
       </c>
       <c r="AG122" t="n">
-        <v>14.032</v>
+        <v>13.893</v>
       </c>
       <c r="AH122" t="n">
-        <v>5.637</v>
+        <v>5.639</v>
       </c>
       <c r="AI122" t="n">
-        <v>2.257</v>
+        <v>2.24</v>
       </c>
       <c r="AJ122" t="n">
-        <v>17.221</v>
+        <v>17.279</v>
       </c>
       <c r="AK122" t="n">
-        <v>-1.2</v>
+        <v>2.2</v>
       </c>
       <c r="AL122" t="n">
-        <v>0.8</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="123">
@@ -15626,22 +15626,22 @@
         </is>
       </c>
       <c r="E127" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F127" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G127" t="b">
         <v>1</v>
       </c>
       <c r="H127" t="n">
-        <v>1860.117</v>
+        <v>1896.858</v>
       </c>
       <c r="I127" t="n">
-        <v>3.0379</v>
+        <v>2.8676</v>
       </c>
       <c r="J127" t="n">
-        <v>1717.1</v>
+        <v>1722.3</v>
       </c>
       <c r="K127" t="n">
         <v>25</v>
@@ -15662,70 +15662,70 @@
         <v>27</v>
       </c>
       <c r="Q127" t="n">
-        <v>119.224</v>
+        <v>119.243</v>
       </c>
       <c r="R127" t="n">
-        <v>105.017</v>
+        <v>105.476</v>
       </c>
       <c r="S127" t="n">
-        <v>14.206</v>
+        <v>13.767</v>
       </c>
       <c r="T127" t="n">
-        <v>0.29176</v>
+        <v>0.29258</v>
       </c>
       <c r="U127" t="n">
-        <v>0.14178</v>
+        <v>0.1441</v>
       </c>
       <c r="V127" t="n">
         <v>74.90000000000001</v>
       </c>
       <c r="W127" t="n">
-        <v>65.78</v>
+        <v>66.05</v>
       </c>
       <c r="X127" t="n">
-        <v>0.6503</v>
+        <v>0.6601</v>
       </c>
       <c r="Y127" t="n">
-        <v>26.283</v>
+        <v>26.2</v>
       </c>
       <c r="Z127" t="n">
-        <v>53.854</v>
+        <v>53.562</v>
       </c>
       <c r="AA127" t="n">
-        <v>8.038</v>
+        <v>7.954</v>
       </c>
       <c r="AB127" t="n">
-        <v>22.533</v>
+        <v>22.37</v>
       </c>
       <c r="AC127" t="n">
-        <v>14.061</v>
+        <v>14.336</v>
       </c>
       <c r="AD127" t="n">
-        <v>18.323</v>
+        <v>18.702</v>
       </c>
       <c r="AE127" t="n">
-        <v>8.048</v>
+        <v>8.065</v>
       </c>
       <c r="AF127" t="n">
-        <v>19.506</v>
+        <v>19.473</v>
       </c>
       <c r="AG127" t="n">
-        <v>15.205</v>
+        <v>15.338</v>
       </c>
       <c r="AH127" t="n">
-        <v>7.001</v>
+        <v>7.028</v>
       </c>
       <c r="AI127" t="n">
-        <v>2</v>
+        <v>1.963</v>
       </c>
       <c r="AJ127" t="n">
-        <v>17.766</v>
+        <v>17.745</v>
       </c>
       <c r="AK127" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="AL127" t="n">
-        <v>-1.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="128">
@@ -15746,22 +15746,22 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F128" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G128" t="b">
         <v>1</v>
       </c>
       <c r="H128" t="n">
-        <v>2040.699</v>
+        <v>2057.221</v>
       </c>
       <c r="I128" t="n">
-        <v>1.9908</v>
+        <v>1.8048</v>
       </c>
       <c r="J128" t="n">
-        <v>1704.9</v>
+        <v>1720.3</v>
       </c>
       <c r="K128" t="n">
         <v>6</v>
@@ -15782,70 +15782,70 @@
         <v>6</v>
       </c>
       <c r="Q128" t="n">
-        <v>119.647</v>
+        <v>119.437</v>
       </c>
       <c r="R128" t="n">
-        <v>95.52800000000001</v>
+        <v>95.352</v>
       </c>
       <c r="S128" t="n">
-        <v>24.119</v>
+        <v>24.085</v>
       </c>
       <c r="T128" t="n">
-        <v>0.32421</v>
+        <v>0.32237</v>
       </c>
       <c r="U128" t="n">
-        <v>0.14659</v>
+        <v>0.14503</v>
       </c>
       <c r="V128" t="n">
-        <v>82.73</v>
+        <v>82.52</v>
       </c>
       <c r="W128" t="n">
-        <v>65.45999999999999</v>
+        <v>65.31999999999999</v>
       </c>
       <c r="X128" t="n">
-        <v>0.8015</v>
+        <v>0.8069</v>
       </c>
       <c r="Y128" t="n">
-        <v>29.492</v>
+        <v>29.379</v>
       </c>
       <c r="Z128" t="n">
-        <v>60.655</v>
+        <v>60.586</v>
       </c>
       <c r="AA128" t="n">
-        <v>9.157</v>
+        <v>9.138</v>
       </c>
       <c r="AB128" t="n">
-        <v>23.688</v>
+        <v>23.834</v>
       </c>
       <c r="AC128" t="n">
-        <v>13.966</v>
+        <v>14.021</v>
       </c>
       <c r="AD128" t="n">
-        <v>20.59</v>
+        <v>20.662</v>
       </c>
       <c r="AE128" t="n">
-        <v>10.938</v>
+        <v>10.821</v>
       </c>
       <c r="AF128" t="n">
-        <v>22.731</v>
+        <v>22.69</v>
       </c>
       <c r="AG128" t="n">
-        <v>17.392</v>
+        <v>17.331</v>
       </c>
       <c r="AH128" t="n">
-        <v>8.914999999999999</v>
+        <v>9.021000000000001</v>
       </c>
       <c r="AI128" t="n">
-        <v>2.788</v>
+        <v>2.676</v>
       </c>
       <c r="AJ128" t="n">
-        <v>15.922</v>
+        <v>15.917</v>
       </c>
       <c r="AK128" t="n">
-        <v>24.8</v>
+        <v>24.4</v>
       </c>
       <c r="AL128" t="n">
-        <v>10.8</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="129">
@@ -16586,22 +16586,22 @@
         </is>
       </c>
       <c r="E135" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F135" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G135" t="b">
         <v>1</v>
       </c>
       <c r="H135" t="n">
-        <v>1979.25</v>
+        <v>1953.755</v>
       </c>
       <c r="I135" t="n">
-        <v>9.864800000000001</v>
+        <v>9.4422</v>
       </c>
       <c r="J135" t="n">
-        <v>1780.1</v>
+        <v>1795</v>
       </c>
       <c r="K135" t="n">
         <v>21</v>
@@ -16622,70 +16622,70 @@
         <v>21</v>
       </c>
       <c r="Q135" t="n">
-        <v>109.767</v>
+        <v>109.195</v>
       </c>
       <c r="R135" t="n">
-        <v>100.723</v>
+        <v>100.635</v>
       </c>
       <c r="S135" t="n">
-        <v>9.044</v>
+        <v>8.561</v>
       </c>
       <c r="T135" t="n">
-        <v>0.25343</v>
+        <v>0.25554</v>
       </c>
       <c r="U135" t="n">
-        <v>0.14997</v>
+        <v>0.14891</v>
       </c>
       <c r="V135" t="n">
-        <v>75.33</v>
+        <v>75.01000000000001</v>
       </c>
       <c r="W135" t="n">
-        <v>69.02</v>
+        <v>69.04000000000001</v>
       </c>
       <c r="X135" t="n">
-        <v>0.7091</v>
+        <v>0.6787</v>
       </c>
       <c r="Y135" t="n">
-        <v>26.727</v>
+        <v>26.669</v>
       </c>
       <c r="Z135" t="n">
-        <v>59.269</v>
+        <v>59.583</v>
       </c>
       <c r="AA135" t="n">
-        <v>7.229</v>
+        <v>7.408</v>
       </c>
       <c r="AB135" t="n">
-        <v>20.978</v>
+        <v>21.538</v>
       </c>
       <c r="AC135" t="n">
-        <v>14.647</v>
+        <v>14.343</v>
       </c>
       <c r="AD135" t="n">
-        <v>19.033</v>
+        <v>18.777</v>
       </c>
       <c r="AE135" t="n">
-        <v>9.446999999999999</v>
+        <v>9.500999999999999</v>
       </c>
       <c r="AF135" t="n">
-        <v>27.684</v>
+        <v>27.545</v>
       </c>
       <c r="AG135" t="n">
-        <v>14.022</v>
+        <v>14.008</v>
       </c>
       <c r="AH135" t="n">
-        <v>5.465</v>
+        <v>5.529</v>
       </c>
       <c r="AI135" t="n">
-        <v>5.658</v>
+        <v>5.574</v>
       </c>
       <c r="AJ135" t="n">
-        <v>14.436</v>
+        <v>14.54</v>
       </c>
       <c r="AK135" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="AL135" t="n">
-        <v>-3.2</v>
+        <v>-1.6</v>
       </c>
     </row>
     <row r="136">
@@ -17066,22 +17066,22 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F139" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G139" t="b">
         <v>1</v>
       </c>
       <c r="H139" t="n">
-        <v>1905.506</v>
+        <v>1888.985</v>
       </c>
       <c r="I139" t="n">
-        <v>4.5369</v>
+        <v>4.416</v>
       </c>
       <c r="J139" t="n">
-        <v>1734</v>
+        <v>1743.2</v>
       </c>
       <c r="K139" t="n">
         <v>28</v>
@@ -17102,70 +17102,70 @@
         <v>28</v>
       </c>
       <c r="Q139" t="n">
-        <v>116.168</v>
+        <v>115.322</v>
       </c>
       <c r="R139" t="n">
-        <v>106.38</v>
+        <v>106.864</v>
       </c>
       <c r="S139" t="n">
-        <v>9.788</v>
+        <v>8.458</v>
       </c>
       <c r="T139" t="n">
-        <v>0.30777</v>
+        <v>0.30343</v>
       </c>
       <c r="U139" t="n">
-        <v>0.14633</v>
+        <v>0.15168</v>
       </c>
       <c r="V139" t="n">
-        <v>81.06999999999999</v>
+        <v>80.36</v>
       </c>
       <c r="W139" t="n">
-        <v>74.2</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="X139" t="n">
-        <v>0.6318</v>
+        <v>0.6061</v>
       </c>
       <c r="Y139" t="n">
-        <v>28.205</v>
+        <v>27.915</v>
       </c>
       <c r="Z139" t="n">
-        <v>60.593</v>
+        <v>60.015</v>
       </c>
       <c r="AA139" t="n">
-        <v>8.131</v>
+        <v>8.146000000000001</v>
       </c>
       <c r="AB139" t="n">
-        <v>23.638</v>
+        <v>23.65</v>
       </c>
       <c r="AC139" t="n">
-        <v>16.359</v>
+        <v>16.215</v>
       </c>
       <c r="AD139" t="n">
-        <v>22.614</v>
+        <v>22.428</v>
       </c>
       <c r="AE139" t="n">
-        <v>10.954</v>
+        <v>10.758</v>
       </c>
       <c r="AF139" t="n">
-        <v>24.656</v>
+        <v>24.614</v>
       </c>
       <c r="AG139" t="n">
-        <v>15.885</v>
+        <v>15.684</v>
       </c>
       <c r="AH139" t="n">
-        <v>7.011</v>
+        <v>6.92</v>
       </c>
       <c r="AI139" t="n">
-        <v>4.458</v>
+        <v>4.35</v>
       </c>
       <c r="AJ139" t="n">
-        <v>18.359</v>
+        <v>18.358</v>
       </c>
       <c r="AK139" t="n">
-        <v>0.2</v>
+        <v>-2.2</v>
       </c>
       <c r="AL139" t="n">
-        <v>0.4</v>
+        <v>-0.7</v>
       </c>
     </row>
     <row r="140">
@@ -20426,22 +20426,22 @@
         </is>
       </c>
       <c r="E167" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F167" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G167" t="b">
         <v>1</v>
       </c>
       <c r="H167" t="n">
-        <v>1794.728</v>
+        <v>1783.017</v>
       </c>
       <c r="I167" t="n">
-        <v>11.4257</v>
+        <v>11.1893</v>
       </c>
       <c r="J167" t="n">
-        <v>1636.7</v>
+        <v>1646.6</v>
       </c>
       <c r="K167" t="n">
         <v>31</v>
@@ -20462,70 +20462,70 @@
         <v>32</v>
       </c>
       <c r="Q167" t="n">
-        <v>117.437</v>
+        <v>116.933</v>
       </c>
       <c r="R167" t="n">
-        <v>102.471</v>
+        <v>103.198</v>
       </c>
       <c r="S167" t="n">
-        <v>14.966</v>
+        <v>13.735</v>
       </c>
       <c r="T167" t="n">
-        <v>0.31068</v>
+        <v>0.31465</v>
       </c>
       <c r="U167" t="n">
-        <v>0.15663</v>
+        <v>0.15787</v>
       </c>
       <c r="V167" t="n">
-        <v>81.86</v>
+        <v>81.39</v>
       </c>
       <c r="W167" t="n">
-        <v>70.97</v>
+        <v>71.34</v>
       </c>
       <c r="X167" t="n">
-        <v>0.7673</v>
+        <v>0.7353</v>
       </c>
       <c r="Y167" t="n">
-        <v>29.84</v>
+        <v>29.81</v>
       </c>
       <c r="Z167" t="n">
-        <v>59.855</v>
+        <v>59.974</v>
       </c>
       <c r="AA167" t="n">
-        <v>6.753</v>
+        <v>6.64</v>
       </c>
       <c r="AB167" t="n">
-        <v>19.142</v>
+        <v>19.085</v>
       </c>
       <c r="AC167" t="n">
-        <v>15.429</v>
+        <v>15.127</v>
       </c>
       <c r="AD167" t="n">
-        <v>22.687</v>
+        <v>22.132</v>
       </c>
       <c r="AE167" t="n">
-        <v>11.055</v>
+        <v>11.115</v>
       </c>
       <c r="AF167" t="n">
-        <v>24.356</v>
+        <v>24.09</v>
       </c>
       <c r="AG167" t="n">
-        <v>16.207</v>
+        <v>16.208</v>
       </c>
       <c r="AH167" t="n">
-        <v>7.844</v>
+        <v>7.897</v>
       </c>
       <c r="AI167" t="n">
-        <v>3.338</v>
+        <v>3.301</v>
       </c>
       <c r="AJ167" t="n">
-        <v>15.476</v>
+        <v>15.491</v>
       </c>
       <c r="AK167" t="n">
-        <v>0.4</v>
+        <v>-3.2</v>
       </c>
       <c r="AL167" t="n">
-        <v>3.3</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="168">
@@ -24146,22 +24146,22 @@
         </is>
       </c>
       <c r="E198" t="n">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="F198" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G198" t="b">
         <v>1</v>
       </c>
       <c r="H198" t="n">
-        <v>1802.429</v>
+        <v>1808.195</v>
       </c>
       <c r="I198" t="n">
-        <v>2.3893</v>
+        <v>2.0968</v>
       </c>
       <c r="J198" t="n">
-        <v>1593.2</v>
+        <v>1592</v>
       </c>
       <c r="K198" t="n">
         <v>50</v>
@@ -24182,70 +24182,70 @@
         <v>46</v>
       </c>
       <c r="Q198" t="n">
-        <v>116.178</v>
+        <v>116.354</v>
       </c>
       <c r="R198" t="n">
-        <v>103.208</v>
+        <v>102.654</v>
       </c>
       <c r="S198" t="n">
-        <v>12.971</v>
+        <v>13.7</v>
       </c>
       <c r="T198" t="n">
-        <v>0.28453</v>
+        <v>0.28594</v>
       </c>
       <c r="U198" t="n">
-        <v>0.14214</v>
+        <v>0.14241</v>
       </c>
       <c r="V198" t="n">
-        <v>81.06999999999999</v>
+        <v>81.04000000000001</v>
       </c>
       <c r="W198" t="n">
-        <v>72</v>
+        <v>71.51000000000001</v>
       </c>
       <c r="X198" t="n">
-        <v>0.6995</v>
+        <v>0.7082000000000001</v>
       </c>
       <c r="Y198" t="n">
-        <v>28.062</v>
+        <v>28.082</v>
       </c>
       <c r="Z198" t="n">
-        <v>60.478</v>
+        <v>60.535</v>
       </c>
       <c r="AA198" t="n">
-        <v>9.183999999999999</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="AB198" t="n">
-        <v>25.376</v>
+        <v>25.366</v>
       </c>
       <c r="AC198" t="n">
-        <v>15.76</v>
+        <v>15.655</v>
       </c>
       <c r="AD198" t="n">
-        <v>21.653</v>
+        <v>21.605</v>
       </c>
       <c r="AE198" t="n">
-        <v>9.994999999999999</v>
+        <v>10.156</v>
       </c>
       <c r="AF198" t="n">
-        <v>24.618</v>
+        <v>24.806</v>
       </c>
       <c r="AG198" t="n">
-        <v>14.78</v>
+        <v>14.886</v>
       </c>
       <c r="AH198" t="n">
-        <v>7.935</v>
+        <v>7.987</v>
       </c>
       <c r="AI198" t="n">
-        <v>2.776</v>
+        <v>2.878</v>
       </c>
       <c r="AJ198" t="n">
-        <v>17.614</v>
+        <v>17.316</v>
       </c>
       <c r="AK198" t="n">
-        <v>5.2</v>
+        <v>11.8</v>
       </c>
       <c r="AL198" t="n">
-        <v>6.9</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="199">
@@ -26666,22 +26666,22 @@
         </is>
       </c>
       <c r="E219" t="n">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="F219" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G219" t="b">
         <v>1</v>
       </c>
       <c r="H219" t="n">
-        <v>1713.594</v>
+        <v>1686.949</v>
       </c>
       <c r="I219" t="n">
-        <v>-1.1886</v>
+        <v>-1.1802</v>
       </c>
       <c r="J219" t="n">
-        <v>1685</v>
+        <v>1684.5</v>
       </c>
       <c r="K219" t="n">
         <v>66</v>
@@ -26702,70 +26702,70 @@
         <v>74</v>
       </c>
       <c r="Q219" t="n">
-        <v>111.537</v>
+        <v>110.918</v>
       </c>
       <c r="R219" t="n">
-        <v>110.394</v>
+        <v>111.177</v>
       </c>
       <c r="S219" t="n">
-        <v>1.144</v>
+        <v>-0.259</v>
       </c>
       <c r="T219" t="n">
-        <v>0.27727</v>
+        <v>0.27908</v>
       </c>
       <c r="U219" t="n">
-        <v>0.15255</v>
+        <v>0.15287</v>
       </c>
       <c r="V219" t="n">
-        <v>84.26000000000001</v>
+        <v>83.73999999999999</v>
       </c>
       <c r="W219" t="n">
-        <v>82.8</v>
+        <v>83.31</v>
       </c>
       <c r="X219" t="n">
-        <v>0.5921</v>
+        <v>0.5664</v>
       </c>
       <c r="Y219" t="n">
-        <v>29.049</v>
+        <v>28.983</v>
       </c>
       <c r="Z219" t="n">
-        <v>62.876</v>
+        <v>63.017</v>
       </c>
       <c r="AA219" t="n">
-        <v>7.758</v>
+        <v>7.699</v>
       </c>
       <c r="AB219" t="n">
-        <v>22.663</v>
+        <v>22.634</v>
       </c>
       <c r="AC219" t="n">
-        <v>18.145</v>
+        <v>17.817</v>
       </c>
       <c r="AD219" t="n">
-        <v>24.464</v>
+        <v>24.174</v>
       </c>
       <c r="AE219" t="n">
-        <v>9.779</v>
+        <v>9.867000000000001</v>
       </c>
       <c r="AF219" t="n">
-        <v>25.404</v>
+        <v>25.386</v>
       </c>
       <c r="AG219" t="n">
-        <v>14.748</v>
+        <v>14.551</v>
       </c>
       <c r="AH219" t="n">
-        <v>7.098</v>
+        <v>7.002</v>
       </c>
       <c r="AI219" t="n">
-        <v>2.544</v>
+        <v>2.649</v>
       </c>
       <c r="AJ219" t="n">
-        <v>17.08</v>
+        <v>16.993</v>
       </c>
       <c r="AK219" t="n">
-        <v>1.2</v>
+        <v>-5.4</v>
       </c>
       <c r="AL219" t="n">
-        <v>-3.9</v>
+        <v>-6.2</v>
       </c>
     </row>
     <row r="220">
@@ -28586,22 +28586,22 @@
         </is>
       </c>
       <c r="E235" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F235" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G235" t="b">
         <v>1</v>
       </c>
       <c r="H235" t="n">
-        <v>2011.512</v>
+        <v>2023.223</v>
       </c>
       <c r="I235" t="n">
-        <v>-0.6772</v>
+        <v>-0.6463</v>
       </c>
       <c r="J235" t="n">
-        <v>1753.9</v>
+        <v>1767</v>
       </c>
       <c r="K235" t="n">
         <v>8</v>
@@ -28622,70 +28622,70 @@
         <v>9</v>
       </c>
       <c r="Q235" t="n">
-        <v>125.909</v>
+        <v>125.552</v>
       </c>
       <c r="R235" t="n">
-        <v>107.355</v>
+        <v>107.346</v>
       </c>
       <c r="S235" t="n">
-        <v>18.555</v>
+        <v>18.206</v>
       </c>
       <c r="T235" t="n">
-        <v>0.31279</v>
+        <v>0.3071</v>
       </c>
       <c r="U235" t="n">
-        <v>0.13549</v>
+        <v>0.13688</v>
       </c>
       <c r="V235" t="n">
-        <v>82.45999999999999</v>
+        <v>82.16</v>
       </c>
       <c r="W235" t="n">
-        <v>70.17</v>
+        <v>70.13</v>
       </c>
       <c r="X235" t="n">
-        <v>0.7796</v>
+        <v>0.7854</v>
       </c>
       <c r="Y235" t="n">
-        <v>30.117</v>
+        <v>29.854</v>
       </c>
       <c r="Z235" t="n">
-        <v>60.234</v>
+        <v>59.739</v>
       </c>
       <c r="AA235" t="n">
-        <v>9.454000000000001</v>
+        <v>9.368</v>
       </c>
       <c r="AB235" t="n">
-        <v>24.523</v>
+        <v>24.165</v>
       </c>
       <c r="AC235" t="n">
-        <v>11.912</v>
+        <v>12.257</v>
       </c>
       <c r="AD235" t="n">
-        <v>16.133</v>
+        <v>16.368</v>
       </c>
       <c r="AE235" t="n">
-        <v>10.702</v>
+        <v>10.437</v>
       </c>
       <c r="AF235" t="n">
-        <v>23.08</v>
+        <v>22.985</v>
       </c>
       <c r="AG235" t="n">
-        <v>19.674</v>
+        <v>19.548</v>
       </c>
       <c r="AH235" t="n">
-        <v>5.496</v>
+        <v>5.586</v>
       </c>
       <c r="AI235" t="n">
-        <v>2.777</v>
+        <v>2.759</v>
       </c>
       <c r="AJ235" t="n">
-        <v>14.901</v>
+        <v>14.713</v>
       </c>
       <c r="AK235" t="n">
-        <v>15.4</v>
+        <v>14.8</v>
       </c>
       <c r="AL235" t="n">
-        <v>9.6</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="236">
@@ -31466,22 +31466,22 @@
         </is>
       </c>
       <c r="E259" t="n">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="F259" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G259" t="b">
         <v>1</v>
       </c>
       <c r="H259" t="n">
-        <v>1560.056</v>
+        <v>1554.391</v>
       </c>
       <c r="I259" t="n">
-        <v>2.1732</v>
+        <v>2.0584</v>
       </c>
       <c r="J259" t="n">
-        <v>1524.1</v>
+        <v>1535.5</v>
       </c>
       <c r="K259" t="n">
         <v>119</v>
@@ -31502,70 +31502,70 @@
         <v>122</v>
       </c>
       <c r="Q259" t="n">
-        <v>100.859</v>
+        <v>101.572</v>
       </c>
       <c r="R259" t="n">
-        <v>97.512</v>
+        <v>98.834</v>
       </c>
       <c r="S259" t="n">
-        <v>3.347</v>
+        <v>2.738</v>
       </c>
       <c r="T259" t="n">
-        <v>0.25248</v>
+        <v>0.24514</v>
       </c>
       <c r="U259" t="n">
-        <v>0.16788</v>
+        <v>0.1658</v>
       </c>
       <c r="V259" t="n">
-        <v>69.59999999999999</v>
+        <v>70.22</v>
       </c>
       <c r="W259" t="n">
-        <v>67.36</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="X259" t="n">
-        <v>0.5974</v>
+        <v>0.5709</v>
       </c>
       <c r="Y259" t="n">
-        <v>24.212</v>
+        <v>24.51</v>
       </c>
       <c r="Z259" t="n">
-        <v>56.508</v>
+        <v>56.665</v>
       </c>
       <c r="AA259" t="n">
-        <v>7.266</v>
+        <v>7.587</v>
       </c>
       <c r="AB259" t="n">
-        <v>22.022</v>
+        <v>22.376</v>
       </c>
       <c r="AC259" t="n">
-        <v>13.912</v>
+        <v>13.611</v>
       </c>
       <c r="AD259" t="n">
-        <v>19.646</v>
+        <v>19.293</v>
       </c>
       <c r="AE259" t="n">
-        <v>7.663</v>
+        <v>7.43</v>
       </c>
       <c r="AF259" t="n">
-        <v>22.049</v>
+        <v>22.03</v>
       </c>
       <c r="AG259" t="n">
-        <v>12.987</v>
+        <v>13.201</v>
       </c>
       <c r="AH259" t="n">
-        <v>7.823</v>
+        <v>7.82</v>
       </c>
       <c r="AI259" t="n">
-        <v>4.863</v>
+        <v>4.85</v>
       </c>
       <c r="AJ259" t="n">
-        <v>16.574</v>
+        <v>16.678</v>
       </c>
       <c r="AK259" t="n">
-        <v>5.2</v>
+        <v>2.6</v>
       </c>
       <c r="AL259" t="n">
-        <v>3.3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="260">
@@ -33146,22 +33146,22 @@
         </is>
       </c>
       <c r="E273" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F273" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G273" t="b">
         <v>1</v>
       </c>
       <c r="H273" t="n">
-        <v>1989.246</v>
+        <v>2014.742</v>
       </c>
       <c r="I273" t="n">
-        <v>5.7241</v>
+        <v>5.7703</v>
       </c>
       <c r="J273" t="n">
-        <v>1684.5</v>
+        <v>1698.7</v>
       </c>
       <c r="K273" t="n">
         <v>17</v>
@@ -33182,70 +33182,70 @@
         <v>16</v>
       </c>
       <c r="Q273" t="n">
-        <v>114.409</v>
+        <v>113.755</v>
       </c>
       <c r="R273" t="n">
-        <v>97.80200000000001</v>
+        <v>97.798</v>
       </c>
       <c r="S273" t="n">
-        <v>16.607</v>
+        <v>15.957</v>
       </c>
       <c r="T273" t="n">
-        <v>0.32084</v>
+        <v>0.31722</v>
       </c>
       <c r="U273" t="n">
-        <v>0.14183</v>
+        <v>0.1451</v>
       </c>
       <c r="V273" t="n">
-        <v>81.47</v>
+        <v>80.98999999999999</v>
       </c>
       <c r="W273" t="n">
-        <v>69.36</v>
+        <v>69.33</v>
       </c>
       <c r="X273" t="n">
-        <v>0.8298</v>
+        <v>0.8345</v>
       </c>
       <c r="Y273" t="n">
-        <v>27.908</v>
+        <v>27.779</v>
       </c>
       <c r="Z273" t="n">
-        <v>61.396</v>
+        <v>61.172</v>
       </c>
       <c r="AA273" t="n">
-        <v>7.022</v>
+        <v>6.931</v>
       </c>
       <c r="AB273" t="n">
-        <v>21.087</v>
+        <v>20.786</v>
       </c>
       <c r="AC273" t="n">
-        <v>18.63</v>
+        <v>18.428</v>
       </c>
       <c r="AD273" t="n">
-        <v>25.659</v>
+        <v>25.386</v>
       </c>
       <c r="AE273" t="n">
-        <v>11.631</v>
+        <v>11.538</v>
       </c>
       <c r="AF273" t="n">
-        <v>24.889</v>
+        <v>25.179</v>
       </c>
       <c r="AG273" t="n">
-        <v>16.148</v>
+        <v>15.924</v>
       </c>
       <c r="AH273" t="n">
-        <v>7.736</v>
+        <v>7.607</v>
       </c>
       <c r="AI273" t="n">
-        <v>4.922</v>
+        <v>5.055</v>
       </c>
       <c r="AJ273" t="n">
-        <v>17.105</v>
+        <v>17.034</v>
       </c>
       <c r="AK273" t="n">
-        <v>15.2</v>
+        <v>14.2</v>
       </c>
       <c r="AL273" t="n">
-        <v>11.4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="274">
@@ -33266,22 +33266,22 @@
         </is>
       </c>
       <c r="E274" t="n">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="F274" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G274" t="b">
         <v>1</v>
       </c>
       <c r="H274" t="n">
-        <v>1633.092</v>
+        <v>1659.458</v>
       </c>
       <c r="I274" t="n">
-        <v>1.7131</v>
+        <v>1.9645</v>
       </c>
       <c r="J274" t="n">
-        <v>1521.6</v>
+        <v>1527.6</v>
       </c>
       <c r="K274" t="n">
         <v>116</v>
@@ -33302,70 +33302,70 @@
         <v>121</v>
       </c>
       <c r="Q274" t="n">
-        <v>105.758</v>
+        <v>106.077</v>
       </c>
       <c r="R274" t="n">
-        <v>102.729</v>
+        <v>103.137</v>
       </c>
       <c r="S274" t="n">
-        <v>3.029</v>
+        <v>2.94</v>
       </c>
       <c r="T274" t="n">
-        <v>0.28861</v>
+        <v>0.29071</v>
       </c>
       <c r="U274" t="n">
-        <v>0.16399</v>
+        <v>0.16258</v>
       </c>
       <c r="V274" t="n">
-        <v>71.88</v>
+        <v>72.06</v>
       </c>
       <c r="W274" t="n">
-        <v>70.08</v>
+        <v>70.31</v>
       </c>
       <c r="X274" t="n">
-        <v>0.6588000000000001</v>
+        <v>0.669</v>
       </c>
       <c r="Y274" t="n">
-        <v>25.078</v>
+        <v>25.275</v>
       </c>
       <c r="Z274" t="n">
-        <v>59.396</v>
+        <v>59.725</v>
       </c>
       <c r="AA274" t="n">
-        <v>8.241</v>
+        <v>8.278</v>
       </c>
       <c r="AB274" t="n">
-        <v>26.784</v>
+        <v>26.782</v>
       </c>
       <c r="AC274" t="n">
-        <v>13.488</v>
+        <v>13.229</v>
       </c>
       <c r="AD274" t="n">
-        <v>18.139</v>
+        <v>17.935</v>
       </c>
       <c r="AE274" t="n">
-        <v>10.464</v>
+        <v>10.644</v>
       </c>
       <c r="AF274" t="n">
-        <v>25.604</v>
+        <v>25.72</v>
       </c>
       <c r="AG274" t="n">
-        <v>15.025</v>
+        <v>15.171</v>
       </c>
       <c r="AH274" t="n">
-        <v>5.519</v>
+        <v>5.481</v>
       </c>
       <c r="AI274" t="n">
-        <v>4.659</v>
+        <v>4.558</v>
       </c>
       <c r="AJ274" t="n">
-        <v>14.232</v>
+        <v>14.137</v>
       </c>
       <c r="AK274" t="n">
-        <v>3.8</v>
+        <v>3.4</v>
       </c>
       <c r="AL274" t="n">
-        <v>5.9</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="275">
@@ -34586,22 +34586,22 @@
         </is>
       </c>
       <c r="E285" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F285" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G285" t="b">
         <v>1</v>
       </c>
       <c r="H285" t="n">
-        <v>1914.838</v>
+        <v>1944.981</v>
       </c>
       <c r="I285" t="n">
-        <v>-1.3934</v>
+        <v>-1.2526</v>
       </c>
       <c r="J285" t="n">
-        <v>1716.9</v>
+        <v>1724</v>
       </c>
       <c r="K285" t="n">
         <v>16</v>
@@ -34622,70 +34622,70 @@
         <v>20</v>
       </c>
       <c r="Q285" t="n">
-        <v>116.955</v>
+        <v>117.137</v>
       </c>
       <c r="R285" t="n">
-        <v>101.617</v>
+        <v>102.163</v>
       </c>
       <c r="S285" t="n">
-        <v>15.338</v>
+        <v>14.975</v>
       </c>
       <c r="T285" t="n">
-        <v>0.35639</v>
+        <v>0.36076</v>
       </c>
       <c r="U285" t="n">
-        <v>0.16761</v>
+        <v>0.16454</v>
       </c>
       <c r="V285" t="n">
         <v>79.40000000000001</v>
       </c>
       <c r="W285" t="n">
-        <v>68.83</v>
+        <v>69.09</v>
       </c>
       <c r="X285" t="n">
-        <v>0.68</v>
+        <v>0.6889</v>
       </c>
       <c r="Y285" t="n">
-        <v>28.382</v>
+        <v>28.301</v>
       </c>
       <c r="Z285" t="n">
-        <v>61.036</v>
+        <v>61.364</v>
       </c>
       <c r="AA285" t="n">
-        <v>6.585</v>
+        <v>6.768</v>
       </c>
       <c r="AB285" t="n">
-        <v>19.418</v>
+        <v>20.011</v>
       </c>
       <c r="AC285" t="n">
-        <v>16.047</v>
+        <v>15.757</v>
       </c>
       <c r="AD285" t="n">
-        <v>23.12</v>
+        <v>22.793</v>
       </c>
       <c r="AE285" t="n">
-        <v>14.687</v>
+        <v>14.756</v>
       </c>
       <c r="AF285" t="n">
-        <v>25.945</v>
+        <v>25.646</v>
       </c>
       <c r="AG285" t="n">
-        <v>16.993</v>
+        <v>16.779</v>
       </c>
       <c r="AH285" t="n">
-        <v>7.415</v>
+        <v>7.347</v>
       </c>
       <c r="AI285" t="n">
-        <v>3.542</v>
+        <v>3.614</v>
       </c>
       <c r="AJ285" t="n">
-        <v>17.724</v>
+        <v>17.812</v>
       </c>
       <c r="AK285" t="n">
-        <v>8</v>
+        <v>5.6</v>
       </c>
       <c r="AL285" t="n">
-        <v>7.1</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="286">
@@ -35306,22 +35306,22 @@
         </is>
       </c>
       <c r="E291" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F291" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G291" t="b">
         <v>1</v>
       </c>
       <c r="H291" t="n">
-        <v>2018.552</v>
+        <v>1987.529</v>
       </c>
       <c r="I291" t="n">
-        <v>8.9857</v>
+        <v>8.4871</v>
       </c>
       <c r="J291" t="n">
-        <v>1767</v>
+        <v>1776.6</v>
       </c>
       <c r="K291" t="n">
         <v>20</v>
@@ -35342,70 +35342,70 @@
         <v>19</v>
       </c>
       <c r="Q291" t="n">
-        <v>118.539</v>
+        <v>117.459</v>
       </c>
       <c r="R291" t="n">
-        <v>106.753</v>
+        <v>107.736</v>
       </c>
       <c r="S291" t="n">
-        <v>11.786</v>
+        <v>9.722</v>
       </c>
       <c r="T291" t="n">
-        <v>0.28763</v>
+        <v>0.29262</v>
       </c>
       <c r="U291" t="n">
-        <v>0.15503</v>
+        <v>0.15476</v>
       </c>
       <c r="V291" t="n">
-        <v>80.83</v>
+        <v>80.12</v>
       </c>
       <c r="W291" t="n">
-        <v>72.56</v>
+        <v>73.25</v>
       </c>
       <c r="X291" t="n">
-        <v>0.7</v>
+        <v>0.6702</v>
       </c>
       <c r="Y291" t="n">
-        <v>29.08</v>
+        <v>28.721</v>
       </c>
       <c r="Z291" t="n">
-        <v>60.71</v>
+        <v>60.796</v>
       </c>
       <c r="AA291" t="n">
-        <v>11.45</v>
+        <v>11.168</v>
       </c>
       <c r="AB291" t="n">
-        <v>28.61</v>
+        <v>28.555</v>
       </c>
       <c r="AC291" t="n">
-        <v>11.88</v>
+        <v>12.153</v>
       </c>
       <c r="AD291" t="n">
-        <v>16.75</v>
+        <v>17.007</v>
       </c>
       <c r="AE291" t="n">
-        <v>10.39</v>
+        <v>10.562</v>
       </c>
       <c r="AF291" t="n">
-        <v>24.58</v>
+        <v>24.438</v>
       </c>
       <c r="AG291" t="n">
-        <v>15.98</v>
+        <v>15.663</v>
       </c>
       <c r="AH291" t="n">
-        <v>5.97</v>
+        <v>6.057</v>
       </c>
       <c r="AI291" t="n">
-        <v>3.77</v>
+        <v>3.767</v>
       </c>
       <c r="AJ291" t="n">
-        <v>16.45</v>
+        <v>16.36</v>
       </c>
       <c r="AK291" t="n">
-        <v>-1.4</v>
+        <v>-8.199999999999999</v>
       </c>
       <c r="AL291" t="n">
-        <v>6.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="292">
@@ -36026,22 +36026,22 @@
         </is>
       </c>
       <c r="E297" t="n">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="F297" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G297" t="b">
         <v>1</v>
       </c>
       <c r="H297" t="n">
-        <v>1682.437</v>
+        <v>1698.087</v>
       </c>
       <c r="I297" t="n">
-        <v>8.0585</v>
+        <v>7.7327</v>
       </c>
       <c r="J297" t="n">
-        <v>1510.5</v>
+        <v>1515.8</v>
       </c>
       <c r="K297" t="n">
         <v>63</v>
@@ -36062,70 +36062,70 @@
         <v>52</v>
       </c>
       <c r="Q297" t="n">
-        <v>121.034</v>
+        <v>121</v>
       </c>
       <c r="R297" t="n">
-        <v>106.412</v>
+        <v>106.231</v>
       </c>
       <c r="S297" t="n">
-        <v>14.622</v>
+        <v>14.769</v>
       </c>
       <c r="T297" t="n">
-        <v>0.28053</v>
+        <v>0.2826</v>
       </c>
       <c r="U297" t="n">
-        <v>0.14866</v>
+        <v>0.15151</v>
       </c>
       <c r="V297" t="n">
-        <v>84.47</v>
+        <v>84.16</v>
       </c>
       <c r="W297" t="n">
-        <v>74.31999999999999</v>
+        <v>73.94</v>
       </c>
       <c r="X297" t="n">
-        <v>0.7829</v>
+        <v>0.7894</v>
       </c>
       <c r="Y297" t="n">
-        <v>27.381</v>
+        <v>27.391</v>
       </c>
       <c r="Z297" t="n">
-        <v>58.439</v>
+        <v>58.361</v>
       </c>
       <c r="AA297" t="n">
-        <v>10.582</v>
+        <v>10.572</v>
       </c>
       <c r="AB297" t="n">
-        <v>27.231</v>
+        <v>27.218</v>
       </c>
       <c r="AC297" t="n">
-        <v>19.128</v>
+        <v>18.808</v>
       </c>
       <c r="AD297" t="n">
-        <v>24.437</v>
+        <v>24.227</v>
       </c>
       <c r="AE297" t="n">
-        <v>9.747999999999999</v>
+        <v>9.965</v>
       </c>
       <c r="AF297" t="n">
-        <v>24.402</v>
+        <v>24.62</v>
       </c>
       <c r="AG297" t="n">
-        <v>15.226</v>
+        <v>15.278</v>
       </c>
       <c r="AH297" t="n">
-        <v>6.665</v>
+        <v>6.528</v>
       </c>
       <c r="AI297" t="n">
-        <v>2.387</v>
+        <v>2.287</v>
       </c>
       <c r="AJ297" t="n">
-        <v>16.156</v>
+        <v>16.032</v>
       </c>
       <c r="AK297" t="n">
-        <v>5.4</v>
+        <v>2.2</v>
       </c>
       <c r="AL297" t="n">
-        <v>8.300000000000001</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="298">
@@ -36986,22 +36986,22 @@
         </is>
       </c>
       <c r="E305" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F305" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G305" t="b">
         <v>1</v>
       </c>
       <c r="H305" t="n">
-        <v>1897.052</v>
+        <v>1881.876</v>
       </c>
       <c r="I305" t="n">
-        <v>2.9774</v>
+        <v>3.1818</v>
       </c>
       <c r="J305" t="n">
-        <v>1708.6</v>
+        <v>1716.2</v>
       </c>
       <c r="K305" t="n">
         <v>27</v>
@@ -37022,70 +37022,70 @@
         <v>30</v>
       </c>
       <c r="Q305" t="n">
-        <v>116.926</v>
+        <v>116.161</v>
       </c>
       <c r="R305" t="n">
-        <v>107.231</v>
+        <v>107.674</v>
       </c>
       <c r="S305" t="n">
-        <v>9.695</v>
+        <v>8.487</v>
       </c>
       <c r="T305" t="n">
-        <v>0.30733</v>
+        <v>0.30781</v>
       </c>
       <c r="U305" t="n">
-        <v>0.1316</v>
+        <v>0.13337</v>
       </c>
       <c r="V305" t="n">
-        <v>77.64</v>
+        <v>76.94</v>
       </c>
       <c r="W305" t="n">
-        <v>71</v>
+        <v>71.06999999999999</v>
       </c>
       <c r="X305" t="n">
-        <v>0.6879999999999999</v>
+        <v>0.6621</v>
       </c>
       <c r="Y305" t="n">
-        <v>27.397</v>
+        <v>27.11</v>
       </c>
       <c r="Z305" t="n">
-        <v>58.839</v>
+        <v>58.434</v>
       </c>
       <c r="AA305" t="n">
-        <v>7.957</v>
+        <v>7.869</v>
       </c>
       <c r="AB305" t="n">
-        <v>21.057</v>
+        <v>20.779</v>
       </c>
       <c r="AC305" t="n">
-        <v>14.9</v>
+        <v>14.883</v>
       </c>
       <c r="AD305" t="n">
-        <v>19.56</v>
+        <v>19.621</v>
       </c>
       <c r="AE305" t="n">
-        <v>9.640000000000001</v>
+        <v>9.545</v>
       </c>
       <c r="AF305" t="n">
-        <v>21.576</v>
+        <v>21.352</v>
       </c>
       <c r="AG305" t="n">
-        <v>16.332</v>
+        <v>16.29</v>
       </c>
       <c r="AH305" t="n">
-        <v>6.449</v>
+        <v>6.317</v>
       </c>
       <c r="AI305" t="n">
-        <v>3.158</v>
+        <v>3.041</v>
       </c>
       <c r="AJ305" t="n">
-        <v>16.872</v>
+        <v>16.89</v>
       </c>
       <c r="AK305" t="n">
-        <v>7</v>
+        <v>-0.4</v>
       </c>
       <c r="AL305" t="n">
-        <v>4.7</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="306">
@@ -37826,22 +37826,22 @@
         </is>
       </c>
       <c r="E312" t="n">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="F312" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G312" t="b">
         <v>1</v>
       </c>
       <c r="H312" t="n">
-        <v>1662.23</v>
+        <v>1646.58</v>
       </c>
       <c r="I312" t="n">
-        <v>1.8215</v>
+        <v>1.9334</v>
       </c>
       <c r="J312" t="n">
-        <v>1625.4</v>
+        <v>1627.7</v>
       </c>
       <c r="K312" t="n">
         <v>107</v>
@@ -37862,70 +37862,70 @@
         <v>111</v>
       </c>
       <c r="Q312" t="n">
-        <v>110.869</v>
+        <v>110.556</v>
       </c>
       <c r="R312" t="n">
-        <v>110.996</v>
+        <v>111.362</v>
       </c>
       <c r="S312" t="n">
-        <v>-0.126</v>
+        <v>-0.806</v>
       </c>
       <c r="T312" t="n">
-        <v>0.29015</v>
+        <v>0.29018</v>
       </c>
       <c r="U312" t="n">
-        <v>0.16844</v>
+        <v>0.16506</v>
       </c>
       <c r="V312" t="n">
-        <v>78.93000000000001</v>
+        <v>78.47</v>
       </c>
       <c r="W312" t="n">
-        <v>79.26000000000001</v>
+        <v>79.23999999999999</v>
       </c>
       <c r="X312" t="n">
-        <v>0.52</v>
+        <v>0.4953</v>
       </c>
       <c r="Y312" t="n">
-        <v>27.56</v>
+        <v>27.524</v>
       </c>
       <c r="Z312" t="n">
-        <v>58.32</v>
+        <v>58.388</v>
       </c>
       <c r="AA312" t="n">
-        <v>7.55</v>
+        <v>7.457</v>
       </c>
       <c r="AB312" t="n">
-        <v>21.12</v>
+        <v>21.28</v>
       </c>
       <c r="AC312" t="n">
-        <v>16.26</v>
+        <v>15.965</v>
       </c>
       <c r="AD312" t="n">
-        <v>23.95</v>
+        <v>23.635</v>
       </c>
       <c r="AE312" t="n">
-        <v>9.57</v>
+        <v>9.467000000000001</v>
       </c>
       <c r="AF312" t="n">
-        <v>23.03</v>
+        <v>22.74</v>
       </c>
       <c r="AG312" t="n">
-        <v>14.24</v>
+        <v>14.089</v>
       </c>
       <c r="AH312" t="n">
-        <v>7.23</v>
+        <v>7.31</v>
       </c>
       <c r="AI312" t="n">
-        <v>4.7</v>
+        <v>4.641</v>
       </c>
       <c r="AJ312" t="n">
-        <v>21.55</v>
+        <v>21.438</v>
       </c>
       <c r="AK312" t="n">
-        <v>2</v>
+        <v>-5.6</v>
       </c>
       <c r="AL312" t="n">
-        <v>2.2</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="313">
@@ -38426,22 +38426,22 @@
         </is>
       </c>
       <c r="E317" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F317" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G317" t="b">
         <v>1</v>
       </c>
       <c r="H317" t="n">
-        <v>1917.024</v>
+        <v>1911.017</v>
       </c>
       <c r="I317" t="n">
-        <v>0.2638</v>
+        <v>0.436</v>
       </c>
       <c r="J317" t="n">
-        <v>1617</v>
+        <v>1632.8</v>
       </c>
       <c r="K317" t="n">
         <v>30</v>
@@ -38462,70 +38462,70 @@
         <v>26</v>
       </c>
       <c r="Q317" t="n">
-        <v>119.887</v>
+        <v>119.218</v>
       </c>
       <c r="R317" t="n">
-        <v>103.861</v>
+        <v>104.375</v>
       </c>
       <c r="S317" t="n">
-        <v>16.026</v>
+        <v>14.843</v>
       </c>
       <c r="T317" t="n">
-        <v>0.30557</v>
+        <v>0.30523</v>
       </c>
       <c r="U317" t="n">
-        <v>0.14772</v>
+        <v>0.14484</v>
       </c>
       <c r="V317" t="n">
-        <v>81.84999999999999</v>
+        <v>81.28</v>
       </c>
       <c r="W317" t="n">
-        <v>71.03</v>
+        <v>71.23999999999999</v>
       </c>
       <c r="X317" t="n">
-        <v>0.8247</v>
+        <v>0.7951</v>
       </c>
       <c r="Y317" t="n">
-        <v>28.701</v>
+        <v>28.578</v>
       </c>
       <c r="Z317" t="n">
-        <v>58.266</v>
+        <v>58.434</v>
       </c>
       <c r="AA317" t="n">
-        <v>8.506</v>
+        <v>8.454000000000001</v>
       </c>
       <c r="AB317" t="n">
-        <v>23.893</v>
+        <v>24.134</v>
       </c>
       <c r="AC317" t="n">
-        <v>15.526</v>
+        <v>15.327</v>
       </c>
       <c r="AD317" t="n">
-        <v>22.146</v>
+        <v>21.819</v>
       </c>
       <c r="AE317" t="n">
-        <v>9.679</v>
+        <v>9.619</v>
       </c>
       <c r="AF317" t="n">
-        <v>21.88</v>
+        <v>21.777</v>
       </c>
       <c r="AG317" t="n">
-        <v>17.14</v>
+        <v>17.039</v>
       </c>
       <c r="AH317" t="n">
-        <v>8.571</v>
+        <v>8.602</v>
       </c>
       <c r="AI317" t="n">
-        <v>2.776</v>
+        <v>2.87</v>
       </c>
       <c r="AJ317" t="n">
-        <v>19.042</v>
+        <v>19.235</v>
       </c>
       <c r="AK317" t="n">
-        <v>11.6</v>
+        <v>8.4</v>
       </c>
       <c r="AL317" t="n">
-        <v>3.5</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="318">
@@ -39386,22 +39386,22 @@
         </is>
       </c>
       <c r="E325" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F325" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G325" t="b">
         <v>1</v>
       </c>
       <c r="H325" t="n">
-        <v>1966.747</v>
+        <v>1936.604</v>
       </c>
       <c r="I325" t="n">
-        <v>11.7947</v>
+        <v>11.404</v>
       </c>
       <c r="J325" t="n">
-        <v>1654.9</v>
+        <v>1670.5</v>
       </c>
       <c r="K325" t="n">
         <v>13</v>
@@ -39422,70 +39422,70 @@
         <v>12</v>
       </c>
       <c r="Q325" t="n">
-        <v>119.416</v>
+        <v>119.058</v>
       </c>
       <c r="R325" t="n">
-        <v>101.187</v>
+        <v>101.799</v>
       </c>
       <c r="S325" t="n">
-        <v>18.229</v>
+        <v>17.259</v>
       </c>
       <c r="T325" t="n">
-        <v>0.31319</v>
+        <v>0.31252</v>
       </c>
       <c r="U325" t="n">
-        <v>0.15637</v>
+        <v>0.15584</v>
       </c>
       <c r="V325" t="n">
-        <v>80.7</v>
+        <v>80.39</v>
       </c>
       <c r="W325" t="n">
-        <v>68.58</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="X325" t="n">
-        <v>0.8582</v>
+        <v>0.8276</v>
       </c>
       <c r="Y325" t="n">
-        <v>28.17</v>
+        <v>28.097</v>
       </c>
       <c r="Z325" t="n">
-        <v>60.58</v>
+        <v>60.434</v>
       </c>
       <c r="AA325" t="n">
-        <v>10.221</v>
+        <v>10.124</v>
       </c>
       <c r="AB325" t="n">
-        <v>27.957</v>
+        <v>27.662</v>
       </c>
       <c r="AC325" t="n">
-        <v>14.021</v>
+        <v>14.2</v>
       </c>
       <c r="AD325" t="n">
-        <v>19.133</v>
+        <v>19.372</v>
       </c>
       <c r="AE325" t="n">
-        <v>11.815</v>
+        <v>11.8</v>
       </c>
       <c r="AF325" t="n">
-        <v>25.568</v>
+        <v>25.628</v>
       </c>
       <c r="AG325" t="n">
-        <v>16.396</v>
+        <v>16.552</v>
       </c>
       <c r="AH325" t="n">
-        <v>6.411</v>
+        <v>6.345</v>
       </c>
       <c r="AI325" t="n">
-        <v>6.333</v>
+        <v>6.331</v>
       </c>
       <c r="AJ325" t="n">
-        <v>17.572</v>
+        <v>17.503</v>
       </c>
       <c r="AK325" t="n">
-        <v>7.6</v>
+        <v>5.4</v>
       </c>
       <c r="AL325" t="n">
-        <v>7.5</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="326">
@@ -40346,22 +40346,22 @@
         </is>
       </c>
       <c r="E333" t="n">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="F333" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G333" t="b">
         <v>1</v>
       </c>
       <c r="H333" t="n">
-        <v>1661.239</v>
+        <v>1638.451</v>
       </c>
       <c r="I333" t="n">
-        <v>-2.4181</v>
+        <v>-2.2356</v>
       </c>
       <c r="J333" t="n">
-        <v>1665.4</v>
+        <v>1665.2</v>
       </c>
       <c r="K333" t="n">
         <v>74</v>
@@ -40382,70 +40382,70 @@
         <v>66</v>
       </c>
       <c r="Q333" t="n">
-        <v>112.962</v>
+        <v>112.689</v>
       </c>
       <c r="R333" t="n">
-        <v>110.155</v>
+        <v>110.294</v>
       </c>
       <c r="S333" t="n">
-        <v>2.807</v>
+        <v>2.395</v>
       </c>
       <c r="T333" t="n">
-        <v>0.2982</v>
+        <v>0.29456</v>
       </c>
       <c r="U333" t="n">
-        <v>0.15295</v>
+        <v>0.15274</v>
       </c>
       <c r="V333" t="n">
-        <v>78.97</v>
+        <v>78.79000000000001</v>
       </c>
       <c r="W333" t="n">
-        <v>76.86</v>
+        <v>76.95</v>
       </c>
       <c r="X333" t="n">
-        <v>0.5345</v>
+        <v>0.509</v>
       </c>
       <c r="Y333" t="n">
-        <v>26.825</v>
+        <v>26.869</v>
       </c>
       <c r="Z333" t="n">
-        <v>59.782</v>
+        <v>59.676</v>
       </c>
       <c r="AA333" t="n">
-        <v>8.930999999999999</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="AB333" t="n">
-        <v>26.276</v>
+        <v>25.842</v>
       </c>
       <c r="AC333" t="n">
-        <v>16.218</v>
+        <v>16.093</v>
       </c>
       <c r="AD333" t="n">
-        <v>20.825</v>
+        <v>20.83</v>
       </c>
       <c r="AE333" t="n">
-        <v>9.548999999999999</v>
+        <v>9.442</v>
       </c>
       <c r="AF333" t="n">
-        <v>22.145</v>
+        <v>22.334</v>
       </c>
       <c r="AG333" t="n">
-        <v>14.353</v>
+        <v>14.35</v>
       </c>
       <c r="AH333" t="n">
-        <v>7.589</v>
+        <v>7.594</v>
       </c>
       <c r="AI333" t="n">
-        <v>3.516</v>
+        <v>3.519</v>
       </c>
       <c r="AJ333" t="n">
-        <v>18.578</v>
+        <v>18.479</v>
       </c>
       <c r="AK333" t="n">
-        <v>1.8</v>
+        <v>2.2</v>
       </c>
       <c r="AL333" t="n">
-        <v>0.7</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="334">
@@ -41186,22 +41186,22 @@
         </is>
       </c>
       <c r="E340" t="n">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="F340" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G340" t="b">
         <v>1</v>
       </c>
       <c r="H340" t="n">
-        <v>1632.359</v>
+        <v>1659.004</v>
       </c>
       <c r="I340" t="n">
-        <v>1.9753</v>
+        <v>2.095</v>
       </c>
       <c r="J340" t="n">
-        <v>1543.7</v>
+        <v>1550.5</v>
       </c>
       <c r="K340" t="n">
         <v>82</v>
@@ -41222,70 +41222,70 @@
         <v>78</v>
       </c>
       <c r="Q340" t="n">
-        <v>111.467</v>
+        <v>112.335</v>
       </c>
       <c r="R340" t="n">
-        <v>101.995</v>
+        <v>101.819</v>
       </c>
       <c r="S340" t="n">
-        <v>9.473000000000001</v>
+        <v>10.517</v>
       </c>
       <c r="T340" t="n">
-        <v>0.34362</v>
+        <v>0.34245</v>
       </c>
       <c r="U340" t="n">
-        <v>0.14702</v>
+        <v>0.14448</v>
       </c>
       <c r="V340" t="n">
-        <v>76.97</v>
+        <v>77.73</v>
       </c>
       <c r="W340" t="n">
-        <v>70.45</v>
+        <v>70.44</v>
       </c>
       <c r="X340" t="n">
-        <v>0.67</v>
+        <v>0.6795</v>
       </c>
       <c r="Y340" t="n">
-        <v>27.28</v>
+        <v>27.608</v>
       </c>
       <c r="Z340" t="n">
-        <v>62.39</v>
+        <v>62.773</v>
       </c>
       <c r="AA340" t="n">
-        <v>7.04</v>
+        <v>7.328</v>
       </c>
       <c r="AB340" t="n">
-        <v>21.12</v>
+        <v>21.338</v>
       </c>
       <c r="AC340" t="n">
-        <v>15.37</v>
+        <v>15.186</v>
       </c>
       <c r="AD340" t="n">
-        <v>22.52</v>
+        <v>22.265</v>
       </c>
       <c r="AE340" t="n">
-        <v>13.43</v>
+        <v>13.417</v>
       </c>
       <c r="AF340" t="n">
-        <v>25.67</v>
+        <v>25.794</v>
       </c>
       <c r="AG340" t="n">
-        <v>11.42</v>
+        <v>11.446</v>
       </c>
       <c r="AH340" t="n">
-        <v>6.01</v>
+        <v>6.068</v>
       </c>
       <c r="AI340" t="n">
-        <v>3.92</v>
+        <v>3.865</v>
       </c>
       <c r="AJ340" t="n">
-        <v>17.46</v>
+        <v>17.312</v>
       </c>
       <c r="AK340" t="n">
-        <v>7.4</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="AL340" t="n">
-        <v>5.4</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="341">

</xml_diff>

<commit_message>
Update team snapshot (2026-03-27)
</commit_message>
<xml_diff>
--- a/team_snapshot_2026.xlsx
+++ b/team_snapshot_2026.xlsx
@@ -1826,22 +1826,22 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="F12" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G12" t="b">
         <v>1</v>
       </c>
       <c r="H12" t="n">
-        <v>2278.515</v>
+        <v>2286.821</v>
       </c>
       <c r="I12" t="n">
-        <v>6.3904</v>
+        <v>6.212</v>
       </c>
       <c r="J12" t="n">
-        <v>1771.6</v>
+        <v>1773.8</v>
       </c>
       <c r="K12" t="n">
         <v>2</v>
@@ -1862,70 +1862,70 @@
         <v>3</v>
       </c>
       <c r="Q12" t="n">
-        <v>121.646</v>
+        <v>122.042</v>
       </c>
       <c r="R12" t="n">
-        <v>96.95099999999999</v>
+        <v>97.27200000000001</v>
       </c>
       <c r="S12" t="n">
-        <v>24.694</v>
+        <v>24.77</v>
       </c>
       <c r="T12" t="n">
-        <v>0.29711</v>
+        <v>0.29313</v>
       </c>
       <c r="U12" t="n">
-        <v>0.15073</v>
+        <v>0.15046</v>
       </c>
       <c r="V12" t="n">
-        <v>86.03</v>
+        <v>86.84999999999999</v>
       </c>
       <c r="W12" t="n">
-        <v>68.40000000000001</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="X12" t="n">
-        <v>0.9448</v>
+        <v>0.9463</v>
       </c>
       <c r="Y12" t="n">
-        <v>30.303</v>
+        <v>30.582</v>
       </c>
       <c r="Z12" t="n">
-        <v>60.662</v>
+        <v>60.605</v>
       </c>
       <c r="AA12" t="n">
-        <v>5.924</v>
+        <v>5.886</v>
       </c>
       <c r="AB12" t="n">
-        <v>16.255</v>
+        <v>15.975</v>
       </c>
       <c r="AC12" t="n">
-        <v>19.497</v>
+        <v>19.796</v>
       </c>
       <c r="AD12" t="n">
-        <v>26.724</v>
+        <v>27.051</v>
       </c>
       <c r="AE12" t="n">
-        <v>12.455</v>
+        <v>12.176</v>
       </c>
       <c r="AF12" t="n">
-        <v>28.993</v>
+        <v>28.806</v>
       </c>
       <c r="AG12" t="n">
-        <v>16.607</v>
+        <v>16.744</v>
       </c>
       <c r="AH12" t="n">
-        <v>7.448</v>
+        <v>7.35</v>
       </c>
       <c r="AI12" t="n">
-        <v>4.421</v>
+        <v>4.369</v>
       </c>
       <c r="AJ12" t="n">
-        <v>15.821</v>
+        <v>15.839</v>
       </c>
       <c r="AK12" t="n">
-        <v>15</v>
+        <v>14.8</v>
       </c>
       <c r="AL12" t="n">
-        <v>13.8</v>
+        <v>15.2</v>
       </c>
     </row>
     <row r="13">
@@ -2306,22 +2306,22 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="F16" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G16" t="b">
         <v>1</v>
       </c>
       <c r="H16" t="n">
-        <v>1988.127</v>
+        <v>1979.821</v>
       </c>
       <c r="I16" t="n">
-        <v>5.0738</v>
+        <v>5.0525</v>
       </c>
       <c r="J16" t="n">
-        <v>1731.7</v>
+        <v>1752.3</v>
       </c>
       <c r="K16" t="n">
         <v>15</v>
@@ -2342,70 +2342,70 @@
         <v>15</v>
       </c>
       <c r="Q16" t="n">
-        <v>122.969</v>
+        <v>122.701</v>
       </c>
       <c r="R16" t="n">
-        <v>109.338</v>
+        <v>110.401</v>
       </c>
       <c r="S16" t="n">
-        <v>13.631</v>
+        <v>12.3</v>
       </c>
       <c r="T16" t="n">
-        <v>0.29609</v>
+        <v>0.29747</v>
       </c>
       <c r="U16" t="n">
-        <v>0.11967</v>
+        <v>0.11979</v>
       </c>
       <c r="V16" t="n">
-        <v>90.28</v>
+        <v>90.17</v>
       </c>
       <c r="W16" t="n">
-        <v>80.3</v>
+        <v>81.20999999999999</v>
       </c>
       <c r="X16" t="n">
-        <v>0.7793</v>
+        <v>0.7519</v>
       </c>
       <c r="Y16" t="n">
-        <v>32.379</v>
+        <v>32.316</v>
       </c>
       <c r="Z16" t="n">
-        <v>64.524</v>
+        <v>64.517</v>
       </c>
       <c r="AA16" t="n">
-        <v>8.228</v>
+        <v>8.115</v>
       </c>
       <c r="AB16" t="n">
-        <v>21.214</v>
+        <v>21.308</v>
       </c>
       <c r="AC16" t="n">
-        <v>17.29</v>
+        <v>17.429</v>
       </c>
       <c r="AD16" t="n">
-        <v>23.062</v>
+        <v>23.181</v>
       </c>
       <c r="AE16" t="n">
-        <v>10.014</v>
+        <v>9.994</v>
       </c>
       <c r="AF16" t="n">
-        <v>23.869</v>
+        <v>23.672</v>
       </c>
       <c r="AG16" t="n">
-        <v>17.283</v>
+        <v>17.135</v>
       </c>
       <c r="AH16" t="n">
-        <v>7.31</v>
+        <v>7.362</v>
       </c>
       <c r="AI16" t="n">
-        <v>5.145</v>
+        <v>5.134</v>
       </c>
       <c r="AJ16" t="n">
-        <v>16.448</v>
+        <v>16.817</v>
       </c>
       <c r="AK16" t="n">
-        <v>8.4</v>
+        <v>3.6</v>
       </c>
       <c r="AL16" t="n">
-        <v>5.5</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="17">
@@ -2666,22 +2666,22 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="F19" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G19" t="b">
         <v>1</v>
       </c>
       <c r="H19" t="n">
-        <v>1836.183</v>
+        <v>1853.815</v>
       </c>
       <c r="I19" t="n">
-        <v>-7.1903</v>
+        <v>-6.9997</v>
       </c>
       <c r="J19" t="n">
-        <v>1743</v>
+        <v>1745.4</v>
       </c>
       <c r="K19" t="n">
         <v>38</v>
@@ -2702,70 +2702,70 @@
         <v>38</v>
       </c>
       <c r="Q19" t="n">
-        <v>118.616</v>
+        <v>118.556</v>
       </c>
       <c r="R19" t="n">
-        <v>113.595</v>
+        <v>113.403</v>
       </c>
       <c r="S19" t="n">
-        <v>5.021</v>
+        <v>5.153</v>
       </c>
       <c r="T19" t="n">
-        <v>0.34374</v>
+        <v>0.34498</v>
       </c>
       <c r="U19" t="n">
-        <v>0.14484</v>
+        <v>0.14368</v>
       </c>
       <c r="V19" t="n">
-        <v>82.90000000000001</v>
+        <v>82.55</v>
       </c>
       <c r="W19" t="n">
-        <v>79.25</v>
+        <v>78.84</v>
       </c>
       <c r="X19" t="n">
-        <v>0.5468</v>
+        <v>0.5592</v>
       </c>
       <c r="Y19" t="n">
-        <v>27.386</v>
+        <v>27.465</v>
       </c>
       <c r="Z19" t="n">
-        <v>59.983</v>
+        <v>60.036</v>
       </c>
       <c r="AA19" t="n">
-        <v>8.207000000000001</v>
+        <v>8.121</v>
       </c>
       <c r="AB19" t="n">
-        <v>24.187</v>
+        <v>24.165</v>
       </c>
       <c r="AC19" t="n">
-        <v>19.922</v>
+        <v>19.497</v>
       </c>
       <c r="AD19" t="n">
-        <v>26.732</v>
+        <v>26.233</v>
       </c>
       <c r="AE19" t="n">
-        <v>11.983</v>
+        <v>11.964</v>
       </c>
       <c r="AF19" t="n">
-        <v>22.56</v>
+        <v>22.397</v>
       </c>
       <c r="AG19" t="n">
-        <v>12.904</v>
+        <v>12.818</v>
       </c>
       <c r="AH19" t="n">
-        <v>7.229</v>
+        <v>7.319</v>
       </c>
       <c r="AI19" t="n">
-        <v>4.198</v>
+        <v>4.157</v>
       </c>
       <c r="AJ19" t="n">
-        <v>17.155</v>
+        <v>17.05</v>
       </c>
       <c r="AK19" t="n">
-        <v>2.6</v>
+        <v>6.2</v>
       </c>
       <c r="AL19" t="n">
-        <v>0.4</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="20">
@@ -8546,22 +8546,22 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="F68" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G68" t="b">
         <v>1</v>
       </c>
       <c r="H68" t="n">
-        <v>1719.075</v>
+        <v>1691.801</v>
       </c>
       <c r="I68" t="n">
-        <v>-1.4928</v>
+        <v>-1.1741</v>
       </c>
       <c r="J68" t="n">
-        <v>1578.5</v>
+        <v>1578.8</v>
       </c>
       <c r="K68" t="n">
         <v>78</v>
@@ -8582,70 +8582,70 @@
         <v>69</v>
       </c>
       <c r="Q68" t="n">
-        <v>110.613</v>
+        <v>109.611</v>
       </c>
       <c r="R68" t="n">
-        <v>102.177</v>
+        <v>102.017</v>
       </c>
       <c r="S68" t="n">
-        <v>8.436</v>
+        <v>7.595</v>
       </c>
       <c r="T68" t="n">
-        <v>0.24972</v>
+        <v>0.2537</v>
       </c>
       <c r="U68" t="n">
-        <v>0.16976</v>
+        <v>0.16647</v>
       </c>
       <c r="V68" t="n">
-        <v>74.72</v>
+        <v>73.95999999999999</v>
       </c>
       <c r="W68" t="n">
-        <v>69.45</v>
+        <v>69.22</v>
       </c>
       <c r="X68" t="n">
-        <v>0.6974</v>
+        <v>0.6696</v>
       </c>
       <c r="Y68" t="n">
-        <v>24.213</v>
+        <v>23.982</v>
       </c>
       <c r="Z68" t="n">
-        <v>53.414</v>
+        <v>53.732</v>
       </c>
       <c r="AA68" t="n">
-        <v>7.734</v>
+        <v>7.554</v>
       </c>
       <c r="AB68" t="n">
-        <v>22.331</v>
+        <v>22.402</v>
       </c>
       <c r="AC68" t="n">
-        <v>18.53</v>
+        <v>18.42</v>
       </c>
       <c r="AD68" t="n">
-        <v>24.557</v>
+        <v>24.438</v>
       </c>
       <c r="AE68" t="n">
-        <v>7.919</v>
+        <v>8.071</v>
       </c>
       <c r="AF68" t="n">
-        <v>23.258</v>
+        <v>23.179</v>
       </c>
       <c r="AG68" t="n">
-        <v>14.377</v>
+        <v>14.17</v>
       </c>
       <c r="AH68" t="n">
-        <v>8.073</v>
+        <v>8.08</v>
       </c>
       <c r="AI68" t="n">
-        <v>3.971</v>
+        <v>3.964</v>
       </c>
       <c r="AJ68" t="n">
-        <v>16.761</v>
+        <v>16.857</v>
       </c>
       <c r="AK68" t="n">
-        <v>6.2</v>
+        <v>4</v>
       </c>
       <c r="AL68" t="n">
-        <v>5.9</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="69">
@@ -14186,22 +14186,22 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="F115" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G115" t="b">
         <v>1</v>
       </c>
       <c r="H115" t="n">
-        <v>2122.165</v>
+        <v>2086.9</v>
       </c>
       <c r="I115" t="n">
-        <v>1.0162</v>
+        <v>0.9762</v>
       </c>
       <c r="J115" t="n">
-        <v>1741.9</v>
+        <v>1746.8</v>
       </c>
       <c r="K115" t="n">
         <v>5</v>
@@ -14222,70 +14222,70 @@
         <v>5</v>
       </c>
       <c r="Q115" t="n">
-        <v>117.91</v>
+        <v>117.051</v>
       </c>
       <c r="R115" t="n">
-        <v>94.52</v>
+        <v>95.251</v>
       </c>
       <c r="S115" t="n">
-        <v>23.39</v>
+        <v>21.799</v>
       </c>
       <c r="T115" t="n">
-        <v>0.33619</v>
+        <v>0.33361</v>
       </c>
       <c r="U115" t="n">
-        <v>0.12241</v>
+        <v>0.12375</v>
       </c>
       <c r="V115" t="n">
-        <v>77.56</v>
+        <v>76.7</v>
       </c>
       <c r="W115" t="n">
-        <v>62.21</v>
+        <v>62.34</v>
       </c>
       <c r="X115" t="n">
-        <v>0.8347</v>
+        <v>0.8046</v>
       </c>
       <c r="Y115" t="n">
-        <v>27.934</v>
+        <v>27.713</v>
       </c>
       <c r="Z115" t="n">
-        <v>61.966</v>
+        <v>61.54</v>
       </c>
       <c r="AA115" t="n">
-        <v>8.744</v>
+        <v>8.759</v>
       </c>
       <c r="AB115" t="n">
-        <v>25.104</v>
+        <v>24.985</v>
       </c>
       <c r="AC115" t="n">
-        <v>12.947</v>
+        <v>12.858</v>
       </c>
       <c r="AD115" t="n">
-        <v>16.762</v>
+        <v>16.843</v>
       </c>
       <c r="AE115" t="n">
-        <v>11.671</v>
+        <v>11.625</v>
       </c>
       <c r="AF115" t="n">
-        <v>23.17</v>
+        <v>23.41</v>
       </c>
       <c r="AG115" t="n">
-        <v>14.523</v>
+        <v>14.475</v>
       </c>
       <c r="AH115" t="n">
-        <v>7.609</v>
+        <v>7.444</v>
       </c>
       <c r="AI115" t="n">
-        <v>3.887</v>
+        <v>3.831</v>
       </c>
       <c r="AJ115" t="n">
-        <v>17.873</v>
+        <v>17.755</v>
       </c>
       <c r="AK115" t="n">
-        <v>17.2</v>
+        <v>13.8</v>
       </c>
       <c r="AL115" t="n">
-        <v>12.6</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="116">
@@ -14906,22 +14906,22 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="F121" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G121" t="b">
         <v>1</v>
       </c>
       <c r="H121" t="n">
-        <v>1997.795</v>
+        <v>2033.06</v>
       </c>
       <c r="I121" t="n">
-        <v>6.9704</v>
+        <v>6.6485</v>
       </c>
       <c r="J121" t="n">
-        <v>1718.8</v>
+        <v>1730.7</v>
       </c>
       <c r="K121" t="n">
         <v>7</v>
@@ -14942,70 +14942,70 @@
         <v>8</v>
       </c>
       <c r="Q121" t="n">
-        <v>125.89</v>
+        <v>125.389</v>
       </c>
       <c r="R121" t="n">
-        <v>102.84</v>
+        <v>102.649</v>
       </c>
       <c r="S121" t="n">
-        <v>23.05</v>
+        <v>22.739</v>
       </c>
       <c r="T121" t="n">
-        <v>0.32312</v>
+        <v>0.32365</v>
       </c>
       <c r="U121" t="n">
-        <v>0.12769</v>
+        <v>0.12572</v>
       </c>
       <c r="V121" t="n">
-        <v>84.65000000000001</v>
+        <v>84</v>
       </c>
       <c r="W121" t="n">
-        <v>69.25</v>
+        <v>68.84999999999999</v>
       </c>
       <c r="X121" t="n">
-        <v>0.7669</v>
+        <v>0.7734</v>
       </c>
       <c r="Y121" t="n">
-        <v>28.699</v>
+        <v>28.458</v>
       </c>
       <c r="Z121" t="n">
-        <v>62.079</v>
+        <v>62.187</v>
       </c>
       <c r="AA121" t="n">
-        <v>10.981</v>
+        <v>10.926</v>
       </c>
       <c r="AB121" t="n">
-        <v>31.576</v>
+        <v>31.66</v>
       </c>
       <c r="AC121" t="n">
-        <v>16.361</v>
+        <v>15.878</v>
       </c>
       <c r="AD121" t="n">
-        <v>20.73</v>
+        <v>20.07</v>
       </c>
       <c r="AE121" t="n">
-        <v>12.554</v>
+        <v>12.501</v>
       </c>
       <c r="AF121" t="n">
-        <v>26.502</v>
+        <v>26.314</v>
       </c>
       <c r="AG121" t="n">
-        <v>14.738</v>
+        <v>14.819</v>
       </c>
       <c r="AH121" t="n">
-        <v>3.864</v>
+        <v>3.858</v>
       </c>
       <c r="AI121" t="n">
-        <v>4.563</v>
+        <v>4.464</v>
       </c>
       <c r="AJ121" t="n">
-        <v>13.184</v>
+        <v>13.466</v>
       </c>
       <c r="AK121" t="n">
-        <v>17</v>
+        <v>13.8</v>
       </c>
       <c r="AL121" t="n">
-        <v>12.4</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="122">
@@ -15026,22 +15026,22 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="F122" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G122" t="b">
         <v>1</v>
       </c>
       <c r="H122" t="n">
-        <v>1617.365</v>
+        <v>1644.639</v>
       </c>
       <c r="I122" t="n">
-        <v>2.1828</v>
+        <v>2.2958</v>
       </c>
       <c r="J122" t="n">
-        <v>1513.3</v>
+        <v>1519.7</v>
       </c>
       <c r="K122" t="n">
         <v>103</v>
@@ -15062,70 +15062,70 @@
         <v>95</v>
       </c>
       <c r="Q122" t="n">
-        <v>110.138</v>
+        <v>109.747</v>
       </c>
       <c r="R122" t="n">
-        <v>101.764</v>
+        <v>101.285</v>
       </c>
       <c r="S122" t="n">
-        <v>8.374000000000001</v>
+        <v>8.462</v>
       </c>
       <c r="T122" t="n">
-        <v>0.25849</v>
+        <v>0.25045</v>
       </c>
       <c r="U122" t="n">
-        <v>0.15917</v>
+        <v>0.16263</v>
       </c>
       <c r="V122" t="n">
-        <v>74.81</v>
+        <v>74.28</v>
       </c>
       <c r="W122" t="n">
-        <v>68.98999999999999</v>
+        <v>68.42</v>
       </c>
       <c r="X122" t="n">
-        <v>0.6394</v>
+        <v>0.6498</v>
       </c>
       <c r="Y122" t="n">
-        <v>26.923</v>
+        <v>26.756</v>
       </c>
       <c r="Z122" t="n">
-        <v>58.025</v>
+        <v>57.333</v>
       </c>
       <c r="AA122" t="n">
-        <v>8.827999999999999</v>
+        <v>8.714</v>
       </c>
       <c r="AB122" t="n">
-        <v>25.007</v>
+        <v>24.608</v>
       </c>
       <c r="AC122" t="n">
-        <v>12.802</v>
+        <v>12.692</v>
       </c>
       <c r="AD122" t="n">
-        <v>17.875</v>
+        <v>17.854</v>
       </c>
       <c r="AE122" t="n">
-        <v>8.678000000000001</v>
+        <v>8.42</v>
       </c>
       <c r="AF122" t="n">
-        <v>25.177</v>
+        <v>25.538</v>
       </c>
       <c r="AG122" t="n">
-        <v>13.893</v>
+        <v>13.838</v>
       </c>
       <c r="AH122" t="n">
-        <v>5.639</v>
+        <v>5.502</v>
       </c>
       <c r="AI122" t="n">
-        <v>2.24</v>
+        <v>2.27</v>
       </c>
       <c r="AJ122" t="n">
-        <v>17.279</v>
+        <v>17.189</v>
       </c>
       <c r="AK122" t="n">
-        <v>2.2</v>
+        <v>3</v>
       </c>
       <c r="AL122" t="n">
-        <v>0.1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="123">
@@ -15626,22 +15626,22 @@
         </is>
       </c>
       <c r="E127" t="n">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="F127" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G127" t="b">
         <v>1</v>
       </c>
       <c r="H127" t="n">
-        <v>1896.858</v>
+        <v>1916.673</v>
       </c>
       <c r="I127" t="n">
-        <v>2.8676</v>
+        <v>2.8861</v>
       </c>
       <c r="J127" t="n">
-        <v>1722.3</v>
+        <v>1722.1</v>
       </c>
       <c r="K127" t="n">
         <v>25</v>
@@ -15662,70 +15662,70 @@
         <v>27</v>
       </c>
       <c r="Q127" t="n">
-        <v>119.243</v>
+        <v>119.481</v>
       </c>
       <c r="R127" t="n">
-        <v>105.476</v>
+        <v>105.751</v>
       </c>
       <c r="S127" t="n">
-        <v>13.767</v>
+        <v>13.73</v>
       </c>
       <c r="T127" t="n">
-        <v>0.29258</v>
+        <v>0.29403</v>
       </c>
       <c r="U127" t="n">
-        <v>0.1441</v>
+        <v>0.14449</v>
       </c>
       <c r="V127" t="n">
-        <v>74.90000000000001</v>
+        <v>74.98999999999999</v>
       </c>
       <c r="W127" t="n">
-        <v>66.05</v>
+        <v>66.18000000000001</v>
       </c>
       <c r="X127" t="n">
-        <v>0.6601</v>
+        <v>0.6694</v>
       </c>
       <c r="Y127" t="n">
-        <v>26.2</v>
+        <v>26.149</v>
       </c>
       <c r="Z127" t="n">
-        <v>53.562</v>
+        <v>53.785</v>
       </c>
       <c r="AA127" t="n">
-        <v>7.954</v>
+        <v>8.151</v>
       </c>
       <c r="AB127" t="n">
-        <v>22.37</v>
+        <v>22.957</v>
       </c>
       <c r="AC127" t="n">
-        <v>14.336</v>
+        <v>14.133</v>
       </c>
       <c r="AD127" t="n">
-        <v>18.702</v>
+        <v>18.356</v>
       </c>
       <c r="AE127" t="n">
-        <v>8.065</v>
+        <v>8.198</v>
       </c>
       <c r="AF127" t="n">
-        <v>19.473</v>
+        <v>19.611</v>
       </c>
       <c r="AG127" t="n">
-        <v>15.338</v>
+        <v>15.446</v>
       </c>
       <c r="AH127" t="n">
-        <v>7.028</v>
+        <v>6.885</v>
       </c>
       <c r="AI127" t="n">
-        <v>1.963</v>
+        <v>2.08</v>
       </c>
       <c r="AJ127" t="n">
-        <v>17.745</v>
+        <v>17.609</v>
       </c>
       <c r="AK127" t="n">
-        <v>1.2</v>
+        <v>4.2</v>
       </c>
       <c r="AL127" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="128">
@@ -23786,22 +23786,22 @@
         </is>
       </c>
       <c r="E195" t="n">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="F195" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G195" t="b">
         <v>1</v>
       </c>
       <c r="H195" t="n">
-        <v>2012.467</v>
+        <v>1992.651</v>
       </c>
       <c r="I195" t="n">
-        <v>8.516999999999999</v>
+        <v>8.0527</v>
       </c>
       <c r="J195" t="n">
-        <v>1683.9</v>
+        <v>1681</v>
       </c>
       <c r="K195" t="n">
         <v>14</v>
@@ -23822,70 +23822,70 @@
         <v>14</v>
       </c>
       <c r="Q195" t="n">
-        <v>115.192</v>
+        <v>115.348</v>
       </c>
       <c r="R195" t="n">
-        <v>98.636</v>
+        <v>99.65900000000001</v>
       </c>
       <c r="S195" t="n">
-        <v>16.556</v>
+        <v>15.689</v>
       </c>
       <c r="T195" t="n">
-        <v>0.24223</v>
+        <v>0.23826</v>
       </c>
       <c r="U195" t="n">
-        <v>0.14089</v>
+        <v>0.13836</v>
       </c>
       <c r="V195" t="n">
-        <v>77.12</v>
+        <v>76.92</v>
       </c>
       <c r="W195" t="n">
-        <v>65.88</v>
+        <v>66.23999999999999</v>
       </c>
       <c r="X195" t="n">
-        <v>0.8252</v>
+        <v>0.793</v>
       </c>
       <c r="Y195" t="n">
-        <v>27.572</v>
+        <v>27.538</v>
       </c>
       <c r="Z195" t="n">
-        <v>58.847</v>
+        <v>58.656</v>
       </c>
       <c r="AA195" t="n">
-        <v>10.573</v>
+        <v>10.678</v>
       </c>
       <c r="AB195" t="n">
-        <v>29.723</v>
+        <v>29.83</v>
       </c>
       <c r="AC195" t="n">
-        <v>11.866</v>
+        <v>11.841</v>
       </c>
       <c r="AD195" t="n">
-        <v>15.624</v>
+        <v>15.54</v>
       </c>
       <c r="AE195" t="n">
-        <v>8.292999999999999</v>
+        <v>8.125999999999999</v>
       </c>
       <c r="AF195" t="n">
-        <v>25.33</v>
+        <v>25.237</v>
       </c>
       <c r="AG195" t="n">
-        <v>18.098</v>
+        <v>18.113</v>
       </c>
       <c r="AH195" t="n">
-        <v>7.302</v>
+        <v>7.275</v>
       </c>
       <c r="AI195" t="n">
-        <v>2.418</v>
+        <v>2.388</v>
       </c>
       <c r="AJ195" t="n">
-        <v>14.3</v>
+        <v>13.996</v>
       </c>
       <c r="AK195" t="n">
-        <v>0.8</v>
+        <v>3.6</v>
       </c>
       <c r="AL195" t="n">
-        <v>6.9</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="196">
@@ -23906,22 +23906,22 @@
         </is>
       </c>
       <c r="E196" t="n">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="F196" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G196" t="b">
         <v>1</v>
       </c>
       <c r="H196" t="n">
-        <v>1767.735</v>
+        <v>1750.102</v>
       </c>
       <c r="I196" t="n">
-        <v>5.1312</v>
+        <v>4.9871</v>
       </c>
       <c r="J196" t="n">
-        <v>1608.4</v>
+        <v>1615.3</v>
       </c>
       <c r="K196" t="n">
         <v>75</v>
@@ -23942,70 +23942,70 @@
         <v>70</v>
       </c>
       <c r="Q196" t="n">
-        <v>113.135</v>
+        <v>112.852</v>
       </c>
       <c r="R196" t="n">
-        <v>105.56</v>
+        <v>105.962</v>
       </c>
       <c r="S196" t="n">
-        <v>7.575</v>
+        <v>6.89</v>
       </c>
       <c r="T196" t="n">
-        <v>0.30057</v>
+        <v>0.30034</v>
       </c>
       <c r="U196" t="n">
-        <v>0.14388</v>
+        <v>0.14519</v>
       </c>
       <c r="V196" t="n">
-        <v>76.19</v>
+        <v>75.95999999999999</v>
       </c>
       <c r="W196" t="n">
-        <v>71.36</v>
+        <v>71.56999999999999</v>
       </c>
       <c r="X196" t="n">
-        <v>0.6698</v>
+        <v>0.6429</v>
       </c>
       <c r="Y196" t="n">
-        <v>25.138</v>
+        <v>25.134</v>
       </c>
       <c r="Z196" t="n">
-        <v>56.916</v>
+        <v>56.839</v>
       </c>
       <c r="AA196" t="n">
-        <v>6.614</v>
+        <v>6.652</v>
       </c>
       <c r="AB196" t="n">
-        <v>18.458</v>
+        <v>18.527</v>
       </c>
       <c r="AC196" t="n">
-        <v>19.193</v>
+        <v>18.938</v>
       </c>
       <c r="AD196" t="n">
-        <v>25.503</v>
+        <v>25.25</v>
       </c>
       <c r="AE196" t="n">
-        <v>10.239</v>
+        <v>10.179</v>
       </c>
       <c r="AF196" t="n">
-        <v>23.727</v>
+        <v>23.607</v>
       </c>
       <c r="AG196" t="n">
-        <v>14.533</v>
+        <v>14.518</v>
       </c>
       <c r="AH196" t="n">
-        <v>6.577</v>
+        <v>6.518</v>
       </c>
       <c r="AI196" t="n">
-        <v>3.725</v>
+        <v>3.732</v>
       </c>
       <c r="AJ196" t="n">
-        <v>17.999</v>
+        <v>17.884</v>
       </c>
       <c r="AK196" t="n">
-        <v>10</v>
+        <v>1.8</v>
       </c>
       <c r="AL196" t="n">
-        <v>6.3</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="197">
@@ -24146,22 +24146,22 @@
         </is>
       </c>
       <c r="E198" t="n">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F198" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G198" t="b">
         <v>1</v>
       </c>
       <c r="H198" t="n">
-        <v>1808.195</v>
+        <v>1819.199</v>
       </c>
       <c r="I198" t="n">
-        <v>2.0968</v>
+        <v>1.8714</v>
       </c>
       <c r="J198" t="n">
-        <v>1592</v>
+        <v>1594.7</v>
       </c>
       <c r="K198" t="n">
         <v>50</v>
@@ -24182,70 +24182,70 @@
         <v>46</v>
       </c>
       <c r="Q198" t="n">
-        <v>116.354</v>
+        <v>116.155</v>
       </c>
       <c r="R198" t="n">
-        <v>102.654</v>
+        <v>102.4</v>
       </c>
       <c r="S198" t="n">
-        <v>13.7</v>
+        <v>13.755</v>
       </c>
       <c r="T198" t="n">
-        <v>0.28594</v>
+        <v>0.28162</v>
       </c>
       <c r="U198" t="n">
-        <v>0.14241</v>
+        <v>0.1422</v>
       </c>
       <c r="V198" t="n">
-        <v>81.04000000000001</v>
+        <v>81.11</v>
       </c>
       <c r="W198" t="n">
-        <v>71.51000000000001</v>
+        <v>71.5</v>
       </c>
       <c r="X198" t="n">
-        <v>0.7082000000000001</v>
+        <v>0.7164</v>
       </c>
       <c r="Y198" t="n">
-        <v>28.082</v>
+        <v>28.057</v>
       </c>
       <c r="Z198" t="n">
-        <v>60.535</v>
+        <v>60.446</v>
       </c>
       <c r="AA198" t="n">
-        <v>9.220000000000001</v>
+        <v>9.090999999999999</v>
       </c>
       <c r="AB198" t="n">
-        <v>25.366</v>
+        <v>25.162</v>
       </c>
       <c r="AC198" t="n">
-        <v>15.655</v>
+        <v>15.902</v>
       </c>
       <c r="AD198" t="n">
-        <v>21.605</v>
+        <v>21.846</v>
       </c>
       <c r="AE198" t="n">
-        <v>10.156</v>
+        <v>10.006</v>
       </c>
       <c r="AF198" t="n">
-        <v>24.806</v>
+        <v>25.059</v>
       </c>
       <c r="AG198" t="n">
-        <v>14.886</v>
+        <v>14.787</v>
       </c>
       <c r="AH198" t="n">
-        <v>7.987</v>
+        <v>7.9</v>
       </c>
       <c r="AI198" t="n">
-        <v>2.878</v>
+        <v>2.787</v>
       </c>
       <c r="AJ198" t="n">
-        <v>17.316</v>
+        <v>17.154</v>
       </c>
       <c r="AK198" t="n">
-        <v>11.8</v>
+        <v>15.6</v>
       </c>
       <c r="AL198" t="n">
-        <v>8.800000000000001</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="199">
@@ -28586,22 +28586,22 @@
         </is>
       </c>
       <c r="E235" t="n">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="F235" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G235" t="b">
         <v>1</v>
       </c>
       <c r="H235" t="n">
-        <v>2023.223</v>
+        <v>2037.083</v>
       </c>
       <c r="I235" t="n">
-        <v>-0.6463</v>
+        <v>-0.5673</v>
       </c>
       <c r="J235" t="n">
-        <v>1767</v>
+        <v>1768.6</v>
       </c>
       <c r="K235" t="n">
         <v>8</v>
@@ -28622,70 +28622,70 @@
         <v>9</v>
       </c>
       <c r="Q235" t="n">
-        <v>125.552</v>
+        <v>125.585</v>
       </c>
       <c r="R235" t="n">
-        <v>107.346</v>
+        <v>107.86</v>
       </c>
       <c r="S235" t="n">
-        <v>18.206</v>
+        <v>17.726</v>
       </c>
       <c r="T235" t="n">
-        <v>0.3071</v>
+        <v>0.31046</v>
       </c>
       <c r="U235" t="n">
-        <v>0.13688</v>
+        <v>0.13408</v>
       </c>
       <c r="V235" t="n">
-        <v>82.16</v>
+        <v>82.08</v>
       </c>
       <c r="W235" t="n">
-        <v>70.13</v>
+        <v>70.36</v>
       </c>
       <c r="X235" t="n">
-        <v>0.7854</v>
+        <v>0.791</v>
       </c>
       <c r="Y235" t="n">
-        <v>29.854</v>
+        <v>29.895</v>
       </c>
       <c r="Z235" t="n">
-        <v>59.739</v>
+        <v>59.91</v>
       </c>
       <c r="AA235" t="n">
-        <v>9.368</v>
+        <v>9.199</v>
       </c>
       <c r="AB235" t="n">
-        <v>24.165</v>
+        <v>24.102</v>
       </c>
       <c r="AC235" t="n">
-        <v>12.257</v>
+        <v>12.283</v>
       </c>
       <c r="AD235" t="n">
-        <v>16.368</v>
+        <v>16.447</v>
       </c>
       <c r="AE235" t="n">
-        <v>10.437</v>
+        <v>10.537</v>
       </c>
       <c r="AF235" t="n">
-        <v>22.985</v>
+        <v>22.9</v>
       </c>
       <c r="AG235" t="n">
-        <v>19.548</v>
+        <v>19.315</v>
       </c>
       <c r="AH235" t="n">
-        <v>5.586</v>
+        <v>5.482</v>
       </c>
       <c r="AI235" t="n">
-        <v>2.759</v>
+        <v>2.665</v>
       </c>
       <c r="AJ235" t="n">
-        <v>14.713</v>
+        <v>14.732</v>
       </c>
       <c r="AK235" t="n">
-        <v>14.8</v>
+        <v>12</v>
       </c>
       <c r="AL235" t="n">
-        <v>7.7</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="236">
@@ -33266,22 +33266,22 @@
         </is>
       </c>
       <c r="E274" t="n">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F274" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G274" t="b">
         <v>1</v>
       </c>
       <c r="H274" t="n">
-        <v>1659.458</v>
+        <v>1648.453</v>
       </c>
       <c r="I274" t="n">
-        <v>1.9645</v>
+        <v>2.3034</v>
       </c>
       <c r="J274" t="n">
-        <v>1527.6</v>
+        <v>1536.4</v>
       </c>
       <c r="K274" t="n">
         <v>116</v>
@@ -33302,70 +33302,70 @@
         <v>121</v>
       </c>
       <c r="Q274" t="n">
-        <v>106.077</v>
+        <v>105.666</v>
       </c>
       <c r="R274" t="n">
-        <v>103.137</v>
+        <v>103.567</v>
       </c>
       <c r="S274" t="n">
-        <v>2.94</v>
+        <v>2.099</v>
       </c>
       <c r="T274" t="n">
-        <v>0.29071</v>
+        <v>0.28855</v>
       </c>
       <c r="U274" t="n">
-        <v>0.16258</v>
+        <v>0.16193</v>
       </c>
       <c r="V274" t="n">
-        <v>72.06</v>
+        <v>71.92</v>
       </c>
       <c r="W274" t="n">
-        <v>70.31</v>
+        <v>70.76000000000001</v>
       </c>
       <c r="X274" t="n">
-        <v>0.669</v>
+        <v>0.6429</v>
       </c>
       <c r="Y274" t="n">
-        <v>25.275</v>
+        <v>25.269</v>
       </c>
       <c r="Z274" t="n">
-        <v>59.725</v>
+        <v>59.857</v>
       </c>
       <c r="AA274" t="n">
-        <v>8.278</v>
+        <v>8.298999999999999</v>
       </c>
       <c r="AB274" t="n">
-        <v>26.782</v>
+        <v>27.01</v>
       </c>
       <c r="AC274" t="n">
-        <v>13.229</v>
+        <v>13.084</v>
       </c>
       <c r="AD274" t="n">
-        <v>17.935</v>
+        <v>17.721</v>
       </c>
       <c r="AE274" t="n">
-        <v>10.644</v>
+        <v>10.513</v>
       </c>
       <c r="AF274" t="n">
-        <v>25.72</v>
+        <v>25.672</v>
       </c>
       <c r="AG274" t="n">
-        <v>15.171</v>
+        <v>15.039</v>
       </c>
       <c r="AH274" t="n">
-        <v>5.481</v>
+        <v>5.539</v>
       </c>
       <c r="AI274" t="n">
-        <v>4.558</v>
+        <v>4.591</v>
       </c>
       <c r="AJ274" t="n">
-        <v>14.137</v>
+        <v>14.36</v>
       </c>
       <c r="AK274" t="n">
-        <v>3.4</v>
+        <v>-2</v>
       </c>
       <c r="AL274" t="n">
-        <v>6.4</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="275">
@@ -34946,22 +34946,22 @@
         </is>
       </c>
       <c r="E288" t="n">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="F288" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G288" t="b">
         <v>1</v>
       </c>
       <c r="H288" t="n">
-        <v>1845.111</v>
+        <v>1831.251</v>
       </c>
       <c r="I288" t="n">
-        <v>2.8244</v>
+        <v>3.1749</v>
       </c>
       <c r="J288" t="n">
-        <v>1711</v>
+        <v>1708.8</v>
       </c>
       <c r="K288" t="n">
         <v>37</v>
@@ -34982,70 +34982,70 @@
         <v>42</v>
       </c>
       <c r="Q288" t="n">
-        <v>119.114</v>
+        <v>119.651</v>
       </c>
       <c r="R288" t="n">
-        <v>110.731</v>
+        <v>111.7</v>
       </c>
       <c r="S288" t="n">
-        <v>8.382999999999999</v>
+        <v>7.951</v>
       </c>
       <c r="T288" t="n">
-        <v>0.30206</v>
+        <v>0.30538</v>
       </c>
       <c r="U288" t="n">
-        <v>0.14233</v>
+        <v>0.14182</v>
       </c>
       <c r="V288" t="n">
-        <v>81.79000000000001</v>
+        <v>81.68000000000001</v>
       </c>
       <c r="W288" t="n">
-        <v>75.97</v>
+        <v>76.14</v>
       </c>
       <c r="X288" t="n">
-        <v>0.5915</v>
+        <v>0.5672</v>
       </c>
       <c r="Y288" t="n">
-        <v>27.7</v>
+        <v>27.752</v>
       </c>
       <c r="Z288" t="n">
-        <v>58.074</v>
+        <v>57.985</v>
       </c>
       <c r="AA288" t="n">
-        <v>6.86</v>
+        <v>7.029</v>
       </c>
       <c r="AB288" t="n">
-        <v>20.29</v>
+        <v>20.491</v>
       </c>
       <c r="AC288" t="n">
-        <v>19.309</v>
+        <v>18.976</v>
       </c>
       <c r="AD288" t="n">
-        <v>25.627</v>
+        <v>25.352</v>
       </c>
       <c r="AE288" t="n">
-        <v>10.43</v>
+        <v>10.497</v>
       </c>
       <c r="AF288" t="n">
-        <v>24.154</v>
+        <v>23.963</v>
       </c>
       <c r="AG288" t="n">
-        <v>11.925</v>
+        <v>11.787</v>
       </c>
       <c r="AH288" t="n">
-        <v>5.963</v>
+        <v>5.829</v>
       </c>
       <c r="AI288" t="n">
-        <v>2.897</v>
+        <v>2.843</v>
       </c>
       <c r="AJ288" t="n">
-        <v>18.6</v>
+        <v>18.652</v>
       </c>
       <c r="AK288" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="AL288" t="n">
-        <v>-3.2</v>
+        <v>-3.7</v>
       </c>
     </row>
     <row r="289">
@@ -36026,22 +36026,22 @@
         </is>
       </c>
       <c r="E297" t="n">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F297" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G297" t="b">
         <v>1</v>
       </c>
       <c r="H297" t="n">
-        <v>1698.087</v>
+        <v>1706.594</v>
       </c>
       <c r="I297" t="n">
-        <v>7.7327</v>
+        <v>7.505</v>
       </c>
       <c r="J297" t="n">
-        <v>1515.8</v>
+        <v>1519.9</v>
       </c>
       <c r="K297" t="n">
         <v>63</v>
@@ -36062,70 +36062,70 @@
         <v>52</v>
       </c>
       <c r="Q297" t="n">
-        <v>121</v>
+        <v>120.722</v>
       </c>
       <c r="R297" t="n">
-        <v>106.231</v>
+        <v>106.301</v>
       </c>
       <c r="S297" t="n">
-        <v>14.769</v>
+        <v>14.421</v>
       </c>
       <c r="T297" t="n">
-        <v>0.2826</v>
+        <v>0.28201</v>
       </c>
       <c r="U297" t="n">
-        <v>0.15151</v>
+        <v>0.14993</v>
       </c>
       <c r="V297" t="n">
-        <v>84.16</v>
+        <v>84.17</v>
       </c>
       <c r="W297" t="n">
-        <v>73.94</v>
+        <v>74.18000000000001</v>
       </c>
       <c r="X297" t="n">
-        <v>0.7894</v>
+        <v>0.7955</v>
       </c>
       <c r="Y297" t="n">
-        <v>27.391</v>
+        <v>27.308</v>
       </c>
       <c r="Z297" t="n">
-        <v>58.361</v>
+        <v>58.601</v>
       </c>
       <c r="AA297" t="n">
-        <v>10.572</v>
+        <v>10.627</v>
       </c>
       <c r="AB297" t="n">
-        <v>27.218</v>
+        <v>27.276</v>
       </c>
       <c r="AC297" t="n">
-        <v>18.808</v>
+        <v>18.925</v>
       </c>
       <c r="AD297" t="n">
-        <v>24.227</v>
+        <v>24.234</v>
       </c>
       <c r="AE297" t="n">
-        <v>9.965</v>
+        <v>9.948</v>
       </c>
       <c r="AF297" t="n">
-        <v>24.62</v>
+        <v>24.698</v>
       </c>
       <c r="AG297" t="n">
-        <v>15.278</v>
+        <v>15.156</v>
       </c>
       <c r="AH297" t="n">
-        <v>6.528</v>
+        <v>6.562</v>
       </c>
       <c r="AI297" t="n">
-        <v>2.287</v>
+        <v>2.292</v>
       </c>
       <c r="AJ297" t="n">
-        <v>16.032</v>
+        <v>16.308</v>
       </c>
       <c r="AK297" t="n">
-        <v>2.2</v>
+        <v>2.6</v>
       </c>
       <c r="AL297" t="n">
-        <v>9.9</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="298">
@@ -41186,22 +41186,22 @@
         </is>
       </c>
       <c r="E340" t="n">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F340" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G340" t="b">
         <v>1</v>
       </c>
       <c r="H340" t="n">
-        <v>1659.004</v>
+        <v>1650.496</v>
       </c>
       <c r="I340" t="n">
-        <v>2.095</v>
+        <v>2.3186</v>
       </c>
       <c r="J340" t="n">
-        <v>1550.5</v>
+        <v>1554.5</v>
       </c>
       <c r="K340" t="n">
         <v>82</v>
@@ -41222,70 +41222,70 @@
         <v>78</v>
       </c>
       <c r="Q340" t="n">
-        <v>112.335</v>
+        <v>111.921</v>
       </c>
       <c r="R340" t="n">
-        <v>101.819</v>
+        <v>102.22</v>
       </c>
       <c r="S340" t="n">
-        <v>10.517</v>
+        <v>9.701000000000001</v>
       </c>
       <c r="T340" t="n">
-        <v>0.34245</v>
+        <v>0.34105</v>
       </c>
       <c r="U340" t="n">
-        <v>0.14448</v>
+        <v>0.14454</v>
       </c>
       <c r="V340" t="n">
-        <v>77.73</v>
+        <v>77.61</v>
       </c>
       <c r="W340" t="n">
-        <v>70.44</v>
+        <v>70.91</v>
       </c>
       <c r="X340" t="n">
-        <v>0.6795</v>
+        <v>0.6514</v>
       </c>
       <c r="Y340" t="n">
-        <v>27.608</v>
+        <v>27.399</v>
       </c>
       <c r="Z340" t="n">
-        <v>62.773</v>
+        <v>62.725</v>
       </c>
       <c r="AA340" t="n">
-        <v>7.328</v>
+        <v>7.07</v>
       </c>
       <c r="AB340" t="n">
-        <v>21.338</v>
+        <v>21.209</v>
       </c>
       <c r="AC340" t="n">
-        <v>15.186</v>
+        <v>15.745</v>
       </c>
       <c r="AD340" t="n">
-        <v>22.265</v>
+        <v>22.645</v>
       </c>
       <c r="AE340" t="n">
-        <v>13.417</v>
+        <v>13.397</v>
       </c>
       <c r="AF340" t="n">
-        <v>25.794</v>
+        <v>25.93</v>
       </c>
       <c r="AG340" t="n">
-        <v>11.446</v>
+        <v>11.277</v>
       </c>
       <c r="AH340" t="n">
-        <v>6.068</v>
+        <v>6.02</v>
       </c>
       <c r="AI340" t="n">
-        <v>3.865</v>
+        <v>3.776</v>
       </c>
       <c r="AJ340" t="n">
-        <v>17.312</v>
+        <v>17.488</v>
       </c>
       <c r="AK340" t="n">
-        <v>9.199999999999999</v>
+        <v>4.8</v>
       </c>
       <c r="AL340" t="n">
-        <v>8.800000000000001</v>
+        <v>8</v>
       </c>
     </row>
     <row r="341">

</xml_diff>

<commit_message>
Update team snapshot (2026-03-28)
</commit_message>
<xml_diff>
--- a/team_snapshot_2026.xlsx
+++ b/team_snapshot_2026.xlsx
@@ -986,22 +986,22 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="F5" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G5" t="b">
         <v>1</v>
       </c>
       <c r="H5" t="n">
-        <v>1985.69</v>
+        <v>1972.781</v>
       </c>
       <c r="I5" t="n">
-        <v>-1.3006</v>
+        <v>-1.1118</v>
       </c>
       <c r="J5" t="n">
-        <v>1777.2</v>
+        <v>1782.7</v>
       </c>
       <c r="K5" t="n">
         <v>18</v>
@@ -1022,70 +1022,70 @@
         <v>18</v>
       </c>
       <c r="Q5" t="n">
-        <v>122.085</v>
+        <v>121.534</v>
       </c>
       <c r="R5" t="n">
-        <v>109.744</v>
+        <v>110.466</v>
       </c>
       <c r="S5" t="n">
-        <v>12.341</v>
+        <v>11.068</v>
       </c>
       <c r="T5" t="n">
-        <v>0.28781</v>
+        <v>0.28909</v>
       </c>
       <c r="U5" t="n">
-        <v>0.13149</v>
+        <v>0.12988</v>
       </c>
       <c r="V5" t="n">
-        <v>91.59999999999999</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="W5" t="n">
-        <v>82.39</v>
+        <v>82.8</v>
       </c>
       <c r="X5" t="n">
-        <v>0.7374000000000001</v>
+        <v>0.709</v>
       </c>
       <c r="Y5" t="n">
-        <v>30.35</v>
+        <v>30.162</v>
       </c>
       <c r="Z5" t="n">
-        <v>66.074</v>
+        <v>66.164</v>
       </c>
       <c r="AA5" t="n">
-        <v>12.843</v>
+        <v>12.837</v>
       </c>
       <c r="AB5" t="n">
-        <v>35.318</v>
+        <v>35.684</v>
       </c>
       <c r="AC5" t="n">
-        <v>18.091</v>
+        <v>17.963</v>
       </c>
       <c r="AD5" t="n">
-        <v>23.696</v>
+        <v>23.416</v>
       </c>
       <c r="AE5" t="n">
-        <v>11.318</v>
+        <v>11.255</v>
       </c>
       <c r="AF5" t="n">
-        <v>27.599</v>
+        <v>27.353</v>
       </c>
       <c r="AG5" t="n">
-        <v>16.45</v>
+        <v>16.297</v>
       </c>
       <c r="AH5" t="n">
-        <v>6.424</v>
+        <v>6.361</v>
       </c>
       <c r="AI5" t="n">
-        <v>5.117</v>
+        <v>4.971</v>
       </c>
       <c r="AJ5" t="n">
-        <v>18.666</v>
+        <v>18.66</v>
       </c>
       <c r="AK5" t="n">
-        <v>9.199999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="AL5" t="n">
-        <v>9.6</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="6">
@@ -7346,22 +7346,22 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="F58" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G58" t="b">
         <v>1</v>
       </c>
       <c r="H58" t="n">
-        <v>2068.556</v>
+        <v>2093.053</v>
       </c>
       <c r="I58" t="n">
-        <v>6.1349</v>
+        <v>5.7678</v>
       </c>
       <c r="J58" t="n">
-        <v>1675.6</v>
+        <v>1680.4</v>
       </c>
       <c r="K58" t="n">
         <v>11</v>
@@ -7382,70 +7382,70 @@
         <v>10</v>
       </c>
       <c r="Q58" t="n">
-        <v>116.645</v>
+        <v>116.297</v>
       </c>
       <c r="R58" t="n">
-        <v>97.91500000000001</v>
+        <v>98.047</v>
       </c>
       <c r="S58" t="n">
-        <v>18.73</v>
+        <v>18.25</v>
       </c>
       <c r="T58" t="n">
-        <v>0.30311</v>
+        <v>0.29954</v>
       </c>
       <c r="U58" t="n">
-        <v>0.16219</v>
+        <v>0.16135</v>
       </c>
       <c r="V58" t="n">
-        <v>77.45999999999999</v>
+        <v>77.14</v>
       </c>
       <c r="W58" t="n">
-        <v>64.98999999999999</v>
+        <v>64.98</v>
       </c>
       <c r="X58" t="n">
-        <v>0.8622</v>
+        <v>0.8659</v>
       </c>
       <c r="Y58" t="n">
-        <v>28.207</v>
+        <v>28.103</v>
       </c>
       <c r="Z58" t="n">
-        <v>58.478</v>
+        <v>58.33</v>
       </c>
       <c r="AA58" t="n">
-        <v>8.220000000000001</v>
+        <v>8.249000000000001</v>
       </c>
       <c r="AB58" t="n">
-        <v>23.697</v>
+        <v>23.602</v>
       </c>
       <c r="AC58" t="n">
-        <v>12.829</v>
+        <v>12.682</v>
       </c>
       <c r="AD58" t="n">
-        <v>17.721</v>
+        <v>17.636</v>
       </c>
       <c r="AE58" t="n">
-        <v>10.642</v>
+        <v>10.479</v>
       </c>
       <c r="AF58" t="n">
-        <v>24.036</v>
+        <v>24.027</v>
       </c>
       <c r="AG58" t="n">
-        <v>18.397</v>
+        <v>18.471</v>
       </c>
       <c r="AH58" t="n">
-        <v>6.89</v>
+        <v>6.927</v>
       </c>
       <c r="AI58" t="n">
-        <v>5.138</v>
+        <v>5.169</v>
       </c>
       <c r="AJ58" t="n">
-        <v>18.127</v>
+        <v>18.107</v>
       </c>
       <c r="AK58" t="n">
-        <v>9.6</v>
+        <v>5.4</v>
       </c>
       <c r="AL58" t="n">
-        <v>8.1</v>
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="59">
@@ -9506,22 +9506,22 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="F76" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G76" t="b">
         <v>1</v>
       </c>
       <c r="H76" t="n">
-        <v>2203.313</v>
+        <v>2216.567</v>
       </c>
       <c r="I76" t="n">
-        <v>3.7385</v>
+        <v>3.7533</v>
       </c>
       <c r="J76" t="n">
-        <v>1715.1</v>
+        <v>1720.4</v>
       </c>
       <c r="K76" t="n">
         <v>1</v>
@@ -9542,67 +9542,67 @@
         <v>1</v>
       </c>
       <c r="Q76" t="n">
-        <v>122.582</v>
+        <v>122.717</v>
       </c>
       <c r="R76" t="n">
-        <v>94.554</v>
+        <v>95.46599999999999</v>
       </c>
       <c r="S76" t="n">
-        <v>28.028</v>
+        <v>27.25</v>
       </c>
       <c r="T76" t="n">
-        <v>0.29512</v>
+        <v>0.29604</v>
       </c>
       <c r="U76" t="n">
-        <v>0.15728</v>
+        <v>0.15583</v>
       </c>
       <c r="V76" t="n">
-        <v>81.94</v>
+        <v>81.88</v>
       </c>
       <c r="W76" t="n">
-        <v>63.01</v>
+        <v>63.48</v>
       </c>
       <c r="X76" t="n">
-        <v>0.945</v>
+        <v>0.9464</v>
       </c>
       <c r="Y76" t="n">
-        <v>28.431</v>
+        <v>28.5</v>
       </c>
       <c r="Z76" t="n">
-        <v>58.079</v>
+        <v>58.089</v>
       </c>
       <c r="AA76" t="n">
-        <v>8.898</v>
+        <v>8.776999999999999</v>
       </c>
       <c r="AB76" t="n">
-        <v>25.732</v>
+        <v>25.357</v>
       </c>
       <c r="AC76" t="n">
-        <v>16.176</v>
+        <v>16.098</v>
       </c>
       <c r="AD76" t="n">
-        <v>22.065</v>
+        <v>22.125</v>
       </c>
       <c r="AE76" t="n">
-        <v>11.559</v>
+        <v>11.598</v>
       </c>
       <c r="AF76" t="n">
-        <v>27.25</v>
+        <v>27.223</v>
       </c>
       <c r="AG76" t="n">
-        <v>16.78</v>
+        <v>16.643</v>
       </c>
       <c r="AH76" t="n">
-        <v>7.559</v>
+        <v>7.455</v>
       </c>
       <c r="AI76" t="n">
-        <v>3.285</v>
+        <v>3.339</v>
       </c>
       <c r="AJ76" t="n">
-        <v>15.523</v>
+        <v>15.438</v>
       </c>
       <c r="AK76" t="n">
-        <v>9.199999999999999</v>
+        <v>10</v>
       </c>
       <c r="AL76" t="n">
         <v>16.5</v>
@@ -15746,22 +15746,22 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="F128" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G128" t="b">
         <v>1</v>
       </c>
       <c r="H128" t="n">
-        <v>2057.221</v>
+        <v>2022.773</v>
       </c>
       <c r="I128" t="n">
-        <v>1.8048</v>
+        <v>1.7144</v>
       </c>
       <c r="J128" t="n">
-        <v>1720.3</v>
+        <v>1721.4</v>
       </c>
       <c r="K128" t="n">
         <v>6</v>
@@ -15782,70 +15782,70 @@
         <v>6</v>
       </c>
       <c r="Q128" t="n">
-        <v>119.437</v>
+        <v>118.569</v>
       </c>
       <c r="R128" t="n">
-        <v>95.352</v>
+        <v>96.009</v>
       </c>
       <c r="S128" t="n">
-        <v>24.085</v>
+        <v>22.56</v>
       </c>
       <c r="T128" t="n">
-        <v>0.32237</v>
+        <v>0.32424</v>
       </c>
       <c r="U128" t="n">
-        <v>0.14503</v>
+        <v>0.149</v>
       </c>
       <c r="V128" t="n">
-        <v>82.52</v>
+        <v>81.84</v>
       </c>
       <c r="W128" t="n">
-        <v>65.31999999999999</v>
+        <v>65.69</v>
       </c>
       <c r="X128" t="n">
-        <v>0.8069</v>
+        <v>0.7786999999999999</v>
       </c>
       <c r="Y128" t="n">
-        <v>29.379</v>
+        <v>29.409</v>
       </c>
       <c r="Z128" t="n">
-        <v>60.586</v>
+        <v>60.531</v>
       </c>
       <c r="AA128" t="n">
-        <v>9.138</v>
+        <v>9.068</v>
       </c>
       <c r="AB128" t="n">
-        <v>23.834</v>
+        <v>23.745</v>
       </c>
       <c r="AC128" t="n">
-        <v>14.021</v>
+        <v>13.833</v>
       </c>
       <c r="AD128" t="n">
-        <v>20.662</v>
+        <v>20.451</v>
       </c>
       <c r="AE128" t="n">
-        <v>10.821</v>
+        <v>11.006</v>
       </c>
       <c r="AF128" t="n">
-        <v>22.69</v>
+        <v>22.838</v>
       </c>
       <c r="AG128" t="n">
-        <v>17.331</v>
+        <v>17.489</v>
       </c>
       <c r="AH128" t="n">
-        <v>9.021000000000001</v>
+        <v>8.867000000000001</v>
       </c>
       <c r="AI128" t="n">
-        <v>2.676</v>
+        <v>2.838</v>
       </c>
       <c r="AJ128" t="n">
-        <v>15.917</v>
+        <v>16.119</v>
       </c>
       <c r="AK128" t="n">
-        <v>24.4</v>
+        <v>11.8</v>
       </c>
       <c r="AL128" t="n">
-        <v>12.4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="129">
@@ -20666,22 +20666,22 @@
         </is>
       </c>
       <c r="E169" t="n">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="F169" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G169" t="b">
         <v>1</v>
       </c>
       <c r="H169" t="n">
-        <v>2180.38</v>
+        <v>2193.288</v>
       </c>
       <c r="I169" t="n">
-        <v>5.8798</v>
+        <v>5.6231</v>
       </c>
       <c r="J169" t="n">
-        <v>1779.7</v>
+        <v>1785.2</v>
       </c>
       <c r="K169" t="n">
         <v>3</v>
@@ -20702,70 +20702,70 @@
         <v>2</v>
       </c>
       <c r="Q169" t="n">
-        <v>121.931</v>
+        <v>122.06</v>
       </c>
       <c r="R169" t="n">
-        <v>97.663</v>
+        <v>98.041</v>
       </c>
       <c r="S169" t="n">
-        <v>24.268</v>
+        <v>24.02</v>
       </c>
       <c r="T169" t="n">
-        <v>0.25601</v>
+        <v>0.25685</v>
       </c>
       <c r="U169" t="n">
-        <v>0.16069</v>
+        <v>0.15936</v>
       </c>
       <c r="V169" t="n">
-        <v>87.5</v>
+        <v>87.53</v>
       </c>
       <c r="W169" t="n">
-        <v>69.59999999999999</v>
+        <v>69.83</v>
       </c>
       <c r="X169" t="n">
-        <v>0.9172</v>
+        <v>0.9194</v>
       </c>
       <c r="Y169" t="n">
-        <v>30.717</v>
+        <v>30.771</v>
       </c>
       <c r="Z169" t="n">
-        <v>59.869</v>
+        <v>60.066</v>
       </c>
       <c r="AA169" t="n">
-        <v>9.097</v>
+        <v>9.214</v>
       </c>
       <c r="AB169" t="n">
-        <v>24.766</v>
+        <v>24.852</v>
       </c>
       <c r="AC169" t="n">
-        <v>17.186</v>
+        <v>16.988</v>
       </c>
       <c r="AD169" t="n">
-        <v>23.055</v>
+        <v>22.954</v>
       </c>
       <c r="AE169" t="n">
-        <v>9.814</v>
+        <v>9.912000000000001</v>
       </c>
       <c r="AF169" t="n">
-        <v>28.186</v>
+        <v>28.328</v>
       </c>
       <c r="AG169" t="n">
-        <v>18.924</v>
+        <v>19.019</v>
       </c>
       <c r="AH169" t="n">
-        <v>5.586</v>
+        <v>5.557</v>
       </c>
       <c r="AI169" t="n">
-        <v>6.103</v>
+        <v>6.147</v>
       </c>
       <c r="AJ169" t="n">
-        <v>15.317</v>
+        <v>15.222</v>
       </c>
       <c r="AK169" t="n">
-        <v>8.6</v>
+        <v>10.4</v>
       </c>
       <c r="AL169" t="n">
-        <v>7.5</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="170">
@@ -20786,22 +20786,22 @@
         </is>
       </c>
       <c r="E170" t="n">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="F170" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G170" t="b">
         <v>1</v>
       </c>
       <c r="H170" t="n">
-        <v>2045.301</v>
+        <v>2020.805</v>
       </c>
       <c r="I170" t="n">
-        <v>-0.0252</v>
+        <v>-0.0373</v>
       </c>
       <c r="J170" t="n">
-        <v>1733.5</v>
+        <v>1741.2</v>
       </c>
       <c r="K170" t="n">
         <v>9</v>
@@ -20822,70 +20822,70 @@
         <v>11</v>
       </c>
       <c r="Q170" t="n">
-        <v>117.697</v>
+        <v>117.077</v>
       </c>
       <c r="R170" t="n">
-        <v>101.519</v>
+        <v>101.694</v>
       </c>
       <c r="S170" t="n">
-        <v>16.178</v>
+        <v>15.383</v>
       </c>
       <c r="T170" t="n">
-        <v>0.29109</v>
+        <v>0.29273</v>
       </c>
       <c r="U170" t="n">
-        <v>0.16361</v>
+        <v>0.1629</v>
       </c>
       <c r="V170" t="n">
-        <v>79.23999999999999</v>
+        <v>78.66</v>
       </c>
       <c r="W170" t="n">
-        <v>68.39</v>
+        <v>68.33</v>
       </c>
       <c r="X170" t="n">
-        <v>0.796</v>
+        <v>0.7647</v>
       </c>
       <c r="Y170" t="n">
-        <v>27.719</v>
+        <v>27.56</v>
       </c>
       <c r="Z170" t="n">
-        <v>58.118</v>
+        <v>58.142</v>
       </c>
       <c r="AA170" t="n">
-        <v>7.911</v>
+        <v>7.739</v>
       </c>
       <c r="AB170" t="n">
-        <v>21.571</v>
+        <v>21.325</v>
       </c>
       <c r="AC170" t="n">
-        <v>16.01</v>
+        <v>15.917</v>
       </c>
       <c r="AD170" t="n">
-        <v>20.923</v>
+        <v>20.832</v>
       </c>
       <c r="AE170" t="n">
-        <v>11.029</v>
+        <v>11.102</v>
       </c>
       <c r="AF170" t="n">
-        <v>26.427</v>
+        <v>26.397</v>
       </c>
       <c r="AG170" t="n">
-        <v>18.707</v>
+        <v>18.466</v>
       </c>
       <c r="AH170" t="n">
-        <v>5.34</v>
+        <v>5.377</v>
       </c>
       <c r="AI170" t="n">
-        <v>4.213</v>
+        <v>4.161</v>
       </c>
       <c r="AJ170" t="n">
-        <v>16.128</v>
+        <v>16.133</v>
       </c>
       <c r="AK170" t="n">
-        <v>4.6</v>
+        <v>3</v>
       </c>
       <c r="AL170" t="n">
-        <v>4.6</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="171">
@@ -33146,22 +33146,22 @@
         </is>
       </c>
       <c r="E273" t="n">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="F273" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G273" t="b">
         <v>1</v>
       </c>
       <c r="H273" t="n">
-        <v>2014.742</v>
+        <v>2001.488</v>
       </c>
       <c r="I273" t="n">
-        <v>5.7703</v>
+        <v>5.8981</v>
       </c>
       <c r="J273" t="n">
-        <v>1698.7</v>
+        <v>1705.8</v>
       </c>
       <c r="K273" t="n">
         <v>17</v>
@@ -33182,70 +33182,70 @@
         <v>16</v>
       </c>
       <c r="Q273" t="n">
-        <v>113.755</v>
+        <v>114.005</v>
       </c>
       <c r="R273" t="n">
-        <v>97.798</v>
+        <v>98.755</v>
       </c>
       <c r="S273" t="n">
-        <v>15.957</v>
+        <v>15.25</v>
       </c>
       <c r="T273" t="n">
-        <v>0.31722</v>
+        <v>0.31974</v>
       </c>
       <c r="U273" t="n">
-        <v>0.1451</v>
+        <v>0.14281</v>
       </c>
       <c r="V273" t="n">
-        <v>80.98999999999999</v>
+        <v>80.88</v>
       </c>
       <c r="W273" t="n">
-        <v>69.33</v>
+        <v>69.72</v>
       </c>
       <c r="X273" t="n">
-        <v>0.8345</v>
+        <v>0.8056</v>
       </c>
       <c r="Y273" t="n">
-        <v>27.779</v>
+        <v>27.845</v>
       </c>
       <c r="Z273" t="n">
-        <v>61.172</v>
+        <v>61.315</v>
       </c>
       <c r="AA273" t="n">
-        <v>6.931</v>
+        <v>7.146</v>
       </c>
       <c r="AB273" t="n">
-        <v>20.786</v>
+        <v>21.206</v>
       </c>
       <c r="AC273" t="n">
-        <v>18.428</v>
+        <v>17.99</v>
       </c>
       <c r="AD273" t="n">
-        <v>25.386</v>
+        <v>24.863</v>
       </c>
       <c r="AE273" t="n">
-        <v>11.538</v>
+        <v>11.504</v>
       </c>
       <c r="AF273" t="n">
-        <v>25.179</v>
+        <v>24.841</v>
       </c>
       <c r="AG273" t="n">
-        <v>15.924</v>
+        <v>16.073</v>
       </c>
       <c r="AH273" t="n">
-        <v>7.607</v>
+        <v>7.618</v>
       </c>
       <c r="AI273" t="n">
-        <v>5.055</v>
+        <v>4.96</v>
       </c>
       <c r="AJ273" t="n">
-        <v>17.034</v>
+        <v>17.154</v>
       </c>
       <c r="AK273" t="n">
-        <v>14.2</v>
+        <v>10.6</v>
       </c>
       <c r="AL273" t="n">
-        <v>11</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="274">
@@ -34586,22 +34586,22 @@
         </is>
       </c>
       <c r="E285" t="n">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="F285" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G285" t="b">
         <v>1</v>
       </c>
       <c r="H285" t="n">
-        <v>1944.981</v>
+        <v>1979.428</v>
       </c>
       <c r="I285" t="n">
-        <v>-1.2526</v>
+        <v>-0.9851</v>
       </c>
       <c r="J285" t="n">
-        <v>1724</v>
+        <v>1727</v>
       </c>
       <c r="K285" t="n">
         <v>16</v>
@@ -34622,70 +34622,70 @@
         <v>20</v>
       </c>
       <c r="Q285" t="n">
-        <v>117.137</v>
+        <v>116.892</v>
       </c>
       <c r="R285" t="n">
-        <v>102.163</v>
+        <v>101.668</v>
       </c>
       <c r="S285" t="n">
-        <v>14.975</v>
+        <v>15.224</v>
       </c>
       <c r="T285" t="n">
-        <v>0.36076</v>
+        <v>0.35992</v>
       </c>
       <c r="U285" t="n">
-        <v>0.16454</v>
+        <v>0.16499</v>
       </c>
       <c r="V285" t="n">
-        <v>79.40000000000001</v>
+        <v>79.27</v>
       </c>
       <c r="W285" t="n">
-        <v>69.09</v>
+        <v>68.8</v>
       </c>
       <c r="X285" t="n">
-        <v>0.6889</v>
+        <v>0.6974</v>
       </c>
       <c r="Y285" t="n">
-        <v>28.301</v>
+        <v>28.043</v>
       </c>
       <c r="Z285" t="n">
-        <v>61.364</v>
+        <v>61.016</v>
       </c>
       <c r="AA285" t="n">
-        <v>6.768</v>
+        <v>6.651</v>
       </c>
       <c r="AB285" t="n">
-        <v>20.011</v>
+        <v>19.974</v>
       </c>
       <c r="AC285" t="n">
-        <v>15.757</v>
+        <v>15.825</v>
       </c>
       <c r="AD285" t="n">
-        <v>22.793</v>
+        <v>22.992</v>
       </c>
       <c r="AE285" t="n">
-        <v>14.756</v>
+        <v>14.493</v>
       </c>
       <c r="AF285" t="n">
-        <v>25.646</v>
+        <v>25.28</v>
       </c>
       <c r="AG285" t="n">
-        <v>16.779</v>
+        <v>16.798</v>
       </c>
       <c r="AH285" t="n">
-        <v>7.347</v>
+        <v>7.358</v>
       </c>
       <c r="AI285" t="n">
-        <v>3.614</v>
+        <v>3.467</v>
       </c>
       <c r="AJ285" t="n">
-        <v>17.812</v>
+        <v>17.696</v>
       </c>
       <c r="AK285" t="n">
-        <v>5.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="AL285" t="n">
-        <v>6.8</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="286">

</xml_diff>

<commit_message>
Update team snapshot (2026-03-29)
</commit_message>
<xml_diff>
--- a/team_snapshot_2026.xlsx
+++ b/team_snapshot_2026.xlsx
@@ -1826,22 +1826,22 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F12" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G12" t="b">
         <v>1</v>
       </c>
       <c r="H12" t="n">
-        <v>2286.821</v>
+        <v>2296.897</v>
       </c>
       <c r="I12" t="n">
-        <v>6.212</v>
+        <v>6.07</v>
       </c>
       <c r="J12" t="n">
-        <v>1773.8</v>
+        <v>1775.1</v>
       </c>
       <c r="K12" t="n">
         <v>2</v>
@@ -1862,70 +1862,70 @@
         <v>3</v>
       </c>
       <c r="Q12" t="n">
-        <v>122.042</v>
+        <v>122.029</v>
       </c>
       <c r="R12" t="n">
-        <v>97.27200000000001</v>
+        <v>97.306</v>
       </c>
       <c r="S12" t="n">
-        <v>24.77</v>
+        <v>24.724</v>
       </c>
       <c r="T12" t="n">
-        <v>0.29313</v>
+        <v>0.29298</v>
       </c>
       <c r="U12" t="n">
-        <v>0.15046</v>
+        <v>0.14866</v>
       </c>
       <c r="V12" t="n">
-        <v>86.84999999999999</v>
+        <v>86.45</v>
       </c>
       <c r="W12" t="n">
-        <v>69.06999999999999</v>
+        <v>68.79000000000001</v>
       </c>
       <c r="X12" t="n">
-        <v>0.9463</v>
+        <v>0.9477</v>
       </c>
       <c r="Y12" t="n">
-        <v>30.582</v>
+        <v>30.426</v>
       </c>
       <c r="Z12" t="n">
-        <v>60.605</v>
+        <v>60.537</v>
       </c>
       <c r="AA12" t="n">
-        <v>5.886</v>
+        <v>5.863</v>
       </c>
       <c r="AB12" t="n">
-        <v>15.975</v>
+        <v>15.994</v>
       </c>
       <c r="AC12" t="n">
-        <v>19.796</v>
+        <v>19.738</v>
       </c>
       <c r="AD12" t="n">
-        <v>27.051</v>
+        <v>26.813</v>
       </c>
       <c r="AE12" t="n">
-        <v>12.176</v>
+        <v>12.145</v>
       </c>
       <c r="AF12" t="n">
-        <v>28.806</v>
+        <v>28.779</v>
       </c>
       <c r="AG12" t="n">
-        <v>16.744</v>
+        <v>16.674</v>
       </c>
       <c r="AH12" t="n">
-        <v>7.35</v>
+        <v>7.302</v>
       </c>
       <c r="AI12" t="n">
-        <v>4.369</v>
+        <v>4.269</v>
       </c>
       <c r="AJ12" t="n">
-        <v>15.839</v>
+        <v>15.779</v>
       </c>
       <c r="AK12" t="n">
-        <v>14.8</v>
+        <v>17.4</v>
       </c>
       <c r="AL12" t="n">
-        <v>15.2</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13">
@@ -14906,22 +14906,22 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F121" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G121" t="b">
         <v>1</v>
       </c>
       <c r="H121" t="n">
-        <v>2033.06</v>
+        <v>2043.215</v>
       </c>
       <c r="I121" t="n">
-        <v>6.6485</v>
+        <v>6.515</v>
       </c>
       <c r="J121" t="n">
-        <v>1730.7</v>
+        <v>1722.8</v>
       </c>
       <c r="K121" t="n">
         <v>7</v>
@@ -14942,70 +14942,70 @@
         <v>8</v>
       </c>
       <c r="Q121" t="n">
-        <v>125.389</v>
+        <v>125.713</v>
       </c>
       <c r="R121" t="n">
-        <v>102.649</v>
+        <v>102.946</v>
       </c>
       <c r="S121" t="n">
-        <v>22.739</v>
+        <v>22.766</v>
       </c>
       <c r="T121" t="n">
-        <v>0.32365</v>
+        <v>0.32713</v>
       </c>
       <c r="U121" t="n">
-        <v>0.12572</v>
+        <v>0.12684</v>
       </c>
       <c r="V121" t="n">
-        <v>84</v>
+        <v>83.7</v>
       </c>
       <c r="W121" t="n">
-        <v>68.84999999999999</v>
+        <v>68.62</v>
       </c>
       <c r="X121" t="n">
-        <v>0.7734</v>
+        <v>0.7796</v>
       </c>
       <c r="Y121" t="n">
-        <v>28.458</v>
+        <v>28.389</v>
       </c>
       <c r="Z121" t="n">
-        <v>62.187</v>
+        <v>61.844</v>
       </c>
       <c r="AA121" t="n">
-        <v>10.926</v>
+        <v>10.659</v>
       </c>
       <c r="AB121" t="n">
-        <v>31.66</v>
+        <v>31.134</v>
       </c>
       <c r="AC121" t="n">
-        <v>15.878</v>
+        <v>16.071</v>
       </c>
       <c r="AD121" t="n">
-        <v>20.07</v>
+        <v>20.256</v>
       </c>
       <c r="AE121" t="n">
-        <v>12.501</v>
+        <v>12.639</v>
       </c>
       <c r="AF121" t="n">
-        <v>26.314</v>
+        <v>26.188</v>
       </c>
       <c r="AG121" t="n">
-        <v>14.819</v>
+        <v>14.557</v>
       </c>
       <c r="AH121" t="n">
-        <v>3.858</v>
+        <v>3.934</v>
       </c>
       <c r="AI121" t="n">
-        <v>4.464</v>
+        <v>4.504</v>
       </c>
       <c r="AJ121" t="n">
-        <v>13.466</v>
+        <v>13.386</v>
       </c>
       <c r="AK121" t="n">
-        <v>13.8</v>
+        <v>15</v>
       </c>
       <c r="AL121" t="n">
-        <v>13.6</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="122">
@@ -15626,22 +15626,22 @@
         </is>
       </c>
       <c r="E127" t="n">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F127" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G127" t="b">
         <v>1</v>
       </c>
       <c r="H127" t="n">
-        <v>1916.673</v>
+        <v>1906.518</v>
       </c>
       <c r="I127" t="n">
-        <v>2.8861</v>
+        <v>2.978</v>
       </c>
       <c r="J127" t="n">
-        <v>1722.1</v>
+        <v>1722.5</v>
       </c>
       <c r="K127" t="n">
         <v>25</v>
@@ -15662,70 +15662,70 @@
         <v>27</v>
       </c>
       <c r="Q127" t="n">
-        <v>119.481</v>
+        <v>119.061</v>
       </c>
       <c r="R127" t="n">
-        <v>105.751</v>
+        <v>106.538</v>
       </c>
       <c r="S127" t="n">
-        <v>13.73</v>
+        <v>12.523</v>
       </c>
       <c r="T127" t="n">
-        <v>0.29403</v>
+        <v>0.29664</v>
       </c>
       <c r="U127" t="n">
-        <v>0.14449</v>
+        <v>0.14508</v>
       </c>
       <c r="V127" t="n">
-        <v>74.98999999999999</v>
+        <v>74.42</v>
       </c>
       <c r="W127" t="n">
-        <v>66.18000000000001</v>
+        <v>66.31</v>
       </c>
       <c r="X127" t="n">
-        <v>0.6694</v>
+        <v>0.6437</v>
       </c>
       <c r="Y127" t="n">
-        <v>26.149</v>
+        <v>25.885</v>
       </c>
       <c r="Z127" t="n">
-        <v>53.785</v>
+        <v>53.517</v>
       </c>
       <c r="AA127" t="n">
-        <v>8.151</v>
+        <v>8.211</v>
       </c>
       <c r="AB127" t="n">
-        <v>22.957</v>
+        <v>23.08</v>
       </c>
       <c r="AC127" t="n">
-        <v>14.133</v>
+        <v>14.092</v>
       </c>
       <c r="AD127" t="n">
-        <v>18.356</v>
+        <v>18.264</v>
       </c>
       <c r="AE127" t="n">
-        <v>8.198</v>
+        <v>8.161</v>
       </c>
       <c r="AF127" t="n">
-        <v>19.611</v>
+        <v>19.356</v>
       </c>
       <c r="AG127" t="n">
-        <v>15.446</v>
+        <v>15.299</v>
       </c>
       <c r="AH127" t="n">
-        <v>6.885</v>
+        <v>6.851</v>
       </c>
       <c r="AI127" t="n">
-        <v>2.08</v>
+        <v>2.088</v>
       </c>
       <c r="AJ127" t="n">
-        <v>17.609</v>
+        <v>17.72</v>
       </c>
       <c r="AK127" t="n">
-        <v>4.2</v>
+        <v>-0.4</v>
       </c>
       <c r="AL127" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="128">
@@ -28586,22 +28586,22 @@
         </is>
       </c>
       <c r="E235" t="n">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F235" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G235" t="b">
         <v>1</v>
       </c>
       <c r="H235" t="n">
-        <v>2037.083</v>
+        <v>2027.007</v>
       </c>
       <c r="I235" t="n">
-        <v>-0.5673</v>
+        <v>-0.4418</v>
       </c>
       <c r="J235" t="n">
-        <v>1768.6</v>
+        <v>1782.8</v>
       </c>
       <c r="K235" t="n">
         <v>8</v>
@@ -28622,70 +28622,70 @@
         <v>9</v>
       </c>
       <c r="Q235" t="n">
-        <v>125.585</v>
+        <v>124.674</v>
       </c>
       <c r="R235" t="n">
-        <v>107.86</v>
+        <v>108.154</v>
       </c>
       <c r="S235" t="n">
-        <v>17.726</v>
+        <v>16.52</v>
       </c>
       <c r="T235" t="n">
-        <v>0.31046</v>
+        <v>0.31253</v>
       </c>
       <c r="U235" t="n">
-        <v>0.13408</v>
+        <v>0.13564</v>
       </c>
       <c r="V235" t="n">
-        <v>82.08</v>
+        <v>81.52</v>
       </c>
       <c r="W235" t="n">
-        <v>70.36</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="X235" t="n">
-        <v>0.791</v>
+        <v>0.764</v>
       </c>
       <c r="Y235" t="n">
-        <v>29.895</v>
+        <v>29.705</v>
       </c>
       <c r="Z235" t="n">
-        <v>59.91</v>
+        <v>59.995</v>
       </c>
       <c r="AA235" t="n">
-        <v>9.199</v>
+        <v>9.196999999999999</v>
       </c>
       <c r="AB235" t="n">
-        <v>24.102</v>
+        <v>24.063</v>
       </c>
       <c r="AC235" t="n">
-        <v>12.283</v>
+        <v>12.126</v>
       </c>
       <c r="AD235" t="n">
-        <v>16.447</v>
+        <v>16.311</v>
       </c>
       <c r="AE235" t="n">
-        <v>10.537</v>
+        <v>10.638</v>
       </c>
       <c r="AF235" t="n">
-        <v>22.9</v>
+        <v>22.891</v>
       </c>
       <c r="AG235" t="n">
-        <v>19.315</v>
+        <v>19.195</v>
       </c>
       <c r="AH235" t="n">
-        <v>5.482</v>
+        <v>5.452</v>
       </c>
       <c r="AI235" t="n">
-        <v>2.665</v>
+        <v>2.727</v>
       </c>
       <c r="AJ235" t="n">
-        <v>14.732</v>
+        <v>14.778</v>
       </c>
       <c r="AK235" t="n">
-        <v>12</v>
+        <v>7.6</v>
       </c>
       <c r="AL235" t="n">
-        <v>8.1</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="236">

</xml_diff>

<commit_message>
Update team snapshot (2026-03-30)
</commit_message>
<xml_diff>
--- a/team_snapshot_2026.xlsx
+++ b/team_snapshot_2026.xlsx
@@ -7346,22 +7346,22 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F58" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G58" t="b">
         <v>1</v>
       </c>
       <c r="H58" t="n">
-        <v>2093.053</v>
+        <v>2128.26</v>
       </c>
       <c r="I58" t="n">
-        <v>5.7678</v>
+        <v>5.5371</v>
       </c>
       <c r="J58" t="n">
-        <v>1680.4</v>
+        <v>1685.7</v>
       </c>
       <c r="K58" t="n">
         <v>11</v>
@@ -7382,70 +7382,70 @@
         <v>10</v>
       </c>
       <c r="Q58" t="n">
-        <v>116.297</v>
+        <v>116.505</v>
       </c>
       <c r="R58" t="n">
-        <v>98.047</v>
+        <v>98.72</v>
       </c>
       <c r="S58" t="n">
-        <v>18.25</v>
+        <v>17.786</v>
       </c>
       <c r="T58" t="n">
-        <v>0.29954</v>
+        <v>0.3001</v>
       </c>
       <c r="U58" t="n">
-        <v>0.16135</v>
+        <v>0.16313</v>
       </c>
       <c r="V58" t="n">
-        <v>77.14</v>
+        <v>77.08</v>
       </c>
       <c r="W58" t="n">
-        <v>64.98</v>
+        <v>65.23</v>
       </c>
       <c r="X58" t="n">
-        <v>0.8659</v>
+        <v>0.8694</v>
       </c>
       <c r="Y58" t="n">
-        <v>28.103</v>
+        <v>28.031</v>
       </c>
       <c r="Z58" t="n">
-        <v>58.33</v>
+        <v>58.032</v>
       </c>
       <c r="AA58" t="n">
-        <v>8.249000000000001</v>
+        <v>8.167999999999999</v>
       </c>
       <c r="AB58" t="n">
-        <v>23.602</v>
+        <v>23.334</v>
       </c>
       <c r="AC58" t="n">
-        <v>12.682</v>
+        <v>12.813</v>
       </c>
       <c r="AD58" t="n">
-        <v>17.636</v>
+        <v>17.794</v>
       </c>
       <c r="AE58" t="n">
-        <v>10.479</v>
+        <v>10.496</v>
       </c>
       <c r="AF58" t="n">
-        <v>24.027</v>
+        <v>24.026</v>
       </c>
       <c r="AG58" t="n">
-        <v>18.471</v>
+        <v>18.411</v>
       </c>
       <c r="AH58" t="n">
-        <v>6.927</v>
+        <v>6.822</v>
       </c>
       <c r="AI58" t="n">
-        <v>5.169</v>
+        <v>5.19</v>
       </c>
       <c r="AJ58" t="n">
-        <v>18.107</v>
+        <v>18.038</v>
       </c>
       <c r="AK58" t="n">
-        <v>5.4</v>
+        <v>2.4</v>
       </c>
       <c r="AL58" t="n">
-        <v>9.199999999999999</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="59">
@@ -9506,22 +9506,22 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F76" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G76" t="b">
         <v>1</v>
       </c>
       <c r="H76" t="n">
-        <v>2216.567</v>
+        <v>2181.359</v>
       </c>
       <c r="I76" t="n">
-        <v>3.7533</v>
+        <v>3.8063</v>
       </c>
       <c r="J76" t="n">
-        <v>1720.4</v>
+        <v>1722.7</v>
       </c>
       <c r="K76" t="n">
         <v>1</v>
@@ -9542,70 +9542,70 @@
         <v>1</v>
       </c>
       <c r="Q76" t="n">
-        <v>122.717</v>
+        <v>122.369</v>
       </c>
       <c r="R76" t="n">
-        <v>95.46599999999999</v>
+        <v>95.944</v>
       </c>
       <c r="S76" t="n">
-        <v>27.25</v>
+        <v>26.425</v>
       </c>
       <c r="T76" t="n">
-        <v>0.29604</v>
+        <v>0.30181</v>
       </c>
       <c r="U76" t="n">
-        <v>0.15583</v>
+        <v>0.15329</v>
       </c>
       <c r="V76" t="n">
-        <v>81.88</v>
+        <v>81.55</v>
       </c>
       <c r="W76" t="n">
-        <v>63.48</v>
+        <v>63.71</v>
       </c>
       <c r="X76" t="n">
-        <v>0.9464</v>
+        <v>0.9133</v>
       </c>
       <c r="Y76" t="n">
-        <v>28.5</v>
+        <v>28.47</v>
       </c>
       <c r="Z76" t="n">
-        <v>58.089</v>
+        <v>58.311</v>
       </c>
       <c r="AA76" t="n">
-        <v>8.776999999999999</v>
+        <v>8.679</v>
       </c>
       <c r="AB76" t="n">
-        <v>25.357</v>
+        <v>25.375</v>
       </c>
       <c r="AC76" t="n">
-        <v>16.098</v>
+        <v>15.966</v>
       </c>
       <c r="AD76" t="n">
-        <v>22.125</v>
+        <v>21.932</v>
       </c>
       <c r="AE76" t="n">
-        <v>11.598</v>
+        <v>11.643</v>
       </c>
       <c r="AF76" t="n">
-        <v>27.223</v>
+        <v>26.795</v>
       </c>
       <c r="AG76" t="n">
-        <v>16.643</v>
+        <v>16.652</v>
       </c>
       <c r="AH76" t="n">
-        <v>7.455</v>
+        <v>7.47</v>
       </c>
       <c r="AI76" t="n">
-        <v>3.339</v>
+        <v>3.486</v>
       </c>
       <c r="AJ76" t="n">
-        <v>15.438</v>
+        <v>15.513</v>
       </c>
       <c r="AK76" t="n">
-        <v>10</v>
+        <v>7.4</v>
       </c>
       <c r="AL76" t="n">
-        <v>16.5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="77">
@@ -20666,22 +20666,22 @@
         </is>
       </c>
       <c r="E169" t="n">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F169" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G169" t="b">
         <v>1</v>
       </c>
       <c r="H169" t="n">
-        <v>2193.288</v>
+        <v>2205.153</v>
       </c>
       <c r="I169" t="n">
-        <v>5.6231</v>
+        <v>5.4369</v>
       </c>
       <c r="J169" t="n">
-        <v>1785.2</v>
+        <v>1784.8</v>
       </c>
       <c r="K169" t="n">
         <v>3</v>
@@ -20702,70 +20702,70 @@
         <v>2</v>
       </c>
       <c r="Q169" t="n">
-        <v>122.06</v>
+        <v>122.15</v>
       </c>
       <c r="R169" t="n">
-        <v>98.041</v>
+        <v>97.45699999999999</v>
       </c>
       <c r="S169" t="n">
-        <v>24.02</v>
+        <v>24.693</v>
       </c>
       <c r="T169" t="n">
-        <v>0.25685</v>
+        <v>0.25455</v>
       </c>
       <c r="U169" t="n">
-        <v>0.15936</v>
+        <v>0.15921</v>
       </c>
       <c r="V169" t="n">
-        <v>87.53</v>
+        <v>87.76000000000001</v>
       </c>
       <c r="W169" t="n">
-        <v>69.83</v>
+        <v>69.53</v>
       </c>
       <c r="X169" t="n">
-        <v>0.9194</v>
+        <v>0.9215</v>
       </c>
       <c r="Y169" t="n">
-        <v>30.771</v>
+        <v>30.7</v>
       </c>
       <c r="Z169" t="n">
-        <v>60.066</v>
+        <v>59.897</v>
       </c>
       <c r="AA169" t="n">
-        <v>9.214</v>
+        <v>9.215</v>
       </c>
       <c r="AB169" t="n">
-        <v>24.852</v>
+        <v>24.908</v>
       </c>
       <c r="AC169" t="n">
-        <v>16.988</v>
+        <v>17.349</v>
       </c>
       <c r="AD169" t="n">
-        <v>22.954</v>
+        <v>23.425</v>
       </c>
       <c r="AE169" t="n">
-        <v>9.912000000000001</v>
+        <v>9.831</v>
       </c>
       <c r="AF169" t="n">
-        <v>28.328</v>
+        <v>28.481</v>
       </c>
       <c r="AG169" t="n">
-        <v>19.019</v>
+        <v>19</v>
       </c>
       <c r="AH169" t="n">
-        <v>5.557</v>
+        <v>5.582</v>
       </c>
       <c r="AI169" t="n">
-        <v>6.147</v>
+        <v>6.195</v>
       </c>
       <c r="AJ169" t="n">
-        <v>15.222</v>
+        <v>15.332</v>
       </c>
       <c r="AK169" t="n">
-        <v>10.4</v>
+        <v>16.4</v>
       </c>
       <c r="AL169" t="n">
-        <v>9.300000000000001</v>
+        <v>11.6</v>
       </c>
     </row>
     <row r="170">
@@ -34586,22 +34586,22 @@
         </is>
       </c>
       <c r="E285" t="n">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F285" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G285" t="b">
         <v>1</v>
       </c>
       <c r="H285" t="n">
-        <v>1979.428</v>
+        <v>1967.563</v>
       </c>
       <c r="I285" t="n">
-        <v>-0.9851</v>
+        <v>-0.6001</v>
       </c>
       <c r="J285" t="n">
-        <v>1727</v>
+        <v>1731.4</v>
       </c>
       <c r="K285" t="n">
         <v>16</v>
@@ -34622,70 +34622,70 @@
         <v>20</v>
       </c>
       <c r="Q285" t="n">
-        <v>116.892</v>
+        <v>115.778</v>
       </c>
       <c r="R285" t="n">
-        <v>101.668</v>
+        <v>102.752</v>
       </c>
       <c r="S285" t="n">
-        <v>15.224</v>
+        <v>13.026</v>
       </c>
       <c r="T285" t="n">
-        <v>0.35992</v>
+        <v>0.36318</v>
       </c>
       <c r="U285" t="n">
-        <v>0.16499</v>
+        <v>0.16351</v>
       </c>
       <c r="V285" t="n">
-        <v>79.27</v>
+        <v>78.69</v>
       </c>
       <c r="W285" t="n">
-        <v>68.8</v>
+        <v>69.79000000000001</v>
       </c>
       <c r="X285" t="n">
-        <v>0.6974</v>
+        <v>0.6696</v>
       </c>
       <c r="Y285" t="n">
-        <v>28.043</v>
+        <v>27.964</v>
       </c>
       <c r="Z285" t="n">
-        <v>61.016</v>
+        <v>61.616</v>
       </c>
       <c r="AA285" t="n">
-        <v>6.651</v>
+        <v>6.607</v>
       </c>
       <c r="AB285" t="n">
-        <v>19.974</v>
+        <v>20.161</v>
       </c>
       <c r="AC285" t="n">
-        <v>15.825</v>
+        <v>15.589</v>
       </c>
       <c r="AD285" t="n">
-        <v>22.992</v>
+        <v>22.759</v>
       </c>
       <c r="AE285" t="n">
-        <v>14.493</v>
+        <v>14.714</v>
       </c>
       <c r="AF285" t="n">
-        <v>25.28</v>
+        <v>25.304</v>
       </c>
       <c r="AG285" t="n">
-        <v>16.798</v>
+        <v>16.634</v>
       </c>
       <c r="AH285" t="n">
-        <v>7.358</v>
+        <v>7.384</v>
       </c>
       <c r="AI285" t="n">
-        <v>3.467</v>
+        <v>3.446</v>
       </c>
       <c r="AJ285" t="n">
-        <v>17.696</v>
+        <v>17.946</v>
       </c>
       <c r="AK285" t="n">
-        <v>9.199999999999999</v>
+        <v>0.6</v>
       </c>
       <c r="AL285" t="n">
-        <v>5.9</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="286">

</xml_diff>

<commit_message>
Update team snapshot (2026-04-05)
</commit_message>
<xml_diff>
--- a/team_snapshot_2026.xlsx
+++ b/team_snapshot_2026.xlsx
@@ -1826,22 +1826,22 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="F12" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G12" t="b">
         <v>1</v>
       </c>
       <c r="H12" t="n">
-        <v>2296.897</v>
+        <v>2263.872</v>
       </c>
       <c r="I12" t="n">
-        <v>6.07</v>
+        <v>5.9654</v>
       </c>
       <c r="J12" t="n">
-        <v>1775.1</v>
+        <v>1780.1</v>
       </c>
       <c r="K12" t="n">
         <v>2</v>
@@ -1862,70 +1862,70 @@
         <v>3</v>
       </c>
       <c r="Q12" t="n">
-        <v>122.029</v>
+        <v>121.127</v>
       </c>
       <c r="R12" t="n">
-        <v>97.306</v>
+        <v>97.89</v>
       </c>
       <c r="S12" t="n">
-        <v>24.724</v>
+        <v>23.237</v>
       </c>
       <c r="T12" t="n">
-        <v>0.29298</v>
+        <v>0.29255</v>
       </c>
       <c r="U12" t="n">
-        <v>0.14866</v>
+        <v>0.14954</v>
       </c>
       <c r="V12" t="n">
-        <v>86.45</v>
+        <v>86.08</v>
       </c>
       <c r="W12" t="n">
-        <v>68.79000000000001</v>
+        <v>69.51000000000001</v>
       </c>
       <c r="X12" t="n">
-        <v>0.9477</v>
+        <v>0.9177999999999999</v>
       </c>
       <c r="Y12" t="n">
-        <v>30.426</v>
+        <v>30.527</v>
       </c>
       <c r="Z12" t="n">
-        <v>60.537</v>
+        <v>60.817</v>
       </c>
       <c r="AA12" t="n">
-        <v>5.863</v>
+        <v>6.06</v>
       </c>
       <c r="AB12" t="n">
-        <v>15.994</v>
+        <v>16.344</v>
       </c>
       <c r="AC12" t="n">
-        <v>19.738</v>
+        <v>19.526</v>
       </c>
       <c r="AD12" t="n">
-        <v>26.813</v>
+        <v>26.503</v>
       </c>
       <c r="AE12" t="n">
-        <v>12.145</v>
+        <v>12.122</v>
       </c>
       <c r="AF12" t="n">
-        <v>28.779</v>
+        <v>28.796</v>
       </c>
       <c r="AG12" t="n">
-        <v>16.674</v>
+        <v>16.85</v>
       </c>
       <c r="AH12" t="n">
-        <v>7.302</v>
+        <v>7.306</v>
       </c>
       <c r="AI12" t="n">
-        <v>4.269</v>
+        <v>4.249</v>
       </c>
       <c r="AJ12" t="n">
-        <v>15.779</v>
+        <v>15.89</v>
       </c>
       <c r="AK12" t="n">
-        <v>17.4</v>
+        <v>12.8</v>
       </c>
       <c r="AL12" t="n">
-        <v>16</v>
+        <v>11.9</v>
       </c>
     </row>
     <row r="13">
@@ -2666,22 +2666,22 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="F19" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G19" t="b">
         <v>1</v>
       </c>
       <c r="H19" t="n">
-        <v>1853.815</v>
+        <v>1864.699</v>
       </c>
       <c r="I19" t="n">
-        <v>-6.9997</v>
+        <v>-6.7282</v>
       </c>
       <c r="J19" t="n">
-        <v>1745.4</v>
+        <v>1741.8</v>
       </c>
       <c r="K19" t="n">
         <v>38</v>
@@ -2702,70 +2702,70 @@
         <v>38</v>
       </c>
       <c r="Q19" t="n">
-        <v>118.556</v>
+        <v>119.295</v>
       </c>
       <c r="R19" t="n">
-        <v>113.403</v>
+        <v>113.147</v>
       </c>
       <c r="S19" t="n">
-        <v>5.153</v>
+        <v>6.148</v>
       </c>
       <c r="T19" t="n">
-        <v>0.34498</v>
+        <v>0.34229</v>
       </c>
       <c r="U19" t="n">
-        <v>0.14368</v>
+        <v>0.14393</v>
       </c>
       <c r="V19" t="n">
-        <v>82.55</v>
+        <v>82.8</v>
       </c>
       <c r="W19" t="n">
-        <v>78.84</v>
+        <v>78.47</v>
       </c>
       <c r="X19" t="n">
-        <v>0.5592</v>
+        <v>0.5709</v>
       </c>
       <c r="Y19" t="n">
-        <v>27.465</v>
+        <v>27.67</v>
       </c>
       <c r="Z19" t="n">
-        <v>60.036</v>
+        <v>59.889</v>
       </c>
       <c r="AA19" t="n">
-        <v>8.121</v>
+        <v>8.272</v>
       </c>
       <c r="AB19" t="n">
-        <v>24.165</v>
+        <v>24.057</v>
       </c>
       <c r="AC19" t="n">
-        <v>19.497</v>
+        <v>19.184</v>
       </c>
       <c r="AD19" t="n">
-        <v>26.233</v>
+        <v>25.805</v>
       </c>
       <c r="AE19" t="n">
-        <v>11.964</v>
+        <v>11.801</v>
       </c>
       <c r="AF19" t="n">
-        <v>22.397</v>
+        <v>22.299</v>
       </c>
       <c r="AG19" t="n">
-        <v>12.818</v>
+        <v>13.08</v>
       </c>
       <c r="AH19" t="n">
-        <v>7.319</v>
+        <v>7.502</v>
       </c>
       <c r="AI19" t="n">
-        <v>4.157</v>
+        <v>4.161</v>
       </c>
       <c r="AJ19" t="n">
-        <v>17.05</v>
+        <v>16.874</v>
       </c>
       <c r="AK19" t="n">
-        <v>6.2</v>
+        <v>7</v>
       </c>
       <c r="AL19" t="n">
-        <v>1.6</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="20">
@@ -3026,22 +3026,22 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>127</v>
+        <v>152</v>
       </c>
       <c r="F22" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G22" t="b">
         <v>1</v>
       </c>
       <c r="H22" t="n">
-        <v>1667.154</v>
+        <v>1664.088</v>
       </c>
       <c r="I22" t="n">
-        <v>-5.9263</v>
+        <v>-5.3935</v>
       </c>
       <c r="J22" t="n">
-        <v>1727.4</v>
+        <v>1724.7</v>
       </c>
       <c r="K22" t="n">
         <v>49</v>
@@ -3062,70 +3062,70 @@
         <v>50</v>
       </c>
       <c r="Q22" t="n">
-        <v>116.311</v>
+        <v>115.661</v>
       </c>
       <c r="R22" t="n">
-        <v>111.717</v>
+        <v>111.037</v>
       </c>
       <c r="S22" t="n">
-        <v>4.594</v>
+        <v>4.623</v>
       </c>
       <c r="T22" t="n">
-        <v>0.33352</v>
+        <v>0.32183</v>
       </c>
       <c r="U22" t="n">
-        <v>0.16197</v>
+        <v>0.15935</v>
       </c>
       <c r="V22" t="n">
-        <v>81.2</v>
+        <v>80.33</v>
       </c>
       <c r="W22" t="n">
-        <v>77.73</v>
+        <v>76.95</v>
       </c>
       <c r="X22" t="n">
-        <v>0.4792</v>
+        <v>0.4808</v>
       </c>
       <c r="Y22" t="n">
-        <v>28.831</v>
+        <v>28.588</v>
       </c>
       <c r="Z22" t="n">
-        <v>60.707</v>
+        <v>60.27</v>
       </c>
       <c r="AA22" t="n">
-        <v>8.510999999999999</v>
+        <v>8.331</v>
       </c>
       <c r="AB22" t="n">
-        <v>24.088</v>
+        <v>23.893</v>
       </c>
       <c r="AC22" t="n">
-        <v>15.3</v>
+        <v>15.022</v>
       </c>
       <c r="AD22" t="n">
-        <v>20.865</v>
+        <v>20.537</v>
       </c>
       <c r="AE22" t="n">
-        <v>11.496</v>
+        <v>11.048</v>
       </c>
       <c r="AF22" t="n">
-        <v>22.492</v>
+        <v>22.733</v>
       </c>
       <c r="AG22" t="n">
-        <v>15.482</v>
+        <v>15.364</v>
       </c>
       <c r="AH22" t="n">
-        <v>6.413</v>
+        <v>6.279</v>
       </c>
       <c r="AI22" t="n">
-        <v>3.821</v>
+        <v>3.781</v>
       </c>
       <c r="AJ22" t="n">
-        <v>16.486</v>
+        <v>16.21</v>
       </c>
       <c r="AK22" t="n">
-        <v>0.6</v>
+        <v>3</v>
       </c>
       <c r="AL22" t="n">
-        <v>-2.7</v>
+        <v>-1.3</v>
       </c>
     </row>
     <row r="23">
@@ -6986,22 +6986,22 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>127</v>
+        <v>149</v>
       </c>
       <c r="F55" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G55" t="b">
         <v>1</v>
       </c>
       <c r="H55" t="n">
-        <v>1605.175</v>
+        <v>1592.288</v>
       </c>
       <c r="I55" t="n">
-        <v>-4.1723</v>
+        <v>-4.0223</v>
       </c>
       <c r="J55" t="n">
-        <v>1689.7</v>
+        <v>1690.8</v>
       </c>
       <c r="K55" t="n">
         <v>70</v>
@@ -7022,70 +7022,70 @@
         <v>76</v>
       </c>
       <c r="Q55" t="n">
-        <v>114.138</v>
+        <v>113.742</v>
       </c>
       <c r="R55" t="n">
-        <v>113.853</v>
+        <v>113.529</v>
       </c>
       <c r="S55" t="n">
-        <v>0.285</v>
+        <v>0.213</v>
       </c>
       <c r="T55" t="n">
-        <v>0.28499</v>
+        <v>0.28564</v>
       </c>
       <c r="U55" t="n">
-        <v>0.13951</v>
+        <v>0.13875</v>
       </c>
       <c r="V55" t="n">
-        <v>80</v>
+        <v>80.20999999999999</v>
       </c>
       <c r="W55" t="n">
-        <v>79.56999999999999</v>
+        <v>79.86</v>
       </c>
       <c r="X55" t="n">
-        <v>0.5255</v>
+        <v>0.51</v>
       </c>
       <c r="Y55" t="n">
-        <v>28.073</v>
+        <v>27.98</v>
       </c>
       <c r="Z55" t="n">
-        <v>59.858</v>
+        <v>60.26</v>
       </c>
       <c r="AA55" t="n">
-        <v>7.257</v>
+        <v>7.39</v>
       </c>
       <c r="AB55" t="n">
-        <v>20.648</v>
+        <v>21.34</v>
       </c>
       <c r="AC55" t="n">
-        <v>16.974</v>
+        <v>17.29</v>
       </c>
       <c r="AD55" t="n">
-        <v>22.171</v>
+        <v>22.43</v>
       </c>
       <c r="AE55" t="n">
-        <v>9.311999999999999</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="AF55" t="n">
-        <v>23.065</v>
+        <v>23.12</v>
       </c>
       <c r="AG55" t="n">
-        <v>15.671</v>
+        <v>15.63</v>
       </c>
       <c r="AH55" t="n">
-        <v>6.371</v>
+        <v>6.48</v>
       </c>
       <c r="AI55" t="n">
-        <v>3.423</v>
+        <v>3.63</v>
       </c>
       <c r="AJ55" t="n">
-        <v>17.495</v>
+        <v>17.76</v>
       </c>
       <c r="AK55" t="n">
-        <v>-7.2</v>
+        <v>-9.800000000000001</v>
       </c>
       <c r="AL55" t="n">
-        <v>-7.1</v>
+        <v>-5.6</v>
       </c>
     </row>
     <row r="56">
@@ -7346,22 +7346,22 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="F58" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G58" t="b">
         <v>1</v>
       </c>
       <c r="H58" t="n">
-        <v>2128.26</v>
+        <v>2148.21</v>
       </c>
       <c r="I58" t="n">
-        <v>5.5371</v>
+        <v>5.461</v>
       </c>
       <c r="J58" t="n">
-        <v>1685.7</v>
+        <v>1679.5</v>
       </c>
       <c r="K58" t="n">
         <v>11</v>
@@ -7382,70 +7382,70 @@
         <v>10</v>
       </c>
       <c r="Q58" t="n">
-        <v>116.505</v>
+        <v>116.328</v>
       </c>
       <c r="R58" t="n">
-        <v>98.72</v>
+        <v>98.54600000000001</v>
       </c>
       <c r="S58" t="n">
-        <v>17.786</v>
+        <v>17.783</v>
       </c>
       <c r="T58" t="n">
-        <v>0.3001</v>
+        <v>0.29918</v>
       </c>
       <c r="U58" t="n">
-        <v>0.16313</v>
+        <v>0.15954</v>
       </c>
       <c r="V58" t="n">
-        <v>77.08</v>
+        <v>76.91</v>
       </c>
       <c r="W58" t="n">
-        <v>65.23</v>
+        <v>65.08</v>
       </c>
       <c r="X58" t="n">
-        <v>0.8694</v>
+        <v>0.8727</v>
       </c>
       <c r="Y58" t="n">
-        <v>28.031</v>
+        <v>27.857</v>
       </c>
       <c r="Z58" t="n">
-        <v>58.032</v>
+        <v>58.231</v>
       </c>
       <c r="AA58" t="n">
-        <v>8.167999999999999</v>
+        <v>8.307</v>
       </c>
       <c r="AB58" t="n">
-        <v>23.334</v>
+        <v>23.705</v>
       </c>
       <c r="AC58" t="n">
-        <v>12.813</v>
+        <v>12.861</v>
       </c>
       <c r="AD58" t="n">
-        <v>17.794</v>
+        <v>17.739</v>
       </c>
       <c r="AE58" t="n">
-        <v>10.496</v>
+        <v>10.484</v>
       </c>
       <c r="AF58" t="n">
-        <v>24.026</v>
+        <v>24.122</v>
       </c>
       <c r="AG58" t="n">
-        <v>18.411</v>
+        <v>18.278</v>
       </c>
       <c r="AH58" t="n">
-        <v>6.822</v>
+        <v>6.815</v>
       </c>
       <c r="AI58" t="n">
-        <v>5.19</v>
+        <v>5.049</v>
       </c>
       <c r="AJ58" t="n">
-        <v>18.038</v>
+        <v>18.148</v>
       </c>
       <c r="AK58" t="n">
-        <v>2.4</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="AL58" t="n">
-        <v>8.300000000000001</v>
+        <v>6</v>
       </c>
     </row>
     <row r="59">
@@ -7706,22 +7706,22 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>129</v>
+        <v>152</v>
       </c>
       <c r="F61" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G61" t="b">
         <v>1</v>
       </c>
       <c r="H61" t="n">
-        <v>1663.553</v>
+        <v>1657.487</v>
       </c>
       <c r="I61" t="n">
-        <v>-2.2846</v>
+        <v>-2.2458</v>
       </c>
       <c r="J61" t="n">
-        <v>1664.6</v>
+        <v>1664.1</v>
       </c>
       <c r="K61" t="n">
         <v>76</v>
@@ -7742,70 +7742,70 @@
         <v>83</v>
       </c>
       <c r="Q61" t="n">
-        <v>109.303</v>
+        <v>109.345</v>
       </c>
       <c r="R61" t="n">
-        <v>109.715</v>
+        <v>110.038</v>
       </c>
       <c r="S61" t="n">
-        <v>-0.411</v>
+        <v>-0.694</v>
       </c>
       <c r="T61" t="n">
-        <v>0.24848</v>
+        <v>0.24532</v>
       </c>
       <c r="U61" t="n">
-        <v>0.15439</v>
+        <v>0.1514</v>
       </c>
       <c r="V61" t="n">
-        <v>74.97</v>
+        <v>75.13</v>
       </c>
       <c r="W61" t="n">
-        <v>75</v>
+        <v>75.31999999999999</v>
       </c>
       <c r="X61" t="n">
-        <v>0.4637</v>
+        <v>0.4662</v>
       </c>
       <c r="Y61" t="n">
-        <v>26.399</v>
+        <v>26.812</v>
       </c>
       <c r="Z61" t="n">
-        <v>59.103</v>
+        <v>59.357</v>
       </c>
       <c r="AA61" t="n">
-        <v>9.824</v>
+        <v>9.872999999999999</v>
       </c>
       <c r="AB61" t="n">
-        <v>28.559</v>
+        <v>28.543</v>
       </c>
       <c r="AC61" t="n">
-        <v>12.351</v>
+        <v>12.284</v>
       </c>
       <c r="AD61" t="n">
-        <v>16.269</v>
+        <v>16.274</v>
       </c>
       <c r="AE61" t="n">
-        <v>8.331</v>
+        <v>8.291</v>
       </c>
       <c r="AF61" t="n">
-        <v>24.517</v>
+        <v>24.939</v>
       </c>
       <c r="AG61" t="n">
-        <v>15.442</v>
+        <v>15.466</v>
       </c>
       <c r="AH61" t="n">
-        <v>5.762</v>
+        <v>5.661</v>
       </c>
       <c r="AI61" t="n">
-        <v>2.671</v>
+        <v>2.787</v>
       </c>
       <c r="AJ61" t="n">
-        <v>14.394</v>
+        <v>14.697</v>
       </c>
       <c r="AK61" t="n">
-        <v>-5.4</v>
+        <v>-0.2</v>
       </c>
       <c r="AL61" t="n">
-        <v>-3.9</v>
+        <v>-3.6</v>
       </c>
     </row>
     <row r="62">
@@ -14906,22 +14906,22 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="F121" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G121" t="b">
         <v>1</v>
       </c>
       <c r="H121" t="n">
-        <v>2043.215</v>
+        <v>2023.265</v>
       </c>
       <c r="I121" t="n">
-        <v>6.515</v>
+        <v>6.4189</v>
       </c>
       <c r="J121" t="n">
-        <v>1722.8</v>
+        <v>1729.9</v>
       </c>
       <c r="K121" t="n">
         <v>7</v>
@@ -14942,70 +14942,70 @@
         <v>8</v>
       </c>
       <c r="Q121" t="n">
-        <v>125.713</v>
+        <v>124.778</v>
       </c>
       <c r="R121" t="n">
-        <v>102.946</v>
+        <v>103.291</v>
       </c>
       <c r="S121" t="n">
-        <v>22.766</v>
+        <v>21.487</v>
       </c>
       <c r="T121" t="n">
-        <v>0.32713</v>
+        <v>0.3245</v>
       </c>
       <c r="U121" t="n">
-        <v>0.12684</v>
+        <v>0.12675</v>
       </c>
       <c r="V121" t="n">
-        <v>83.7</v>
+        <v>83.05</v>
       </c>
       <c r="W121" t="n">
-        <v>68.62</v>
+        <v>68.77</v>
       </c>
       <c r="X121" t="n">
-        <v>0.7796</v>
+        <v>0.751</v>
       </c>
       <c r="Y121" t="n">
-        <v>28.389</v>
+        <v>28.092</v>
       </c>
       <c r="Z121" t="n">
-        <v>61.844</v>
+        <v>61.713</v>
       </c>
       <c r="AA121" t="n">
-        <v>10.659</v>
+        <v>10.559</v>
       </c>
       <c r="AB121" t="n">
-        <v>31.134</v>
+        <v>31.069</v>
       </c>
       <c r="AC121" t="n">
-        <v>16.071</v>
+        <v>16.123</v>
       </c>
       <c r="AD121" t="n">
-        <v>20.256</v>
+        <v>20.345</v>
       </c>
       <c r="AE121" t="n">
-        <v>12.639</v>
+        <v>12.59</v>
       </c>
       <c r="AF121" t="n">
-        <v>26.188</v>
+        <v>26.421</v>
       </c>
       <c r="AG121" t="n">
-        <v>14.557</v>
+        <v>14.211</v>
       </c>
       <c r="AH121" t="n">
-        <v>3.934</v>
+        <v>3.851</v>
       </c>
       <c r="AI121" t="n">
-        <v>4.504</v>
+        <v>4.552</v>
       </c>
       <c r="AJ121" t="n">
-        <v>13.386</v>
+        <v>13.513</v>
       </c>
       <c r="AK121" t="n">
-        <v>15</v>
+        <v>13.8</v>
       </c>
       <c r="AL121" t="n">
-        <v>12.8</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="122">
@@ -15026,22 +15026,22 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="F122" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G122" t="b">
         <v>1</v>
       </c>
       <c r="H122" t="n">
-        <v>1644.639</v>
+        <v>1633.755</v>
       </c>
       <c r="I122" t="n">
-        <v>2.2958</v>
+        <v>2.516</v>
       </c>
       <c r="J122" t="n">
-        <v>1519.7</v>
+        <v>1530.1</v>
       </c>
       <c r="K122" t="n">
         <v>103</v>
@@ -15062,70 +15062,70 @@
         <v>95</v>
       </c>
       <c r="Q122" t="n">
-        <v>109.747</v>
+        <v>109.523</v>
       </c>
       <c r="R122" t="n">
-        <v>101.285</v>
+        <v>102.581</v>
       </c>
       <c r="S122" t="n">
-        <v>8.462</v>
+        <v>6.941</v>
       </c>
       <c r="T122" t="n">
-        <v>0.25045</v>
+        <v>0.25673</v>
       </c>
       <c r="U122" t="n">
-        <v>0.16263</v>
+        <v>0.16606</v>
       </c>
       <c r="V122" t="n">
-        <v>74.28</v>
+        <v>74.08</v>
       </c>
       <c r="W122" t="n">
-        <v>68.42</v>
+        <v>69.22</v>
       </c>
       <c r="X122" t="n">
-        <v>0.6498</v>
+        <v>0.6239</v>
       </c>
       <c r="Y122" t="n">
-        <v>26.756</v>
+        <v>26.73</v>
       </c>
       <c r="Z122" t="n">
-        <v>57.333</v>
+        <v>57.347</v>
       </c>
       <c r="AA122" t="n">
-        <v>8.714</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="AB122" t="n">
-        <v>24.608</v>
+        <v>24.688</v>
       </c>
       <c r="AC122" t="n">
-        <v>12.692</v>
+        <v>12.466</v>
       </c>
       <c r="AD122" t="n">
-        <v>17.854</v>
+        <v>17.465</v>
       </c>
       <c r="AE122" t="n">
-        <v>8.42</v>
+        <v>8.525</v>
       </c>
       <c r="AF122" t="n">
-        <v>25.538</v>
+        <v>25.132</v>
       </c>
       <c r="AG122" t="n">
-        <v>13.838</v>
+        <v>13.894</v>
       </c>
       <c r="AH122" t="n">
-        <v>5.502</v>
+        <v>5.403</v>
       </c>
       <c r="AI122" t="n">
-        <v>2.27</v>
+        <v>2.291</v>
       </c>
       <c r="AJ122" t="n">
-        <v>17.189</v>
+        <v>17.056</v>
       </c>
       <c r="AK122" t="n">
-        <v>3</v>
+        <v>-2.8</v>
       </c>
       <c r="AL122" t="n">
-        <v>1.5</v>
+        <v>-2.9</v>
       </c>
     </row>
     <row r="123">
@@ -20666,22 +20666,22 @@
         </is>
       </c>
       <c r="E169" t="n">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="F169" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G169" t="b">
         <v>1</v>
       </c>
       <c r="H169" t="n">
-        <v>2205.153</v>
+        <v>2238.177</v>
       </c>
       <c r="I169" t="n">
-        <v>5.4369</v>
+        <v>5.3046</v>
       </c>
       <c r="J169" t="n">
-        <v>1784.8</v>
+        <v>1794.5</v>
       </c>
       <c r="K169" t="n">
         <v>3</v>
@@ -20702,70 +20702,70 @@
         <v>2</v>
       </c>
       <c r="Q169" t="n">
-        <v>122.15</v>
+        <v>122.018</v>
       </c>
       <c r="R169" t="n">
-        <v>97.45699999999999</v>
+        <v>97.477</v>
       </c>
       <c r="S169" t="n">
-        <v>24.693</v>
+        <v>24.541</v>
       </c>
       <c r="T169" t="n">
-        <v>0.25455</v>
+        <v>0.25976</v>
       </c>
       <c r="U169" t="n">
-        <v>0.15921</v>
+        <v>0.16002</v>
       </c>
       <c r="V169" t="n">
-        <v>87.76000000000001</v>
+        <v>87.81</v>
       </c>
       <c r="W169" t="n">
-        <v>69.53</v>
+        <v>69.69</v>
       </c>
       <c r="X169" t="n">
-        <v>0.9215</v>
+        <v>0.9235</v>
       </c>
       <c r="Y169" t="n">
-        <v>30.7</v>
+        <v>30.563</v>
       </c>
       <c r="Z169" t="n">
-        <v>59.897</v>
+        <v>60.267</v>
       </c>
       <c r="AA169" t="n">
-        <v>9.215</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="AB169" t="n">
-        <v>24.908</v>
+        <v>24.648</v>
       </c>
       <c r="AC169" t="n">
-        <v>17.349</v>
+        <v>17.218</v>
       </c>
       <c r="AD169" t="n">
-        <v>23.425</v>
+        <v>23.3</v>
       </c>
       <c r="AE169" t="n">
-        <v>9.831</v>
+        <v>10.097</v>
       </c>
       <c r="AF169" t="n">
-        <v>28.481</v>
+        <v>28.371</v>
       </c>
       <c r="AG169" t="n">
-        <v>19</v>
+        <v>18.562</v>
       </c>
       <c r="AH169" t="n">
-        <v>5.582</v>
+        <v>5.686</v>
       </c>
       <c r="AI169" t="n">
-        <v>6.195</v>
+        <v>6.053</v>
       </c>
       <c r="AJ169" t="n">
-        <v>15.332</v>
+        <v>15.431</v>
       </c>
       <c r="AK169" t="n">
-        <v>16.4</v>
+        <v>21.6</v>
       </c>
       <c r="AL169" t="n">
-        <v>11.6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="170">
@@ -20906,22 +20906,22 @@
         </is>
       </c>
       <c r="E171" t="n">
-        <v>128</v>
+        <v>149</v>
       </c>
       <c r="F171" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G171" t="b">
         <v>1</v>
       </c>
       <c r="H171" t="n">
-        <v>1613.709</v>
+        <v>1598.564</v>
       </c>
       <c r="I171" t="n">
-        <v>0.3599</v>
+        <v>0.401</v>
       </c>
       <c r="J171" t="n">
-        <v>1670.6</v>
+        <v>1671.6</v>
       </c>
       <c r="K171" t="n">
         <v>77</v>
@@ -20942,70 +20942,70 @@
         <v>81</v>
       </c>
       <c r="Q171" t="n">
-        <v>110.457</v>
+        <v>109.316</v>
       </c>
       <c r="R171" t="n">
-        <v>108.577</v>
+        <v>108.686</v>
       </c>
       <c r="S171" t="n">
-        <v>1.88</v>
+        <v>0.629</v>
       </c>
       <c r="T171" t="n">
-        <v>0.24991</v>
+        <v>0.24699</v>
       </c>
       <c r="U171" t="n">
-        <v>0.15774</v>
+        <v>0.15479</v>
       </c>
       <c r="V171" t="n">
-        <v>70</v>
+        <v>69.15000000000001</v>
       </c>
       <c r="W171" t="n">
-        <v>68.56999999999999</v>
+        <v>68.47</v>
       </c>
       <c r="X171" t="n">
-        <v>0.4637</v>
+        <v>0.45</v>
       </c>
       <c r="Y171" t="n">
-        <v>24.134</v>
+        <v>24.24</v>
       </c>
       <c r="Z171" t="n">
-        <v>52.609</v>
+        <v>52.81</v>
       </c>
       <c r="AA171" t="n">
-        <v>8.640000000000001</v>
+        <v>8.52</v>
       </c>
       <c r="AB171" t="n">
-        <v>24.762</v>
+        <v>24.55</v>
       </c>
       <c r="AC171" t="n">
-        <v>13.298</v>
+        <v>13.06</v>
       </c>
       <c r="AD171" t="n">
-        <v>18.978</v>
+        <v>18.56</v>
       </c>
       <c r="AE171" t="n">
-        <v>7.474</v>
+        <v>7.45</v>
       </c>
       <c r="AF171" t="n">
-        <v>21.442</v>
+        <v>21.81</v>
       </c>
       <c r="AG171" t="n">
-        <v>17.394</v>
+        <v>17.01</v>
       </c>
       <c r="AH171" t="n">
-        <v>6.505</v>
+        <v>6.44</v>
       </c>
       <c r="AI171" t="n">
-        <v>2.754</v>
+        <v>2.77</v>
       </c>
       <c r="AJ171" t="n">
-        <v>14.462</v>
+        <v>14.56</v>
       </c>
       <c r="AK171" t="n">
-        <v>-7.8</v>
+        <v>-9.6</v>
       </c>
       <c r="AL171" t="n">
-        <v>-1.7</v>
+        <v>-3.9</v>
       </c>
     </row>
     <row r="172">
@@ -24146,22 +24146,22 @@
         </is>
       </c>
       <c r="E198" t="n">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F198" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G198" t="b">
         <v>1</v>
       </c>
       <c r="H198" t="n">
-        <v>1819.199</v>
+        <v>1787.285</v>
       </c>
       <c r="I198" t="n">
-        <v>1.8714</v>
+        <v>1.726</v>
       </c>
       <c r="J198" t="n">
-        <v>1594.7</v>
+        <v>1598.1</v>
       </c>
       <c r="K198" t="n">
         <v>50</v>
@@ -24182,70 +24182,70 @@
         <v>46</v>
       </c>
       <c r="Q198" t="n">
-        <v>116.155</v>
+        <v>115.624</v>
       </c>
       <c r="R198" t="n">
-        <v>102.4</v>
+        <v>102.64</v>
       </c>
       <c r="S198" t="n">
-        <v>13.755</v>
+        <v>12.984</v>
       </c>
       <c r="T198" t="n">
-        <v>0.28162</v>
+        <v>0.28239</v>
       </c>
       <c r="U198" t="n">
-        <v>0.1422</v>
+        <v>0.14436</v>
       </c>
       <c r="V198" t="n">
-        <v>81.11</v>
+        <v>80.67</v>
       </c>
       <c r="W198" t="n">
-        <v>71.5</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="X198" t="n">
-        <v>0.7164</v>
+        <v>0.6897</v>
       </c>
       <c r="Y198" t="n">
-        <v>28.057</v>
+        <v>27.917</v>
       </c>
       <c r="Z198" t="n">
-        <v>60.446</v>
+        <v>60.372</v>
       </c>
       <c r="AA198" t="n">
-        <v>9.090999999999999</v>
+        <v>9.214</v>
       </c>
       <c r="AB198" t="n">
-        <v>25.162</v>
+        <v>25.434</v>
       </c>
       <c r="AC198" t="n">
-        <v>15.902</v>
+        <v>15.793</v>
       </c>
       <c r="AD198" t="n">
-        <v>21.846</v>
+        <v>21.669</v>
       </c>
       <c r="AE198" t="n">
-        <v>10.006</v>
+        <v>10.062</v>
       </c>
       <c r="AF198" t="n">
-        <v>25.059</v>
+        <v>25.103</v>
       </c>
       <c r="AG198" t="n">
-        <v>14.787</v>
+        <v>14.876</v>
       </c>
       <c r="AH198" t="n">
-        <v>7.9</v>
+        <v>7.883</v>
       </c>
       <c r="AI198" t="n">
-        <v>2.787</v>
+        <v>2.945</v>
       </c>
       <c r="AJ198" t="n">
-        <v>17.154</v>
+        <v>17.159</v>
       </c>
       <c r="AK198" t="n">
-        <v>15.6</v>
+        <v>11.4</v>
       </c>
       <c r="AL198" t="n">
-        <v>6.6</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="199">
@@ -26546,22 +26546,22 @@
         </is>
       </c>
       <c r="E218" t="n">
-        <v>130</v>
+        <v>152</v>
       </c>
       <c r="F218" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G218" t="b">
         <v>1</v>
       </c>
       <c r="H218" t="n">
-        <v>1722.461</v>
+        <v>1753.558</v>
       </c>
       <c r="I218" t="n">
-        <v>-1.4338</v>
+        <v>-0.8196</v>
       </c>
       <c r="J218" t="n">
-        <v>1675.4</v>
+        <v>1671.3</v>
       </c>
       <c r="K218" t="n">
         <v>40</v>
@@ -26582,70 +26582,70 @@
         <v>48</v>
       </c>
       <c r="Q218" t="n">
-        <v>120.005</v>
+        <v>119.738</v>
       </c>
       <c r="R218" t="n">
-        <v>111.633</v>
+        <v>110.983</v>
       </c>
       <c r="S218" t="n">
-        <v>8.372999999999999</v>
+        <v>8.755000000000001</v>
       </c>
       <c r="T218" t="n">
-        <v>0.30897</v>
+        <v>0.30841</v>
       </c>
       <c r="U218" t="n">
-        <v>0.14018</v>
+        <v>0.14278</v>
       </c>
       <c r="V218" t="n">
-        <v>82.7</v>
+        <v>82.91</v>
       </c>
       <c r="W218" t="n">
-        <v>77.13</v>
+        <v>77.04000000000001</v>
       </c>
       <c r="X218" t="n">
-        <v>0.5536</v>
+        <v>0.5867</v>
       </c>
       <c r="Y218" t="n">
-        <v>28.184</v>
+        <v>27.885</v>
       </c>
       <c r="Z218" t="n">
-        <v>60.221</v>
+        <v>60.237</v>
       </c>
       <c r="AA218" t="n">
-        <v>9.682</v>
+        <v>9.526999999999999</v>
       </c>
       <c r="AB218" t="n">
-        <v>26.402</v>
+        <v>26.529</v>
       </c>
       <c r="AC218" t="n">
-        <v>16.068</v>
+        <v>16.488</v>
       </c>
       <c r="AD218" t="n">
-        <v>21.603</v>
+        <v>22.039</v>
       </c>
       <c r="AE218" t="n">
-        <v>10.213</v>
+        <v>10.328</v>
       </c>
       <c r="AF218" t="n">
-        <v>22.494</v>
+        <v>22.879</v>
       </c>
       <c r="AG218" t="n">
-        <v>14.164</v>
+        <v>13.758</v>
       </c>
       <c r="AH218" t="n">
-        <v>6.205</v>
+        <v>6.185</v>
       </c>
       <c r="AI218" t="n">
-        <v>3.641</v>
+        <v>3.65</v>
       </c>
       <c r="AJ218" t="n">
-        <v>17.534</v>
+        <v>17.626</v>
       </c>
       <c r="AK218" t="n">
-        <v>9.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="AL218" t="n">
-        <v>6.5</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="219">
@@ -29546,22 +29546,22 @@
         </is>
       </c>
       <c r="E243" t="n">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="F243" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G243" t="b">
         <v>1</v>
       </c>
       <c r="H243" t="n">
-        <v>1563.92</v>
+        <v>1552.046</v>
       </c>
       <c r="I243" t="n">
-        <v>-2.5391</v>
+        <v>-2.3595</v>
       </c>
       <c r="J243" t="n">
-        <v>1691.9</v>
+        <v>1688.9</v>
       </c>
       <c r="K243" t="n">
         <v>124</v>
@@ -29582,70 +29582,70 @@
         <v>134</v>
       </c>
       <c r="Q243" t="n">
-        <v>104.259</v>
+        <v>104.103</v>
       </c>
       <c r="R243" t="n">
-        <v>111.496</v>
+        <v>111.635</v>
       </c>
       <c r="S243" t="n">
-        <v>-7.237</v>
+        <v>-7.531</v>
       </c>
       <c r="T243" t="n">
-        <v>0.31226</v>
+        <v>0.3133</v>
       </c>
       <c r="U243" t="n">
-        <v>0.15056</v>
+        <v>0.1485</v>
       </c>
       <c r="V243" t="n">
-        <v>70.44</v>
+        <v>70.51000000000001</v>
       </c>
       <c r="W243" t="n">
-        <v>75.08</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="X243" t="n">
-        <v>0.4193</v>
+        <v>0.4073</v>
       </c>
       <c r="Y243" t="n">
-        <v>24.216</v>
+        <v>24.233</v>
       </c>
       <c r="Z243" t="n">
-        <v>57.76</v>
+        <v>58.047</v>
       </c>
       <c r="AA243" t="n">
-        <v>6.539</v>
+        <v>6.364</v>
       </c>
       <c r="AB243" t="n">
-        <v>19.988</v>
+        <v>19.76</v>
       </c>
       <c r="AC243" t="n">
-        <v>15.319</v>
+        <v>15.538</v>
       </c>
       <c r="AD243" t="n">
-        <v>20.661</v>
+        <v>20.996</v>
       </c>
       <c r="AE243" t="n">
-        <v>9.486000000000001</v>
+        <v>9.615</v>
       </c>
       <c r="AF243" t="n">
-        <v>21.083</v>
+        <v>21.258</v>
       </c>
       <c r="AG243" t="n">
-        <v>12.323</v>
+        <v>12.131</v>
       </c>
       <c r="AH243" t="n">
-        <v>6.078</v>
+        <v>6.047</v>
       </c>
       <c r="AI243" t="n">
-        <v>3.371</v>
+        <v>3.309</v>
       </c>
       <c r="AJ243" t="n">
-        <v>16.76</v>
+        <v>16.807</v>
       </c>
       <c r="AK243" t="n">
-        <v>0.8</v>
+        <v>-2.6</v>
       </c>
       <c r="AL243" t="n">
-        <v>-1</v>
+        <v>-1.1</v>
       </c>
     </row>
     <row r="244">
@@ -33746,22 +33746,22 @@
         </is>
       </c>
       <c r="E278" t="n">
-        <v>127</v>
+        <v>150</v>
       </c>
       <c r="F278" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G278" t="b">
         <v>1</v>
       </c>
       <c r="H278" t="n">
-        <v>1734.155</v>
+        <v>1710.236</v>
       </c>
       <c r="I278" t="n">
-        <v>2.5276</v>
+        <v>2.3442</v>
       </c>
       <c r="J278" t="n">
-        <v>1622.5</v>
+        <v>1626.8</v>
       </c>
       <c r="K278" t="n">
         <v>58</v>
@@ -33782,70 +33782,70 @@
         <v>61</v>
       </c>
       <c r="Q278" t="n">
-        <v>111.896</v>
+        <v>111.763</v>
       </c>
       <c r="R278" t="n">
-        <v>107.42</v>
+        <v>107.68</v>
       </c>
       <c r="S278" t="n">
-        <v>4.476</v>
+        <v>4.083</v>
       </c>
       <c r="T278" t="n">
-        <v>0.3248</v>
+        <v>0.32373</v>
       </c>
       <c r="U278" t="n">
-        <v>0.14394</v>
+        <v>0.14366</v>
       </c>
       <c r="V278" t="n">
-        <v>75.83</v>
+        <v>76.01000000000001</v>
       </c>
       <c r="W278" t="n">
-        <v>72.59</v>
+        <v>73.06</v>
       </c>
       <c r="X278" t="n">
-        <v>0.6183</v>
+        <v>0.6</v>
       </c>
       <c r="Y278" t="n">
-        <v>25.836</v>
+        <v>25.9</v>
       </c>
       <c r="Z278" t="n">
-        <v>59.168</v>
+        <v>59.49</v>
       </c>
       <c r="AA278" t="n">
-        <v>8.997</v>
+        <v>8.94</v>
       </c>
       <c r="AB278" t="n">
-        <v>25.718</v>
+        <v>25.86</v>
       </c>
       <c r="AC278" t="n">
-        <v>15.202</v>
+        <v>15.3</v>
       </c>
       <c r="AD278" t="n">
-        <v>20.902</v>
+        <v>20.99</v>
       </c>
       <c r="AE278" t="n">
-        <v>10.448</v>
+        <v>10.57</v>
       </c>
       <c r="AF278" t="n">
-        <v>21.309</v>
+        <v>21.7</v>
       </c>
       <c r="AG278" t="n">
-        <v>11.875</v>
+        <v>11.79</v>
       </c>
       <c r="AH278" t="n">
-        <v>7.927</v>
+        <v>7.78</v>
       </c>
       <c r="AI278" t="n">
-        <v>3.598</v>
+        <v>3.77</v>
       </c>
       <c r="AJ278" t="n">
-        <v>17.492</v>
+        <v>17.58</v>
       </c>
       <c r="AK278" t="n">
-        <v>7.2</v>
+        <v>4.6</v>
       </c>
       <c r="AL278" t="n">
-        <v>5.2</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="279">
@@ -36026,22 +36026,22 @@
         </is>
       </c>
       <c r="E297" t="n">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F297" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G297" t="b">
         <v>1</v>
       </c>
       <c r="H297" t="n">
-        <v>1706.594</v>
+        <v>1738.508</v>
       </c>
       <c r="I297" t="n">
-        <v>7.505</v>
+        <v>7.3202</v>
       </c>
       <c r="J297" t="n">
-        <v>1519.9</v>
+        <v>1529.3</v>
       </c>
       <c r="K297" t="n">
         <v>63</v>
@@ -36062,67 +36062,67 @@
         <v>52</v>
       </c>
       <c r="Q297" t="n">
-        <v>120.722</v>
+        <v>120.157</v>
       </c>
       <c r="R297" t="n">
-        <v>106.301</v>
+        <v>105.937</v>
       </c>
       <c r="S297" t="n">
-        <v>14.421</v>
+        <v>14.22</v>
       </c>
       <c r="T297" t="n">
-        <v>0.28201</v>
+        <v>0.28533</v>
       </c>
       <c r="U297" t="n">
-        <v>0.14993</v>
+        <v>0.14972</v>
       </c>
       <c r="V297" t="n">
-        <v>84.17</v>
+        <v>83.83</v>
       </c>
       <c r="W297" t="n">
-        <v>74.18000000000001</v>
+        <v>73.97</v>
       </c>
       <c r="X297" t="n">
-        <v>0.7955</v>
+        <v>0.8012</v>
       </c>
       <c r="Y297" t="n">
-        <v>27.308</v>
+        <v>27.209</v>
       </c>
       <c r="Z297" t="n">
-        <v>58.601</v>
+        <v>58.884</v>
       </c>
       <c r="AA297" t="n">
-        <v>10.627</v>
+        <v>10.493</v>
       </c>
       <c r="AB297" t="n">
-        <v>27.276</v>
+        <v>27.462</v>
       </c>
       <c r="AC297" t="n">
-        <v>18.925</v>
+        <v>18.742</v>
       </c>
       <c r="AD297" t="n">
-        <v>24.234</v>
+        <v>24.02</v>
       </c>
       <c r="AE297" t="n">
-        <v>9.948</v>
+        <v>10.081</v>
       </c>
       <c r="AF297" t="n">
-        <v>24.698</v>
+        <v>24.619</v>
       </c>
       <c r="AG297" t="n">
-        <v>15.156</v>
+        <v>15.101</v>
       </c>
       <c r="AH297" t="n">
-        <v>6.562</v>
+        <v>6.609</v>
       </c>
       <c r="AI297" t="n">
-        <v>2.292</v>
+        <v>2.215</v>
       </c>
       <c r="AJ297" t="n">
-        <v>16.308</v>
+        <v>16.29</v>
       </c>
       <c r="AK297" t="n">
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
       <c r="AL297" t="n">
         <v>10.7</v>
@@ -40826,22 +40826,22 @@
         </is>
       </c>
       <c r="E337" t="n">
-        <v>128</v>
+        <v>152</v>
       </c>
       <c r="F337" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G337" t="b">
         <v>1</v>
       </c>
       <c r="H337" t="n">
-        <v>1703.642</v>
+        <v>1745.5</v>
       </c>
       <c r="I337" t="n">
-        <v>0.6918</v>
+        <v>1.0412</v>
       </c>
       <c r="J337" t="n">
-        <v>1669</v>
+        <v>1668.5</v>
       </c>
       <c r="K337" t="n">
         <v>59</v>
@@ -40862,70 +40862,70 @@
         <v>59</v>
       </c>
       <c r="Q337" t="n">
-        <v>106.362</v>
+        <v>107.709</v>
       </c>
       <c r="R337" t="n">
-        <v>99.998</v>
+        <v>100.214</v>
       </c>
       <c r="S337" t="n">
-        <v>6.364</v>
+        <v>7.495</v>
       </c>
       <c r="T337" t="n">
-        <v>0.29519</v>
+        <v>0.28466</v>
       </c>
       <c r="U337" t="n">
-        <v>0.16549</v>
+        <v>0.16026</v>
       </c>
       <c r="V337" t="n">
-        <v>68.95999999999999</v>
+        <v>70.25</v>
       </c>
       <c r="W337" t="n">
-        <v>64.78</v>
+        <v>65.31</v>
       </c>
       <c r="X337" t="n">
-        <v>0.5565</v>
+        <v>0.5921</v>
       </c>
       <c r="Y337" t="n">
-        <v>24.569</v>
+        <v>24.603</v>
       </c>
       <c r="Z337" t="n">
-        <v>55.435</v>
+        <v>55.564</v>
       </c>
       <c r="AA337" t="n">
-        <v>7.731</v>
+        <v>7.515</v>
       </c>
       <c r="AB337" t="n">
-        <v>23.441</v>
+        <v>23.456</v>
       </c>
       <c r="AC337" t="n">
-        <v>12.925</v>
+        <v>13.455</v>
       </c>
       <c r="AD337" t="n">
-        <v>19.089</v>
+        <v>19.533</v>
       </c>
       <c r="AE337" t="n">
-        <v>9.724</v>
+        <v>9.381</v>
       </c>
       <c r="AF337" t="n">
-        <v>22.648</v>
+        <v>22.97</v>
       </c>
       <c r="AG337" t="n">
-        <v>12.864</v>
+        <v>12.709</v>
       </c>
       <c r="AH337" t="n">
-        <v>6.496</v>
+        <v>6.283</v>
       </c>
       <c r="AI337" t="n">
-        <v>2.949</v>
+        <v>3</v>
       </c>
       <c r="AJ337" t="n">
-        <v>15.402</v>
+        <v>15.263</v>
       </c>
       <c r="AK337" t="n">
-        <v>-1.2</v>
+        <v>3</v>
       </c>
       <c r="AL337" t="n">
-        <v>-1.2</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="338">

</xml_diff>

<commit_message>
Update team snapshot (2026-04-10)
</commit_message>
<xml_diff>
--- a/team_snapshot_2026.xlsx
+++ b/team_snapshot_2026.xlsx
@@ -8302,22 +8302,22 @@
         <v>417</v>
       </c>
       <c r="E58">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F58">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G58" t="b">
         <v>1</v>
       </c>
       <c r="H58">
-        <v>2148.21</v>
+        <v>2128.609</v>
       </c>
       <c r="I58">
-        <v>5.461</v>
+        <v>5.4518</v>
       </c>
       <c r="J58">
-        <v>1679.5</v>
+        <v>1685.2</v>
       </c>
       <c r="K58">
         <v>9</v>
@@ -8338,70 +8338,70 @@
         <v>9</v>
       </c>
       <c r="Q58">
-        <v>116.328</v>
+        <v>115.797</v>
       </c>
       <c r="R58">
-        <v>98.54600000000001</v>
+        <v>98.839</v>
       </c>
       <c r="S58">
-        <v>17.783</v>
+        <v>16.958</v>
       </c>
       <c r="T58">
-        <v>0.29918</v>
+        <v>0.30497</v>
       </c>
       <c r="U58">
-        <v>0.15954</v>
+        <v>0.16056</v>
       </c>
       <c r="V58">
-        <v>76.91</v>
+        <v>76.51000000000001</v>
       </c>
       <c r="W58">
-        <v>65.08</v>
+        <v>65.22</v>
       </c>
       <c r="X58">
-        <v>0.8727</v>
+        <v>0.8446</v>
       </c>
       <c r="Y58">
-        <v>27.857</v>
+        <v>27.682</v>
       </c>
       <c r="Z58">
-        <v>58.231</v>
+        <v>58.511</v>
       </c>
       <c r="AA58">
-        <v>8.307</v>
+        <v>8.304</v>
       </c>
       <c r="AB58">
-        <v>23.705</v>
+        <v>23.933</v>
       </c>
       <c r="AC58">
-        <v>12.861</v>
+        <v>12.82</v>
       </c>
       <c r="AD58">
-        <v>17.739</v>
+        <v>17.689</v>
       </c>
       <c r="AE58">
-        <v>10.484</v>
+        <v>10.847</v>
       </c>
       <c r="AF58">
-        <v>24.122</v>
+        <v>24.099</v>
       </c>
       <c r="AG58">
-        <v>18.278</v>
+        <v>18.017</v>
       </c>
       <c r="AH58">
-        <v>6.815</v>
+        <v>6.732</v>
       </c>
       <c r="AI58">
-        <v>5.049</v>
+        <v>4.981</v>
       </c>
       <c r="AJ58">
-        <v>18.148</v>
+        <v>18.249</v>
       </c>
       <c r="AK58">
-        <v>8.199999999999999</v>
+        <v>4.8</v>
       </c>
       <c r="AL58">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="59" spans="1:38">
@@ -8427,7 +8427,7 @@
         <v>1</v>
       </c>
       <c r="H59">
-        <v>1180.884</v>
+        <v>1183.618</v>
       </c>
       <c r="I59">
         <v>-2.2819</v>
@@ -21178,22 +21178,22 @@
         <v>433</v>
       </c>
       <c r="E169">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F169">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G169" t="b">
         <v>1</v>
       </c>
       <c r="H169">
-        <v>2238.177</v>
+        <v>2257.778</v>
       </c>
       <c r="I169">
-        <v>5.3046</v>
+        <v>5.2983</v>
       </c>
       <c r="J169">
-        <v>1794.5</v>
+        <v>1789.5</v>
       </c>
       <c r="K169">
         <v>1</v>
@@ -21214,70 +21214,70 @@
         <v>1</v>
       </c>
       <c r="Q169">
-        <v>122.018</v>
+        <v>121.54</v>
       </c>
       <c r="R169">
-        <v>97.477</v>
+        <v>97.458</v>
       </c>
       <c r="S169">
-        <v>24.541</v>
+        <v>24.082</v>
       </c>
       <c r="T169">
-        <v>0.25976</v>
+        <v>0.26038</v>
       </c>
       <c r="U169">
-        <v>0.16002</v>
+        <v>0.15968</v>
       </c>
       <c r="V169">
-        <v>87.81</v>
+        <v>87.23</v>
       </c>
       <c r="W169">
-        <v>69.69</v>
+        <v>69.45999999999999</v>
       </c>
       <c r="X169">
-        <v>0.9235</v>
+        <v>0.9254</v>
       </c>
       <c r="Y169">
-        <v>30.563</v>
+        <v>30.299</v>
       </c>
       <c r="Z169">
-        <v>60.267</v>
+        <v>60.047</v>
       </c>
       <c r="AA169">
-        <v>9.109999999999999</v>
+        <v>8.912000000000001</v>
       </c>
       <c r="AB169">
-        <v>24.648</v>
+        <v>24.399</v>
       </c>
       <c r="AC169">
-        <v>17.218</v>
+        <v>17.466</v>
       </c>
       <c r="AD169">
-        <v>23.3</v>
+        <v>23.45</v>
       </c>
       <c r="AE169">
-        <v>10.097</v>
+        <v>10.11</v>
       </c>
       <c r="AF169">
-        <v>28.371</v>
+        <v>28.343</v>
       </c>
       <c r="AG169">
-        <v>18.562</v>
+        <v>18.288</v>
       </c>
       <c r="AH169">
-        <v>5.686</v>
+        <v>5.677</v>
       </c>
       <c r="AI169">
-        <v>6.053</v>
+        <v>6.075</v>
       </c>
       <c r="AJ169">
-        <v>15.431</v>
+        <v>15.337</v>
       </c>
       <c r="AK169">
-        <v>21.6</v>
+        <v>18.6</v>
       </c>
       <c r="AL169">
-        <v>12</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="170" spans="1:38">
@@ -22573,19 +22573,19 @@
         <v>128</v>
       </c>
       <c r="F181">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G181" t="b">
         <v>1</v>
       </c>
       <c r="H181">
-        <v>1266.451</v>
+        <v>1271.112</v>
       </c>
       <c r="I181">
         <v>-0.0021</v>
       </c>
       <c r="J181">
-        <v>1356.2</v>
+        <v>1356.5</v>
       </c>
       <c r="K181">
         <v>353</v>
@@ -22606,64 +22606,64 @@
         <v>352</v>
       </c>
       <c r="Q181">
-        <v>99.72799999999999</v>
+        <v>99.742</v>
       </c>
       <c r="R181">
-        <v>111.487</v>
+        <v>111.513</v>
       </c>
       <c r="S181">
-        <v>-11.758</v>
+        <v>-11.771</v>
       </c>
       <c r="T181">
-        <v>0.29397</v>
+        <v>0.29399</v>
       </c>
       <c r="U181">
-        <v>0.17056</v>
+        <v>0.17059</v>
       </c>
       <c r="V181">
         <v>71.72</v>
       </c>
       <c r="W181">
-        <v>80.01000000000001</v>
+        <v>80.02</v>
       </c>
       <c r="X181">
-        <v>0.4019</v>
+        <v>0.4029</v>
       </c>
       <c r="Y181">
-        <v>23.662</v>
+        <v>23.656</v>
       </c>
       <c r="Z181">
-        <v>58.187</v>
+        <v>58.179</v>
       </c>
       <c r="AA181">
-        <v>6.335</v>
+        <v>6.348</v>
       </c>
       <c r="AB181">
-        <v>19.902</v>
+        <v>19.927</v>
       </c>
       <c r="AC181">
-        <v>18.31</v>
+        <v>18.3</v>
       </c>
       <c r="AD181">
-        <v>24.665</v>
+        <v>24.652</v>
       </c>
       <c r="AE181">
-        <v>9.333</v>
+        <v>9.326000000000001</v>
       </c>
       <c r="AF181">
-        <v>21.523</v>
+        <v>21.502</v>
       </c>
       <c r="AG181">
-        <v>12.265</v>
+        <v>12.271</v>
       </c>
       <c r="AH181">
-        <v>4.329</v>
+        <v>4.33</v>
       </c>
       <c r="AI181">
-        <v>3.342</v>
+        <v>3.341</v>
       </c>
       <c r="AJ181">
-        <v>21.575</v>
+        <v>21.571</v>
       </c>
       <c r="AK181">
         <v>-2.6</v>
@@ -22689,7 +22689,7 @@
         <v>126</v>
       </c>
       <c r="F182">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G182" t="b">
         <v>1</v>
@@ -22701,7 +22701,7 @@
         <v>-2.8469</v>
       </c>
       <c r="J182">
-        <v>1371.1</v>
+        <v>1371.2</v>
       </c>
       <c r="K182">
         <v>365</v>
@@ -22722,64 +22722,64 @@
         <v>365</v>
       </c>
       <c r="Q182">
-        <v>90.483</v>
+        <v>90.5</v>
       </c>
       <c r="R182">
         <v>119.095</v>
       </c>
       <c r="S182">
-        <v>-28.613</v>
+        <v>-28.595</v>
       </c>
       <c r="T182">
-        <v>0.291</v>
+        <v>0.29086</v>
       </c>
       <c r="U182">
-        <v>0.2104</v>
+        <v>0.21028</v>
       </c>
       <c r="V182">
-        <v>63.1</v>
+        <v>63.12</v>
       </c>
       <c r="W182">
-        <v>83.62</v>
+        <v>83.63</v>
       </c>
       <c r="X182">
-        <v>0.0618</v>
+        <v>0.0619</v>
       </c>
       <c r="Y182">
-        <v>22.421</v>
+        <v>22.428</v>
       </c>
       <c r="Z182">
-        <v>55.122</v>
+        <v>55.128</v>
       </c>
       <c r="AA182">
         <v>4.907</v>
       </c>
       <c r="AB182">
-        <v>16.638</v>
+        <v>16.641</v>
       </c>
       <c r="AC182">
-        <v>13.349</v>
+        <v>13.354</v>
       </c>
       <c r="AD182">
-        <v>18.669</v>
+        <v>18.672</v>
       </c>
       <c r="AE182">
-        <v>8.177</v>
+        <v>8.169</v>
       </c>
       <c r="AF182">
-        <v>19.743</v>
+        <v>19.739</v>
       </c>
       <c r="AG182">
-        <v>11.898</v>
+        <v>11.894</v>
       </c>
       <c r="AH182">
-        <v>7.094</v>
+        <v>7.089</v>
       </c>
       <c r="AI182">
-        <v>2.567</v>
+        <v>2.566</v>
       </c>
       <c r="AJ182">
-        <v>21.503</v>
+        <v>21.512</v>
       </c>
       <c r="AK182">
         <v>-11.2</v>
@@ -24893,7 +24893,7 @@
         <v>118</v>
       </c>
       <c r="F201">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G201" t="b">
         <v>1</v>
@@ -24905,7 +24905,7 @@
         <v>-3.5334</v>
       </c>
       <c r="J201">
-        <v>1425.9</v>
+        <v>1425.7</v>
       </c>
       <c r="K201">
         <v>337</v>
@@ -24926,64 +24926,64 @@
         <v>340</v>
       </c>
       <c r="Q201">
-        <v>100.711</v>
+        <v>100.691</v>
       </c>
       <c r="R201">
-        <v>113.555</v>
+        <v>113.538</v>
       </c>
       <c r="S201">
-        <v>-12.844</v>
+        <v>-12.847</v>
       </c>
       <c r="T201">
-        <v>0.25156</v>
+        <v>0.25146</v>
       </c>
       <c r="U201">
-        <v>0.17493</v>
+        <v>0.17473</v>
       </c>
       <c r="V201">
         <v>63.31</v>
       </c>
       <c r="W201">
-        <v>71.70999999999999</v>
+        <v>71.7</v>
       </c>
       <c r="X201">
-        <v>0.2381</v>
+        <v>0.2386</v>
       </c>
       <c r="Y201">
-        <v>22.973</v>
+        <v>22.977</v>
       </c>
       <c r="Z201">
-        <v>52.537</v>
+        <v>52.557</v>
       </c>
       <c r="AA201">
         <v>7.17</v>
       </c>
       <c r="AB201">
-        <v>21.265</v>
+        <v>21.273</v>
       </c>
       <c r="AC201">
-        <v>10.197</v>
+        <v>10.182</v>
       </c>
       <c r="AD201">
-        <v>14.068</v>
+        <v>14.057</v>
       </c>
       <c r="AE201">
-        <v>6.639</v>
+        <v>6.636</v>
       </c>
       <c r="AF201">
-        <v>19.986</v>
+        <v>19.989</v>
       </c>
       <c r="AG201">
-        <v>13.796</v>
+        <v>13.795</v>
       </c>
       <c r="AH201">
-        <v>5.619</v>
+        <v>5.614</v>
       </c>
       <c r="AI201">
         <v>2.83</v>
       </c>
       <c r="AJ201">
-        <v>15.388</v>
+        <v>15.386</v>
       </c>
       <c r="AK201">
         <v>-4.2</v>
@@ -33129,7 +33129,7 @@
         <v>117</v>
       </c>
       <c r="F272">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G272" t="b">
         <v>1</v>
@@ -33141,7 +33141,7 @@
         <v>-1.7292</v>
       </c>
       <c r="J272">
-        <v>1423.6</v>
+        <v>1423.5</v>
       </c>
       <c r="K272">
         <v>354</v>
@@ -33162,64 +33162,64 @@
         <v>353</v>
       </c>
       <c r="Q272">
-        <v>99.95999999999999</v>
+        <v>99.96299999999999</v>
       </c>
       <c r="R272">
-        <v>117.777</v>
+        <v>117.803</v>
       </c>
       <c r="S272">
-        <v>-17.817</v>
+        <v>-17.84</v>
       </c>
       <c r="T272">
-        <v>0.2987</v>
+        <v>0.29857</v>
       </c>
       <c r="U272">
-        <v>0.17427</v>
+        <v>0.17422</v>
       </c>
       <c r="V272">
-        <v>69.95</v>
+        <v>69.97</v>
       </c>
       <c r="W272">
-        <v>82.88</v>
+        <v>82.91</v>
       </c>
       <c r="X272">
-        <v>0.1701</v>
+        <v>0.1705</v>
       </c>
       <c r="Y272">
-        <v>24.918</v>
+        <v>24.92</v>
       </c>
       <c r="Z272">
-        <v>58.639</v>
+        <v>58.648</v>
       </c>
       <c r="AA272">
-        <v>7.524</v>
+        <v>7.534</v>
       </c>
       <c r="AB272">
-        <v>22.088</v>
+        <v>22.102</v>
       </c>
       <c r="AC272">
-        <v>12.592</v>
+        <v>12.591</v>
       </c>
       <c r="AD272">
         <v>18.102</v>
       </c>
       <c r="AE272">
-        <v>8.755000000000001</v>
+        <v>8.75</v>
       </c>
       <c r="AF272">
         <v>19.932</v>
       </c>
       <c r="AG272">
-        <v>12.81</v>
+        <v>12.818</v>
       </c>
       <c r="AH272">
-        <v>7.395</v>
+        <v>7.398</v>
       </c>
       <c r="AI272">
-        <v>1.66</v>
+        <v>1.659</v>
       </c>
       <c r="AJ272">
-        <v>18.619</v>
+        <v>18.625</v>
       </c>
       <c r="AK272">
         <v>-7.2</v>
@@ -34521,7 +34521,7 @@
         <v>128</v>
       </c>
       <c r="F284">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G284" t="b">
         <v>1</v>
@@ -34533,7 +34533,7 @@
         <v>-1.7447</v>
       </c>
       <c r="J284">
-        <v>1501.2</v>
+        <v>1501.1</v>
       </c>
       <c r="K284">
         <v>159</v>
@@ -34554,64 +34554,64 @@
         <v>167</v>
       </c>
       <c r="Q284">
-        <v>110.657</v>
+        <v>110.701</v>
       </c>
       <c r="R284">
-        <v>108.259</v>
+        <v>108.286</v>
       </c>
       <c r="S284">
-        <v>2.398</v>
+        <v>2.415</v>
       </c>
       <c r="T284">
-        <v>0.27641</v>
+        <v>0.27617</v>
       </c>
       <c r="U284">
-        <v>0.13004</v>
+        <v>0.13</v>
       </c>
       <c r="V284">
-        <v>72.81</v>
+        <v>72.84</v>
       </c>
       <c r="W284">
-        <v>71.08</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="X284">
-        <v>0.4773</v>
+        <v>0.4783</v>
       </c>
       <c r="Y284">
-        <v>24.655</v>
+        <v>24.658</v>
       </c>
       <c r="Z284">
-        <v>55.927</v>
+        <v>55.919</v>
       </c>
       <c r="AA284">
-        <v>6.645</v>
+        <v>6.655</v>
       </c>
       <c r="AB284">
-        <v>19.818</v>
+        <v>19.841</v>
       </c>
       <c r="AC284">
-        <v>16.855</v>
+        <v>16.867</v>
       </c>
       <c r="AD284">
-        <v>22.586</v>
+        <v>22.6</v>
       </c>
       <c r="AE284">
-        <v>8.550000000000001</v>
+        <v>8.545</v>
       </c>
       <c r="AF284">
-        <v>21.964</v>
+        <v>21.974</v>
       </c>
       <c r="AG284">
-        <v>11.795</v>
+        <v>11.812</v>
       </c>
       <c r="AH284">
-        <v>5.745</v>
+        <v>5.73</v>
       </c>
       <c r="AI284">
-        <v>3.973</v>
+        <v>3.977</v>
       </c>
       <c r="AJ284">
-        <v>17.268</v>
+        <v>17.281</v>
       </c>
       <c r="AK284">
         <v>2.6</v>
@@ -42757,7 +42757,7 @@
         <v>128</v>
       </c>
       <c r="F355">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G355" t="b">
         <v>1</v>
@@ -42769,7 +42769,7 @@
         <v>-1.08</v>
       </c>
       <c r="J355">
-        <v>1467.7</v>
+        <v>1467.9</v>
       </c>
       <c r="K355">
         <v>220</v>
@@ -42790,64 +42790,64 @@
         <v>230</v>
       </c>
       <c r="Q355">
-        <v>100.944</v>
+        <v>100.938</v>
       </c>
       <c r="R355">
-        <v>105.941</v>
+        <v>105.928</v>
       </c>
       <c r="S355">
-        <v>-4.997</v>
+        <v>-4.99</v>
       </c>
       <c r="T355">
-        <v>0.32108</v>
+        <v>0.32105</v>
       </c>
       <c r="U355">
-        <v>0.19124</v>
+        <v>0.19129</v>
       </c>
       <c r="V355">
-        <v>72.55</v>
+        <v>72.53</v>
       </c>
       <c r="W355">
-        <v>75.87</v>
+        <v>75.84999999999999</v>
       </c>
       <c r="X355">
-        <v>0.3519</v>
+        <v>0.3527</v>
       </c>
       <c r="Y355">
-        <v>25.161</v>
+        <v>25.164</v>
       </c>
       <c r="Z355">
-        <v>56.769</v>
+        <v>56.765</v>
       </c>
       <c r="AA355">
-        <v>4.472</v>
+        <v>4.471</v>
       </c>
       <c r="AB355">
-        <v>13.739</v>
+        <v>13.741</v>
       </c>
       <c r="AC355">
-        <v>17.752</v>
+        <v>17.734</v>
       </c>
       <c r="AD355">
-        <v>23.952</v>
+        <v>23.924</v>
       </c>
       <c r="AE355">
-        <v>9.311</v>
+        <v>9.307</v>
       </c>
       <c r="AF355">
-        <v>19.502</v>
+        <v>19.496</v>
       </c>
       <c r="AG355">
-        <v>10.478</v>
+        <v>10.481</v>
       </c>
       <c r="AH355">
-        <v>9.704000000000001</v>
+        <v>9.705</v>
       </c>
       <c r="AI355">
-        <v>3.07</v>
+        <v>3.071</v>
       </c>
       <c r="AJ355">
-        <v>20.635</v>
+        <v>20.607</v>
       </c>
       <c r="AK355">
         <v>-8.199999999999999</v>

</xml_diff>